<commit_message>
blank related hadith removed
</commit_message>
<xml_diff>
--- a/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_TARGIB WATTAHRIB.xlsx
+++ b/SINGLE HADITH CONTENT/BOOK WISE FINAL UPDATED CONTENT/BN/BN_TARGIB WATTAHRIB.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1021,19 +1021,15 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>121</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম গোপন করার ভয়াবহ সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. জিজ্ঞাসিত ইলম জানা সত্ত্বেও গোপন করলে কিয়ামতের দিনে আগুনের লাগামের কঠিন সতর্কতা এসেছে।"},"heading":{"title":"ইলম গোপন করা: জিজ্ঞাসিত জ্ঞান লুকানোর ভয়াবহ পরিণতি","description":"কোর টপিক: ইলম প্রচার। এই হাদিসে বলা হয়েছে, কাউকে যদি কোনো বিষয়ে ইলম সম্পর্কে জিজ্ঞাসা করা হয়, আর সে তা গোপন রাখে, তবে কিয়ামতের দিনে তার মুখে আগুনের লাগাম পরানো হবে। ইবনে মাজাহর আরেক বর্ণনায়ও একই অর্থ এসেছে—যে জ্ঞান রাখে অথচ গোপন করে, সে আগুনের লাগাম পরানো অবস্থায় উপস্থিত হবে। এখানে জ্ঞান গোপন করার বিপদ বোঝানো হয়েছে। তবে কথা বলার আগে জানা জরুরি যে মানুষ সত্যিই জানে কি না। যে জানে না, তার জন্য না জানা স্বীকার করা নিরাপদ। কিন্তু যে জানে, আর প্রয়োজনের সময় মানুষকে উপকারী ইলম জানায় না, তার জন্য হাদিসে কঠিন সতর্কতা এসেছে।"},"teachings":["জানা ইলম প্রয়োজনের সময় গোপন করা বিপজ্জনক।","যে জানে না, তার উচিত না জানা স্বীকার করা।","উপকারী জ্ঞান মানুষের কাছে পৌঁছানো দায়িত্বের অংশ।","ইলমের সাথে আমানতদারির সম্পর্ক আছে।"],"related_hadiths":[]}</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[0]: unknown book label "রিয়াদুস সালেহিন ১৩৯৮"; related_hadiths[1]: unknown book label "হাদিস সম্ভার ১৫৬৮ (প্রাসঙ্গিক বর্ণনা)"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম গোপন করার ভয়াবহ পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম জানার পর তা গোপন রাখা কঠিন জবাবদিহির কারণ; হাদিসটি জ্ঞান প্রচারের দায়িত্ব স্মরণ করায়।"},"heading":{"title":"ইলম গোপন করার শাস্তি: জ্ঞান প্রচারের দায়িত্ব","description":"এই হাদিসে ইলম গোপন করার বিষয়ে কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি এলেম গোপন করে রাখবে, কিয়ামতের দিন আল্লাহ তাকে আগুনের লাগাম পরাবেন। তাই ইসলামী জ্ঞান শুধু নিজের কাছে রেখে দেওয়ার বিষয় নয়। কেউ যদি এমন জ্ঞান জানে যা মানুষের উপকারে আসতে পারে, তাহলে তা যথাযথভাবে পৌঁছে দেওয়া তার দায়িত্ব। এখানে মূল শিক্ষা হলো—দ্বীনি জ্ঞান আমানত। এই আমানতকে অহংকার, ভয়, স্বার্থ বা অবহেলার কারণে লুকিয়ে রাখা উচিত নয়। তবে জ্ঞান প্রচার করতে হবে সততা, বুঝে বলা এবং দায়িত্ববোধের সঙ্গে।"},"teachings":["দ্বীনি ইলম মানুষের কাছে পৌঁছে দেওয়া একটি গুরুত্বপূর্ণ দায়িত্ব।","উপকারী জ্ঞান জেনেও গোপন রাখা কিয়ামতের জবাবদিহির কারণ হতে পারে।","জ্ঞানকে ব্যক্তিগত সম্পদ না ভেবে আমানত হিসেবে দেখা উচিত।","ইলম প্রচারে সততা ও দায়িত্ববোধ থাকা দরকার।"],"related_hadiths":[{"id":"3658","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2649","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"261","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1048,12 +1044,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>122</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম গোপন করার ভয়াবহ পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম জানার পর তা গোপন রাখা কঠিন জবাবদিহির কারণ; হাদিসটি জ্ঞান প্রচারের দায়িত্ব স্মরণ করায়।"},"heading":{"title":"ইলম গোপন করার শাস্তি: জ্ঞান প্রচারের দায়িত্ব","description":"এই হাদিসে ইলম গোপন করার বিষয়ে কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি এলেম গোপন করে রাখবে, কিয়ামতের দিন আল্লাহ তাকে আগুনের লাগাম পরাবেন। তাই ইসলামী জ্ঞান শুধু নিজের কাছে রেখে দেওয়ার বিষয় নয়। কেউ যদি এমন জ্ঞান জানে যা মানুষের উপকারে আসতে পারে, তাহলে তা যথাযথভাবে পৌঁছে দেওয়া তার দায়িত্ব। এখানে মূল শিক্ষা হলো—দ্বীনি জ্ঞান আমানত। এই আমানতকে অহংকার, ভয়, স্বার্থ বা অবহেলার কারণে লুকিয়ে রাখা উচিত নয়। তবে জ্ঞান প্রচার করতে হবে সততা, বুঝে বলা এবং দায়িত্ববোধের সঙ্গে।"},"teachings":["দ্বীনি ইলম মানুষের কাছে পৌঁছে দেওয়া একটি গুরুত্বপূর্ণ দায়িত্ব।","উপকারী জ্ঞান জেনেও গোপন রাখা কিয়ামতের জবাবদিহির কারণ হতে পারে।","জ্ঞানকে ব্যক্তিগত সম্পদ না ভেবে আমানত হিসেবে দেখা উচিত।","ইলম প্রচারে সততা ও দায়িত্ববোধ থাকা দরকার।"],"related_hadiths":[{"id":"3658","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2649","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"261","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান শিখে আলোচনা না করার ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদ্যা শিখে তা না বলা গচ্ছিত ধন ব্যয় না করার মতো; হাদিসটি জ্ঞান ভাগ করার শিক্ষা দেয়।"},"heading":{"title":"বিদ্যা শিখে না বলা: গচ্ছিত সম্পদের মতো অপচয়","description":"এই হাদিসে জ্ঞান শিখে তা আলোচনা না করার একটি সহজ উপমা দেওয়া হয়েছে। যে ব্যক্তি বিদ্যা শিক্ষা করে, কিন্তু তা মানুষের কাছে বলে না বা উপকারীভাবে আলোচনা করে না, তার উদাহরণ সেই ব্যক্তির মতো, যে সম্পদ জমিয়ে রাখে কিন্তু তা থেকে খরচ করে না। এখানে মূল বিষয় হলো—উপকারী ইলম আটকে রাখলে তার লাভ কমে যায়। জ্ঞান তখনই বেশি উপকারী হয়, যখন তা নিজের আমলের সঙ্গে যুক্ত হয় এবং অন্যদেরও উপকারে আসে। হাদিসটি আমাদের শেখায়, দ্বীনি বিদ্যা কেবল জানার জন্য নয়; তা শেখানো, আলোচনা করা ও মানুষের কল্যাণে ব্যবহার করার জন্যও।"},"teachings":["শেখা জ্ঞান উপকারীভাবে আলোচনা করা উচিত।","ইলমকে গচ্ছিত সম্পদের মতো আটকে রাখা ঠিক নয়।","জ্ঞান নিজের আমল ও অন্যের উপকার—দুই দিকেই কাজে লাগানো দরকার।","বিদ্যা শেখার পর দায়িত্ব আরও বেড়ে যায়।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E25" s="4" t="n"/>
@@ -1071,12 +1067,12 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>123</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান শিখে আলোচনা না করার ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদ্যা শিখে তা না বলা গচ্ছিত ধন ব্যয় না করার মতো; হাদিসটি জ্ঞান ভাগ করার শিক্ষা দেয়।"},"heading":{"title":"বিদ্যা শিখে না বলা: গচ্ছিত সম্পদের মতো অপচয়","description":"এই হাদিসে জ্ঞান শিখে তা আলোচনা না করার একটি সহজ উপমা দেওয়া হয়েছে। যে ব্যক্তি বিদ্যা শিক্ষা করে, কিন্তু তা মানুষের কাছে বলে না বা উপকারীভাবে আলোচনা করে না, তার উদাহরণ সেই ব্যক্তির মতো, যে সম্পদ জমিয়ে রাখে কিন্তু তা থেকে খরচ করে না। এখানে মূল বিষয় হলো—উপকারী ইলম আটকে রাখলে তার লাভ কমে যায়। জ্ঞান তখনই বেশি উপকারী হয়, যখন তা নিজের আমলের সঙ্গে যুক্ত হয় এবং অন্যদেরও উপকারে আসে। হাদিসটি আমাদের শেখায়, দ্বীনি বিদ্যা কেবল জানার জন্য নয়; তা শেখানো, আলোচনা করা ও মানুষের কল্যাণে ব্যবহার করার জন্যও।"},"teachings":["শেখা জ্ঞান উপকারীভাবে আলোচনা করা উচিত।","ইলমকে গচ্ছিত সম্পদের মতো আটকে রাখা ঠিক নয়।","জ্ঞান নিজের আমল ও অন্যের উপকার—দুই দিকেই কাজে লাগানো দরকার।","বিদ্যা শেখার পর দায়িত্ব আরও বেড়ে যায়।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উপকারী ইলমের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি উপকারহীন বিদ্যা, ভীতিহীন অন্তর, অতৃপ্ত আত্মা ও কবুল না হওয়া দোয়া থেকে আশ্রয় চাইতেন।"},"heading":{"title":"উপকারী ইলমের দোয়া ও অন্তরের ভয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর একটি গুরুত্বপূর্ণ দোয়া এসেছে। তিনি আল্লাহর কাছে আশ্রয় চাইতেন এমন বিদ্যা থেকে যা উপকারে আসে না, এমন অন্তর থেকে যা ভীত হয় না, এমন আত্মা থেকে যা পরিতৃপ্ত হয় না এবং এমন দোয়া থেকে যা কবুল হয় না। এখানে উপকারী ইলমের গুরুত্ব খুব স্পষ্ট। শুধু জানা যথেষ্ট নয়; সেই জ্ঞান যেন অন্তরকে নরম করে, আমলে প্রভাব ফেলে এবং মানুষকে আল্লাহর দিকে নিয়ে যায়—এটাই কাম্য। একই সঙ্গে এই দোয়া আমাদের নিজের ভেতরের অবস্থাও ভাবতে শেখায়: আমার জ্ঞান কি কাজে লাগছে, আমার অন্তর কি আল্লাহকে ভয় করছে, আমার চাওয়া কি সীমাহীন হয়ে যাচ্ছে?"},"teachings":["উপকারী ইলমের জন্য আল্লাহর কাছে দোয়া করা উচিত।","জ্ঞান যদি আমল ও অন্তরের পরিবর্তনে না আসে, তবে তা নিয়ে ভাবা দরকার।","অতৃপ্ত নফস ও ভীতিহীন অন্তর থেকে আশ্রয় চাওয়া নববী শিক্ষা।","দোয়ার কবুলিয়াত আল্লাহর হাতে—তাই বিনয় নিয়ে দোয়া করা উচিত।"],"related_hadiths":[{"id":"2722","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3482","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2472","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E26" s="4" t="n"/>
@@ -1094,12 +1090,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>124</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উপকারী ইলমের দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি উপকারহীন বিদ্যা, ভীতিহীন অন্তর, অতৃপ্ত আত্মা ও কবুল না হওয়া দোয়া থেকে আশ্রয় চাইতেন।"},"heading":{"title":"উপকারী ইলমের দোয়া ও অন্তরের ভয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর একটি গুরুত্বপূর্ণ দোয়া এসেছে। তিনি আল্লাহর কাছে আশ্রয় চাইতেন এমন বিদ্যা থেকে যা উপকারে আসে না, এমন অন্তর থেকে যা ভীত হয় না, এমন আত্মা থেকে যা পরিতৃপ্ত হয় না এবং এমন দোয়া থেকে যা কবুল হয় না। এখানে উপকারী ইলমের গুরুত্ব খুব স্পষ্ট। শুধু জানা যথেষ্ট নয়; সেই জ্ঞান যেন অন্তরকে নরম করে, আমলে প্রভাব ফেলে এবং মানুষকে আল্লাহর দিকে নিয়ে যায়—এটাই কাম্য। একই সঙ্গে এই দোয়া আমাদের নিজের ভেতরের অবস্থাও ভাবতে শেখায়: আমার জ্ঞান কি কাজে লাগছে, আমার অন্তর কি আল্লাহকে ভয় করছে, আমার চাওয়া কি সীমাহীন হয়ে যাচ্ছে?"},"teachings":["উপকারী ইলমের জন্য আল্লাহর কাছে দোয়া করা উচিত।","জ্ঞান যদি আমল ও অন্তরের পরিবর্তনে না আসে, তবে তা নিয়ে ভাবা দরকার।","অতৃপ্ত নফস ও ভীতিহীন অন্তর থেকে আশ্রয় চাওয়া নববী শিক্ষা।","দোয়ার কবুলিয়াত আল্লাহর হাতে—তাই বিনয় নিয়ে দোয়া করা উচিত।"],"related_hadiths":[{"id":"2722","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3482","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2472","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কথার সঙ্গে আমলের মিল","description":"$book_name$ $hadith_number$ - $chapter_name$. সৎকাজের আদেশ করে নিজে না মানা ও মন্দ থেকে নিষেধ করে নিজে করা কঠিন পরিণতির কারণ হতে পারে।"},"heading":{"title":"কথা ও আমলের অমিল: সৎকাজের আদেশের আগে নিজের হিসাব","description":"এই হাদিসে এমন ব্যক্তির ভয়াবহ পরিণতি বলা হয়েছে, যে মানুষকে সৎকাজের আদেশ করত কিন্তু নিজে তা করত না; আবার মন্দ কাজ থেকে নিষেধ করত, অথচ নিজেই সেই কাজ করত। কিয়ামতের দিনের দৃশ্যটি খুব কঠিন ভাষায় এসেছে, যাতে মানুষ নিজের কথার সঙ্গে নিজের আমল মিলিয়ে দেখে। এর মানে এই নয় যে কেউ নিজে দুর্বল হলে ভালো কথা বলবে না; বরং হাদিসটি সতর্ক করছে—অন্যকে নসীহত করার সঙ্গে সঙ্গে নিজের আমলকে ভুলে যাওয়া বিপজ্জনক। সৎকাজের আদেশ ও অসৎ কাজ থেকে নিষেধ একটি বড় দায়িত্ব, আর সেই দায়িত্বের সঙ্গে নিজের সংশোধনও জরুরি।"},"teachings":["মানুষকে ভালো কথা বলার পাশাপাশি নিজের আমলের দিকেও নজর দিতে হবে।","সৎকাজের আদেশ করে নিজে তা না করা কঠিন জবাবদিহির কারণ হতে পারে।","মন্দ থেকে নিষেধ করে নিজে সেই মন্দে জড়ানো বড় সতর্কতার বিষয়।","নসীহত করার আগে ও পরে নিজের হিসাব নেওয়া দরকার।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"198","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E27" s="4" t="n"/>
@@ -1117,12 +1113,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>125</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কথার সঙ্গে আমলের মিল","description":"$book_name$ $hadith_number$ - $chapter_name$. সৎকাজের আদেশ করে নিজে না মানা ও মন্দ থেকে নিষেধ করে নিজে করা কঠিন পরিণতির কারণ হতে পারে।"},"heading":{"title":"কথা ও আমলের অমিল: সৎকাজের আদেশের আগে নিজের হিসাব","description":"এই হাদিসে এমন ব্যক্তির ভয়াবহ পরিণতি বলা হয়েছে, যে মানুষকে সৎকাজের আদেশ করত কিন্তু নিজে তা করত না; আবার মন্দ কাজ থেকে নিষেধ করত, অথচ নিজেই সেই কাজ করত। কিয়ামতের দিনের দৃশ্যটি খুব কঠিন ভাষায় এসেছে, যাতে মানুষ নিজের কথার সঙ্গে নিজের আমল মিলিয়ে দেখে। এর মানে এই নয় যে কেউ নিজে দুর্বল হলে ভালো কথা বলবে না; বরং হাদিসটি সতর্ক করছে—অন্যকে নসীহত করার সঙ্গে সঙ্গে নিজের আমলকে ভুলে যাওয়া বিপজ্জনক। সৎকাজের আদেশ ও অসৎ কাজ থেকে নিষেধ একটি বড় দায়িত্ব, আর সেই দায়িত্বের সঙ্গে নিজের সংশোধনও জরুরি।"},"teachings":["মানুষকে ভালো কথা বলার পাশাপাশি নিজের আমলের দিকেও নজর দিতে হবে।","সৎকাজের আদেশ করে নিজে তা না করা কঠিন জবাবদিহির কারণ হতে পারে।","মন্দ থেকে নিষেধ করে নিজে সেই মন্দে জড়ানো বড় সতর্কতার বিষয়।","নসীহত করার আগে ও পরে নিজের হিসাব নেওয়া দরকার।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"198","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বক্তার কথা ও আমলের মিল","description":"$book_name$ $hadith_number$ - $chapter_name$. যারা বলে কিন্তু নিজেরা আমল করে না, তাদের বিষয়ে মেরাজের রাতের কঠিন সতর্কতা এই হাদিসে এসেছে।"},"heading":{"title":"বক্তার দায়িত্ব: যা বলি, তা আমলে আনার চেষ্টা","description":"এই হাদিসে মেরাজের রাতের একটি দৃশ্য এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন একদল লোককে দেখলেন, যাদের ঠোঁট আগুনের কাঁচি দিয়ে কাটা হচ্ছিল। জিবরীল (আলাইহিস সালাম) জানালেন, তারা উম্মতের বক্তাশ্রেণী; তারা এমন কথা বলত যা নিজেরা আমল করত না। বর্ণনার শেষে আরও এসেছে, তারা আল্লাহর কিতাব পাঠ করত কিন্তু তার প্রতি আমল করত না। হাদিসটি বক্তা, শিক্ষক, লেখক এবং নসীহতকারীদের জন্য বিশেষ সতর্কতা। কথা বলা সহজ, কিন্তু সেই কথার দাবি নিজের জীবনে রাখা কঠিন। তাই জ্ঞানী কথা বলার আগে নিজেকে ভুলে না যাওয়াই এই হাদিসের মূল শিক্ষা।"},"teachings":["বক্তা বা শিক্ষককে নিজের আমলের বিষয়ে বেশি সচেতন হতে হবে।","কুরআন পড়া ও বলা যথেষ্ট নয়; তার নির্দেশ মানার চেষ্টা দরকার।","যা বলা হয়, তা নিজের জীবনে আনার চেষ্টা না থাকলে বড় জবাবদিহি হতে পারে।","নসীহতের আগে আত্মসংশোধন জরুরি।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2989","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E28" s="4" t="n"/>
@@ -1140,12 +1136,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>126</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বক্তার কথা ও আমলের মিল","description":"$book_name$ $hadith_number$ - $chapter_name$. যারা বলে কিন্তু নিজেরা আমল করে না, তাদের বিষয়ে মেরাজের রাতের কঠিন সতর্কতা এই হাদিসে এসেছে।"},"heading":{"title":"বক্তার দায়িত্ব: যা বলি, তা আমলে আনার চেষ্টা","description":"এই হাদিসে মেরাজের রাতের একটি দৃশ্য এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন একদল লোককে দেখলেন, যাদের ঠোঁট আগুনের কাঁচি দিয়ে কাটা হচ্ছিল। জিবরীল (আলাইহিস সালাম) জানালেন, তারা উম্মতের বক্তাশ্রেণী; তারা এমন কথা বলত যা নিজেরা আমল করত না। বর্ণনার শেষে আরও এসেছে, তারা আল্লাহর কিতাব পাঠ করত কিন্তু তার প্রতি আমল করত না। হাদিসটি বক্তা, শিক্ষক, লেখক এবং নসীহতকারীদের জন্য বিশেষ সতর্কতা। কথা বলা সহজ, কিন্তু সেই কথার দাবি নিজের জীবনে রাখা কঠিন। তাই জ্ঞানী কথা বলার আগে নিজেকে ভুলে না যাওয়াই এই হাদিসের মূল শিক্ষা।"},"teachings":["বক্তা বা শিক্ষককে নিজের আমলের বিষয়ে বেশি সচেতন হতে হবে।","কুরআন পড়া ও বলা যথেষ্ট নয়; তার নির্দেশ মানার চেষ্টা দরকার।","যা বলা হয়, তা নিজের জীবনে আনার চেষ্টা না থাকলে বড় জবাবদিহি হতে পারে।","নসীহতের আগে আত্মসংশোধন জরুরি।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2989","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কিয়ামতের জবাবদিহি","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, জ্ঞান, সম্পদ ও শরীর—কিয়ামতের দিনে এসব নেয়ামত সম্পর্কে বান্দাকে প্রশ্ন করা হবে।"},"heading":{"title":"কিয়ামতের জবাবদিহি: বয়স, জ্ঞান, সম্পদ ও শরীর","description":"এই হাদিসে কিয়ামতের দিনের জবাবদিহির কয়েকটি বড় বিষয় এসেছে। বান্দার পা সরবে না, যতক্ষণ না তাকে বয়স সম্পর্কে জিজ্ঞাসা করা হয়—কীভাবে তা শেষ করেছে; জ্ঞান সম্পর্কে—তা দিয়ে কী করেছে; সম্পদ সম্পর্কে—কোথা থেকে উপার্জন করেছে এবং কোথায় ব্যয় করেছে; শরীর সম্পর্কে—কীভাবে তা ক্ষয় করেছে। হাদিসটি আমাদের জীবনকে হিসাবের চোখে দেখতে শেখায়। বয়স, জ্ঞান, টাকা-পয়সা ও শরীর—এসবই আল্লাহর দেওয়া নেয়ামত। এগুলো শুধু ব্যবহার করার জিনিস নয়; এগুলোর ব্যবহার সম্পর্কে একদিন জবাব দিতে হবে। তাই সময় নষ্ট, জ্ঞান অবহেলা, অন্যায় উপার্জন ও শরীরের অপব্যবহার থেকে সাবধান থাকা দরকার।"},"teachings":["জীবনের সময় কীভাবে কাটছে, তা নিয়ে নিয়মিত ভাবা উচিত।","জ্ঞান অর্জনের পর তা দিয়ে কী আমল করা হয়েছে—এ প্রশ্ন গুরুত্বপূর্ণ।","সম্পদের আয় ও ব্যয়—দুই দিকেই জবাবদিহি আছে।","শরীরকে আল্লাহর নেয়ামত মনে করে ভালো কাজে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2417","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E29" s="4" t="n"/>
@@ -1163,12 +1159,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>127</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কিয়ামতের জবাবদিহি","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, জ্ঞান, সম্পদ ও শরীর—কিয়ামতের দিনে এসব নেয়ামত সম্পর্কে বান্দাকে প্রশ্ন করা হবে।"},"heading":{"title":"কিয়ামতের জবাবদিহি: বয়স, জ্ঞান, সম্পদ ও শরীর","description":"এই হাদিসে কিয়ামতের দিনের জবাবদিহির কয়েকটি বড় বিষয় এসেছে। বান্দার পা সরবে না, যতক্ষণ না তাকে বয়স সম্পর্কে জিজ্ঞাসা করা হয়—কীভাবে তা শেষ করেছে; জ্ঞান সম্পর্কে—তা দিয়ে কী করেছে; সম্পদ সম্পর্কে—কোথা থেকে উপার্জন করেছে এবং কোথায় ব্যয় করেছে; শরীর সম্পর্কে—কীভাবে তা ক্ষয় করেছে। হাদিসটি আমাদের জীবনকে হিসাবের চোখে দেখতে শেখায়। বয়স, জ্ঞান, টাকা-পয়সা ও শরীর—এসবই আল্লাহর দেওয়া নেয়ামত। এগুলো শুধু ব্যবহার করার জিনিস নয়; এগুলোর ব্যবহার সম্পর্কে একদিন জবাব দিতে হবে। তাই সময় নষ্ট, জ্ঞান অবহেলা, অন্যায় উপার্জন ও শরীরের অপব্যবহার থেকে সাবধান থাকা দরকার।"},"teachings":["জীবনের সময় কীভাবে কাটছে, তা নিয়ে নিয়মিত ভাবা উচিত।","জ্ঞান অর্জনের পর তা দিয়ে কী আমল করা হয়েছে—এ প্রশ্ন গুরুত্বপূর্ণ।","সম্পদের আয় ও ব্যয়—দুই দিকেই জবাবদিহি আছে।","শরীরকে আল্লাহর নেয়ামত মনে করে ভালো কাজে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2417","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চার বিষয়ের হিসাব","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, যৌবন, সম্পদ ও বিদ্যা—কিয়ামতের দিনে এসব বিষয়ে বান্দাকে প্রশ্ন করা হবে।"},"heading":{"title":"চার বিষয়ের হিসাব: বয়স, যৌবন, সম্পদ ও বিদ্যা","description":"এই হাদিসে কিয়ামতের দিনে চারটি বিষয়ে প্রশ্নের কথা বলা হয়েছে। বান্দার পা নড়বে না, যতক্ষণ না তাকে তার বয়স, যৌবন, সম্পদ এবং বিদ্যা সম্পর্কে জিজ্ঞাসা করা হয়। বয়স কীভাবে কাটাল, যৌবন কীভাবে পুরাতন করল, সম্পদ কীভাবে উপার্জন করল এবং কোন পথে খরচ করল, আর বিদ্যা দিয়ে কী আমল করল—এসব প্রশ্ন মানুষকে নিজের জীবন নিয়ে ভাবতে শেখায়। বিশেষ করে যৌবনের কথা আলাদা করে আসা আমাদের সতর্ক করে। শক্তি, সময়, শেখার ক্ষমতা ও কাজ করার সুযোগ—এসব সময়ের সঙ্গে কমে যায়। তাই এই নেয়ামতগুলোকে হালকা করে দেখা ঠিক নয়।"},"teachings":["বয়স ও যৌবন আল্লাহর নেয়ামত; এগুলো অবহেলায় নষ্ট করা উচিত নয়।","সম্পদের উৎস ও ব্যয়—দুই দিকেই হিসাব হবে।","বিদ্যা শেখার পর তা অনুযায়ী আমল করা জরুরি।","কিয়ামতের জবাবদিহির চিন্তা জীবনকে সোজা রাখতে সাহায্য করে।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"6412","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E30" s="4" t="n"/>
@@ -1186,12 +1182,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>128</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চার বিষয়ের হিসাব","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, যৌবন, সম্পদ ও বিদ্যা—কিয়ামতের দিনে এসব বিষয়ে বান্দাকে প্রশ্ন করা হবে।"},"heading":{"title":"চার বিষয়ের হিসাব: বয়স, যৌবন, সম্পদ ও বিদ্যা","description":"এই হাদিসে কিয়ামতের দিনে চারটি বিষয়ে প্রশ্নের কথা বলা হয়েছে। বান্দার পা নড়বে না, যতক্ষণ না তাকে তার বয়স, যৌবন, সম্পদ এবং বিদ্যা সম্পর্কে জিজ্ঞাসা করা হয়। বয়স কীভাবে কাটাল, যৌবন কীভাবে পুরাতন করল, সম্পদ কীভাবে উপার্জন করল এবং কোন পথে খরচ করল, আর বিদ্যা দিয়ে কী আমল করল—এসব প্রশ্ন মানুষকে নিজের জীবন নিয়ে ভাবতে শেখায়। বিশেষ করে যৌবনের কথা আলাদা করে আসা আমাদের সতর্ক করে। শক্তি, সময়, শেখার ক্ষমতা ও কাজ করার সুযোগ—এসব সময়ের সঙ্গে কমে যায়। তাই এই নেয়ামতগুলোকে হালকা করে দেখা ঠিক নয়।"},"teachings":["বয়স ও যৌবন আল্লাহর নেয়ামত; এগুলো অবহেলায় নষ্ট করা উচিত নয়।","সম্পদের উৎস ও ব্যয়—দুই দিকেই হিসাব হবে।","বিদ্যা শেখার পর তা অনুযায়ী আমল করা জরুরি।","কিয়ামতের জবাবদিহির চিন্তা জীবনকে সোজা রাখতে সাহায্য করে।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"6412","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পাঁচ বিষয়ের প্রশ্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, যৌবন, সম্পদ আয়-ব্যয় ও শেখা জ্ঞানের আমল—এসব বিষয়ে কিয়ামতে প্রশ্ন হবে।"},"heading":{"title":"পাঁচ বিষয়ের প্রশ্ন: জীবনের প্রতিটি নেয়ামতের হিসাব","description":"এই হাদিসে কিয়ামতের দিনে আদম সন্তানের পাঁচটি বিষয়ে প্রশ্নের কথা এসেছে। তার বয়স কীভাবে ক্ষয় করেছে, যৌবন কীভাবে অতিবাহিত করেছে, সম্পদ কীভাবে উপার্জন করেছে, কোন পথে খরচ করেছে, এবং যা শিখেছে সে অনুযায়ী কী আমল করেছে। এখানে সম্পদের আয় ও ব্যয় আলাদা করে বলা হয়েছে। অর্থাৎ শুধু টাকা খরচের জায়গা নয়, টাকা আসার পথও গুরুত্বপূর্ণ। আবার জ্ঞান শেখার পর আমল না করলে সেটিও জবাবদিহির বিষয়। হাদিসটি আমাদের দৈনন্দিন জীবনকে আল্লাহর সামনে দাঁড়ানোর মতো করে সাজাতে শেখায়—সময়, শক্তি, অর্থ ও জ্ঞান যেন অবহেলায় নষ্ট না হয়।"},"teachings":["বয়স ও যৌবন কীভাবে যাচ্ছে, সে বিষয়ে সচেতন থাকা দরকার।","হালাল উপার্জন ও সঠিক ব্যয়—দুইটিই গুরুত্বপূর্ণ।","শেখা জ্ঞানের দাবি হলো আমল করার চেষ্টা।","কিয়ামতের হিসাবের চিন্তা মানুষকে দায়িত্বশীল করে।"],"related_hadiths":[{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E31" s="4" t="n"/>
@@ -1209,12 +1205,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>129</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পাঁচ বিষয়ের প্রশ্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. বয়স, যৌবন, সম্পদ আয়-ব্যয় ও শেখা জ্ঞানের আমল—এসব বিষয়ে কিয়ামতে প্রশ্ন হবে।"},"heading":{"title":"পাঁচ বিষয়ের প্রশ্ন: জীবনের প্রতিটি নেয়ামতের হিসাব","description":"এই হাদিসে কিয়ামতের দিনে আদম সন্তানের পাঁচটি বিষয়ে প্রশ্নের কথা এসেছে। তার বয়স কীভাবে ক্ষয় করেছে, যৌবন কীভাবে অতিবাহিত করেছে, সম্পদ কীভাবে উপার্জন করেছে, কোন পথে খরচ করেছে, এবং যা শিখেছে সে অনুযায়ী কী আমল করেছে। এখানে সম্পদের আয় ও ব্যয় আলাদা করে বলা হয়েছে। অর্থাৎ শুধু টাকা খরচের জায়গা নয়, টাকা আসার পথও গুরুত্বপূর্ণ। আবার জ্ঞান শেখার পর আমল না করলে সেটিও জবাবদিহির বিষয়। হাদিসটি আমাদের দৈনন্দিন জীবনকে আল্লাহর সামনে দাঁড়ানোর মতো করে সাজাতে শেখায়—সময়, শক্তি, অর্থ ও জ্ঞান যেন অবহেলায় নষ্ট না হয়।"},"teachings":["বয়স ও যৌবন কীভাবে যাচ্ছে, সে বিষয়ে সচেতন থাকা দরকার।","হালাল উপার্জন ও সঠিক ব্যয়—দুইটিই গুরুত্বপূর্ণ।","শেখা জ্ঞানের দাবি হলো আমল করার চেষ্টা।","কিয়ামতের হিসাবের চিন্তা মানুষকে দায়িত্বশীল করে।"],"related_hadiths":[{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শেখা জ্ঞানের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. আবু দারদা (রাঃ) শেখা জ্ঞান অনুযায়ী আমল করেছেন কি না—এই প্রশ্নকে ভয় করতেন।"},"heading":{"title":"শেখা জ্ঞানের আমল: আবু দারদা (রাঃ)-এর ভয়","description":"এই বর্ণনায় আবু দারদা (রাঃ)-এর গভীর আত্মভয় দেখা যায়। তিনি বলতেন, কিয়ামতের দিন আল্লাহ যদি সকল সৃষ্টির সামনে তাকে ডাকেন এবং জিজ্ঞেস করেন—যা শিক্ষা লাভ করেছিলে, সে অনুযায়ী কী আমল করেছিলে?—এই প্রশ্নকে তিনি ভয় করতেন। এখানে জ্ঞানের মর্যাদার পাশাপাশি জ্ঞানের দায়িত্বও স্পষ্ট। মানুষ যত বেশি শেখে, তার ওপর তত বেশি দায়িত্ব আসে। শুধু জানা, বলা বা মনে রাখা যথেষ্ট নয়; শেখা বিষয় জীবনে কতটা কাজে লাগানো হলো, সেটাই বড় প্রশ্ন। এই বর্ণনা আমাদের শেখায়, ইলমের সঙ্গে আমল না থাকলে অন্তরে ভয় থাকা উচিত।"},"teachings":["জ্ঞান অর্জনের পর আমলের হিসাব নিয়ে ভাবা উচিত।","সাহাবীদের মধ্যে আত্মজবাবদিহির গভীর অনুভূতি ছিল।","ইলম মানুষকে দায়িত্বশীল করে, শুধু তথ্যসমৃদ্ধ করে না।","কিয়ামতের প্রশ্নের ভয় আমলকে সুন্দর করতে সাহায্য করে।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E32" s="4" t="n"/>
@@ -1232,12 +1228,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শেখা জ্ঞানের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. আবু দারদা (রাঃ) শেখা জ্ঞান অনুযায়ী আমল করেছেন কি না—এই প্রশ্নকে ভয় করতেন।"},"heading":{"title":"শেখা জ্ঞানের আমল: আবু দারদা (রাঃ)-এর ভয়","description":"এই বর্ণনায় আবু দারদা (রাঃ)-এর গভীর আত্মভয় দেখা যায়। তিনি বলতেন, কিয়ামতের দিন আল্লাহ যদি সকল সৃষ্টির সামনে তাকে ডাকেন এবং জিজ্ঞেস করেন—যা শিক্ষা লাভ করেছিলে, সে অনুযায়ী কী আমল করেছিলে?—এই প্রশ্নকে তিনি ভয় করতেন। এখানে জ্ঞানের মর্যাদার পাশাপাশি জ্ঞানের দায়িত্বও স্পষ্ট। মানুষ যত বেশি শেখে, তার ওপর তত বেশি দায়িত্ব আসে। শুধু জানা, বলা বা মনে রাখা যথেষ্ট নয়; শেখা বিষয় জীবনে কতটা কাজে লাগানো হলো, সেটাই বড় প্রশ্ন। এই বর্ণনা আমাদের শেখায়, ইলমের সঙ্গে আমল না থাকলে অন্তরে ভয় থাকা উচিত।"},"teachings":["জ্ঞান অর্জনের পর আমলের হিসাব নিয়ে ভাবা উচিত।","সাহাবীদের মধ্যে আত্মজবাবদিহির গভীর অনুভূতি ছিল।","ইলম মানুষকে দায়িত্বশীল করে, শুধু তথ্যসমৃদ্ধ করে না।","কিয়ামতের প্রশ্নের ভয় আমলকে সুন্দর করতে সাহায্য করে।"],"related_hadiths":[{"id":"2417","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"2416","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মানুষ উঠবে নিয়ত অনুযায়ী","description":"$book_name$ $hadith_number$ - $chapter_name$. সংক্ষিপ্ত এই হাদিস জানায়, কিয়ামতের দিনে মানুষের পুনরুত্থান হবে তাদের নিয়ত অনুযায়ী।"},"heading":{"title":"নিয়ত অনুযায়ী উঠানো হবে: অন্তরের উদ্দেশ্যের হিসাব","description":"এই হাদিসের বাণী খুব সংক্ষিপ্ত, কিন্তু শিক্ষা বড়। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, মানুষকে তাদের নিয়ত অনুযায়ী উঠানো হবে। এখানে কিয়ামতের দিন পুনরুত্থানের কথা এসেছে এবং সেই দিনের সাথে নিয়তকে যুক্ত করা হয়েছে। মানুষ দুনিয়ায় অনেক কাজ করে, অনেক দলে থাকে, অনেক সিদ্ধান্ত নেয়। বাইরে থেকে সবকিছু একই রকম মনে হলেও আল্লাহ অন্তরের উদ্দেশ্য জানেন। তাই এই হাদিস আমাদের নিয়তকে গুরুত্ব দিতে শেখায়। আমরা কী করছি, তার পাশাপাশি কেন করছি—এ প্রশ্নও জরুরি। ভালো কাজে আল্লাহর সন্তুষ্টি উদ্দেশ্য করা, মন্দ উদ্দেশ্য থেকে বাঁচা এবং নিজের অন্তরকে নিয়মিত পরীক্ষা করা এই হাদিসের প্রধান শিক্ষা। যেহেতু বর্ণনা সংক্ষিপ্ত, তাই এর বাইরে বিস্তারিত ঘটনা যোগ না করে মূল কথাতেই থাকা নিরাপদ।"},"teachings":["কিয়ামতের দিনে নিয়ত গুরুত্বপূর্ণ হিসাবের বিষয় হবে।","কাজের পাশাপাশি উদ্দেশ্যও শুদ্ধ রাখা দরকার।","আল্লাহ মানুষের অন্তরের অবস্থা জানেন।","নিজের নিয়ত নিয়মিত পরীক্ষা করা মুমিনের কাজ।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E33" s="4" t="n"/>
@@ -1255,12 +1251,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>130</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মানুষ উঠবে নিয়ত অনুযায়ী","description":"$book_name$ $hadith_number$ - $chapter_name$. সংক্ষিপ্ত এই হাদিস জানায়, কিয়ামতের দিনে মানুষের পুনরুত্থান হবে তাদের নিয়ত অনুযায়ী।"},"heading":{"title":"নিয়ত অনুযায়ী উঠানো হবে: অন্তরের উদ্দেশ্যের হিসাব","description":"এই হাদিসের বাণী খুব সংক্ষিপ্ত, কিন্তু শিক্ষা বড়। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, মানুষকে তাদের নিয়ত অনুযায়ী উঠানো হবে। এখানে কিয়ামতের দিন পুনরুত্থানের কথা এসেছে এবং সেই দিনের সাথে নিয়তকে যুক্ত করা হয়েছে। মানুষ দুনিয়ায় অনেক কাজ করে, অনেক দলে থাকে, অনেক সিদ্ধান্ত নেয়। বাইরে থেকে সবকিছু একই রকম মনে হলেও আল্লাহ অন্তরের উদ্দেশ্য জানেন। তাই এই হাদিস আমাদের নিয়তকে গুরুত্ব দিতে শেখায়। আমরা কী করছি, তার পাশাপাশি কেন করছি—এ প্রশ্নও জরুরি। ভালো কাজে আল্লাহর সন্তুষ্টি উদ্দেশ্য করা, মন্দ উদ্দেশ্য থেকে বাঁচা এবং নিজের অন্তরকে নিয়মিত পরীক্ষা করা এই হাদিসের প্রধান শিক্ষা। যেহেতু বর্ণনা সংক্ষিপ্ত, তাই এর বাইরে বিস্তারিত ঘটনা যোগ না করে মূল কথাতেই থাকা নিরাপদ।"},"teachings":["কিয়ামতের দিনে নিয়ত গুরুত্বপূর্ণ হিসাবের বিষয় হবে।","কাজের পাশাপাশি উদ্দেশ্যও শুদ্ধ রাখা দরকার।","আল্লাহ মানুষের অন্তরের অবস্থা জানেন।","নিজের নিয়ত নিয়মিত পরীক্ষা করা মুমিনের কাজ।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অন্যকে শেখায় নিজেকে ভুলে যায়","description":"$book_name$ $hadith_number$ - $chapter_name$. কল্যাণ শেখিয়ে নিজে আমল ভুলে গেলে চেরাগের মতো মানুষ উপকৃত হলেও নিজের ক্ষতি হয়।"},"heading":{"title":"চেরাগের উপমা: অন্যকে শেখাই, নিজেকেও ভুলে না যাই","description":"এই হাদিসে খুব সহজ একটি উপমা দেওয়া হয়েছে। যে ব্যক্তি মানুষকে কল্যাণের শিক্ষা দেয়, অথচ নিজের আমলের কথা ভুলে যায়, তার উদাহরণ চেরাগের মতো। চেরাগ মানুষকে আলো দেয়, কিন্তু নিজেকে জ্বালিয়ে দেয়। অর্থাৎ অন্যরা তার কথা থেকে উপকার পেতে পারে, কিন্তু সে নিজে আমল না করলে নিজের ক্ষতি ডেকে আনে। এই হাদিস শিক্ষক, বক্তা, লেখক, অভিভাবক—সবার জন্য সতর্কতা। ভালো কথা বলা অবশ্যই দরকার, তবে নিজের জীবনেও সেই ভালো কাজ আনার চেষ্টা থাকা চাই। অন্যকে আলো দেখাতে গিয়ে নিজের অন্তর অন্ধকারে পড়ে আছে কি না—এই হিসাব নেওয়া জরুরি।"},"teachings":["মানুষকে কল্যাণ শেখানোর সঙ্গে নিজের আমলও জরুরি।","ভালো কথা বললেই নিজের মুক্তি নিশ্চিত—এমন ভাবা ঠিক নয়।","অন্যকে উপকার করেও নিজের ক্ষতি হতে পারে, যদি নিজে আমল ভুলে যায়।","শিক্ষাদান ও আত্মসংশোধন একসঙ্গে চলা উচিত।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"198","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
         </is>
       </c>
       <c r="E34" s="4" t="n"/>
@@ -1278,12 +1274,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>131</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অন্যকে শেখায় নিজেকে ভুলে যায়","description":"$book_name$ $hadith_number$ - $chapter_name$. কল্যাণ শেখিয়ে নিজে আমল ভুলে গেলে চেরাগের মতো মানুষ উপকৃত হলেও নিজের ক্ষতি হয়।"},"heading":{"title":"চেরাগের উপমা: অন্যকে শেখাই, নিজেকেও ভুলে না যাই","description":"এই হাদিসে খুব সহজ একটি উপমা দেওয়া হয়েছে। যে ব্যক্তি মানুষকে কল্যাণের শিক্ষা দেয়, অথচ নিজের আমলের কথা ভুলে যায়, তার উদাহরণ চেরাগের মতো। চেরাগ মানুষকে আলো দেয়, কিন্তু নিজেকে জ্বালিয়ে দেয়। অর্থাৎ অন্যরা তার কথা থেকে উপকার পেতে পারে, কিন্তু সে নিজে আমল না করলে নিজের ক্ষতি ডেকে আনে। এই হাদিস শিক্ষক, বক্তা, লেখক, অভিভাবক—সবার জন্য সতর্কতা। ভালো কথা বলা অবশ্যই দরকার, তবে নিজের জীবনেও সেই ভালো কাজ আনার চেষ্টা থাকা চাই। অন্যকে আলো দেখাতে গিয়ে নিজের অন্তর অন্ধকারে পড়ে আছে কি না—এই হিসাব নেওয়া জরুরি।"},"teachings":["মানুষকে কল্যাণ শেখানোর সঙ্গে নিজের আমলও জরুরি।","ভালো কথা বললেই নিজের মুক্তি নিশ্চিত—এমন ভাবা ঠিক নয়।","অন্যকে উপকার করেও নিজের ক্ষতি হতে পারে, যদি নিজে আমল ভুলে যায়।","শিক্ষাদান ও আত্মসংশোধন একসঙ্গে চলা উচিত।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"198","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বাতির আলো ও নিজের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষকে ভালো শেখিয়ে নিজে আমল ভুলে গেলে বাতির মতো অন্যকে আলো দিয়ে নিজেকে পোড়ায়।"},"heading":{"title":"বাতির উপমা: শিক্ষা দেওয়ার আগে নিজের দিকে তাকানো","description":"এই হাদিসে আগের একই মূল শিক্ষাকে বাতির উপমায় বোঝানো হয়েছে। যে ব্যক্তি মানুষকে কল্যাণ শেখায়, অথচ নিজে নিজের আমলের কথা ভুলে যায়, তার উদাহরণ বাতির মতো। বাতি মানুষকে আলো দেয়, কিন্তু নিজেকে পুড়িয়ে ফেলে। এখানে শিক্ষা হলো—জ্ঞান ও নসীহত শুধু অন্যের জন্য নয়, আগে নিজের জন্যও। কেউ যদি ভালো কথা বলে, মানুষ উপকৃত হতে পারে; কিন্তু সে নিজে যদি সেই ভালো কাজে মন না দেয়, তবে তার নিজের ক্ষতি থেকে যায়। তাই ওয়াজ, লেখা, শিক্ষা বা দাওয়াত—সব ক্ষেত্রেই নিজের আমলকে ভুলে না যাওয়া দরকার।"},"teachings":["অন্যকে ভালো শেখানোর সময় নিজের আমল ভুলে যাওয়া উচিত নয়।","ভালো কথার আসল প্রভাব নিজের জীবনেও দেখা দরকার।","মানুষের উপকার হলেও নিজের জবাবদিহি থেকে মুক্তি নেই।","জ্ঞান, শিক্ষা ও আমলকে একসঙ্গে রাখা দরকার।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E35" s="4" t="n"/>
@@ -1301,12 +1297,12 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>132</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বাতির আলো ও নিজের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষকে ভালো শেখিয়ে নিজে আমল ভুলে গেলে বাতির মতো অন্যকে আলো দিয়ে নিজেকে পোড়ায়।"},"heading":{"title":"বাতির উপমা: শিক্ষা দেওয়ার আগে নিজের দিকে তাকানো","description":"এই হাদিসে আগের একই মূল শিক্ষাকে বাতির উপমায় বোঝানো হয়েছে। যে ব্যক্তি মানুষকে কল্যাণ শেখায়, অথচ নিজে নিজের আমলের কথা ভুলে যায়, তার উদাহরণ বাতির মতো। বাতি মানুষকে আলো দেয়, কিন্তু নিজেকে পুড়িয়ে ফেলে। এখানে শিক্ষা হলো—জ্ঞান ও নসীহত শুধু অন্যের জন্য নয়, আগে নিজের জন্যও। কেউ যদি ভালো কথা বলে, মানুষ উপকৃত হতে পারে; কিন্তু সে নিজে যদি সেই ভালো কাজে মন না দেয়, তবে তার নিজের ক্ষতি থেকে যায়। তাই ওয়াজ, লেখা, শিক্ষা বা দাওয়াত—সব ক্ষেত্রেই নিজের আমলকে ভুলে না যাওয়া দরকার।"},"teachings":["অন্যকে ভালো শেখানোর সময় নিজের আমল ভুলে যাওয়া উচিত নয়।","ভালো কথার আসল প্রভাব নিজের জীবনেও দেখা দরকার।","মানুষের উপকার হলেও নিজের জবাবদিহি থেকে মুক্তি নেই।","জ্ঞান, শিক্ষা ও আমলকে একসঙ্গে রাখা দরকার।"],"related_hadiths":[{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভাষাজ্ঞানী মুনাফিকের ভয়","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দর ভাষা ও জ্ঞান থাকলেও অন্তরের ভ্রষ্টতা থাকলে তা উম্মতের জন্য ভয় ও ক্ষতির কারণ হতে পারে।"},"heading":{"title":"বিজ্ঞ ভাষাবিদ মুনাফিক: কথার চমক নয়, অন্তরের সততা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, তাঁর পরে উম্মতের জন্য তিনি সবচেয়ে বেশি ভয় করেন প্রত্যেক বিজ্ঞ ভাষাবিদ মুনাফিককে। এখানে সতর্কতা ভাষা, বক্তৃতা বা জ্ঞানের বিরুদ্ধে নয়; বরং এমন ব্যক্তির বিরুদ্ধে, যার কথা খুব শক্তিশালী, ভাষা সুন্দর, কিন্তু অন্তরে সত্যতা নেই। মানুষ অনেক সময় সুন্দর কথা শুনে মুগ্ধ হয়, কিন্তু হাদিসটি শেখায়—শুধু ভাষার জোর দেখে কাউকে গ্রহণ করা ঠিক নয়। দ্বীনি কথার সঙ্গে ঈমান, সততা, আমল ও আল্লাহভীতি থাকা দরকার। মুখের জ্ঞান যদি অন্তরের সত্যতার সঙ্গে না মেলে, তা মানুষের জন্য বিভ্রান্তির কারণ হতে পারে।"},"teachings":["সুন্দর ভাষা একা যথেষ্ট নয়; অন্তরের সততা দরকার।","দ্বীনি বক্তার কথার সঙ্গে আমল ও ঈমানের মিল দেখা জরুরি।","ভাষার চমকে মুগ্ধ হয়ে সত্য-মিথ্যা ভুলে যাওয়া ঠিক নয়।","মুনাফিকি স্বভাব থেকে আল্লাহর কাছে আশ্রয় চাওয়া উচিত।"],"related_hadiths":[{"id":"33","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"59","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E36" s="4" t="n"/>
@@ -1324,12 +1320,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>133</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভাষাজ্ঞানী মুনাফিকের ভয়","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দর ভাষা ও জ্ঞান থাকলেও অন্তরের ভ্রষ্টতা থাকলে তা উম্মতের জন্য ভয় ও ক্ষতির কারণ হতে পারে।"},"heading":{"title":"বিজ্ঞ ভাষাবিদ মুনাফিক: কথার চমক নয়, অন্তরের সততা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, তাঁর পরে উম্মতের জন্য তিনি সবচেয়ে বেশি ভয় করেন প্রত্যেক বিজ্ঞ ভাষাবিদ মুনাফিককে। এখানে সতর্কতা ভাষা, বক্তৃতা বা জ্ঞানের বিরুদ্ধে নয়; বরং এমন ব্যক্তির বিরুদ্ধে, যার কথা খুব শক্তিশালী, ভাষা সুন্দর, কিন্তু অন্তরে সত্যতা নেই। মানুষ অনেক সময় সুন্দর কথা শুনে মুগ্ধ হয়, কিন্তু হাদিসটি শেখায়—শুধু ভাষার জোর দেখে কাউকে গ্রহণ করা ঠিক নয়। দ্বীনি কথার সঙ্গে ঈমান, সততা, আমল ও আল্লাহভীতি থাকা দরকার। মুখের জ্ঞান যদি অন্তরের সত্যতার সঙ্গে না মেলে, তা মানুষের জন্য বিভ্রান্তির কারণ হতে পারে।"},"teachings":["সুন্দর ভাষা একা যথেষ্ট নয়; অন্তরের সততা দরকার।","দ্বীনি বক্তার কথার সঙ্গে আমল ও ঈমানের মিল দেখা জরুরি।","ভাষার চমকে মুগ্ধ হয়ে সত্য-মিথ্যা ভুলে যাওয়া ঠিক নয়।","মুনাফিকি স্বভাব থেকে আল্লাহর কাছে আশ্রয় চাওয়া উচিত।"],"related_hadiths":[{"id":"33","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"59","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | একই সতর্কতার আরেক বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. উমার (রাঃ) থেকে একই বিষয়ের বর্ণনা এসেছে; কথার দক্ষতার সঙ্গে সত্যতা থাকা জরুরি।"},"heading":{"title":"ভাষার জ্ঞান ও অন্তরের সততা: উমার (রাঃ)-এর সূত্রে বর্ণনা","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, উক্ত হাদিসটি ইমাম আহমাদ উমার বিন খাত্তাব (রাঃ) থেকে বর্ণনা করেছেন। যেহেতু এটি আগের হাদিসের সঙ্গে যুক্ত, তাই মূল শিক্ষা হলো—কথার দক্ষতা, ভাষার জোর বা বিদ্যার পরিচয় থাকলেই মানুষ নিরাপদ হয়ে যায় না। দ্বীনি কথায় সবচেয়ে দরকার সত্যতা, আমল এবং অন্তরের সঠিক অবস্থা। একজন মানুষ সুন্দরভাবে কথা বলতে পারে, মানুষকে প্রভাবিত করতে পারে, কিন্তু যদি তার ভেতরে মুনাফিকি স্বভাব থাকে, তবে সেই ভাষা মানুষের জন্য ক্ষতির কারণ হতে পারে। তাই জ্ঞান ও ভাষাকে আল্লাহভীতি ও সৎ আমলের সঙ্গে রাখা দরকার।"},"teachings":["একই সতর্কতা একাধিক সূত্রে আসা বিষয়টির গুরুত্ব বোঝায়।","কথার দক্ষতার সঙ্গে অন্তরের সততা থাকা দরকার।","দ্বীনি ভাষণ বা আলোচনা শুনলে শুধু ভাষা নয়, সত্যতাও বিবেচনা করা উচিত।","মুনাফিকি স্বভাব থেকে নিজের অন্তরকে বাঁচাতে চেষ্টা করা দরকার।"],"related_hadiths":[{"id":"33","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"59","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E37" s="4" t="n"/>
@@ -1347,12 +1343,12 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>134</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | একই সতর্কতার আরেক বর্ণনা","description":"$book_name$ $hadith_number$ - $chapter_name$. উমার (রাঃ) থেকে একই বিষয়ের বর্ণনা এসেছে; কথার দক্ষতার সঙ্গে সত্যতা থাকা জরুরি।"},"heading":{"title":"ভাষার জ্ঞান ও অন্তরের সততা: উমার (রাঃ)-এর সূত্রে বর্ণনা","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, উক্ত হাদিসটি ইমাম আহমাদ উমার বিন খাত্তাব (রাঃ) থেকে বর্ণনা করেছেন। যেহেতু এটি আগের হাদিসের সঙ্গে যুক্ত, তাই মূল শিক্ষা হলো—কথার দক্ষতা, ভাষার জোর বা বিদ্যার পরিচয় থাকলেই মানুষ নিরাপদ হয়ে যায় না। দ্বীনি কথায় সবচেয়ে দরকার সত্যতা, আমল এবং অন্তরের সঠিক অবস্থা। একজন মানুষ সুন্দরভাবে কথা বলতে পারে, মানুষকে প্রভাবিত করতে পারে, কিন্তু যদি তার ভেতরে মুনাফিকি স্বভাব থাকে, তবে সেই ভাষা মানুষের জন্য ক্ষতির কারণ হতে পারে। তাই জ্ঞান ও ভাষাকে আল্লাহভীতি ও সৎ আমলের সঙ্গে রাখা দরকার।"},"teachings":["একই সতর্কতা একাধিক সূত্রে আসা বিষয়টির গুরুত্ব বোঝায়।","কথার দক্ষতার সঙ্গে অন্তরের সততা থাকা দরকার।","দ্বীনি ভাষণ বা আলোচনা শুনলে শুধু ভাষা নয়, সত্যতাও বিবেচনা করা উচিত।","মুনাফিকি স্বভাব থেকে নিজের অন্তরকে বাঁচাতে চেষ্টা করা দরকার।"],"related_hadiths":[{"id":"33","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"59","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান আল্লাহর দিকে সমর্পণ","description":"$book_name$ $hadith_number$ - $chapter_name$. মূসা (আঃ) ও খিযিরের ঘটনায় শেখানো হয়েছে—সব জ্ঞানের মালিক আল্লাহ, মানুষের জ্ঞান সীমিত।"},"heading":{"title":"মূসা ও খিযিরের ঘটনা: জ্ঞানের আসল মালিক আল্লাহ","description":"এই হাদিসে মূসা (আলাইহিস সালাম) ও খিযিরের ঘটনা এসেছে। মূসা (আঃ)-কে যখন জিজ্ঞেস করা হলো, সবচেয়ে জ্ঞানী মানুষ কে, তিনি বললেন—আমি সবচেয়ে বেশি জ্ঞানী। আল্লাহ তাঁকে সতর্ক করলেন, কারণ তিনি জ্ঞানকে আল্লাহর দিকে সম্পর্কিত করেননি। পরে আল্লাহ তাঁকে এমন এক বান্দার খবর দিলেন, যিনি তাঁর চেয়ে বেশি জ্ঞানী। নৌকায় চড়ুই পাখির চঞ্চুতে সামান্য পানি তুলে নেওয়ার উপমা দিয়ে খিযির বললেন, তাঁর ও মূসা (আঃ)-এর জ্ঞান মিলেও আল্লাহর জ্ঞানের তুলনায় সমুদ্রের সামনে চড়ুইয়ের ঠোঁটের পানির মতো। হাদিসটি জ্ঞান নিয়ে বিনয়, “আল্লাহই ভালো জানেন” বলা এবং নিজের সীমাবদ্ধতা বুঝতে শেখায়।"},"teachings":["সব জ্ঞানের আসল মালিক আল্লাহ—এ কথা মনে রাখা দরকার।","জ্ঞান বেশি হলেও বিনয় হারানো উচিত নয়।","মানুষের জ্ঞান সীমিত; আল্লাহর জ্ঞানের সঙ্গে তার তুলনা নেই।","না জানা বিষয়ে আল্লাহর দিকে জ্ঞান সমর্পণ করা আদব।"],"related_hadiths":[{"id":"4727","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3401","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6057","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E38" s="4" t="n"/>
@@ -1370,12 +1366,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>135</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান আল্লাহর দিকে সমর্পণ","description":"$book_name$ $hadith_number$ - $chapter_name$. মূসা (আঃ) ও খিযিরের ঘটনায় শেখানো হয়েছে—সব জ্ঞানের মালিক আল্লাহ, মানুষের জ্ঞান সীমিত।"},"heading":{"title":"মূসা ও খিযিরের ঘটনা: জ্ঞানের আসল মালিক আল্লাহ","description":"এই হাদিসে মূসা (আলাইহিস সালাম) ও খিযিরের ঘটনা এসেছে। মূসা (আঃ)-কে যখন জিজ্ঞেস করা হলো, সবচেয়ে জ্ঞানী মানুষ কে, তিনি বললেন—আমি সবচেয়ে বেশি জ্ঞানী। আল্লাহ তাঁকে সতর্ক করলেন, কারণ তিনি জ্ঞানকে আল্লাহর দিকে সম্পর্কিত করেননি। পরে আল্লাহ তাঁকে এমন এক বান্দার খবর দিলেন, যিনি তাঁর চেয়ে বেশি জ্ঞানী। নৌকায় চড়ুই পাখির চঞ্চুতে সামান্য পানি তুলে নেওয়ার উপমা দিয়ে খিযির বললেন, তাঁর ও মূসা (আঃ)-এর জ্ঞান মিলেও আল্লাহর জ্ঞানের তুলনায় সমুদ্রের সামনে চড়ুইয়ের ঠোঁটের পানির মতো। হাদিসটি জ্ঞান নিয়ে বিনয়, “আল্লাহই ভালো জানেন” বলা এবং নিজের সীমাবদ্ধতা বুঝতে শেখায়।"},"teachings":["সব জ্ঞানের আসল মালিক আল্লাহ—এ কথা মনে রাখা দরকার।","জ্ঞান বেশি হলেও বিনয় হারানো উচিত নয়।","মানুষের জ্ঞান সীমিত; আল্লাহর জ্ঞানের সঙ্গে তার তুলনা নেই।","না জানা বিষয়ে আল্লাহর দিকে জ্ঞান সমর্পণ করা আদব।"],"related_hadiths":[{"id":"4727","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3401","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6057","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন জ্ঞান নিয়ে অহংকারের ভয়","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন পড়ে নিজেকে বড় মনে করা কল্যাণের পথ নয়; হাদিসটি জ্ঞান নিয়ে অহংকার থেকে সতর্ক করে।"},"heading":{"title":"কুরআন জ্ঞান নিয়ে অহংকার: নিজের শ্রেষ্ঠত্ব দাবি নয়","description":"এই হাদিসে এমন একদল মানুষের কথা এসেছে যারা কুরআন পড়বে এবং বলবে—আমাদের চেয়ে বেশি কুরআন কে পড়তে পারে, আমাদের চেয়ে বেশি জ্ঞানী কে, আমাদের চেয়ে বেশি বুঝে কে? রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) সাহাবীদের জিজ্ঞেস করলেন, তাদের মধ্যে কি কোনো কল্যাণ আছে? পরে তিনি জানালেন, তারা উম্মতেরই অন্তর্ভুক্ত, কিন্তু তারা জাহান্নামের ইন্ধন হবে। হাদিসটির মূল সতর্কতা হলো—কুরআন পড়া, জ্ঞান অর্জন করা বা বুঝ থাকার দাবি যদি অহংকারে পরিণত হয়, তা বিপজ্জনক। কুরআনের সঙ্গে বিনয়, আমল ও আল্লাহভীতি থাকতে হবে; আত্মপ্রশংসা নয়।"},"teachings":["কুরআন পড়া নিয়ে অহংকার করা ভয়ংকর ভুল।","জ্ঞান ও বুঝের দাবি মানুষকে বিনয়ী না করলে তা ক্ষতির কারণ হতে পারে।","নিজেকে অন্যদের চেয়ে বড় ভাবা দ্বীনি জ্ঞানের আদব নয়।","কুরআন শেখার সঙ্গে আমল ও আল্লাহভীতি থাকা দরকার।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E39" s="4" t="n"/>
@@ -1393,12 +1389,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>136</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন জ্ঞান নিয়ে অহংকারের ভয়","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন পড়ে নিজেকে বড় মনে করা কল্যাণের পথ নয়; হাদিসটি জ্ঞান নিয়ে অহংকার থেকে সতর্ক করে।"},"heading":{"title":"কুরআন জ্ঞান নিয়ে অহংকার: নিজের শ্রেষ্ঠত্ব দাবি নয়","description":"এই হাদিসে এমন একদল মানুষের কথা এসেছে যারা কুরআন পড়বে এবং বলবে—আমাদের চেয়ে বেশি কুরআন কে পড়তে পারে, আমাদের চেয়ে বেশি জ্ঞানী কে, আমাদের চেয়ে বেশি বুঝে কে? রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) সাহাবীদের জিজ্ঞেস করলেন, তাদের মধ্যে কি কোনো কল্যাণ আছে? পরে তিনি জানালেন, তারা উম্মতেরই অন্তর্ভুক্ত, কিন্তু তারা জাহান্নামের ইন্ধন হবে। হাদিসটির মূল সতর্কতা হলো—কুরআন পড়া, জ্ঞান অর্জন করা বা বুঝ থাকার দাবি যদি অহংকারে পরিণত হয়, তা বিপজ্জনক। কুরআনের সঙ্গে বিনয়, আমল ও আল্লাহভীতি থাকতে হবে; আত্মপ্রশংসা নয়।"},"teachings":["কুরআন পড়া নিয়ে অহংকার করা ভয়ংকর ভুল।","জ্ঞান ও বুঝের দাবি মানুষকে বিনয়ী না করলে তা ক্ষতির কারণ হতে পারে।","নিজেকে অন্যদের চেয়ে বড় ভাবা দ্বীনি জ্ঞানের আদব নয়।","কুরআন শেখার সঙ্গে আমল ও আল্লাহভীতি থাকা দরকার।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | একই বিষয়ের অতিরিক্ত সূত্র","description":"$book_name$ $hadith_number$ - $chapter_name$. আব্বাস (রাঃ) সূত্রে একই সতর্কতা এসেছে—কুরআন ও জ্ঞান যেন অহংকারের কারণ না হয়।"},"heading":{"title":"কুরআন জ্ঞান ও বিনয়: অতিরিক্ত সূত্রের শিক্ষা","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, উক্ত হাদিসটি আবু ইয়া'লা, বাযযার ও ত্বাবরানী আব্বাস বিন আবদুল মুত্তালিব থেকে বর্ণনা করেছেন। এটি আগের বিষয়ের আরেকটি সূত্র হিসেবে বোঝায় যে, কুরআন শেখা, পড়া ও জানা—এসব বড় নেয়ামত হলেও এগুলো নিয়ে নিজের শ্রেষ্ঠত্ব দাবি করা ঠিক নয়। কুরআনের জ্ঞান মানুষকে আল্লাহর সামনে বিনয়ী করবে, নিজের অহংকার বাড়াবে না। কেউ যদি বলে, আমাদের চেয়ে কে বেশি জানে বা কে বেশি পড়ে—তাহলে তার কথায় আত্মপ্রশংসার গন্ধ থাকে। হাদিসের শিক্ষা হলো, জ্ঞান যত বাড়ে, নিজের ভয় ও বিনয়ও তত বাড়া উচিত।"},"teachings":["একই সতর্কতা বিভিন্ন সূত্রে আসা বিষয়টির গুরুত্ব বোঝায়।","কুরআন জানা ও পড়া বিনয়ের কারণ হওয়া উচিত।","নিজেকে অন্যদের চেয়ে বড় মনে করা জ্ঞানের আদব নয়।","জ্ঞানকে আমল ও আল্লাহভীতির সঙ্গে রাখা দরকার।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E40" s="4" t="n"/>
@@ -1416,12 +1412,12 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>137</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | একই বিষয়ের অতিরিক্ত সূত্র","description":"$book_name$ $hadith_number$ - $chapter_name$. আব্বাস (রাঃ) সূত্রে একই সতর্কতা এসেছে—কুরআন ও জ্ঞান যেন অহংকারের কারণ না হয়।"},"heading":{"title":"কুরআন জ্ঞান ও বিনয়: অতিরিক্ত সূত্রের শিক্ষা","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, উক্ত হাদিসটি আবু ইয়া'লা, বাযযার ও ত্বাবরানী আব্বাস বিন আবদুল মুত্তালিব থেকে বর্ণনা করেছেন। এটি আগের বিষয়ের আরেকটি সূত্র হিসেবে বোঝায় যে, কুরআন শেখা, পড়া ও জানা—এসব বড় নেয়ামত হলেও এগুলো নিয়ে নিজের শ্রেষ্ঠত্ব দাবি করা ঠিক নয়। কুরআনের জ্ঞান মানুষকে আল্লাহর সামনে বিনয়ী করবে, নিজের অহংকার বাড়াবে না। কেউ যদি বলে, আমাদের চেয়ে কে বেশি জানে বা কে বেশি পড়ে—তাহলে তার কথায় আত্মপ্রশংসার গন্ধ থাকে। হাদিসের শিক্ষা হলো, জ্ঞান যত বাড়ে, নিজের ভয় ও বিনয়ও তত বাড়া উচিত।"},"teachings":["একই সতর্কতা বিভিন্ন সূত্রে আসা বিষয়টির গুরুত্ব বোঝায়।","কুরআন জানা ও পড়া বিনয়ের কারণ হওয়া উচিত।","নিজেকে অন্যদের চেয়ে বড় মনে করা জ্ঞানের আদব নয়।","জ্ঞানকে আমল ও আল্লাহভীতির সঙ্গে রাখা দরকার।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন শেখার পর অহংকার নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন শিখে ‘আমাদের চেয়ে উত্তম কে’ বলা অহংকারের লক্ষণ; হাদিসটি বিনয়ের শিক্ষা দেয়।"},"heading":{"title":"কুরআন শেখার পর বিনয়: আত্মপ্রশংসা থেকে সতর্কতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) ইসলামের বিজয় ও বিস্তারের কথা বলার পর এমন এক সময়ের কথা বলেছেন, যখন মানুষ কুরআন শিক্ষা করবে, পড়বে এবং বলবে—আমরা পড়েছি ও জেনেছি; আমাদের চেয়ে উত্তম আর কে আছে? তিনি জিজ্ঞেস করলেন, তাদের মধ্যে কি কল্যাণ আছে? পরে জানালেন, তারা উম্মতেরই অন্তর্ভুক্ত এবং জাহান্নামের ইন্ধন হবে। হাদিসটি স্পষ্টভাবে শেখায়, কুরআন শেখা ও জানা বড় নেয়ামত, কিন্তু সেটি যদি অহংকার, আত্মপ্রশংসা ও অন্যকে ছোট দেখানোর পথে যায়, তবে তা ভয়ংকর। কুরআনের সঙ্গে বিনয়, আমল ও আল্লাহর ভয় থাকা দরকার।"},"teachings":["কুরআন শেখার পর নিজের শ্রেষ্ঠত্ব দাবি করা উচিত নয়।","জ্ঞান অহংকার বাড়ালে তা বিপজ্জনক হতে পারে।","কুরআন পড়া ও জানা আমল ও বিনয়ের সঙ্গে যুক্ত হওয়া দরকার।","আত্মপ্রশংসা থেকে বেঁচে থাকা দ্বীনি আদবের অংশ।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E41" s="4" t="n"/>
@@ -1439,12 +1435,12 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>138</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন শেখার পর অহংকার নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন শিখে ‘আমাদের চেয়ে উত্তম কে’ বলা অহংকারের লক্ষণ; হাদিসটি বিনয়ের শিক্ষা দেয়।"},"heading":{"title":"কুরআন শেখার পর বিনয়: আত্মপ্রশংসা থেকে সতর্কতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) ইসলামের বিজয় ও বিস্তারের কথা বলার পর এমন এক সময়ের কথা বলেছেন, যখন মানুষ কুরআন শিক্ষা করবে, পড়বে এবং বলবে—আমরা পড়েছি ও জেনেছি; আমাদের চেয়ে উত্তম আর কে আছে? তিনি জিজ্ঞেস করলেন, তাদের মধ্যে কি কল্যাণ আছে? পরে জানালেন, তারা উম্মতেরই অন্তর্ভুক্ত এবং জাহান্নামের ইন্ধন হবে। হাদিসটি স্পষ্টভাবে শেখায়, কুরআন শেখা ও জানা বড় নেয়ামত, কিন্তু সেটি যদি অহংকার, আত্মপ্রশংসা ও অন্যকে ছোট দেখানোর পথে যায়, তবে তা ভয়ংকর। কুরআনের সঙ্গে বিনয়, আমল ও আল্লাহর ভয় থাকা দরকার।"},"teachings":["কুরআন শেখার পর নিজের শ্রেষ্ঠত্ব দাবি করা উচিত নয়।","জ্ঞান অহংকার বাড়ালে তা বিপজ্জনক হতে পারে।","কুরআন পড়া ও জানা আমল ও বিনয়ের সঙ্গে যুক্ত হওয়া দরকার।","আত্মপ্রশংসা থেকে বেঁচে থাকা দ্বীনি আদবের অংশ।"],"related_hadiths":[{"id":"2382","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"3267","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঝগড়া ছাড়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. বাতিল ও সত্য বিষয়েও ঝগড়া ছাড়ার ফজিলত এবং সুন্দর চরিত্রের মর্যাদা এই হাদিসে এসেছে।"},"heading":{"title":"ঝগড়া ছাড়ার ফজিলত ও সুন্দর চরিত্র","description":"এই হাদিসে ঝগড়া পরিত্যাগ ও সুন্দর চরিত্রের বড় ফজিলত বলা হয়েছে। যে ব্যক্তি বাতিল বিষয় নিয়ে ঝগড়া ছেড়ে দেয়, তার জন্য জান্নাতের আশেপাশে ঘরের কথা এসেছে। আর সত্য বিষয়ে থাকা সত্ত্বেও যে ঝগড়া ছেড়ে দেয়, তার জন্য জান্নাতের মধ্যভাগে ঘরের কথা বলা হয়েছে। যে নিজের চরিত্র সুন্দর করে, তার জন্য জান্নাতের উঁচু স্থানে ঘরের কথা এসেছে। হাদিসটি আমাদের শেখায়, সব কথা জিতে যাওয়ার চেষ্টা করা ভালো পথ নয়। অনেক সময় চুপ থাকা, ঝগড়া না বাড়ানো এবং চরিত্র ভালো রাখা বেশি কল্যাণকর। সত্য থাকলেও অহংকার ও তর্কপ্রবণতা থেকে বাঁচা দরকার।"},"teachings":["বাতিল বিষয়ে ঝগড়া না করা মুমিনের সুন্দর গুণ।","সত্য পাশে থাকলেও ঝগড়া না বাড়ানো বড় চরিত্রের পরিচয়।","সুন্দর চরিত্র জান্নাতের মর্যাদা লাভের কারণ হতে পারে।","জেতার জন্য তর্ক না করে শান্তি ও আদব রক্ষা করা উচিত।"],"related_hadiths":[{"id":"4800","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1993","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"51","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E42" s="4" t="n"/>
@@ -1462,12 +1458,12 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঝগড়া ছাড়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. বাতিল ও সত্য বিষয়েও ঝগড়া ছাড়ার ফজিলত এবং সুন্দর চরিত্রের মর্যাদা এই হাদিসে এসেছে।"},"heading":{"title":"ঝগড়া ছাড়ার ফজিলত ও সুন্দর চরিত্র","description":"এই হাদিসে ঝগড়া পরিত্যাগ ও সুন্দর চরিত্রের বড় ফজিলত বলা হয়েছে। যে ব্যক্তি বাতিল বিষয় নিয়ে ঝগড়া ছেড়ে দেয়, তার জন্য জান্নাতের আশেপাশে ঘরের কথা এসেছে। আর সত্য বিষয়ে থাকা সত্ত্বেও যে ঝগড়া ছেড়ে দেয়, তার জন্য জান্নাতের মধ্যভাগে ঘরের কথা বলা হয়েছে। যে নিজের চরিত্র সুন্দর করে, তার জন্য জান্নাতের উঁচু স্থানে ঘরের কথা এসেছে। হাদিসটি আমাদের শেখায়, সব কথা জিতে যাওয়ার চেষ্টা করা ভালো পথ নয়। অনেক সময় চুপ থাকা, ঝগড়া না বাড়ানো এবং চরিত্র ভালো রাখা বেশি কল্যাণকর। সত্য থাকলেও অহংকার ও তর্কপ্রবণতা থেকে বাঁচা দরকার।"},"teachings":["বাতিল বিষয়ে ঝগড়া না করা মুমিনের সুন্দর গুণ।","সত্য পাশে থাকলেও ঝগড়া না বাড়ানো বড় চরিত্রের পরিচয়।","সুন্দর চরিত্র জান্নাতের মর্যাদা লাভের কারণ হতে পারে।","জেতার জন্য তর্ক না করে শান্তি ও আদব রক্ষা করা উচিত।"],"related_hadiths":[{"id":"4800","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1993","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"51","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মিথ্যা ও ঝগড়া ছাড়ার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. সত্য হয়েও ঝগড়া ছাড়া, ঠাট্টাতেও মিথ্যা না বলা ও চরিত্র সুন্দর করার ফজিলত এসেছে।"},"heading":{"title":"ঠাট্টাতেও মিথ্যা নয়, সত্য হয়েও ঝগড়া নয়","description":"এই হাদিসে তিনটি সুন্দর গুণের কথা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন ব্যক্তির জন্য জান্নাতের বিভিন্ন স্থানে ঘরের জিম্মাদার হওয়ার কথা বলেছেন, যে সত্যবাদী হয়েও অনর্থক ঝগড়া ছাড়ে, ঠাট্টা করেও মিথ্যা বলে না, এবং নিজের চরিত্র সুন্দর করে। এখানে ঝগড়া, মিথ্যা ও চরিত্র—তিনটি বিষয় একসঙ্গে এসেছে। অনেক সময় মানুষ ঠাট্টার নামে মিথ্যা বলে, বা সত্য পাশে আছে বলে তর্ক বাড়াতে থাকে। হাদিসটি শেখায়, সত্যবাদিতা শুধু গম্ভীর কথায় নয়; হাসি-ঠাট্টার সময়ও সত্য থাকা দরকার। আর সুন্দর চরিত্র মানুষের দ্বীনি জীবনের বড় অংশ।"},"teachings":["সত্য পাশে থাকলেও অনর্থক ঝগড়া ছেড়ে দেওয়া প্রশংসনীয়।","ঠাট্টা করেও মিথ্যা বলা থেকে বাঁচা উচিত।","সুন্দর চরিত্র আল্লাহর কাছে মর্যাদার কারণ হতে পারে।","ভালো মুসলিম হওয়ার জন্য কথা ও আচরণ দুটোই ঠিক রাখা দরকার।"],"related_hadiths":[{"id":"4800","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1993","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"51","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E43" s="4" t="n"/>
@@ -1485,12 +1481,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মিথ্যা ও ঝগড়া ছাড়ার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. সত্য হয়েও ঝগড়া ছাড়া, ঠাট্টাতেও মিথ্যা না বলা ও চরিত্র সুন্দর করার ফজিলত এসেছে।"},"heading":{"title":"ঠাট্টাতেও মিথ্যা নয়, সত্য হয়েও ঝগড়া নয়","description":"এই হাদিসে তিনটি সুন্দর গুণের কথা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন ব্যক্তির জন্য জান্নাতের বিভিন্ন স্থানে ঘরের জিম্মাদার হওয়ার কথা বলেছেন, যে সত্যবাদী হয়েও অনর্থক ঝগড়া ছাড়ে, ঠাট্টা করেও মিথ্যা বলে না, এবং নিজের চরিত্র সুন্দর করে। এখানে ঝগড়া, মিথ্যা ও চরিত্র—তিনটি বিষয় একসঙ্গে এসেছে। অনেক সময় মানুষ ঠাট্টার নামে মিথ্যা বলে, বা সত্য পাশে আছে বলে তর্ক বাড়াতে থাকে। হাদিসটি শেখায়, সত্যবাদিতা শুধু গম্ভীর কথায় নয়; হাসি-ঠাট্টার সময়ও সত্য থাকা দরকার। আর সুন্দর চরিত্র মানুষের দ্বীনি জীবনের বড় অংশ।"},"teachings":["সত্য পাশে থাকলেও অনর্থক ঝগড়া ছেড়ে দেওয়া প্রশংসনীয়।","ঠাট্টা করেও মিথ্যা বলা থেকে বাঁচা উচিত।","সুন্দর চরিত্র আল্লাহর কাছে মর্যাদার কারণ হতে পারে।","ভালো মুসলিম হওয়ার জন্য কথা ও আচরণ দুটোই ঠিক রাখা দরকার।"],"related_hadiths":[{"id":"4800","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1993","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"51","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাশরে নিয়তের ভিত্তিতে সমাবেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. এই বর্ণনায় বলা হয়েছে, মানুষকে হাশরের মাঠে একত্র করা হবে তাদের নিয়ত অনুযায়ী।"},"heading":{"title":"হাশরের মাঠে নিয়ত: অন্তরের অবস্থার গুরুত্ব","description":"এই অংশে আগের অর্থের কাছাকাছি আরেকটি বর্ণনার কথা এসেছে। ইবনে মাজাহ জাবের রাদিয়াল্লাহু আনহু থেকেও এটি বর্ণনা করেছেন, তবে এখানে শব্দ এসেছে—মানুষকে হাশরের মাঠে একত্রিত করা হবে তাদের নিয়ত অনুযায়ী। এই সংক্ষিপ্ত বাক্য নিয়তের গুরুত্বকে আখিরাতের সাথে যুক্ত করে। দুনিয়ায় মানুষ অনেক সময় বাহ্যিক পরিচয়, দল, কাজ বা অবস্থার কারণে একসাথে দেখা যায়। কিন্তু হাশরের দিনে আল্লাহর কাছে অন্তরের উদ্দেশ্যও গুরুত্বপূর্ণ হবে। তাই একজন মুসলিমের উচিত শুধু কাজের বাহ্যিক রূপ ঠিক করা নয়; ভেতরের লক্ষ্যও ঠিক রাখা। হাদিসটি বেশি কথা নয়, বরং গভীর সতর্কতা দেয়। আল্লাহর সন্তুষ্টির জন্য ভালো কাজ করা এবং মন্দ উদ্দেশ্য থেকে বাঁচা—এটাই এর সহজ শিক্ষা।"},"teachings":["হাশরের মাঠে মানুষের নিয়ত গুরুত্বপূর্ণ হবে।","বাহ্যিক কাজের সাথে অন্তরের উদ্দেশ্যও ঠিক রাখা দরকার।","আল্লাহর সন্তুষ্টির নিয়ত মুমিনের মূল লক্ষ্য হওয়া উচিত।","সংক্ষিপ্ত হাদিস থেকেও বড় শিক্ষা নেওয়া যায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2118","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E44" s="4" t="n"/>
@@ -1508,12 +1504,12 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>140</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাশরে নিয়তের ভিত্তিতে সমাবেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. এই বর্ণনায় বলা হয়েছে, মানুষকে হাশরের মাঠে একত্র করা হবে তাদের নিয়ত অনুযায়ী।"},"heading":{"title":"হাশরের মাঠে নিয়ত: অন্তরের অবস্থার গুরুত্ব","description":"এই অংশে আগের অর্থের কাছাকাছি আরেকটি বর্ণনার কথা এসেছে। ইবনে মাজাহ জাবের রাদিয়াল্লাহু আনহু থেকেও এটি বর্ণনা করেছেন, তবে এখানে শব্দ এসেছে—মানুষকে হাশরের মাঠে একত্রিত করা হবে তাদের নিয়ত অনুযায়ী। এই সংক্ষিপ্ত বাক্য নিয়তের গুরুত্বকে আখিরাতের সাথে যুক্ত করে। দুনিয়ায় মানুষ অনেক সময় বাহ্যিক পরিচয়, দল, কাজ বা অবস্থার কারণে একসাথে দেখা যায়। কিন্তু হাশরের দিনে আল্লাহর কাছে অন্তরের উদ্দেশ্যও গুরুত্বপূর্ণ হবে। তাই একজন মুসলিমের উচিত শুধু কাজের বাহ্যিক রূপ ঠিক করা নয়; ভেতরের লক্ষ্যও ঠিক রাখা। হাদিসটি বেশি কথা নয়, বরং গভীর সতর্কতা দেয়। আল্লাহর সন্তুষ্টির জন্য ভালো কাজ করা এবং মন্দ উদ্দেশ্য থেকে বাঁচা—এটাই এর সহজ শিক্ষা।"},"teachings":["হাশরের মাঠে মানুষের নিয়ত গুরুত্বপূর্ণ হবে।","বাহ্যিক কাজের সাথে অন্তরের উদ্দেশ্যও ঠিক রাখা দরকার।","আল্লাহর সন্তুষ্টির নিয়ত মুমিনের মূল লক্ষ্য হওয়া উচিত।","সংক্ষিপ্ত হাদিস থেকেও বড় শিক্ষা নেওয়া যায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2118","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আয়াত নিয়ে ঝগড়া থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআনের আয়াত টেনে পরস্পর ঝগড়ায় জড়ানো থেকে নবীজি সতর্ক করেছেন এবং বিভেদ এড়াতে বলেছেন।"},"heading":{"title":"কুরআনের আয়াত নিয়ে ঝগড়া নয়: একতার শিক্ষা","description":"এই হাদিসে সাহাবীরা রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর দরজায় বসে আলোচনা করছিলেন। একজন একটি আয়াত টানছিলেন, আরেকজন আরেকটি আয়াত। তখন নবীজি বের হয়ে কঠোরভাবে সতর্ক করলেন। তিনি বললেন, তোমাদের কি এ জন্য প্রেরণ করা হয়েছে, নাকি এ বিষয়ে আদেশ করা হয়েছে? তারপর তিনি সতর্ক করলেন, তাঁর পরে যেন তারা কাফেরদের মতো না হয়ে যায়, যেখানে একজন আরেকজনের ঘাড় মটকাবে। হাদিসটির শিক্ষা হলো, কুরআনের আয়াতকে ঝগড়া, রাগ বা দলাদলির হাতিয়ার বানানো ঠিক নয়। কুরআন মানুষকে হেদায়াত, একতা ও আল্লাহর পথে চলার জন্য এসেছে; ঝগড়া বাড়ানোর জন্য নয়।"},"teachings":["কুরআনের আয়াত নিয়ে ঝগড়া ও দলাদলি করা থেকে বাঁচা উচিত।","দ্বীনি আলোচনা আদব ও শান্তির সঙ্গে হওয়া দরকার।","আয়াতকে পরস্পরকে হারানোর অস্ত্র বানানো ঠিক নয়।","মুসলিমদের মধ্যে বিভেদ ও সংঘাত থেকে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4987","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5669","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E45" s="4" t="n"/>
@@ -1531,12 +1527,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আয়াত নিয়ে ঝগড়া থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআনের আয়াত টেনে পরস্পর ঝগড়ায় জড়ানো থেকে নবীজি সতর্ক করেছেন এবং বিভেদ এড়াতে বলেছেন।"},"heading":{"title":"কুরআনের আয়াত নিয়ে ঝগড়া নয়: একতার শিক্ষা","description":"এই হাদিসে সাহাবীরা রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর দরজায় বসে আলোচনা করছিলেন। একজন একটি আয়াত টানছিলেন, আরেকজন আরেকটি আয়াত। তখন নবীজি বের হয়ে কঠোরভাবে সতর্ক করলেন। তিনি বললেন, তোমাদের কি এ জন্য প্রেরণ করা হয়েছে, নাকি এ বিষয়ে আদেশ করা হয়েছে? তারপর তিনি সতর্ক করলেন, তাঁর পরে যেন তারা কাফেরদের মতো না হয়ে যায়, যেখানে একজন আরেকজনের ঘাড় মটকাবে। হাদিসটির শিক্ষা হলো, কুরআনের আয়াতকে ঝগড়া, রাগ বা দলাদলির হাতিয়ার বানানো ঠিক নয়। কুরআন মানুষকে হেদায়াত, একতা ও আল্লাহর পথে চলার জন্য এসেছে; ঝগড়া বাড়ানোর জন্য নয়।"},"teachings":["কুরআনের আয়াত নিয়ে ঝগড়া ও দলাদলি করা থেকে বাঁচা উচিত।","দ্বীনি আলোচনা আদব ও শান্তির সঙ্গে হওয়া দরকার।","আয়াতকে পরস্পরকে হারানোর অস্ত্র বানানো ঠিক নয়।","মুসলিমদের মধ্যে বিভেদ ও সংঘাত থেকে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"5060","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4987","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5669","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুটতর্ক থেকে সতর্ক থাকার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. হেদায়াতের পর কুটতর্কে জড়ানো পথভ্রষ্টতার লক্ষণ—এই হাদিস বিতর্কপ্রিয়তা থেকে সতর্ক করে।"},"heading":{"title":"কুটতর্ক থেকে বাঁচার হাদিস: হেদায়াতের পর বিতর্কপ্রিয়তা","description":"এই হাদিসে রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কুটতর্কের ভয়াবহ দিকটি খুব পরিষ্কারভাবে বলেছেন। কোনো জাতি হেদায়াতের উপর থাকার পর যখন পথভ্রষ্ট হয়, তখন তাদেরকে কুট বিতর্কে জড়িয়ে দেওয়া হয়। এখানে মূল শিক্ষা হলো, সত্য জানার পর অহেতুক ঝগড়া-বিতর্কে মেতে ওঠা ভালো লক্ষণ নয়। মানুষ যখন হেদায়াত, কুরআনের শিক্ষা ও সঠিক পথের বদলে তর্ক জেতাকে বড় করে দেখে, তখন তার মন নরম থাকে না। হাদিসে রাসূলুল্লাহ্ (সা.) সূরা যুখরুফের আয়াতও পড়েছেন, যেখানে বলা হয়েছে যে তারা উদাহরণ দেয় শুধু বিতর্কের জন্য। তাই কুটতর্ক থেকে বাঁচা, হেদায়াতের উপর থাকা এবং সত্যের সামনে বিনয়ী থাকা একজন মুমিনের জন্য জরুরি শিক্ষা।"},"teachings":["হেদায়াত পাওয়ার পর অহেতুক কুটতর্কে জড়ানো বিপজ্জনক লক্ষণ।","সত্য বোঝার উদ্দেশ্যে কথা বলা ভালো, কিন্তু তর্ক জেতার মনোভাব ক্ষতিকর।","কুরআনের আয়াতকে বিতর্কের হাতিয়ার বানানো থেকে সতর্ক থাকতে হবে।","হেদায়াতের উপর টিকে থাকতে বিনয় ও সংযম দরকার।"],"related_hadiths":[{"id":"48","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3253","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"180","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E46" s="4" t="n"/>
@@ -1554,12 +1550,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>142</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুটতর্ক থেকে সতর্ক থাকার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. হেদায়াতের পর কুটতর্কে জড়ানো পথভ্রষ্টতার লক্ষণ—এই হাদিস বিতর্কপ্রিয়তা থেকে সতর্ক করে।"},"heading":{"title":"কুটতর্ক থেকে বাঁচার হাদিস: হেদায়াতের পর বিতর্কপ্রিয়তা","description":"এই হাদিসে রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কুটতর্কের ভয়াবহ দিকটি খুব পরিষ্কারভাবে বলেছেন। কোনো জাতি হেদায়াতের উপর থাকার পর যখন পথভ্রষ্ট হয়, তখন তাদেরকে কুট বিতর্কে জড়িয়ে দেওয়া হয়। এখানে মূল শিক্ষা হলো, সত্য জানার পর অহেতুক ঝগড়া-বিতর্কে মেতে ওঠা ভালো লক্ষণ নয়। মানুষ যখন হেদায়াত, কুরআনের শিক্ষা ও সঠিক পথের বদলে তর্ক জেতাকে বড় করে দেখে, তখন তার মন নরম থাকে না। হাদিসে রাসূলুল্লাহ্ (সা.) সূরা যুখরুফের আয়াতও পড়েছেন, যেখানে বলা হয়েছে যে তারা উদাহরণ দেয় শুধু বিতর্কের জন্য। তাই কুটতর্ক থেকে বাঁচা, হেদায়াতের উপর থাকা এবং সত্যের সামনে বিনয়ী থাকা একজন মুমিনের জন্য জরুরি শিক্ষা।"},"teachings":["হেদায়াত পাওয়ার পর অহেতুক কুটতর্কে জড়ানো বিপজ্জনক লক্ষণ।","সত্য বোঝার উদ্দেশ্যে কথা বলা ভালো, কিন্তু তর্ক জেতার মনোভাব ক্ষতিকর।","কুরআনের আয়াতকে বিতর্কের হাতিয়ার বানানো থেকে সতর্ক থাকতে হবে।","হেদায়াতের উপর টিকে থাকতে বিনয় ও সংযম দরকার।"],"related_hadiths":[{"id":"48","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3253","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"180","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুটতর্ককারীর অপছন্দনীয় স্বভাব","description":"$book_name$ $hadith_number$ - $chapter_name$. সর্বদা কুটতর্কে লিপ্ত মানুষ আল্লাহর নিকট ঘৃণিত—এই হাদিস কথায় সংযম শেখায়।"},"heading":{"title":"কুটতর্ককারী মানুষ সম্পর্কে হাদিস: কথায় সংযমের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন মানুষের কথা বলেছেন, যে সবসময় কুটতর্ক করে। হাদিসের ভাষায়, আল্লাহর নিকট সবচেয়ে ঘৃণিত মানুষ হলো সর্বদা কুটতর্ককারী। এখানে কোর টপিক হলো কুটতর্ক ও ঝগড়াটে স্বভাব। একজন মানুষ যদি সত্য বোঝার জন্য কথা বলে, তা আলাদা বিষয়। কিন্তু যদি সে সবসময় কথার লড়াই করতে চায়, নিজের কথা চাপিয়ে দিতে চায়, আর বিরোধ তৈরি করে, তাহলে এই স্বভাব নিন্দনীয়। হাদিসটি আমাদের শেখায়, জ্ঞান থাকলেও বিনয় থাকা দরকার। কথা বলার সময় লক্ষ্য হওয়া উচিত সত্য, কল্যাণ ও শান্তি; শুধু কাউকে হারানো নয়। তাই কুটতর্ক থেকে বাঁচা, নরম ভাষা ব্যবহার করা এবং অকারণ ঝগড়া এড়িয়ে চলা এই হাদিসের বড় শিক্ষা।"},"teachings":["সর্বদা কুটতর্ক করা আল্লাহর নিকট অপছন্দনীয় স্বভাব।","কথা বলার উদ্দেশ্য সত্য বোঝা হওয়া উচিত, ঝগড়া করা নয়।","নিজের ভাষা ও আচরণে সংযম রাখা জরুরি।","বিতর্কপ্রিয়তা মানুষের চরিত্রকে ক্ষতিগ্রস্ত করতে পারে।"],"related_hadiths":[{"id":"4523","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2976","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"6781","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E47" s="4" t="n"/>
@@ -1577,12 +1573,12 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুটতর্ককারীর অপছন্দনীয় স্বভাব","description":"$book_name$ $hadith_number$ - $chapter_name$. সর্বদা কুটতর্কে লিপ্ত মানুষ আল্লাহর নিকট ঘৃণিত—এই হাদিস কথায় সংযম শেখায়।"},"heading":{"title":"কুটতর্ককারী মানুষ সম্পর্কে হাদিস: কথায় সংযমের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এমন মানুষের কথা বলেছেন, যে সবসময় কুটতর্ক করে। হাদিসের ভাষায়, আল্লাহর নিকট সবচেয়ে ঘৃণিত মানুষ হলো সর্বদা কুটতর্ককারী। এখানে কোর টপিক হলো কুটতর্ক ও ঝগড়াটে স্বভাব। একজন মানুষ যদি সত্য বোঝার জন্য কথা বলে, তা আলাদা বিষয়। কিন্তু যদি সে সবসময় কথার লড়াই করতে চায়, নিজের কথা চাপিয়ে দিতে চায়, আর বিরোধ তৈরি করে, তাহলে এই স্বভাব নিন্দনীয়। হাদিসটি আমাদের শেখায়, জ্ঞান থাকলেও বিনয় থাকা দরকার। কথা বলার সময় লক্ষ্য হওয়া উচিত সত্য, কল্যাণ ও শান্তি; শুধু কাউকে হারানো নয়। তাই কুটতর্ক থেকে বাঁচা, নরম ভাষা ব্যবহার করা এবং অকারণ ঝগড়া এড়িয়ে চলা এই হাদিসের বড় শিক্ষা।"},"teachings":["সর্বদা কুটতর্ক করা আল্লাহর নিকট অপছন্দনীয় স্বভাব।","কথা বলার উদ্দেশ্য সত্য বোঝা হওয়া উচিত, ঝগড়া করা নয়।","নিজের ভাষা ও আচরণে সংযম রাখা জরুরি।","বিতর্কপ্রিয়তা মানুষের চরিত্রকে ক্ষতিগ্রস্ত করতে পারে।"],"related_hadiths":[{"id":"4523","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2976","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"6781","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন নিয়ে কুটতর্কের ভয়াবহতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন নিয়ে কুটতর্কে জড়ানো গুরুতর বিষয়—এই হাদিস কুরআনের সামনে বিনয় শেখায়।"},"heading":{"title":"কুরআন নিয়ে কুটতর্কের হাদিস: ঈমান ও বিনয়ের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কুরআন নিয়ে কুটতর্ক করার বিষয়ে কঠোর সতর্কতা দিয়েছেন। তিনি বলেছেন, কুরআন নিয়ে কুটতর্কে লিপ্ত হওয়া কুফরী। এখানে মূল বিষয় হলো কুরআনের প্রতি আদব ও বিনয়। কুরআন আল্লাহর কালাম; তাই একে নিজের জেদ, অহংকার বা কথার লড়াইয়ের জায়গা বানানো ঠিক নয়। কেউ যদি বুঝতে না পারে, সে জিজ্ঞেস করবে। কেউ যদি শিখতে চায়, সে বিনয়ের সাথে শিখবে। কিন্তু কুরআনের আয়াত নিয়ে জেদি তর্ক, অপব্যাখ্যা বা অহেতুক বিরোধ তৈরি করা এই হাদিসের আলোকে ভয়াবহ কাজ। তাই কুরআন নিয়ে কথা বলার সময় সতর্কতা, শ্রদ্ধা এবং সত্য জানার নিয়ত রাখা জরুরি।"},"teachings":["কুরআন নিয়ে কুটতর্ক করা গুরুতর সতর্কতার বিষয়।","কুরআনের সামনে বিনয় ও আদব রাখা জরুরি।","না বুঝলে জেদ না করে জিজ্ঞেস করা উচিত।","কুরআনের আয়াতকে অহেতুক বিতর্কের বিষয় বানানো থেকে বাঁচতে হবে।"],"related_hadiths":[{"id":"4603","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"180","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"48","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E48" s="4" t="n"/>
@@ -1600,12 +1596,12 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>145</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন নিয়ে কুটতর্কের ভয়াবহতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন নিয়ে কুটতর্কে জড়ানো গুরুতর বিষয়—এই হাদিস কুরআনের সামনে বিনয় শেখায়।"},"heading":{"title":"কুরআন নিয়ে কুটতর্কের হাদিস: ঈমান ও বিনয়ের শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কুরআন নিয়ে কুটতর্ক করার বিষয়ে কঠোর সতর্কতা দিয়েছেন। তিনি বলেছেন, কুরআন নিয়ে কুটতর্কে লিপ্ত হওয়া কুফরী। এখানে মূল বিষয় হলো কুরআনের প্রতি আদব ও বিনয়। কুরআন আল্লাহর কালাম; তাই একে নিজের জেদ, অহংকার বা কথার লড়াইয়ের জায়গা বানানো ঠিক নয়। কেউ যদি বুঝতে না পারে, সে জিজ্ঞেস করবে। কেউ যদি শিখতে চায়, সে বিনয়ের সাথে শিখবে। কিন্তু কুরআনের আয়াত নিয়ে জেদি তর্ক, অপব্যাখ্যা বা অহেতুক বিরোধ তৈরি করা এই হাদিসের আলোকে ভয়াবহ কাজ। তাই কুরআন নিয়ে কথা বলার সময় সতর্কতা, শ্রদ্ধা এবং সত্য জানার নিয়ত রাখা জরুরি।"},"teachings":["কুরআন নিয়ে কুটতর্ক করা গুরুতর সতর্কতার বিষয়।","কুরআনের সামনে বিনয় ও আদব রাখা জরুরি।","না বুঝলে জেদ না করে জিজ্ঞেস করা উচিত।","কুরআনের আয়াতকে অহেতুক বিতর্কের বিষয় বানানো থেকে বাঁচতে হবে।"],"related_hadiths":[{"id":"4603","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"180","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"48","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাস্তা ও ছায়ায় শৌচকার্য থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের চলার রাস্তা ও ব্যবহৃত ছায়ায় পেশাব-পায়খানা লা‘নত ডেকে আনে—এই হাদিস পরিচ্ছন্নতা শেখায়।"},"heading":{"title":"রাস্তা ও ছায়ায় পেশাব-পায়খানা নিষেধ: পরিচ্ছন্নতার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুইটি কাজ থেকে বেঁচে থাকতে বলেছেন, যা লা‘নত ডেকে আনে। সাহাবিরা জানতে চাইলেন, সে কাজ দু’টি কী? তিনি বললেন, মানুষের চলাচলের রাস্তায় অথবা তাদের ছায়ায় পেশাব-পায়খানা করা। এখানে মূল শিক্ষা হলো জনসাধারণের জায়গা নোংরা করা থেকে বিরত থাকা। রাস্তা মানুষ ব্যবহার করে, আর ছায়ার জায়গাও মানুষ বিশ্রামের জন্য নেয়। এসব স্থানে শৌচকার্য করলে অন্য মানুষ কষ্ট পায় এবং পরিবেশ নোংরা হয়। ইসলামে পবিত্রতা শুধু ব্যক্তিগত বিষয় নয়; অন্যের আরাম ও নিরাপত্তাও এর সাথে জড়িত। তাই পাবলিক রাস্তা, বসার স্থান, ছায়া বা মানুষের ব্যবহৃত জায়গা পরিষ্কার রাখা এই হাদিসের সরাসরি শিক্ষা।"},"teachings":["মানুষের চলার রাস্তা নোংরা করা থেকে বাঁচতে হবে।","যে ছায়া মানুষ ব্যবহার করে সেখানে পেশাব-পায়খানা করা নিষিদ্ধ।","নিজের কাজের কারণে অন্যকে কষ্ট দেওয়া ঠিক নয়।","ইসলামে পরিচ্ছন্নতা সামাজিক দায়িত্বের অংশ।"],"related_hadiths":[{"id":"506","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"146","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E49" s="4" t="n"/>
@@ -1623,12 +1619,12 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>146</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাস্তা ও ছায়ায় শৌচকার্য থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের চলার রাস্তা ও ব্যবহৃত ছায়ায় পেশাব-পায়খানা লা‘নত ডেকে আনে—এই হাদিস পরিচ্ছন্নতা শেখায়।"},"heading":{"title":"রাস্তা ও ছায়ায় পেশাব-পায়খানা নিষেধ: পরিচ্ছন্নতার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুইটি কাজ থেকে বেঁচে থাকতে বলেছেন, যা লা‘নত ডেকে আনে। সাহাবিরা জানতে চাইলেন, সে কাজ দু’টি কী? তিনি বললেন, মানুষের চলাচলের রাস্তায় অথবা তাদের ছায়ায় পেশাব-পায়খানা করা। এখানে মূল শিক্ষা হলো জনসাধারণের জায়গা নোংরা করা থেকে বিরত থাকা। রাস্তা মানুষ ব্যবহার করে, আর ছায়ার জায়গাও মানুষ বিশ্রামের জন্য নেয়। এসব স্থানে শৌচকার্য করলে অন্য মানুষ কষ্ট পায় এবং পরিবেশ নোংরা হয়। ইসলামে পবিত্রতা শুধু ব্যক্তিগত বিষয় নয়; অন্যের আরাম ও নিরাপত্তাও এর সাথে জড়িত। তাই পাবলিক রাস্তা, বসার স্থান, ছায়া বা মানুষের ব্যবহৃত জায়গা পরিষ্কার রাখা এই হাদিসের সরাসরি শিক্ষা।"},"teachings":["মানুষের চলার রাস্তা নোংরা করা থেকে বাঁচতে হবে।","যে ছায়া মানুষ ব্যবহার করে সেখানে পেশাব-পায়খানা করা নিষিদ্ধ।","নিজের কাজের কারণে অন্যকে কষ্ট দেওয়া ঠিক নয়।","ইসলামে পরিচ্ছন্নতা সামাজিক দায়িত্বের অংশ।"],"related_hadiths":[{"id":"506","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"146","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তিন লা‘নতের স্থান থেকে বাঁচার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. পানির ঘাট, চলার রাস্তা ও মানুষের ছায়ায় শৌচকার্য থেকে বাঁচতে এই হাদিস সতর্ক করে।"},"heading":{"title":"তিন লা‘নতের স্থান: পানির ঘাট, রাস্তা ও ছায়ায় শৌচকার্য নিষেধ","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) তিনটি লা‘নতের স্থান থেকে বেঁচে থাকতে বলেছেন। এগুলো হলো পানির ঘাট, চলাচলের রাস্তা এবং যে স্থানের ছায়ায় মানুষ আশ্রয় নেয়। এই তিন জায়গায় পেশাব-পায়খানা করলে মানুষের কষ্ট হয়। পানির ঘাট মানুষের প্রয়োজনের জায়গা। রাস্তা সবার চলাচলের জন্য। আর ছায়া মানুষ বিশ্রাম বা আশ্রয়ের জন্য ব্যবহার করে। তাই এসব জায়গা নোংরা করা শুধু ব্যক্তিগত ভুল নয়, অন্যের অধিকার নষ্ট করার মতো আচরণ। হাদিসটি আমাদের শেখায়, পবিত্রতা ও পরিচ্ছন্নতা এমন বিষয় যা মানুষের সুবিধা, স্বাস্থ্য ও সম্মানের সাথে জড়িত। মুসলমানের আচরণ হওয়া উচিত এমন, যাতে অন্যরা তার কারণে বিরক্ত না হয়।"},"teachings":["পানির ঘাটে পেশাব-পায়খানা করা থেকে বাঁচতে হবে।","চলাচলের রাস্তা সবার অধিকার, তা নোংরা করা ঠিক নয়।","মানুষ যে ছায়ায় আশ্রয় নেয়, সেটি পরিষ্কার রাখা দরকার।","পরিচ্ছন্নতা রক্ষা করা অন্যের কষ্ট দূর করার একটি উপায়।"],"related_hadiths":[{"id":"26","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"328","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E50" s="4" t="n"/>
@@ -1646,12 +1642,12 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তিন লা‘নতের স্থান থেকে বাঁচার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. পানির ঘাট, চলার রাস্তা ও মানুষের ছায়ায় শৌচকার্য থেকে বাঁচতে এই হাদিস সতর্ক করে।"},"heading":{"title":"তিন লা‘নতের স্থান: পানির ঘাট, রাস্তা ও ছায়ায় শৌচকার্য নিষেধ","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) তিনটি লা‘নতের স্থান থেকে বেঁচে থাকতে বলেছেন। এগুলো হলো পানির ঘাট, চলাচলের রাস্তা এবং যে স্থানের ছায়ায় মানুষ আশ্রয় নেয়। এই তিন জায়গায় পেশাব-পায়খানা করলে মানুষের কষ্ট হয়। পানির ঘাট মানুষের প্রয়োজনের জায়গা। রাস্তা সবার চলাচলের জন্য। আর ছায়া মানুষ বিশ্রাম বা আশ্রয়ের জন্য ব্যবহার করে। তাই এসব জায়গা নোংরা করা শুধু ব্যক্তিগত ভুল নয়, অন্যের অধিকার নষ্ট করার মতো আচরণ। হাদিসটি আমাদের শেখায়, পবিত্রতা ও পরিচ্ছন্নতা এমন বিষয় যা মানুষের সুবিধা, স্বাস্থ্য ও সম্মানের সাথে জড়িত। মুসলমানের আচরণ হওয়া উচিত এমন, যাতে অন্যরা তার কারণে বিরক্ত না হয়।"},"teachings":["পানির ঘাটে পেশাব-পায়খানা করা থেকে বাঁচতে হবে।","চলাচলের রাস্তা সবার অধিকার, তা নোংরা করা ঠিক নয়।","মানুষ যে ছায়ায় আশ্রয় নেয়, সেটি পরিষ্কার রাখা দরকার।","পরিচ্ছন্নতা রক্ষা করা অন্যের কষ্ট দূর করার একটি উপায়।"],"related_hadiths":[{"id":"26","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"328","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ছায়া, রাস্তা ও জমা পানিতে শৌচকার্য নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ যে ছায়া নেয়, রাস্তা ও জমা পানির স্থানে শৌচকার্য থেকে বাঁচার শিক্ষা দেয় এই হাদিস।"},"heading":{"title":"জমা পানি, রাস্তা ও ছায়ায় শৌচকার্য নিষেধ: পবিত্রতার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) তিনটি অভিশাপের স্থান থেকে বেঁচে থাকতে বলেছেন। প্রশ্ন করা হলে তিনি বলেন, কেউ যেন এমন ছায়ায় না বসে যেখানে মানুষ ছায়া নেয়, রাস্তায় না বসে এবং যেখানে পানি জমে থাকে সেখানে না বসে। এখানে বসা বলতে পেশাব-পায়খানার জন্য বসা বোঝানো হয়েছে। হাদিসটি খুব বাস্তব শিক্ষা দেয়। মানুষের ব্যবহার করা জায়গা নোংরা করলে মানুষ বিরক্ত হয়, কষ্ট পায় এবং ক্ষতি হতে পারে। জমা পানি নোংরা করা আরও কষ্টের কারণ হতে পারে, কারণ পানি অনেকের প্রয়োজনের সাথে যুক্ত। তাই ইসলাম মানুষকে শুধু নিজের পবিত্রতার কথা বলে না, বরং জনসাধারণের জায়গা পরিষ্কার রাখতেও শেখায়।"},"teachings":["মানুষের ব্যবহৃত ছায়ার জায়গা নোংরা করা থেকে বাঁচতে হবে।","রাস্তায় শৌচকার্য করা মানুষের কষ্টের কারণ।","জমা পানির স্থানে পেশাব-পায়খানা করা নিষিদ্ধ কাজের অন্তর্ভুক্ত।","পবিত্রতা মানে নিজের সঙ্গে অন্যের সুবিধার কথাও ভাবা।"],"related_hadiths":[{"id":"146","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"6","book_id":"9","slug":"bulugul-maram","label":"বুলুগুল মারাম"},{"id":"26","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E51" s="4" t="n"/>
@@ -1669,12 +1665,12 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>148</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ছায়া, রাস্তা ও জমা পানিতে শৌচকার্য নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ যে ছায়া নেয়, রাস্তা ও জমা পানির স্থানে শৌচকার্য থেকে বাঁচার শিক্ষা দেয় এই হাদিস।"},"heading":{"title":"জমা পানি, রাস্তা ও ছায়ায় শৌচকার্য নিষেধ: পবিত্রতার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) তিনটি অভিশাপের স্থান থেকে বেঁচে থাকতে বলেছেন। প্রশ্ন করা হলে তিনি বলেন, কেউ যেন এমন ছায়ায় না বসে যেখানে মানুষ ছায়া নেয়, রাস্তায় না বসে এবং যেখানে পানি জমে থাকে সেখানে না বসে। এখানে বসা বলতে পেশাব-পায়খানার জন্য বসা বোঝানো হয়েছে। হাদিসটি খুব বাস্তব শিক্ষা দেয়। মানুষের ব্যবহার করা জায়গা নোংরা করলে মানুষ বিরক্ত হয়, কষ্ট পায় এবং ক্ষতি হতে পারে। জমা পানি নোংরা করা আরও কষ্টের কারণ হতে পারে, কারণ পানি অনেকের প্রয়োজনের সাথে যুক্ত। তাই ইসলাম মানুষকে শুধু নিজের পবিত্রতার কথা বলে না, বরং জনসাধারণের জায়গা পরিষ্কার রাখতেও শেখায়।"},"teachings":["মানুষের ব্যবহৃত ছায়ার জায়গা নোংরা করা থেকে বাঁচতে হবে।","রাস্তায় শৌচকার্য করা মানুষের কষ্টের কারণ।","জমা পানির স্থানে পেশাব-পায়খানা করা নিষিদ্ধ কাজের অন্তর্ভুক্ত।","পবিত্রতা মানে নিজের সঙ্গে অন্যের সুবিধার কথাও ভাবা।"],"related_hadiths":[{"id":"146","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"6","book_id":"9","slug":"bulugul-maram","label":"বুলুগুল মারাম"},{"id":"26","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাস্তায় মুসলিমদের কষ্ট দেওয়া নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মুসলমানদের চলার পথে কষ্ট দেওয়া লা‘নতের কারণ—এই হাদিস জনপথের অধিকার শেখায়।"},"heading":{"title":"রাস্তার অধিকার সম্পর্কে হাদিস: মুসলমানদের কষ্ট দেওয়া থেকে বাঁচুন","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি মুসলমানদের চলাচলের রাস্তায় তাদেরকে কষ্ট দিল, তার উপর তাদের লা‘নত আবশ্যক হয়ে গেল। এখানে মূল শিক্ষা হলো রাস্তায় অন্যকে কষ্ট দেওয়া থেকে বেঁচে থাকা। কষ্ট দেওয়া অনেকভাবে হতে পারে, কিন্তু এই হাদিসের সরাসরি ভাষা হলো মুসলমানদের চলার পথে কষ্ট দেওয়া। রাস্তা সবার চলাচলের জায়গা। সেখানে এমন কিছু করা উচিত নয়, যার কারণে মানুষ বিরক্ত, বাধাগ্রস্ত বা কষ্টে পড়ে। ইসলামের সৌন্দর্য হলো, এটি মানুষের ইবাদতের পাশাপাশি সামাজিক আচরণও ঠিক করে দেয়। একজন মুসলিমের পরিচয় শুধু নিজের ভালো আমলে নয়, বরং তার কারণে অন্য মানুষ নিরাপদ ও স্বস্তিতে আছে কি না—সেটিও গুরুত্বপূর্ণ।"},"teachings":["মানুষের চলাচলের পথে কষ্ট দেওয়া থেকে বিরত থাকতে হবে।","রাস্তা সবার ব্যবহারের জায়গা, তাই তা নিরাপদ রাখা দরকার।","নিজের আচরণের কারণে অন্য মুসলমান কষ্ট পাচ্ছে কি না, তা ভাবতে হবে।","ইসলামে সামাজিক দায়িত্ব ও পরিচ্ছন্ন আচরণের গুরুত্ব আছে।"],"related_hadiths":[{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"506","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E52" s="4" t="n"/>
@@ -1692,12 +1688,12 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>149</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাস্তায় মুসলিমদের কষ্ট দেওয়া নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মুসলমানদের চলার পথে কষ্ট দেওয়া লা‘নতের কারণ—এই হাদিস জনপথের অধিকার শেখায়।"},"heading":{"title":"রাস্তার অধিকার সম্পর্কে হাদিস: মুসলমানদের কষ্ট দেওয়া থেকে বাঁচুন","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি মুসলমানদের চলাচলের রাস্তায় তাদেরকে কষ্ট দিল, তার উপর তাদের লা‘নত আবশ্যক হয়ে গেল। এখানে মূল শিক্ষা হলো রাস্তায় অন্যকে কষ্ট দেওয়া থেকে বেঁচে থাকা। কষ্ট দেওয়া অনেকভাবে হতে পারে, কিন্তু এই হাদিসের সরাসরি ভাষা হলো মুসলমানদের চলার পথে কষ্ট দেওয়া। রাস্তা সবার চলাচলের জায়গা। সেখানে এমন কিছু করা উচিত নয়, যার কারণে মানুষ বিরক্ত, বাধাগ্রস্ত বা কষ্টে পড়ে। ইসলামের সৌন্দর্য হলো, এটি মানুষের ইবাদতের পাশাপাশি সামাজিক আচরণও ঠিক করে দেয়। একজন মুসলিমের পরিচয় শুধু নিজের ভালো আমলে নয়, বরং তার কারণে অন্য মানুষ নিরাপদ ও স্বস্তিতে আছে কি না—সেটিও গুরুত্বপূর্ণ।"},"teachings":["মানুষের চলাচলের পথে কষ্ট দেওয়া থেকে বিরত থাকতে হবে।","রাস্তা সবার ব্যবহারের জায়গা, তাই তা নিরাপদ রাখা দরকার।","নিজের আচরণের কারণে অন্য মুসলমান কষ্ট পাচ্ছে কি না, তা ভাবতে হবে।","ইসলামে সামাজিক দায়িত্ব ও পরিচ্ছন্ন আচরণের গুরুত্ব আছে।"],"related_hadiths":[{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"506","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের রাস্তায় অবস্থান ও শৌচকার্য থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের রাস্তার মধ্যভাগে থাকা ও সেখানে শৌচকার্য করা থেকে হাদিসটি সতর্ক করে।"},"heading":{"title":"রাতের রাস্তায় অবস্থান ও শৌচকার্য নিষেধ: নিরাপত্তা ও আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) রাতের বেলায় রাস্তার মধ্যভাগে অবস্থান নেওয়া থেকে সাবধান করেছেন। কারণ হিসেবে বলা হয়েছে, তা সাপ ও হিংস্র প্রাণীদের আশ্রয়স্থল হতে পারে। একই সঙ্গে রাস্তার উপর প্রয়োজন পূরণ বা শৌচকার্য থেকেও সাবধান করা হয়েছে, কারণ তা অভিশাপের কাজের অন্তর্ভুক্ত। এখানে দুটি শিক্ষা একসাথে এসেছে। প্রথমটি নিরাপত্তা সম্পর্কিত—রাতের রাস্তায় থাকা ঝুঁকির কারণ হতে পারে। দ্বিতীয়টি পরিচ্ছন্নতা ও মানুষের অধিকার সম্পর্কিত—চলাচলের পথে শৌচকার্য করা অন্যদের কষ্ট দেয়। তাই এই হাদিস মুসলিমকে সাবধান, পরিচ্ছন্ন এবং অন্যের সুবিধার প্রতি যত্নশীল হতে শেখায়।"},"teachings":["রাতে রাস্তার মধ্যভাগে অবস্থান নেওয়া থেকে সাবধান থাকতে হবে।","রাস্তা সাপ ও হিংস্র প্রাণীর আশ্রয় হতে পারে—এই সতর্কতা হাদিসে এসেছে।","রাস্তার উপর শৌচকার্য করা অভিশাপের কাজের অন্তর্ভুক্ত।","নিরাপত্তা ও পরিচ্ছন্নতা—দুই দিকেই সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"148","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E53" s="4" t="n"/>
@@ -1715,12 +1711,12 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাতের রাস্তায় অবস্থান ও শৌচকার্য থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতের রাস্তার মধ্যভাগে থাকা ও সেখানে শৌচকার্য করা থেকে হাদিসটি সতর্ক করে।"},"heading":{"title":"রাতের রাস্তায় অবস্থান ও শৌচকার্য নিষেধ: নিরাপত্তা ও আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) রাতের বেলায় রাস্তার মধ্যভাগে অবস্থান নেওয়া থেকে সাবধান করেছেন। কারণ হিসেবে বলা হয়েছে, তা সাপ ও হিংস্র প্রাণীদের আশ্রয়স্থল হতে পারে। একই সঙ্গে রাস্তার উপর প্রয়োজন পূরণ বা শৌচকার্য থেকেও সাবধান করা হয়েছে, কারণ তা অভিশাপের কাজের অন্তর্ভুক্ত। এখানে দুটি শিক্ষা একসাথে এসেছে। প্রথমটি নিরাপত্তা সম্পর্কিত—রাতের রাস্তায় থাকা ঝুঁকির কারণ হতে পারে। দ্বিতীয়টি পরিচ্ছন্নতা ও মানুষের অধিকার সম্পর্কিত—চলাচলের পথে শৌচকার্য করা অন্যদের কষ্ট দেয়। তাই এই হাদিস মুসলিমকে সাবধান, পরিচ্ছন্ন এবং অন্যের সুবিধার প্রতি যত্নশীল হতে শেখায়।"},"teachings":["রাতে রাস্তার মধ্যভাগে অবস্থান নেওয়া থেকে সাবধান থাকতে হবে।","রাস্তা সাপ ও হিংস্র প্রাণীর আশ্রয় হতে পারে—এই সতর্কতা হাদিসে এসেছে।","রাস্তার উপর শৌচকার্য করা অভিশাপের কাজের অন্তর্ভুক্ত।","নিরাপত্তা ও পরিচ্ছন্নতা—দুই দিকেই সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"148","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহ অন্তর ও আমল দেখেন","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি শেখায়, আল্লাহ মানুষের দেহ বা চেহারা নয়; অন্তর ও আমল দেখেন।"},"heading":{"title":"আল্লাহ অন্তর ও আমল দেখেন: বাহ্যিক রূপ নয়, ভেতরের সত্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, আল্লাহ তোমাদের দেহ এবং আকার-আকৃতি দেখেন না; বরং তিনি তোমাদের অন্তর দেখেন। বর্ণনায় এসেছে, তিনি নিজের বুকের দিকে আঙুল দিয়ে ইঙ্গিত করেন। আরও বলা হয়েছে, আল্লাহ তোমাদের আমলও দেখেন। এখানে বাহ্যিক সৌন্দর্য, শক্তি, দেহ বা চেহারাকে মূল মানদণ্ড করা হয়নি। বরং অন্তরের অবস্থা এবং বাস্তব আমলকে গুরুত্ব দেওয়া হয়েছে। তাই শুধু ভালো দেখানো, সুন্দর কথা বলা বা বাহ্যিক সাজ যথেষ্ট নয়। হৃদয়ে ইখলাস থাকা এবং কাজে তা প্রমাণ হওয়া দরকার। এই হাদিস মানুষকে নিজের ভিতর ঠিক করতে শেখায়। অহংকার কমানো, অন্যকে চেহারা বা অবস্থা দিয়ে বিচার না করা, এবং নিজের আমল ঠিক রাখা—এসব শিক্ষা এতে স্পষ্টভাবে মেলে।"},"teachings":["আল্লাহ মানুষের বাহ্যিক রূপকে আসল মানদণ্ড করেন না।","অন্তরের অবস্থা ও আমল আল্লাহর কাছে গুরুত্বপূর্ণ।","শুধু ভালো দেখানো যথেষ্ট নয়; কাজও ভালো হওয়া দরকার।","অন্যকে চেহারা বা দেহ দেখে বিচার করা থেকে বাঁচা উচিত।"],"related_hadiths":[{"id":"8","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E54" s="4" t="n"/>
@@ -1738,12 +1734,12 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>150</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহ অন্তর ও আমল দেখেন","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি শেখায়, আল্লাহ মানুষের দেহ বা চেহারা নয়; অন্তর ও আমল দেখেন।"},"heading":{"title":"আল্লাহ অন্তর ও আমল দেখেন: বাহ্যিক রূপ নয়, ভেতরের সত্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, আল্লাহ তোমাদের দেহ এবং আকার-আকৃতি দেখেন না; বরং তিনি তোমাদের অন্তর দেখেন। বর্ণনায় এসেছে, তিনি নিজের বুকের দিকে আঙুল দিয়ে ইঙ্গিত করেন। আরও বলা হয়েছে, আল্লাহ তোমাদের আমলও দেখেন। এখানে বাহ্যিক সৌন্দর্য, শক্তি, দেহ বা চেহারাকে মূল মানদণ্ড করা হয়নি। বরং অন্তরের অবস্থা এবং বাস্তব আমলকে গুরুত্ব দেওয়া হয়েছে। তাই শুধু ভালো দেখানো, সুন্দর কথা বলা বা বাহ্যিক সাজ যথেষ্ট নয়। হৃদয়ে ইখলাস থাকা এবং কাজে তা প্রমাণ হওয়া দরকার। এই হাদিস মানুষকে নিজের ভিতর ঠিক করতে শেখায়। অহংকার কমানো, অন্যকে চেহারা বা অবস্থা দিয়ে বিচার না করা, এবং নিজের আমল ঠিক রাখা—এসব শিক্ষা এতে স্পষ্টভাবে মেলে।"},"teachings":["আল্লাহ মানুষের বাহ্যিক রূপকে আসল মানদণ্ড করেন না।","অন্তরের অবস্থা ও আমল আল্লাহর কাছে গুরুত্বপূর্ণ।","শুধু ভালো দেখানো যথেষ্ট নয়; কাজও ভালো হওয়া দরকার।","অন্যকে চেহারা বা দেহ দেখে বিচার করা থেকে বাঁচা উচিত।"],"related_hadiths":[{"id":"8","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদের দরজার পাশে প্রস্রাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদের দরজার আশপাশে প্রস্রাব করতে নিষেধ করা হয়েছে—এটি মসজিদের সম্মান ও পরিচ্ছন্নতার শিক্ষা।"},"heading":{"title":"মসজিদের দরজার পাশে প্রস্রাব নিষেধ: মসজিদের আদব","description":"এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) মসজিদের দরজার আশেপাশে প্রস্রাব করতে নিষেধ করেছেন। এখানে মূল শিক্ষা হলো মসজিদের সম্মান ও পরিচ্ছন্নতা রক্ষা করা। মসজিদ হলো ইবাদতের স্থান। মানুষ সেখানে সালাত, দোয়া ও আল্লাহর স্মরণের জন্য আসে। তাই মসজিদের প্রবেশপথ বা আশেপাশের জায়গা নোংরা করা মসজিদের আদবের বিপরীত। হাদিসটি আমাদের মনে করিয়ে দেয়, পবিত্রতা শুধু মসজিদের ভেতরে নয়; মসজিদের চারপাশের পরিবেশেও দরকার। যে জায়গা দিয়ে মানুষ মসজিদে প্রবেশ করে, সেটি পরিষ্কার ও কষ্টমুক্ত রাখা উচিত। এই হাদিসের শিক্ষা সহজ—ইবাদতের স্থানকে সম্মান করতে হলে তার পরিচ্ছন্নতাও রক্ষা করতে হবে।"},"teachings":["মসজিদের দরজার আশেপাশে প্রস্রাব করা নিষিদ্ধ।","মসজিদের সম্মান রক্ষায় আশপাশ পরিষ্কার রাখা দরকার।","ইবাদতের স্থানে মানুষের কষ্টের কারণ হওয়া ঠিক নয়।","পবিত্রতা মসজিদের ভেতর ও বাইরের পরিবেশের সাথেও যুক্ত।"],"related_hadiths":[{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"148","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E55" s="4" t="n"/>
@@ -1761,12 +1757,12 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>152</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদের দরজার পাশে প্রস্রাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদের দরজার আশপাশে প্রস্রাব করতে নিষেধ করা হয়েছে—এটি মসজিদের সম্মান ও পরিচ্ছন্নতার শিক্ষা।"},"heading":{"title":"মসজিদের দরজার পাশে প্রস্রাব নিষেধ: মসজিদের আদব","description":"এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ্ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) মসজিদের দরজার আশেপাশে প্রস্রাব করতে নিষেধ করেছেন। এখানে মূল শিক্ষা হলো মসজিদের সম্মান ও পরিচ্ছন্নতা রক্ষা করা। মসজিদ হলো ইবাদতের স্থান। মানুষ সেখানে সালাত, দোয়া ও আল্লাহর স্মরণের জন্য আসে। তাই মসজিদের প্রবেশপথ বা আশেপাশের জায়গা নোংরা করা মসজিদের আদবের বিপরীত। হাদিসটি আমাদের মনে করিয়ে দেয়, পবিত্রতা শুধু মসজিদের ভেতরে নয়; মসজিদের চারপাশের পরিবেশেও দরকার। যে জায়গা দিয়ে মানুষ মসজিদে প্রবেশ করে, সেটি পরিষ্কার ও কষ্টমুক্ত রাখা উচিত। এই হাদিসের শিক্ষা সহজ—ইবাদতের স্থানকে সম্মান করতে হলে তার পরিচ্ছন্নতাও রক্ষা করতে হবে।"},"teachings":["মসজিদের দরজার আশেপাশে প্রস্রাব করা নিষিদ্ধ।","মসজিদের সম্মান রক্ষায় আশপাশ পরিষ্কার রাখা দরকার।","ইবাদতের স্থানে মানুষের কষ্টের কারণ হওয়া ঠিক নয়।","পবিত্রতা মসজিদের ভেতর ও বাইরের পরিবেশের সাথেও যুক্ত।"],"related_hadiths":[{"id":"145","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"148","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"25","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্থির পানিতে পেশাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. স্থির পানিতে পেশাব করতে নিষেধ করা হয়েছে—এই হাদিস পানি পরিষ্কার রাখার শিক্ষা দেয়।"},"heading":{"title":"স্থির পানিতে পেশাব করা নিষেধ: পানি পবিত্র রাখার হাদিস","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) স্থির পানিতে পেশাব করতে নিষেধ করেছেন। এখানে মূল শিক্ষা খুব সহজ—যে পানি স্থির আছে, সেটি নোংরা করা যাবে না। পানি মানুষের প্রয়োজনীয় জিনিস। কেউ তা ব্যবহার করতে পারে, কেউ তা থেকে উপকার নিতে পারে। স্থির পানিতে পেশাব করলে পানি নোংরা হয় এবং অন্যের ব্যবহারের জন্য কষ্টের কারণ হতে পারে। হাদিসটি আমাদের শেখায়, পবিত্রতা শুধু শরীরের সাথে নয়; পানির মতো সাধারণ সম্পদ রক্ষার সাথেও যুক্ত। মুসলিমের আচরণ এমন হওয়া উচিত, যাতে তার কারণে কোনো প্রয়োজনীয় জিনিস নষ্ট না হয়। তাই পানি পরিষ্কার রাখা, অপবিত্রতা থেকে বাঁচা এবং অন্যের সুবিধার কথা ভাবা এই হাদিসের সরাসরি শিক্ষা।"},"teachings":["স্থির পানিতে পেশাব করা থেকে বাঁচতে হবে।","পানি মানুষের প্রয়োজনের জিনিস, তা নোংরা করা ঠিক নয়।","পবিত্রতা পরিবেশ ও সাধারণ সম্পদের সাথেও যুক্ত।","নিজের কাজের কারণে অন্যের ব্যবহারযোগ্য পানি নষ্ট করা উচিত নয়।"],"related_hadiths":[{"id":"6","book_id":"9","slug":"bulugul-maram","label":"বুলুগুল মারাম"},{"id":"564","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"35","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
         </is>
       </c>
       <c r="E56" s="4" t="n"/>
@@ -1784,12 +1780,12 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>153</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্থির পানিতে পেশাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. স্থির পানিতে পেশাব করতে নিষেধ করা হয়েছে—এই হাদিস পানি পরিষ্কার রাখার শিক্ষা দেয়।"},"heading":{"title":"স্থির পানিতে পেশাব করা নিষেধ: পানি পবিত্র রাখার হাদিস","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) স্থির পানিতে পেশাব করতে নিষেধ করেছেন। এখানে মূল শিক্ষা খুব সহজ—যে পানি স্থির আছে, সেটি নোংরা করা যাবে না। পানি মানুষের প্রয়োজনীয় জিনিস। কেউ তা ব্যবহার করতে পারে, কেউ তা থেকে উপকার নিতে পারে। স্থির পানিতে পেশাব করলে পানি নোংরা হয় এবং অন্যের ব্যবহারের জন্য কষ্টের কারণ হতে পারে। হাদিসটি আমাদের শেখায়, পবিত্রতা শুধু শরীরের সাথে নয়; পানির মতো সাধারণ সম্পদ রক্ষার সাথেও যুক্ত। মুসলিমের আচরণ এমন হওয়া উচিত, যাতে তার কারণে কোনো প্রয়োজনীয় জিনিস নষ্ট না হয়। তাই পানি পরিষ্কার রাখা, অপবিত্রতা থেকে বাঁচা এবং অন্যের সুবিধার কথা ভাবা এই হাদিসের সরাসরি শিক্ষা।"},"teachings":["স্থির পানিতে পেশাব করা থেকে বাঁচতে হবে।","পানি মানুষের প্রয়োজনের জিনিস, তা নোংরা করা ঠিক নয়।","পবিত্রতা পরিবেশ ও সাধারণ সম্পদের সাথেও যুক্ত।","নিজের কাজের কারণে অন্যের ব্যবহারযোগ্য পানি নষ্ট করা উচিত নয়।"],"related_hadiths":[{"id":"6","book_id":"9","slug":"bulugul-maram","label":"বুলুগুল মারাম"},{"id":"564","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"35","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে পেশাব জমা রাখা ও গোসলখানায় পেশাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে পাত্রে পেশাব জমা রাখা ও গোসলখানায় পেশাব করতে নিষেধ—এটি পবিত্রতার শিক্ষা।"},"heading":{"title":"ঘরে পেশাব জমা রাখা নিষেধ: গোসলখানায় পেশাব থেকে সতর্কতা","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুটি বিষয়ে নিষেধ করেছেন। এক, ঘরের মধ্যে কোনো পাত্রে পেশাব জমা রাখা উচিত নয়। কারণ যে ঘরে পেশাব জমা থাকে, সেখানে রহমতের ফেরেশতা প্রবেশ করে না—হাদিসে এ কথা এসেছে। দুই, গোসলখানায় পেশাব করতে নিষেধ করা হয়েছে। এখানে মূল শিক্ষা হলো ঘর ও গোসলের জায়গা পবিত্র রাখা। ঘর মানুষের থাকার জায়গা, আর গোসলখানা শরীর পরিষ্কারের জায়গা। এসব জায়গা নোংরা হলে পবিত্রতা ও আরামের ক্ষতি হয়। এই হাদিস মুসলমানকে শেখায়, পবিত্রতা শুধু বাহ্যিক নয়; ঘরের পরিবেশ, ব্যবহারযোগ্য পাত্র এবং গোসলের স্থান—সবই পরিষ্কার রাখার বিষয়।"},"teachings":["ঘরে পাত্রে পেশাব জমা রাখা থেকে বাঁচতে হবে।","গোসলখানায় পেশাব করা নিষেধ হিসেবে এসেছে।","ঘর ও গোসলের স্থান পরিষ্কার রাখা পবিত্রতার অংশ।","নোংরা জিনিস ঘরে রেখে দেওয়া থেকে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"27","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"304","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"21","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E57" s="4" t="n"/>
@@ -1807,12 +1803,12 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঘরে পেশাব জমা রাখা ও গোসলখানায় পেশাব নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. ঘরে পাত্রে পেশাব জমা রাখা ও গোসলখানায় পেশাব করতে নিষেধ—এটি পবিত্রতার শিক্ষা।"},"heading":{"title":"ঘরে পেশাব জমা রাখা নিষেধ: গোসলখানায় পেশাব থেকে সতর্কতা","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুটি বিষয়ে নিষেধ করেছেন। এক, ঘরের মধ্যে কোনো পাত্রে পেশাব জমা রাখা উচিত নয়। কারণ যে ঘরে পেশাব জমা থাকে, সেখানে রহমতের ফেরেশতা প্রবেশ করে না—হাদিসে এ কথা এসেছে। দুই, গোসলখানায় পেশাব করতে নিষেধ করা হয়েছে। এখানে মূল শিক্ষা হলো ঘর ও গোসলের জায়গা পবিত্র রাখা। ঘর মানুষের থাকার জায়গা, আর গোসলখানা শরীর পরিষ্কারের জায়গা। এসব জায়গা নোংরা হলে পবিত্রতা ও আরামের ক্ষতি হয়। এই হাদিস মুসলমানকে শেখায়, পবিত্রতা শুধু বাহ্যিক নয়; ঘরের পরিবেশ, ব্যবহারযোগ্য পাত্র এবং গোসলের স্থান—সবই পরিষ্কার রাখার বিষয়।"},"teachings":["ঘরে পাত্রে পেশাব জমা রাখা থেকে বাঁচতে হবে।","গোসলখানায় পেশাব করা নিষেধ হিসেবে এসেছে।","ঘর ও গোসলের স্থান পরিষ্কার রাখা পবিত্রতার অংশ।","নোংরা জিনিস ঘরে রেখে দেওয়া থেকে সতর্ক থাকা দরকার।"],"related_hadiths":[{"id":"27","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"304","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"21","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোসলখানায় পেশাব ও অতিরিক্ত সাজগোজে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রতিদিন চুল আঁচড়ানো ও গোসলখানায় পেশাব থেকে নিষেধ এসেছে—এই হাদিস সংযম ও পবিত্রতা শেখায়।"},"heading":{"title":"গোসলখানায় পেশাব নিষেধ ও দৈনন্দিন সংযমের হাদিস","description":"এই হাদিসে একজন সাহাবীর মাধ্যমে বর্ণিত হয়েছে যে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) প্রতিদিন চুল আঁচড়াতে বা গোসলখানায় পেশাব করতে নিষেধ করেছেন। এখানে দুটি বিষয় আছে। প্রথমটি হলো প্রতিদিন চুল আঁচড়ানো নিয়ে সংযমের শিক্ষা, যা হাদিসের সরাসরি ভাষায় এসেছে। দ্বিতীয়টি হলো গোসলখানায় পেশাব না করা। গোসলখানা শরীর পরিষ্কার করার জায়গা, তাই সেখানে পেশাব করা পবিত্রতার আদবের বিপরীত। হাদিসটি আমাদের দৈনন্দিন জীবনের ছোট কাজেও শিষ্টতা শেখায়। পরিচ্ছন্নতা মানে শুধু গোসল করা নয়; গোসলের জায়গাটিও নোংরা না করা। আর সাজসজ্জার ক্ষেত্রেও অতিরিক্ত অভ্যাস থেকে দূরে থাকা—এই বর্ণনার একটি সহজ শিক্ষা।"},"teachings":["গোসলখানায় পেশাব করা থেকে বাঁচতে হবে।","গোসলের জায়গা পরিষ্কার রাখা পবিত্রতার অংশ।","দৈনন্দিন সাজগোজেও সংযমের শিক্ষা আছে।","ছোট অভ্যাসও ইসলামী আদবের আওতায় আসে।"],"related_hadiths":[{"id":"28","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"27","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"304","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E58" s="4" t="n"/>
@@ -1830,12 +1826,12 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>155</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোসলখানায় পেশাব ও অতিরিক্ত সাজগোজে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রতিদিন চুল আঁচড়ানো ও গোসলখানায় পেশাব থেকে নিষেধ এসেছে—এই হাদিস সংযম ও পবিত্রতা শেখায়।"},"heading":{"title":"গোসলখানায় পেশাব নিষেধ ও দৈনন্দিন সংযমের হাদিস","description":"এই হাদিসে একজন সাহাবীর মাধ্যমে বর্ণিত হয়েছে যে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) প্রতিদিন চুল আঁচড়াতে বা গোসলখানায় পেশাব করতে নিষেধ করেছেন। এখানে দুটি বিষয় আছে। প্রথমটি হলো প্রতিদিন চুল আঁচড়ানো নিয়ে সংযমের শিক্ষা, যা হাদিসের সরাসরি ভাষায় এসেছে। দ্বিতীয়টি হলো গোসলখানায় পেশাব না করা। গোসলখানা শরীর পরিষ্কার করার জায়গা, তাই সেখানে পেশাব করা পবিত্রতার আদবের বিপরীত। হাদিসটি আমাদের দৈনন্দিন জীবনের ছোট কাজেও শিষ্টতা শেখায়। পরিচ্ছন্নতা মানে শুধু গোসল করা নয়; গোসলের জায়গাটিও নোংরা না করা। আর সাজসজ্জার ক্ষেত্রেও অতিরিক্ত অভ্যাস থেকে দূরে থাকা—এই বর্ণনার একটি সহজ শিক্ষা।"},"teachings":["গোসলখানায় পেশাব করা থেকে বাঁচতে হবে।","গোসলের জায়গা পরিষ্কার রাখা পবিত্রতার অংশ।","দৈনন্দিন সাজগোজেও সংযমের শিক্ষা আছে।","ছোট অভ্যাসও ইসলামী আদবের আওতায় আসে।"],"related_hadiths":[{"id":"28","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"27","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"304","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শৌচকার্যে লজ্জাশীলতা ও গোপনীয়তা","description":"$book_name$ $hadith_number$ - $chapter_name$. শৌচকার্যে একে অপরের লজ্জাস্থান দেখা ও কথাবার্তা থেকে নিষেধ—এটি লজ্জাশীলতার শিক্ষা।"},"heading":{"title":"শৌচকার্যে লজ্জাশীলতা: গোপনীয়তা রক্ষার হাদিস","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দু’জন মানুষ যেন একত্রে শৌচকার্যে বসে পরস্পরে গোপনে কথাবার্তা না বলে এবং একজন অপরজনের লজ্জাস্থান না দেখে। কারণ আল্লাহ তা ঘৃণা করেন। এখানে মূল শিক্ষা হলো লজ্জাশীলতা, গোপনীয়তা এবং শৌচকার্যের আদব। শৌচকার্য মানুষের ব্যক্তিগত বিষয়। সেখানে লজ্জাস্থান উন্মুক্ত থাকে, তাই অন্যের দিকে তাকানো বা কথা বলতে বসা শোভন নয়। হাদিসে বিষয়টি শুধু সামাজিক ভদ্রতা হিসেবে নয়, আল্লাহর অপছন্দনীয় কাজ হিসেবে এসেছে। তাই একজন মুসলিমকে একান্ত প্রয়োজনের সময়ও নিজের লজ্জাস্থান ঢাকার চেষ্টা করতে হবে, অন্যের দিকে তাকানো থেকে বাঁচতে হবে এবং অকারণ কথাবার্তা এড়িয়ে চলতে হবে।"},"teachings":["শৌচকার্যে গোপনীয়তা ও লজ্জাশীলতা রক্ষা করতে হবে।","একজন অন্যজনের লজ্জাস্থান দেখা থেকে বাঁচতে হবে।","শৌচকার্যের সময় কথাবার্তা বলা এই হাদিসে অপছন্দনীয় হিসেবে এসেছে।","আল্লাহ যা ঘৃণা করেন, তা থেকে সাবধান থাকা জরুরি।"],"related_hadiths":[{"id":"15","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"342","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"156","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E59" s="4" t="n"/>
@@ -1853,12 +1849,12 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>156</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শৌচকার্যে লজ্জাশীলতা ও গোপনীয়তা","description":"$book_name$ $hadith_number$ - $chapter_name$. শৌচকার্যে একে অপরের লজ্জাস্থান দেখা ও কথাবার্তা থেকে নিষেধ—এটি লজ্জাশীলতার শিক্ষা।"},"heading":{"title":"শৌচকার্যে লজ্জাশীলতা: গোপনীয়তা রক্ষার হাদিস","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দু’জন মানুষ যেন একত্রে শৌচকার্যে বসে পরস্পরে গোপনে কথাবার্তা না বলে এবং একজন অপরজনের লজ্জাস্থান না দেখে। কারণ আল্লাহ তা ঘৃণা করেন। এখানে মূল শিক্ষা হলো লজ্জাশীলতা, গোপনীয়তা এবং শৌচকার্যের আদব। শৌচকার্য মানুষের ব্যক্তিগত বিষয়। সেখানে লজ্জাস্থান উন্মুক্ত থাকে, তাই অন্যের দিকে তাকানো বা কথা বলতে বসা শোভন নয়। হাদিসে বিষয়টি শুধু সামাজিক ভদ্রতা হিসেবে নয়, আল্লাহর অপছন্দনীয় কাজ হিসেবে এসেছে। তাই একজন মুসলিমকে একান্ত প্রয়োজনের সময়ও নিজের লজ্জাস্থান ঢাকার চেষ্টা করতে হবে, অন্যের দিকে তাকানো থেকে বাঁচতে হবে এবং অকারণ কথাবার্তা এড়িয়ে চলতে হবে।"},"teachings":["শৌচকার্যে গোপনীয়তা ও লজ্জাশীলতা রক্ষা করতে হবে।","একজন অন্যজনের লজ্জাস্থান দেখা থেকে বাঁচতে হবে।","শৌচকার্যের সময় কথাবার্তা বলা এই হাদিসে অপছন্দনীয় হিসেবে এসেছে।","আল্লাহ যা ঘৃণা করেন, তা থেকে সাবধান থাকা জরুরি।"],"related_hadiths":[{"id":"15","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"342","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"156","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শৌচকার্যে কথা বলা ও লজ্জাস্থান খোলা নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. দুজন শৌচকার্যে বসে লজ্জাস্থান উন্মুক্ত রেখে কথা বলা আল্লাহ অপছন্দ করেন—হাদিসের শিক্ষা।"},"heading":{"title":"শৌচকার্যে কথা বলা নিষেধ: লজ্জাস্থান ঢাকার আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুজন যেন শৌচকার্যে বের হয়ে একত্রে বসে লজ্জাস্থান উন্মুক্ত রেখে পরস্পরের সাথে কথা না বলে। কারণ আল্লাহ তা ঘৃণা করেন। এই বর্ণনায় বিষয়টি খুব স্পষ্টভাবে এসেছে। শৌচকার্য মানুষের একান্ত ব্যক্তিগত প্রয়োজন। সেখানে অকারণ একসাথে বসা, কথা বলা এবং লজ্জাস্থান উন্মুক্ত রাখা ইসলামী আদবের বিপরীত। হাদিসটি আমাদের শেখায়, লজ্জাশীলতা শুধু মানুষের সামনে পোশাকের বিষয় নয়; ব্যক্তিগত কাজের সময়ও তা মানতে হয়। যে কাজ আল্লাহ ঘৃণা করেন, তা থেকে দূরে থাকা একজন মুমিনের দায়িত্ব। তাই শৌচকার্যে গোপনীয়তা, নীরবতা ও সতর্কতা রাখা জরুরি।"},"teachings":["শৌচকার্যে একত্রে বসে কথাবার্তা বলা থেকে বাঁচতে হবে।","লজ্জাস্থান উন্মুক্ত রেখে অন্যের সামনে থাকা অপছন্দনীয়।","ব্যক্তিগত প্রয়োজনের সময়ও ইসলামী আদব মানা দরকার।","আল্লাহর অপছন্দনীয় কাজ থেকে সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"155","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"15","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"342","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E60" s="4" t="n"/>
@@ -1876,12 +1872,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>157</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শৌচকার্যে কথা বলা ও লজ্জাস্থান খোলা নিষেধ","description":"$book_name$ $hadith_number$ - $chapter_name$. দুজন শৌচকার্যে বসে লজ্জাস্থান উন্মুক্ত রেখে কথা বলা আল্লাহ অপছন্দ করেন—হাদিসের শিক্ষা।"},"heading":{"title":"শৌচকার্যে কথা বলা নিষেধ: লজ্জাস্থান ঢাকার আদব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুজন যেন শৌচকার্যে বের হয়ে একত্রে বসে লজ্জাস্থান উন্মুক্ত রেখে পরস্পরের সাথে কথা না বলে। কারণ আল্লাহ তা ঘৃণা করেন। এই বর্ণনায় বিষয়টি খুব স্পষ্টভাবে এসেছে। শৌচকার্য মানুষের একান্ত ব্যক্তিগত প্রয়োজন। সেখানে অকারণ একসাথে বসা, কথা বলা এবং লজ্জাস্থান উন্মুক্ত রাখা ইসলামী আদবের বিপরীত। হাদিসটি আমাদের শেখায়, লজ্জাশীলতা শুধু মানুষের সামনে পোশাকের বিষয় নয়; ব্যক্তিগত কাজের সময়ও তা মানতে হয়। যে কাজ আল্লাহ ঘৃণা করেন, তা থেকে দূরে থাকা একজন মুমিনের দায়িত্ব। তাই শৌচকার্যে গোপনীয়তা, নীরবতা ও সতর্কতা রাখা জরুরি।"},"teachings":["শৌচকার্যে একত্রে বসে কথাবার্তা বলা থেকে বাঁচতে হবে।","লজ্জাস্থান উন্মুক্ত রেখে অন্যের সামনে থাকা অপছন্দনীয়।","ব্যক্তিগত প্রয়োজনের সময়ও ইসলামী আদব মানা দরকার।","আল্লাহর অপছন্দনীয় কাজ থেকে সতর্ক থাকা উচিত।"],"related_hadiths":[{"id":"155","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"15","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"342","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চুগলখোরি ও পেশাব থেকে সতর্কতার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. কবরের আযাবের দুটি কারণ হিসেবে চুগলখোরি ও পেশাব থেকে সতর্ক না থাকার কথা এসেছে।"},"heading":{"title":"কবরের আযাব সম্পর্কে হাদিস: চুগলখোরি ও পেশাব থেকে সতর্কতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুই কবরের পাশ দিয়ে যাওয়ার সময় বলেন, তাদের দু’জনকে আযাব দেওয়া হচ্ছে। তিনি বলেন, বিষয়টি তাদের কাছে খুব বড় মনে হয়নি; কিন্তু তা বড় পাপই। একজন চুগলখোরি করত, আর অন্যজন পেশাব থেকে সতর্ক থাকত না। বর্ণনায় আরও এসেছে, একজন পেশাবের ব্যাপারে সাবধানতা অবলম্বন করত না এবং অন্যজন চুগলখোরি করে বেড়াত। এখানে দুটি মূল শিক্ষা আছে। প্রথমত, মানুষের মাঝে কথা লাগানো ভয়াবহ কাজ। দ্বিতীয়ত, পেশাবের অপবিত্রতা থেকে বাঁচা খুব গুরুত্বপূর্ণ। অনেক সময় মানুষ ছোট ভেবে কিছু কাজ অবহেলা করে, কিন্তু হাদিস দেখায়—এমন কাজ কবরের আযাবের কারণ হতে পারে।"},"teachings":["চুগলখোরি কবরের আযাবের কারণ হিসেবে এসেছে।","পেশাবের অপবিত্রতা থেকে সতর্ক থাকা জরুরি।","মানুষ যে কাজ ছোট মনে করে, তা বড় পাপ হতে পারে।","জিহ্বা ও পবিত্রতা—দুই বিষয়ে সাবধান থাকা দরকার।"],"related_hadiths":[{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"677","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E61" s="4" t="n"/>
@@ -1899,12 +1895,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>158</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | চুগলখোরি ও পেশাব থেকে সতর্কতার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. কবরের আযাবের দুটি কারণ হিসেবে চুগলখোরি ও পেশাব থেকে সতর্ক না থাকার কথা এসেছে।"},"heading":{"title":"কবরের আযাব সম্পর্কে হাদিস: চুগলখোরি ও পেশাব থেকে সতর্কতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুই কবরের পাশ দিয়ে যাওয়ার সময় বলেন, তাদের দু’জনকে আযাব দেওয়া হচ্ছে। তিনি বলেন, বিষয়টি তাদের কাছে খুব বড় মনে হয়নি; কিন্তু তা বড় পাপই। একজন চুগলখোরি করত, আর অন্যজন পেশাব থেকে সতর্ক থাকত না। বর্ণনায় আরও এসেছে, একজন পেশাবের ব্যাপারে সাবধানতা অবলম্বন করত না এবং অন্যজন চুগলখোরি করে বেড়াত। এখানে দুটি মূল শিক্ষা আছে। প্রথমত, মানুষের মাঝে কথা লাগানো ভয়াবহ কাজ। দ্বিতীয়ত, পেশাবের অপবিত্রতা থেকে বাঁচা খুব গুরুত্বপূর্ণ। অনেক সময় মানুষ ছোট ভেবে কিছু কাজ অবহেলা করে, কিন্তু হাদিস দেখায়—এমন কাজ কবরের আযাবের কারণ হতে পারে।"},"teachings":["চুগলখোরি কবরের আযাবের কারণ হিসেবে এসেছে।","পেশাবের অপবিত্রতা থেকে সতর্ক থাকা জরুরি।","মানুষ যে কাজ ছোট মনে করে, তা বড় পাপ হতে পারে।","জিহ্বা ও পবিত্রতা—দুই বিষয়ে সাবধান থাকা দরকার।"],"related_hadiths":[{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"677","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব থেকে সতর্ক থাকার গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. অধিকাংশ কবরের আযাব পেশাবের কারণে—তাই পেশাব থেকে সতর্ক থাকার শিক্ষা দেয় এই হাদিস।"},"heading":{"title":"পেশাব থেকে সতর্ক থাকার হাদিস: কবরের আযাবের ভয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, অধিকাংশ কবরের আযাব পেশাবের কারণে হয়ে থাকে। তাই তিনি বলেছেন, তোমরা পেশাব থেকে সতর্ক থাক। এখানে মূল শিক্ষা হলো পেশাবের অপবিত্রতা থেকে বাঁচা। মানুষ অনেক সময় এই বিষয়কে ছোট মনে করে, কিন্তু হাদিসে এটিকে খুব গুরুতরভাবে বলা হয়েছে। পেশাবের ছিটা, কাপড় বা শরীরে অপবিত্রতা লেগে থাকা—এসব থেকে সতর্ক থাকা পবিত্রতার অংশ। হাদিসের ভাষা সরাসরি সতর্কতামূলক, তাই ব্যাখ্যাতেও বাড়তি দাবি করার দরকার নেই। সহজ শিক্ষা হলো, শৌচকার্যের পর ভালোভাবে পবিত্র হওয়া, কাপড় ও শরীরকে নাপাকি থেকে বাঁচানো এবং এই বিষয়ে অবহেলা না করা।"},"teachings":["পেশাবের অপবিত্রতা থেকে সতর্ক থাকা জরুরি।","কবরের আযাবের প্রসঙ্গে পেশাবের বিষয়টি গুরুতরভাবে এসেছে।","শরীর ও কাপড় নাপাকি থেকে বাঁচাতে হবে।","ছোট মনে হলেও পবিত্রতার বিষয়ে অবহেলা করা ঠিক নয়।"],"related_hadiths":[{"id":"159","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E62" s="4" t="n"/>
@@ -1922,12 +1918,12 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>159</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব থেকে সতর্ক থাকার গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. অধিকাংশ কবরের আযাব পেশাবের কারণে—তাই পেশাব থেকে সতর্ক থাকার শিক্ষা দেয় এই হাদিস।"},"heading":{"title":"পেশাব থেকে সতর্ক থাকার হাদিস: কবরের আযাবের ভয়","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, অধিকাংশ কবরের আযাব পেশাবের কারণে হয়ে থাকে। তাই তিনি বলেছেন, তোমরা পেশাব থেকে সতর্ক থাক। এখানে মূল শিক্ষা হলো পেশাবের অপবিত্রতা থেকে বাঁচা। মানুষ অনেক সময় এই বিষয়কে ছোট মনে করে, কিন্তু হাদিসে এটিকে খুব গুরুতরভাবে বলা হয়েছে। পেশাবের ছিটা, কাপড় বা শরীরে অপবিত্রতা লেগে থাকা—এসব থেকে সতর্ক থাকা পবিত্রতার অংশ। হাদিসের ভাষা সরাসরি সতর্কতামূলক, তাই ব্যাখ্যাতেও বাড়তি দাবি করার দরকার নেই। সহজ শিক্ষা হলো, শৌচকার্যের পর ভালোভাবে পবিত্র হওয়া, কাপড় ও শরীরকে নাপাকি থেকে বাঁচানো এবং এই বিষয়ে অবহেলা না করা।"},"teachings":["পেশাবের অপবিত্রতা থেকে সতর্ক থাকা জরুরি।","কবরের আযাবের প্রসঙ্গে পেশাবের বিষয়টি গুরুতরভাবে এসেছে।","শরীর ও কাপড় নাপাকি থেকে বাঁচাতে হবে।","ছোট মনে হলেও পবিত্রতার বিষয়ে অবহেলা করা ঠিক নয়।"],"related_hadiths":[{"id":"159","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব থেকে পবিত্র থাকার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে পবিত্র থাকতে বলা হয়েছে, কারণ কবরের আযাবের সঙ্গে এটি জড়িত বলে হাদিসে এসেছে।"},"heading":{"title":"পেশাব থেকে পবিত্র থাকা: কবরের আযাব থেকে সতর্কতার হাদিস","description":"এই হাদিসে রাসুলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, তোমরা পেশাব থেকে পবিত্র থাক। কারণ পেশাবের কারণেই অধিকাংশ কবরের আযাব হয়ে থাকে। হাদিসের ভাষা সংক্ষিপ্ত, কিন্তু শিক্ষা খুব গভীর। শৌচকার্যের পর পবিত্রতা অর্জন করা, শরীর ও কাপড়কে নাপাকি থেকে বাঁচানো এবং পেশাবের ব্যাপারে অবহেলা না করা—এসব বিষয় সরাসরি এই হাদিসের সাথে যুক্ত। এখানে কোনো অতিরিক্ত ব্যাখ্যার প্রয়োজন নেই। রাসূলুল্লাহ (সা.) নিজেই কারণ বলেছেন—কবরের আযাবের একটি বড় অংশ পেশাবের সাথে জড়িত। তাই মুসলিমের উচিত এই বিষয়ে সতর্ক থাকা। পবিত্রতা সালাত ও দৈনন্দিন ইবাদতের সাথেও সম্পর্কিত, তবে এই হাদিসে মূল জোর দেওয়া হয়েছে পেশাব থেকে পবিত্র থাকার উপর।"},"teachings":["পেশাব থেকে পবিত্র থাকা নবীজির সরাসরি নির্দেশ।","পেশাবের ব্যাপারে অবহেলা কবরের আযাবের কারণ হিসেবে এসেছে।","শরীর ও কাপড় নাপাক হওয়া থেকে বাঁচতে হবে।","শৌচকার্যের পর ভালোভাবে পবিত্র হওয়া দরকার।"],"related_hadiths":[{"id":"158","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E63" s="4" t="n"/>
@@ -1945,15 +1941,19 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব থেকে পবিত্র থাকার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে পবিত্র থাকতে বলা হয়েছে, কারণ কবরের আযাবের সঙ্গে এটি জড়িত বলে হাদিসে এসেছে।"},"heading":{"title":"পেশাব থেকে পবিত্র থাকা: কবরের আযাব থেকে সতর্কতার হাদিস","description":"এই হাদিসে রাসুলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, তোমরা পেশাব থেকে পবিত্র থাক। কারণ পেশাবের কারণেই অধিকাংশ কবরের আযাব হয়ে থাকে। হাদিসের ভাষা সংক্ষিপ্ত, কিন্তু শিক্ষা খুব গভীর। শৌচকার্যের পর পবিত্রতা অর্জন করা, শরীর ও কাপড়কে নাপাকি থেকে বাঁচানো এবং পেশাবের ব্যাপারে অবহেলা না করা—এসব বিষয় সরাসরি এই হাদিসের সাথে যুক্ত। এখানে কোনো অতিরিক্ত ব্যাখ্যার প্রয়োজন নেই। রাসূলুল্লাহ (সা.) নিজেই কারণ বলেছেন—কবরের আযাবের একটি বড় অংশ পেশাবের সাথে জড়িত। তাই মুসলিমের উচিত এই বিষয়ে সতর্ক থাকা। পবিত্রতা সালাত ও দৈনন্দিন ইবাদতের সাথেও সম্পর্কিত, তবে এই হাদিসে মূল জোর দেওয়া হয়েছে পেশাব থেকে পবিত্র থাকার উপর।"},"teachings":["পেশাব থেকে পবিত্র থাকা নবীজির সরাসরি নির্দেশ।","পেশাবের ব্যাপারে অবহেলা কবরের আযাবের কারণ হিসেবে এসেছে।","শরীর ও কাপড় নাপাক হওয়া থেকে বাঁচতে হবে।","শৌচকার্যের পর ভালোভাবে পবিত্র হওয়া দরকার।"],"related_hadiths":[{"id":"158","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="n"/>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সম্পদ, জ্ঞান ও নিয়তের ফল","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি চার ধরনের মানুষের উদাহরণ দিয়ে সম্পদ, জ্ঞান ও নিয়তের ভালো-মন্দ ফল বোঝায়।"},"heading":{"title":"সম্পদ, জ্ঞান ও সৎ নিয়ত: চার ধরনের মানুষের শিক্ষা","description":"এই হাদিসে প্রথমে তিনটি বিষয়ের কথা এসেছে। সাদকা করলে বান্দার সম্পদ কমে না; জুলুমের শিকার হয়ে ধৈর্য ধরলে আল্লাহ মর্যাদা বাড়িয়ে দেন; আর ভিক্ষার দরজা খুললে অভাবের দরজা খুলে যেতে পারে। এরপর দুনিয়ার মানুষকে চার ভাগে দেখানো হয়েছে। কেউ সম্পদ ও জ্ঞান পেয়ে আল্লাহকে ভয় করে, আত্মীয়তার সম্পর্ক রাখে এবং আল্লাহর হক আদায় করে। কেউ জ্ঞান পেয়েছে কিন্তু সম্পদ পায়নি; সে সৎ নিয়তে বলে, সম্পদ থাকলে প্রথম ব্যক্তির মতো কাজ করত। সে নিয়ত অনুযায়ী প্রতিদান পায়। আবার কেউ সম্পদ পেয়েছে কিন্তু জ্ঞান নেই; সে অন্যায়ভাবে ব্যয় করে। আর কেউ সম্পদও পায়নি, জ্ঞানও পায়নি; সে খারাপ নিয়তে বলে, সম্পদ থাকলে তৃতীয় ব্যক্তির মতো করত। এই হাদিস নিয়ত, জ্ঞান ও সম্পদের সঠিক ব্যবহারের ভারসাম্য শেখায়।"},"teachings":["সম্পদ ও জ্ঞান থাকলে আল্লাহর হক বুঝে ব্যয় করা উচিত।","সৎ নিয়ত প্রতিদানের কারণ হতে পারে, যদিও সম্পদ না থাকে।","জ্ঞান ছাড়া সম্পদ অন্যায় পথে চলে যেতে পারে।","খারাপ কাজের ইচ্ছাও মানুষের জন্য বিপদের কারণ হতে পারে।"],"related_hadiths":[{"id":"2325","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ৪২২৮ (প্রাসঙ্গিক বর্ণনা)"</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="46" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1968,19 +1968,15 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>160</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সম্পদ, জ্ঞান ও নিয়তের ফল","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি চার ধরনের মানুষের উদাহরণ দিয়ে সম্পদ, জ্ঞান ও নিয়তের ভালো-মন্দ ফল বোঝায়।"},"heading":{"title":"সম্পদ, জ্ঞান ও সৎ নিয়ত: চার ধরনের মানুষের শিক্ষা","description":"এই হাদিসে প্রথমে তিনটি বিষয়ের কথা এসেছে। সাদকা করলে বান্দার সম্পদ কমে না; জুলুমের শিকার হয়ে ধৈর্য ধরলে আল্লাহ মর্যাদা বাড়িয়ে দেন; আর ভিক্ষার দরজা খুললে অভাবের দরজা খুলে যেতে পারে। এরপর দুনিয়ার মানুষকে চার ভাগে দেখানো হয়েছে। কেউ সম্পদ ও জ্ঞান পেয়ে আল্লাহকে ভয় করে, আত্মীয়তার সম্পর্ক রাখে এবং আল্লাহর হক আদায় করে। কেউ জ্ঞান পেয়েছে কিন্তু সম্পদ পায়নি; সে সৎ নিয়তে বলে, সম্পদ থাকলে প্রথম ব্যক্তির মতো কাজ করত। সে নিয়ত অনুযায়ী প্রতিদান পায়। আবার কেউ সম্পদ পেয়েছে কিন্তু জ্ঞান নেই; সে অন্যায়ভাবে ব্যয় করে। আর কেউ সম্পদও পায়নি, জ্ঞানও পায়নি; সে খারাপ নিয়তে বলে, সম্পদ থাকলে তৃতীয় ব্যক্তির মতো করত। এই হাদিস নিয়ত, জ্ঞান ও সম্পদের সঠিক ব্যবহারের ভারসাম্য শেখায়।"},"teachings":["সম্পদ ও জ্ঞান থাকলে আল্লাহর হক বুঝে ব্যয় করা উচিত।","সৎ নিয়ত প্রতিদানের কারণ হতে পারে, যদিও সম্পদ না থাকে।","জ্ঞান ছাড়া সম্পদ অন্যায় পথে চলে যেতে পারে।","খারাপ কাজের ইচ্ছাও মানুষের জন্য বিপদের কারণ হতে পারে।"],"related_hadiths":[{"id":"2325","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ৪২২৮ (প্রাসঙ্গিক বর্ণনা)"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গীবত ও পেশাব থেকে সতর্কতার কবরের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুই কবরের আযাবের ঘটনায় গীবত ও পেশাব থেকে সতর্ক না থাকার শিক্ষা এসেছে।"},"heading":{"title":"গীবত ও পেশাব থেকে সতর্কতার হাদিস: দুই কবরের ঘটনা","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুই কবরের কাছে এসে বলেন, এ দু’কবরের অধিবাসীকে আযাব দেওয়া হচ্ছে। তারপর তিনি একটি খেজুরের ডাল আনতে বলেন, ডালটি দুই ভাগ করে দুই কবরে রাখেন এবং বলেন, যতক্ষণ ডাল দু’টি তাজা থাকবে, আশা করা যায় তাদের কবরের আযাব হালকা করা হবে। এরপর কারণ হিসেবে বলেন, একজন গীবত করত এবং অপরজন পেশাব থেকে সতর্ক থাকত না। এখানে দুটি বিষয় খুব স্পষ্ট। গীবত মানুষের জিহ্বার পাপ, আর পেশাব থেকে সতর্ক না থাকা পবিত্রতার অবহেলা। হাদিসটি আমাদের শেখায়, কথা ও পবিত্রতা—দুই ক্ষেত্রেই সতর্ক থাকতে হয়। ছোট ভেবে অবহেলা করা নিরাপদ নয়।"},"teachings":["গীবত কবরের আযাবের কারণ হিসেবে এই বর্ণনায় এসেছে।","পেশাব থেকে সতর্ক না থাকা গুরুতর অবহেলা।","জিহ্বা ও পবিত্রতা—দুই বিষয়ে মুসলিমকে সাবধান থাকতে হবে।","নবীজি আযাব হালকা হওয়ার আশা প্রকাশ করেছিলেন, নিশ্চিত দাবি করেননি।"],"related_hadiths":[{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"157","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n"/>
     </row>
     <row r="66" ht="46" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
@@ -1995,12 +1991,12 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>161</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গীবত ও পেশাব থেকে সতর্কতার কবরের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুই কবরের আযাবের ঘটনায় গীবত ও পেশাব থেকে সতর্ক না থাকার শিক্ষা এসেছে।"},"heading":{"title":"গীবত ও পেশাব থেকে সতর্কতার হাদিস: দুই কবরের ঘটনা","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) দুই কবরের কাছে এসে বলেন, এ দু’কবরের অধিবাসীকে আযাব দেওয়া হচ্ছে। তারপর তিনি একটি খেজুরের ডাল আনতে বলেন, ডালটি দুই ভাগ করে দুই কবরে রাখেন এবং বলেন, যতক্ষণ ডাল দু’টি তাজা থাকবে, আশা করা যায় তাদের কবরের আযাব হালকা করা হবে। এরপর কারণ হিসেবে বলেন, একজন গীবত করত এবং অপরজন পেশাব থেকে সতর্ক থাকত না। এখানে দুটি বিষয় খুব স্পষ্ট। গীবত মানুষের জিহ্বার পাপ, আর পেশাব থেকে সতর্ক না থাকা পবিত্রতার অবহেলা। হাদিসটি আমাদের শেখায়, কথা ও পবিত্রতা—দুই ক্ষেত্রেই সতর্ক থাকতে হয়। ছোট ভেবে অবহেলা করা নিরাপদ নয়।"},"teachings":["গীবত কবরের আযাবের কারণ হিসেবে এই বর্ণনায় এসেছে।","পেশাব থেকে সতর্ক না থাকা গুরুতর অবহেলা।","জিহ্বা ও পবিত্রতা—দুই বিষয়ে মুসলিমকে সাবধান থাকতে হবে।","নবীজি আযাব হালকা হওয়ার আশা প্রকাশ করেছিলেন, নিশ্চিত দাবি করেননি।"],"related_hadiths":[{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"216","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"157","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাবের পবিত্রতা ও কবরের আযাব","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে সতর্ক থাকা কবরের আযাব থেকে বাঁচার বড় কারণ—এই হাদিসে পবিত্রতার গুরুত্ব স্পষ্ট হয়েছে।"},"heading":{"title":"পেশাবের পবিত্রতা: কবরের আযাব থেকে সতর্ক থাকার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম খুব সংক্ষিপ্ত কিন্তু গভীর একটি সতর্কবার্তা দিয়েছেন। তিনি বলেছেন, বেশিরভাগ কবরের আযাব পেশাবের কারণে হয়ে থাকে। এখানে মূল শিক্ষা হলো পেশাবের পবিত্রতা ও নাপাকী থেকে সতর্ক থাকা। একজন মুসলিমের জন্য পবিত্রতা শুধু নামাজের আগে ওযু করা নয়, বরং শরীর, কাপড় ও চলাফেরার জায়গাকে নাপাকী থেকে বাঁচানোও জরুরি। অনেক সময় মানুষ পেশাবের ছিটা বা নাপাকীকে ছোট মনে করে। কিন্তু এই হাদিস জানিয়ে দেয়, এমন অবহেলা আখিরাতের কঠিন পরিণতির কারণ হতে পারে। তাই ইস্তিঞ্জা, কাপড়ের পরিচ্ছন্নতা এবং পেশাবের সময় সতর্কতা মুসলিম জীবনের গুরুত্বপূর্ণ আদব।"},"teachings":["পেশাবের নাপাকী থেকে সতর্ক থাকা ঈমানদারের পরিচ্ছন্নতার অংশ।","ছোট মনে হওয়া অবহেলাও আখিরাতে কঠিন জবাবদিহির কারণ হতে পারে।","শরীর ও কাপড় পবিত্র রাখা নামাজ ও দৈনন্দিন ইবাদতের জন্য জরুরি।","কবরের আযাব থেকে বাঁচতে পবিত্রতার বিষয়ে সচেতন থাকা দরকার।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E66" s="4" t="n"/>
@@ -2018,12 +2014,12 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>162</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাবের পবিত্রতা ও কবরের আযাব","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে সতর্ক থাকা কবরের আযাব থেকে বাঁচার বড় কারণ—এই হাদিসে পবিত্রতার গুরুত্ব স্পষ্ট হয়েছে।"},"heading":{"title":"পেশাবের পবিত্রতা: কবরের আযাব থেকে সতর্ক থাকার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম খুব সংক্ষিপ্ত কিন্তু গভীর একটি সতর্কবার্তা দিয়েছেন। তিনি বলেছেন, বেশিরভাগ কবরের আযাব পেশাবের কারণে হয়ে থাকে। এখানে মূল শিক্ষা হলো পেশাবের পবিত্রতা ও নাপাকী থেকে সতর্ক থাকা। একজন মুসলিমের জন্য পবিত্রতা শুধু নামাজের আগে ওযু করা নয়, বরং শরীর, কাপড় ও চলাফেরার জায়গাকে নাপাকী থেকে বাঁচানোও জরুরি। অনেক সময় মানুষ পেশাবের ছিটা বা নাপাকীকে ছোট মনে করে। কিন্তু এই হাদিস জানিয়ে দেয়, এমন অবহেলা আখিরাতের কঠিন পরিণতির কারণ হতে পারে। তাই ইস্তিঞ্জা, কাপড়ের পরিচ্ছন্নতা এবং পেশাবের সময় সতর্কতা মুসলিম জীবনের গুরুত্বপূর্ণ আদব।"},"teachings":["পেশাবের নাপাকী থেকে সতর্ক থাকা ঈমানদারের পরিচ্ছন্নতার অংশ।","ছোট মনে হওয়া অবহেলাও আখিরাতে কঠিন জবাবদিহির কারণ হতে পারে।","শরীর ও কাপড় পবিত্র রাখা নামাজ ও দৈনন্দিন ইবাদতের জন্য জরুরি।","কবরের আযাব থেকে বাঁচতে পবিত্রতার বিষয়ে সচেতন থাকা দরকার।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাবের আদব ও বনী ইসরাঈলের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাবের সময় পর্দা, সতর্কতা ও নাপাকীকে হালকা না ভাবার শিক্ষা এই হাদিসে পরিষ্কারভাবে এসেছে।"},"heading":{"title":"পেশাবের আদব: পর্দা ও পবিত্রতার গুরুত্বপূর্ণ শিক্ষা","description":"এই হাদিসে দেখা যায়, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম পেশাবের সময় একটি চামড়ার ঢাল সামনে রেখে পর্দা করলেন। এতে পেশাবের আদব এবং লজ্জাশীলতার শিক্ষা আছে। একজন লোক তাঁর বসার ধরন নিয়ে মন্তব্য করলে নবীজি তাকে বনী ইসরাঈলের এক ঘটনার কথা স্মরণ করিয়ে দেন। তাদের মধ্যে পেশাব লাগলে শরীরের অংশ কেটে ফেলার মতো কঠিন নিয়ম ছিল। এক ব্যক্তি তাদের তা করতে নিষেধ করেছিল, ফলে তাকে কবরে আযাব দেয়া হয় বলে হাদিসে এসেছে। এই বর্ণনা আমাদের শেখায়, পেশাবের নাপাকী নিয়ে অবহেলা করা ঠিক নয়। তবে এই হাদিসে মূল জোর হলো পবিত্রতার ব্যাপারে সতর্কতা, পর্দা রাখা এবং নবীজির কাজ নিয়ে অজ্ঞভাবে মন্তব্য না করা।"},"teachings":["পেশাবের সময় পর্দা রাখা শালীনতার একটি গুরুত্বপূর্ণ আদব।","নাপাকীকে হালকা মনে করে অবহেলা করা উচিত নয়।","নবীজির কাজ বুঝে না নিয়ে মন্তব্য করা বিপজ্জনক হতে পারে।","পবিত্রতার বিধান আল্লাহর কাছে গুরুত্বপূর্ণ বিষয়।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E67" s="4" t="n"/>
@@ -2041,12 +2037,12 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>163</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাবের আদব ও বনী ইসরাঈলের শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাবের সময় পর্দা, সতর্কতা ও নাপাকীকে হালকা না ভাবার শিক্ষা এই হাদিসে পরিষ্কারভাবে এসেছে।"},"heading":{"title":"পেশাবের আদব: পর্দা ও পবিত্রতার গুরুত্বপূর্ণ শিক্ষা","description":"এই হাদিসে দেখা যায়, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম পেশাবের সময় একটি চামড়ার ঢাল সামনে রেখে পর্দা করলেন। এতে পেশাবের আদব এবং লজ্জাশীলতার শিক্ষা আছে। একজন লোক তাঁর বসার ধরন নিয়ে মন্তব্য করলে নবীজি তাকে বনী ইসরাঈলের এক ঘটনার কথা স্মরণ করিয়ে দেন। তাদের মধ্যে পেশাব লাগলে শরীরের অংশ কেটে ফেলার মতো কঠিন নিয়ম ছিল। এক ব্যক্তি তাদের তা করতে নিষেধ করেছিল, ফলে তাকে কবরে আযাব দেয়া হয় বলে হাদিসে এসেছে। এই বর্ণনা আমাদের শেখায়, পেশাবের নাপাকী নিয়ে অবহেলা করা ঠিক নয়। তবে এই হাদিসে মূল জোর হলো পবিত্রতার ব্যাপারে সতর্কতা, পর্দা রাখা এবং নবীজির কাজ নিয়ে অজ্ঞভাবে মন্তব্য না করা।"},"teachings":["পেশাবের সময় পর্দা রাখা শালীনতার একটি গুরুত্বপূর্ণ আদব।","নাপাকীকে হালকা মনে করে অবহেলা করা উচিত নয়।","নবীজির কাজ বুঝে না নিয়ে মন্তব্য করা বিপজ্জনক হতে পারে।","পবিত্রতার বিধান আল্লাহর কাছে গুরুত্বপূর্ণ বিষয়।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব ও চুগলখোরির কবরের শাস্তি","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে সতর্ক না থাকা ও চুগলখোরি—দুটি গুনাহ কবরে কঠিন আযাবের কারণ হতে পারে।"},"heading":{"title":"কবরের আযাবের দুই কারণ: পেশাবের অবহেলা ও চুগলখোরি","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম দু’টি কবরের পাশ দিয়ে যাওয়ার সময় থেমে যান। তিনি জানান, কবরের দুই ব্যক্তিকে কঠিন আযাব দেয়া হচ্ছে। কারণ দুটি মানুষের চোখে সাধারণ মনে হতে পারে, কিন্তু আল্লাহর কাছে তা হালকা নয়। একজন পেশাব থেকে সতর্ক হত না। অর্থাৎ নাপাকী থেকে নিজেকে ঠিকভাবে বাঁচাত না। অন্যজন জিহ্বা দিয়ে মানুষকে কষ্ট দিত এবং চুগলখোরি করত। এতে বোঝা যায়, পবিত্রতা ও জবান—দুইটি বিষয়ে মুসলিমকে খুব সচেতন থাকতে হবে। নবীজি খেজুরের তাজা ডাল কবরের উপর রাখলেন এবং বললেন, ডাল তাজা থাকা পর্যন্ত আযাব হালকা করা হবে। হাদিসের মূল শিক্ষা হলো নাপাকী ও কথার ক্ষতি—দুটিই গুরুতর।"},"teachings":["পেশাবের নাপাকী থেকে সতর্ক না থাকা কবরে শাস্তির কারণ হতে পারে।","চুগলখোরি ও জিহ্বা দিয়ে কষ্ট দেয়া গুরুতর গুনাহ।","মানুষের চোখে ছোট মনে হওয়া কাজও আল্লাহর কাছে বড় হতে পারে।","পবিত্রতা ও কথাবার্তায় সাবধানতা মুসলিম চরিত্রের অংশ।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E68" s="4" t="n"/>
@@ -2064,12 +2060,12 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>164</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেশাব ও চুগলখোরির কবরের শাস্তি","description":"$book_name$ $hadith_number$ - $chapter_name$. পেশাব থেকে সতর্ক না থাকা ও চুগলখোরি—দুটি গুনাহ কবরে কঠিন আযাবের কারণ হতে পারে।"},"heading":{"title":"কবরের আযাবের দুই কারণ: পেশাবের অবহেলা ও চুগলখোরি","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম দু’টি কবরের পাশ দিয়ে যাওয়ার সময় থেমে যান। তিনি জানান, কবরের দুই ব্যক্তিকে কঠিন আযাব দেয়া হচ্ছে। কারণ দুটি মানুষের চোখে সাধারণ মনে হতে পারে, কিন্তু আল্লাহর কাছে তা হালকা নয়। একজন পেশাব থেকে সতর্ক হত না। অর্থাৎ নাপাকী থেকে নিজেকে ঠিকভাবে বাঁচাত না। অন্যজন জিহ্বা দিয়ে মানুষকে কষ্ট দিত এবং চুগলখোরি করত। এতে বোঝা যায়, পবিত্রতা ও জবান—দুইটি বিষয়ে মুসলিমকে খুব সচেতন থাকতে হবে। নবীজি খেজুরের তাজা ডাল কবরের উপর রাখলেন এবং বললেন, ডাল তাজা থাকা পর্যন্ত আযাব হালকা করা হবে। হাদিসের মূল শিক্ষা হলো নাপাকী ও কথার ক্ষতি—দুটিই গুরুতর।"},"teachings":["পেশাবের নাপাকী থেকে সতর্ক না থাকা কবরে শাস্তির কারণ হতে পারে।","চুগলখোরি ও জিহ্বা দিয়ে কষ্ট দেয়া গুরুতর গুনাহ।","মানুষের চোখে ছোট মনে হওয়া কাজও আল্লাহর কাছে বড় হতে পারে।","পবিত্রতা ও কথাবার্তায় সাবধানতা মুসলিম চরিত্রের অংশ।"],"related_hadiths":[{"id":"218","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1361","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6055","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গণগোসলখানায় পর্দা ও শালীনতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমানদারের জন্য গণগোসলখানায় পর্দা রক্ষা ও নারীদের এ স্থান থেকে দূরে রাখার শিক্ষা দেয়া হয়েছে।"},"heading":{"title":"গণগোসলখানায় পর্দা: ঈমানদারের শালীনতার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ঈমানের সাথে শালীনতার সম্পর্ক তুলে ধরেছেন। তিনি বলেছেন, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। অর্থাৎ এমন জায়গায় শরীর ঢেকে রাখা জরুরি, যেখানে অন্য মানুষের সামনে উন্মুক্ত হওয়ার আশঙ্কা থাকে। এরপর তিনি বলেন, কেউ যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। এখানে মূল বিষয় হলো পর্দা, লজ্জাশীলতা এবং দেহের সম্মান রক্ষা। হাদিসটি আমাদের শেখায়, পবিত্রতা অর্জনের স্থান হলেও শালীনতার সীমা ভাঙা যাবে না। গোসলের প্রয়োজন থাকতে পারে, কিন্তু পর্দা ও নিরাপত্তা বজায় রাখা ঈমানদারের আচরণের অংশ।"},"teachings":["গণগোসলখানায় প্রবেশ করলে শরীর ঢেকে রাখা জরুরি।","পর্দা ও লজ্জাশীলতা ঈমানের সাথে যুক্ত একটি আচরণ।","পরিবারের নারীদের পর্দা ও নিরাপত্তার বিষয়ে দায়িত্বশীল হওয়া দরকার।","পবিত্রতা অর্জনের সময়ও শালীনতার সীমা মানতে হয়।"],"related_hadiths":[{"id":"4009","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E69" s="4" t="n"/>
@@ -2087,12 +2083,12 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>166</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গণগোসলখানায় পর্দা ও শালীনতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমানদারের জন্য গণগোসলখানায় পর্দা রক্ষা ও নারীদের এ স্থান থেকে দূরে রাখার শিক্ষা দেয়া হয়েছে।"},"heading":{"title":"গণগোসলখানায় পর্দা: ঈমানদারের শালীনতার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ঈমানের সাথে শালীনতার সম্পর্ক তুলে ধরেছেন। তিনি বলেছেন, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। অর্থাৎ এমন জায়গায় শরীর ঢেকে রাখা জরুরি, যেখানে অন্য মানুষের সামনে উন্মুক্ত হওয়ার আশঙ্কা থাকে। এরপর তিনি বলেন, কেউ যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। এখানে মূল বিষয় হলো পর্দা, লজ্জাশীলতা এবং দেহের সম্মান রক্ষা। হাদিসটি আমাদের শেখায়, পবিত্রতা অর্জনের স্থান হলেও শালীনতার সীমা ভাঙা যাবে না। গোসলের প্রয়োজন থাকতে পারে, কিন্তু পর্দা ও নিরাপত্তা বজায় রাখা ঈমানদারের আচরণের অংশ।"},"teachings":["গণগোসলখানায় প্রবেশ করলে শরীর ঢেকে রাখা জরুরি।","পর্দা ও লজ্জাশীলতা ঈমানের সাথে যুক্ত একটি আচরণ।","পরিবারের নারীদের পর্দা ও নিরাপত্তার বিষয়ে দায়িত্বশীল হওয়া দরকার।","পবিত্রতা অর্জনের সময়ও শালীনতার সীমা মানতে হয়।"],"related_hadiths":[{"id":"4009","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈমান, প্রতিবেশী ও শালীনতার আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রতিবেশীকে সম্মান, ভালো কথা বলা ও গণগোসলখানায় পর্দা—ঈমানদারের কয়েকটি আদব শেখানো হয়েছে।"},"heading":{"title":"ঈমানদারের আদব: প্রতিবেশী, কথা ও গণগোসলখানায় পর্দা","description":"এই হাদিসে কয়েকটি গুরুত্বপূর্ণ আচরণ একসাথে এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন প্রতিবেশীকে সম্মান করে। সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। সে যেন ভালো কথা বলে, না হলে চুপ থাকে। আর নারীদের ব্যাপারে বলা হয়েছে, তারা যেন গণগোসলখানায় প্রবেশ না করে। এসব নির্দেশ এক জায়গায় আসায় বোঝা যায়, ঈমান শুধু মনে রাখার বিষয় নয়; আচরণ, কথা, পর্দা ও সামাজিক দায়িত্বে তার প্রভাব দেখা যায়। হাদিসের শেষ অংশে ওমর বিন আবদুল আযীয এই বর্ণনার সত্যতা যাচাই করে নারীদের গণগোসলখানায় প্রবেশে নিষেধাজ্ঞা দেন। এতে সতর্কতা ও দায়িত্বশীলতার শিক্ষা আছে।"},"teachings":["প্রতিবেশীকে সম্মান করা ঈমানদারের ভালো আচরণের অংশ।","ভালো কথা বলা বা চুপ থাকা জিহ্বা রক্ষার সহজ পথ।","গণগোসলখানায় পর্দা রক্ষা করা জরুরি।","নারীদের পর্দা ও নিরাপত্তার বিষয়ে দায়িত্বশীল ব্যবস্থা নেয়া যায়।"],"related_hadiths":[{"id":"6018","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4009","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E70" s="4" t="n"/>
@@ -2110,12 +2106,12 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>167</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈমান, প্রতিবেশী ও শালীনতার আদব","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রতিবেশীকে সম্মান, ভালো কথা বলা ও গণগোসলখানায় পর্দা—ঈমানদারের কয়েকটি আদব শেখানো হয়েছে।"},"heading":{"title":"ঈমানদারের আদব: প্রতিবেশী, কথা ও গণগোসলখানায় পর্দা","description":"এই হাদিসে কয়েকটি গুরুত্বপূর্ণ আচরণ একসাথে এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন প্রতিবেশীকে সম্মান করে। সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। সে যেন ভালো কথা বলে, না হলে চুপ থাকে। আর নারীদের ব্যাপারে বলা হয়েছে, তারা যেন গণগোসলখানায় প্রবেশ না করে। এসব নির্দেশ এক জায়গায় আসায় বোঝা যায়, ঈমান শুধু মনে রাখার বিষয় নয়; আচরণ, কথা, পর্দা ও সামাজিক দায়িত্বে তার প্রভাব দেখা যায়। হাদিসের শেষ অংশে ওমর বিন আবদুল আযীয এই বর্ণনার সত্যতা যাচাই করে নারীদের গণগোসলখানায় প্রবেশে নিষেধাজ্ঞা দেন। এতে সতর্কতা ও দায়িত্বশীলতার শিক্ষা আছে।"},"teachings":["প্রতিবেশীকে সম্মান করা ঈমানদারের ভালো আচরণের অংশ।","ভালো কথা বলা বা চুপ থাকা জিহ্বা রক্ষার সহজ পথ।","গণগোসলখানায় পর্দা রক্ষা করা জরুরি।","নারীদের পর্দা ও নিরাপত্তার বিষয়ে দায়িত্বশীল ব্যবস্থা নেয়া যায়।"],"related_hadiths":[{"id":"6018","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4009","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মদের আসর ও গণগোসলখানা থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমানদারকে মদের আসর, পর্দাহীন গোসলখানা ও স্ত্রীকে এমন স্থানে পাঠানো থেকে বিরত থাকতে বলা হয়েছে।"},"heading":{"title":"মদের আসর ও পর্দাহীন গোসলখানা: ঈমানদারের সতর্কতা","description":"এই হাদিসে ওমার বিন খাত্তাব রাদিয়াল্লাহু আনহু মানুষের সামনে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের একটি বাণী তুলে ধরেন। এতে তিনটি সতর্কতা এসেছে। প্রথমত, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন এমন দস্তরখানায় না বসে যেখানে মদ বিতরণ করা হয়। দ্বিতীয়ত, সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। তৃতীয়ত, সে যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। এখানে মূল শিক্ষা হলো ঈমান মানুষকে পরিবেশ বাছাই করতে শেখায়। শুধু নিজে মদ না খাওয়া নয়, মদের আসর থেকেও দূরে থাকার শিক্ষা এসেছে। একইভাবে গোসলখানায় পর্দা রক্ষা ও পরিবারের মর্যাদার কথাও বলা হয়েছে।"},"teachings":["মদ বিতরণ হয় এমন আসর থেকে ঈমানদারের দূরে থাকা উচিত।","গণগোসলখানায় প্রবেশ করলে শরীর ঢেকে রাখা জরুরি।","স্ত্রীর পর্দা ও মর্যাদা রক্ষায় দায়িত্বশীল হওয়া দরকার।","ঈমান মানুষের বসার স্থান ও পরিবেশ বাছাইয়ে প্রভাব ফেলে।"],"related_hadiths":[{"id":"5232","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5233","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5566","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E71" s="4" t="n"/>
@@ -2133,12 +2129,12 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>169</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মদের আসর ও গণগোসলখানা থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঈমানদারকে মদের আসর, পর্দাহীন গোসলখানা ও স্ত্রীকে এমন স্থানে পাঠানো থেকে বিরত থাকতে বলা হয়েছে।"},"heading":{"title":"মদের আসর ও পর্দাহীন গোসলখানা: ঈমানদারের সতর্কতা","description":"এই হাদিসে ওমার বিন খাত্তাব রাদিয়াল্লাহু আনহু মানুষের সামনে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের একটি বাণী তুলে ধরেন। এতে তিনটি সতর্কতা এসেছে। প্রথমত, যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন এমন দস্তরখানায় না বসে যেখানে মদ বিতরণ করা হয়। দ্বিতীয়ত, সে যেন লুঙ্গি ছাড়া গণগোসলখানায় প্রবেশ না করে। তৃতীয়ত, সে যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। এখানে মূল শিক্ষা হলো ঈমান মানুষকে পরিবেশ বাছাই করতে শেখায়। শুধু নিজে মদ না খাওয়া নয়, মদের আসর থেকেও দূরে থাকার শিক্ষা এসেছে। একইভাবে গোসলখানায় পর্দা রক্ষা ও পরিবারের মর্যাদার কথাও বলা হয়েছে।"},"teachings":["মদ বিতরণ হয় এমন আসর থেকে ঈমানদারের দূরে থাকা উচিত।","গণগোসলখানায় প্রবেশ করলে শরীর ঢেকে রাখা জরুরি।","স্ত্রীর পর্দা ও মর্যাদা রক্ষায় দায়িত্বশীল হওয়া দরকার।","ঈমান মানুষের বসার স্থান ও পরিবেশ বাছাইয়ে প্রভাব ফেলে।"],"related_hadiths":[{"id":"5232","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5233","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5566","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নারীর পোশাক খোলা ও পর্দার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের নিরাপদ ঘর ছাড়া অন্যত্র পোশাক খোলা নারীর পর্দা ও আল্লাহর সাথে সম্পর্কের জন্য ক্ষতিকর বলা হয়েছে।"},"heading":{"title":"নারীর পর্দা রক্ষা: অন্যের ঘরে পোশাক খোলার সতর্কতা","description":"এই হাদিসে উম্মু দারদা রাদিয়াল্লাহু আনহার ঘটনা এসেছে। তিনি গোসলখানা থেকে বের হলে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁকে জিজ্ঞেস করেন, কোথা থেকে এসেছেন। তিনি বলেন, গোসলখানা থেকে। তখন নবীজি কঠোর ভাষায় সতর্ক করেন যে, যে মহিলা নিজের মাতৃকুলের বাড়ি ছাড়া অন্যের বাড়িতে নিজের বস্ত্র খুলে, সে দয়াময় আল্লাহ ও তার মাঝের পর্দা ধ্বংস করে দেয়। হাদিসের ভাষা খুব সতর্কতামূলক। এখানে মূল শিক্ষা হলো নারীর দেহ, গোপনীয়তা ও পর্দা রক্ষা করা। গোসল, কাপড় বদল বা শরীর খোলার মতো বিষয় নিরাপদ ও সম্মানজনক জায়গায় হওয়া উচিত। ব্যাখ্যায় বাড়তি দাবি না করে বলা যায়, এই হাদিস পর্দা ও লজ্জাশীলতার বড় গুরুত্ব শেখায়।"},"teachings":["নারীর পোশাক খোলার জায়গা নিরাপদ ও পর্দাসম্মত হওয়া দরকার।","গোসলখানা বা অন্যের বাড়িতে গোপনীয়তা নষ্ট হওয়ার আশঙ্কা থাকলে সতর্ক থাকা উচিত।","পর্দা শুধু পোশাক নয়, ব্যক্তিগত নিরাপত্তার সাথেও জড়িত।","শালীনতা রক্ষা আল্লাহর সামনে দায়িত্বের বিষয়।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E72" s="4" t="n"/>
@@ -2156,12 +2152,12 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নারীর পোশাক খোলা ও পর্দার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের নিরাপদ ঘর ছাড়া অন্যত্র পোশাক খোলা নারীর পর্দা ও আল্লাহর সাথে সম্পর্কের জন্য ক্ষতিকর বলা হয়েছে।"},"heading":{"title":"নারীর পর্দা রক্ষা: অন্যের ঘরে পোশাক খোলার সতর্কতা","description":"এই হাদিসে উম্মু দারদা রাদিয়াল্লাহু আনহার ঘটনা এসেছে। তিনি গোসলখানা থেকে বের হলে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁকে জিজ্ঞেস করেন, কোথা থেকে এসেছেন। তিনি বলেন, গোসলখানা থেকে। তখন নবীজি কঠোর ভাষায় সতর্ক করেন যে, যে মহিলা নিজের মাতৃকুলের বাড়ি ছাড়া অন্যের বাড়িতে নিজের বস্ত্র খুলে, সে দয়াময় আল্লাহ ও তার মাঝের পর্দা ধ্বংস করে দেয়। হাদিসের ভাষা খুব সতর্কতামূলক। এখানে মূল শিক্ষা হলো নারীর দেহ, গোপনীয়তা ও পর্দা রক্ষা করা। গোসল, কাপড় বদল বা শরীর খোলার মতো বিষয় নিরাপদ ও সম্মানজনক জায়গায় হওয়া উচিত। ব্যাখ্যায় বাড়তি দাবি না করে বলা যায়, এই হাদিস পর্দা ও লজ্জাশীলতার বড় গুরুত্ব শেখায়।"},"teachings":["নারীর পোশাক খোলার জায়গা নিরাপদ ও পর্দাসম্মত হওয়া দরকার।","গোসলখানা বা অন্যের বাড়িতে গোপনীয়তা নষ্ট হওয়ার আশঙ্কা থাকলে সতর্ক থাকা উচিত।","পর্দা শুধু পোশাক নয়, ব্যক্তিগত নিরাপত্তার সাথেও জড়িত।","শালীনতা রক্ষা আল্লাহর সামনে দায়িত্বের বিষয়।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নেক ইচ্ছার প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসে এসেছে, সৎ কাজের ইচ্ছাও নেকি; আর কাজ করলে তা বহু গুণে লেখা হয়।"},"heading":{"title":"নেক ইচ্ছা ও পাপ থেকে বিরত থাকা: আল্লাহর দয়ার শিক্ষা","description":"এই হাদিসে আল্লাহর দয়া ও হিসাবের সুন্দর নিয়ম এসেছে। নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর রব থেকে বর্ণনা করেন, আল্লাহ সৎকর্ম ও অসৎকর্ম লিখে রেখেছেন এবং তা স্পষ্ট করেছেন। কেউ যদি সৎ কাজের ইচ্ছা করে কিন্তু তা করতে না পারে, আল্লাহ তা পূর্ণ একটি সৎকর্ম হিসেবে লিখে নেন। আর ইচ্ছা করার পর কাজটি করলে তা দশ থেকে সাতশত বা আরও বেশি গুণে লেখা হয়। আবার কেউ পাপের ইচ্ছা করে কিন্তু তা বাস্তবায়ন না করে, আল্লাহ তা একটি পূর্ণ সৎকর্ম হিসেবে লিখে নেন। আর যদি পাপ করে, তা একটিমাত্র পাপ হিসেবে লেখা হয়। মুসলিমের বর্ণনায় পাপ মুছে দেওয়ার কথাও এসেছে। এই হাদিস মানুষকে আশা দেয়, তবে পাপকে হালকা মনে করার শিক্ষা দেয় না; বরং নেক ইচ্ছা ও পাপ থেকে ফিরে আসার মূল্য বোঝায়।"},"teachings":["সৎ কাজের ইচ্ছাও আল্লাহর কাছে নেকি হিসেবে লেখা হতে পারে।","নেক কাজ করলে তা বহু গুণে বাড়িয়ে লেখা হয়।","পাপের ইচ্ছা ছেড়ে দিলে আল্লাহর দয়ার আশা আছে।","আল্লাহ বান্দার ছোট ভালো ইচ্ছাকেও মূল্য দেন।"],"related_hadiths":[{"id":"6491","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"237","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E73" s="4" t="n"/>
@@ -2179,12 +2175,12 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>170</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নেক ইচ্ছার প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসে এসেছে, সৎ কাজের ইচ্ছাও নেকি; আর কাজ করলে তা বহু গুণে লেখা হয়।"},"heading":{"title":"নেক ইচ্ছা ও পাপ থেকে বিরত থাকা: আল্লাহর দয়ার শিক্ষা","description":"এই হাদিসে আল্লাহর দয়া ও হিসাবের সুন্দর নিয়ম এসেছে। নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর রব থেকে বর্ণনা করেন, আল্লাহ সৎকর্ম ও অসৎকর্ম লিখে রেখেছেন এবং তা স্পষ্ট করেছেন। কেউ যদি সৎ কাজের ইচ্ছা করে কিন্তু তা করতে না পারে, আল্লাহ তা পূর্ণ একটি সৎকর্ম হিসেবে লিখে নেন। আর ইচ্ছা করার পর কাজটি করলে তা দশ থেকে সাতশত বা আরও বেশি গুণে লেখা হয়। আবার কেউ পাপের ইচ্ছা করে কিন্তু তা বাস্তবায়ন না করে, আল্লাহ তা একটি পূর্ণ সৎকর্ম হিসেবে লিখে নেন। আর যদি পাপ করে, তা একটিমাত্র পাপ হিসেবে লেখা হয়। মুসলিমের বর্ণনায় পাপ মুছে দেওয়ার কথাও এসেছে। এই হাদিস মানুষকে আশা দেয়, তবে পাপকে হালকা মনে করার শিক্ষা দেয় না; বরং নেক ইচ্ছা ও পাপ থেকে ফিরে আসার মূল্য বোঝায়।"},"teachings":["সৎ কাজের ইচ্ছাও আল্লাহর কাছে নেকি হিসেবে লেখা হতে পারে।","নেক কাজ করলে তা বহু গুণে বাড়িয়ে লেখা হয়।","পাপের ইচ্ছা ছেড়ে দিলে আল্লাহর দয়ার আশা আছে।","আল্লাহ বান্দার ছোট ভালো ইচ্ছাকেও মূল্য দেন।"],"related_hadiths":[{"id":"6491","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"237","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বামীর ঘর ছাড়া পোশাক খোলার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. স্বামীর ঘর ছাড়া অন্যত্র পোশাক খোলার বিষয়ে নারীদের সতর্ক করা হয়েছে, যাতে পর্দা রক্ষা পায়।"},"heading":{"title":"স্বামীর ঘর ছাড়া পোশাক খোলা: নারীর পর্দা বিষয়ে হাদিস","description":"এই হাদিসে হিমস বা শামের কয়েকজন মহিলা আয়েশা রাদিয়াল্লাহু আনহার কাছে এলে তিনি তাদেরকে গোসলখানায় প্রবেশের বিষয় জিজ্ঞেস করেন। এরপর তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের বাণী শুনিয়েছেন। নবীজি বলেছেন, যে নারী তার স্বামীর ঘর ছাড়া অন্যের ঘরে নিজের পোশাক খুলবে, সে তার ও তার প্রভুর মাঝের পর্দা ধ্বংস করে দেয়। এখানে মূল বিষয় হলো নারীর পর্দা, ব্যক্তিগত গোপনীয়তা এবং নিরাপদ জায়গায় থাকা। হাদিসের কথাগুলো কঠোর, তাই বিষয়টি হালকা করে দেখা ঠিক নয়। তবে ব্যাখ্যায় এতটুকুই বলা যায় যে, এমন জায়গা এড়িয়ে চলা উচিত যেখানে পোশাক খোলা বা গোসলের কারণে পর্দা নষ্ট হওয়ার আশঙ্কা থাকে।"},"teachings":["নারীর জন্য পোশাক খোলার ক্ষেত্রে নিরাপদ ও সম্মানজনক জায়গা জরুরি।","স্বামীর ঘর ছাড়া অন্যত্র গোপনীয়তা নষ্ট হওয়ার ভয় থাকলে সতর্ক থাকা দরকার।","গণগোসলখানা নিয়ে সাহাবিয়াদের সতর্কতা ছিল।","পর্দা রক্ষা আল্লাহর সাথে সম্পর্কের আদবের অংশ।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E74" s="4" t="n"/>
@@ -2202,12 +2198,12 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>171</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বামীর ঘর ছাড়া পোশাক খোলার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. স্বামীর ঘর ছাড়া অন্যত্র পোশাক খোলার বিষয়ে নারীদের সতর্ক করা হয়েছে, যাতে পর্দা রক্ষা পায়।"},"heading":{"title":"স্বামীর ঘর ছাড়া পোশাক খোলা: নারীর পর্দা বিষয়ে হাদিস","description":"এই হাদিসে হিমস বা শামের কয়েকজন মহিলা আয়েশা রাদিয়াল্লাহু আনহার কাছে এলে তিনি তাদেরকে গোসলখানায় প্রবেশের বিষয় জিজ্ঞেস করেন। এরপর তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের বাণী শুনিয়েছেন। নবীজি বলেছেন, যে নারী তার স্বামীর ঘর ছাড়া অন্যের ঘরে নিজের পোশাক খুলবে, সে তার ও তার প্রভুর মাঝের পর্দা ধ্বংস করে দেয়। এখানে মূল বিষয় হলো নারীর পর্দা, ব্যক্তিগত গোপনীয়তা এবং নিরাপদ জায়গায় থাকা। হাদিসের কথাগুলো কঠোর, তাই বিষয়টি হালকা করে দেখা ঠিক নয়। তবে ব্যাখ্যায় এতটুকুই বলা যায় যে, এমন জায়গা এড়িয়ে চলা উচিত যেখানে পোশাক খোলা বা গোসলের কারণে পর্দা নষ্ট হওয়ার আশঙ্কা থাকে।"},"teachings":["নারীর জন্য পোশাক খোলার ক্ষেত্রে নিরাপদ ও সম্মানজনক জায়গা জরুরি।","স্বামীর ঘর ছাড়া অন্যত্র গোপনীয়তা নষ্ট হওয়ার ভয় থাকলে সতর্ক থাকা দরকার।","গণগোসলখানা নিয়ে সাহাবিয়াদের সতর্কতা ছিল।","পর্দা রক্ষা আল্লাহর সাথে সম্পর্কের আদবের অংশ।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নিজের ঘর ছাড়া পোশাক খোলার ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের ঘর ছাড়া অন্যত্র পোশাক খোলার বিষয়ে উম্মু সালামা রা. নারীদের কঠোর সতর্কতা শুনিয়েছেন।"},"heading":{"title":"নিজের ঘর ছাড়া পোশাক খোলা: উম্মু সালামা রা.-এর সতর্কতা","description":"এই বর্ণনায় কিছু মহিলা উম্মু সালামা রাদিয়াল্লাহু আনহার কাছে এলে তিনি তাদের পরিচয় জানতে চান। তারা জানায়, তারা হিমসের অধিবাসী। তখন তিনি বুঝতে চান, তারা কি গোসলখানায় প্রবেশকারীদের মধ্যে। তারা জিজ্ঞেস করে, এতে কোনো সমস্যা আছে কি না। উম্মু সালামা রাদিয়াল্লাহু আনহা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের বাণী শুনিয়ে বলেন, যে মহিলা নিজের ঘর ছাড়া অন্যের ঘরে নিজের পোশাক খুলে, আল্লাহ তার পর্দা ছিন্ন করে দেন। এই হাদিসের মূল কথা হলো, নারীর পর্দা ও গোপনীয়তা রক্ষার ব্যাপারে অবহেলা করা যাবে না। গোসলখানা বা অন্য জায়গা যদি পর্দার জন্য নিরাপদ না হয়, সেখানে সতর্ক থাকা প্রয়োজন।"},"teachings":["নারীর নিজ ঘর পর্দা ও গোপনীয়তার নিরাপদ জায়গা।","গোসলখানায় প্রবেশের আগে পর্দা নষ্ট হওয়ার আশঙ্কা ভাবতে হবে।","সাহাবিয়ারা নারীদের শালীনতা বিষয়ে সতর্ক করতেন।","পোশাক খোলা ব্যক্তিগত বিষয়, তাই তা নিরাপদ জায়গায় হওয়া দরকার।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E75" s="4" t="n"/>
@@ -2225,12 +2221,12 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>172</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নিজের ঘর ছাড়া পোশাক খোলার ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. নিজের ঘর ছাড়া অন্যত্র পোশাক খোলার বিষয়ে উম্মু সালামা রা. নারীদের কঠোর সতর্কতা শুনিয়েছেন।"},"heading":{"title":"নিজের ঘর ছাড়া পোশাক খোলা: উম্মু সালামা রা.-এর সতর্কতা","description":"এই বর্ণনায় কিছু মহিলা উম্মু সালামা রাদিয়াল্লাহু আনহার কাছে এলে তিনি তাদের পরিচয় জানতে চান। তারা জানায়, তারা হিমসের অধিবাসী। তখন তিনি বুঝতে চান, তারা কি গোসলখানায় প্রবেশকারীদের মধ্যে। তারা জিজ্ঞেস করে, এতে কোনো সমস্যা আছে কি না। উম্মু সালামা রাদিয়াল্লাহু আনহা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের বাণী শুনিয়ে বলেন, যে মহিলা নিজের ঘর ছাড়া অন্যের ঘরে নিজের পোশাক খুলে, আল্লাহ তার পর্দা ছিন্ন করে দেন। এই হাদিসের মূল কথা হলো, নারীর পর্দা ও গোপনীয়তা রক্ষার ব্যাপারে অবহেলা করা যাবে না। গোসলখানা বা অন্য জায়গা যদি পর্দার জন্য নিরাপদ না হয়, সেখানে সতর্ক থাকা প্রয়োজন।"},"teachings":["নারীর নিজ ঘর পর্দা ও গোপনীয়তার নিরাপদ জায়গা।","গোসলখানায় প্রবেশের আগে পর্দা নষ্ট হওয়ার আশঙ্কা ভাবতে হবে।","সাহাবিয়ারা নারীদের শালীনতা বিষয়ে সতর্ক করতেন।","পোশাক খোলা ব্যক্তিগত বিষয়, তাই তা নিরাপদ জায়গায় হওয়া দরকার।"],"related_hadiths":[{"id":"4010","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2803","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"3750","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈমানদারের পাঁচ সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. গোসলখানায় পর্দা, স্ত্রীকে রক্ষা, মদ থেকে দূরে থাকা ও মাহরাম ছাড়া নির্জনতা এড়ানোর শিক্ষা এসেছে।"},"heading":{"title":"ঈমানদারের সতর্কতা: পর্দা, মদ ও নির্জনতা থেকে বাঁচা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম কয়েকটি সতর্কতা একসাথে বলেছেন। যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন গোসলখানায় পর্দাহীনভাবে প্রবেশ না করে। সে যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। সে যেন মদ পান না করে এবং এমন দস্তরখানায় না বসে যেখানে মদ পান করা হয়। আরও বলা হয়েছে, মাহরাম পুরুষ না থাকলে কোনো নারীর সাথে নির্জনে থাকা যাবে না। এখানে মূল শিক্ষা হলো, ঈমান মানুষকে শুধু ইবাদতে নয়, পরিবেশ, সম্পর্ক ও আচরণেও সতর্ক করে। মদ, পর্দাহীনতা এবং গায়রে মাহরাম নির্জনতা—এসব বিষয় মানুষকে গুনাহের দিকে নিতে পারে। তাই হাদিসটি দৈনন্দিন জীবনে সীমা মানার শিক্ষা দেয়।"},"teachings":["গোসলখানায় পর্দা ও শালীনতা বজায় রাখা জরুরি।","মদ পান এবং মদের আসর—দুইটি থেকেই দূরে থাকার শিক্ষা এসেছে।","মাহরাম ছাড়া নারীর সাথে নির্জনে থাকা থেকে বিরত থাকতে বলা হয়েছে।","ঈমান মানুষের ব্যক্তিগত ও সামাজিক আচরণকে নিয়ন্ত্রণ করে।"],"related_hadiths":[{"id":"5232","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5233","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5566","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E76" s="4" t="n"/>
@@ -2248,12 +2244,12 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>175</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ঈমানদারের পাঁচ সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. গোসলখানায় পর্দা, স্ত্রীকে রক্ষা, মদ থেকে দূরে থাকা ও মাহরাম ছাড়া নির্জনতা এড়ানোর শিক্ষা এসেছে।"},"heading":{"title":"ঈমানদারের সতর্কতা: পর্দা, মদ ও নির্জনতা থেকে বাঁচা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম কয়েকটি সতর্কতা একসাথে বলেছেন। যে আল্লাহ ও শেষ দিবসে ঈমান রাখে, সে যেন গোসলখানায় পর্দাহীনভাবে প্রবেশ না করে। সে যেন তার স্ত্রীকে গণগোসলখানায় প্রবেশ না করায়। সে যেন মদ পান না করে এবং এমন দস্তরখানায় না বসে যেখানে মদ পান করা হয়। আরও বলা হয়েছে, মাহরাম পুরুষ না থাকলে কোনো নারীর সাথে নির্জনে থাকা যাবে না। এখানে মূল শিক্ষা হলো, ঈমান মানুষকে শুধু ইবাদতে নয়, পরিবেশ, সম্পর্ক ও আচরণেও সতর্ক করে। মদ, পর্দাহীনতা এবং গায়রে মাহরাম নির্জনতা—এসব বিষয় মানুষকে গুনাহের দিকে নিতে পারে। তাই হাদিসটি দৈনন্দিন জীবনে সীমা মানার শিক্ষা দেয়।"},"teachings":["গোসলখানায় পর্দা ও শালীনতা বজায় রাখা জরুরি।","মদ পান এবং মদের আসর—দুইটি থেকেই দূরে থাকার শিক্ষা এসেছে।","মাহরাম ছাড়া নারীর সাথে নির্জনে থাকা থেকে বিরত থাকতে বলা হয়েছে।","ঈমান মানুষের ব্যক্তিগত ও সামাজিক আচরণকে নিয়ন্ত্রণ করে।"],"related_hadiths":[{"id":"5232","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5233","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5566","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের মূল ভিত্তি ও পবিত্রতা","description":"$book_name$ $hadith_number$ - $chapter_name$. জিবরীল আ.-এর প্রশ্নে ইসলাম, নামাজ, যাকাত, হজ্জ, ওমরাহ, গোসল, ওযু ও রোজার শিক্ষা এসেছে।"},"heading":{"title":"ইসলামের পরিচয়: সাক্ষ্য, নামাজ, যাকাত, হজ্জ, ওযু ও রোজা","description":"এই হাদিসে জিবরীল আলাইহিস সালামের প্রশ্নের জবাবে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ইসলাম কী তা ব্যাখ্যা করেছেন। তিনি বলেন, ইসলাম হলো আল্লাহ ছাড়া সত্য কোনো মা’বুদ নেই এবং মুহাম্মদ আল্লাহর রাসূল—এ সাক্ষ্য দেয়া। এরপর নামাজ কায়েম করা, যাকাত দেয়া, হজ্জ ও ওমরাহ আদায় করা, জানাবাত থেকে গোসল করা, পরিপূর্ণভাবে ওযু করা এবং রমযানের সিয়াম পালন করার কথা এসেছে। এই বর্ণনায় পবিত্রতা বিশেষভাবে উল্লেখিত হয়েছে—জানাবাত থেকে গোসল এবং ওযু পূর্ণ করা। এতে বোঝা যায়, ইসলাম শুধু বিশ্বাসের নাম নয়; ইবাদত, পবিত্রতা এবং নিয়মিত আমলের মাধ্যমে তা জীবনে প্রকাশ পায়। জিবরীল আলাইহিস সালাম জিজ্ঞেস করলে নবীজি বলেন, এগুলো করলে সে মুসলিম।"},"teachings":["ইসলামের শুরু তাওহীদ ও রাসূলের রিসালাতের সাক্ষ্য দিয়ে।","নামাজ, যাকাত, হজ্জ, ওমরাহ ও রোজা ইসলামের বড় আমল।","জানাবাত থেকে গোসল ও পূর্ণ ওযু ইসলামের পবিত্রতার অংশ।","ইসলাম বিশ্বাস ও কাজ—দুইয়ের সমন্বয়ে জীবনে প্রকাশ পায়।"],"related_hadiths":[{"id":"50","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"8","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E77" s="4" t="n"/>
@@ -2271,12 +2267,12 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>177</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের মূল ভিত্তি ও পবিত্রতা","description":"$book_name$ $hadith_number$ - $chapter_name$. জিবরীল আ.-এর প্রশ্নে ইসলাম, নামাজ, যাকাত, হজ্জ, ওমরাহ, গোসল, ওযু ও রোজার শিক্ষা এসেছে।"},"heading":{"title":"ইসলামের পরিচয়: সাক্ষ্য, নামাজ, যাকাত, হজ্জ, ওযু ও রোজা","description":"এই হাদিসে জিবরীল আলাইহিস সালামের প্রশ্নের জবাবে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ইসলাম কী তা ব্যাখ্যা করেছেন। তিনি বলেন, ইসলাম হলো আল্লাহ ছাড়া সত্য কোনো মা’বুদ নেই এবং মুহাম্মদ আল্লাহর রাসূল—এ সাক্ষ্য দেয়া। এরপর নামাজ কায়েম করা, যাকাত দেয়া, হজ্জ ও ওমরাহ আদায় করা, জানাবাত থেকে গোসল করা, পরিপূর্ণভাবে ওযু করা এবং রমযানের সিয়াম পালন করার কথা এসেছে। এই বর্ণনায় পবিত্রতা বিশেষভাবে উল্লেখিত হয়েছে—জানাবাত থেকে গোসল এবং ওযু পূর্ণ করা। এতে বোঝা যায়, ইসলাম শুধু বিশ্বাসের নাম নয়; ইবাদত, পবিত্রতা এবং নিয়মিত আমলের মাধ্যমে তা জীবনে প্রকাশ পায়। জিবরীল আলাইহিস সালাম জিজ্ঞেস করলে নবীজি বলেন, এগুলো করলে সে মুসলিম।"},"teachings":["ইসলামের শুরু তাওহীদ ও রাসূলের রিসালাতের সাক্ষ্য দিয়ে।","নামাজ, যাকাত, হজ্জ, ওমরাহ ও রোজা ইসলামের বড় আমল।","জানাবাত থেকে গোসল ও পূর্ণ ওযু ইসলামের পবিত্রতার অংশ।","ইসলাম বিশ্বাস ও কাজ—দুইয়ের সমন্বয়ে জীবনে প্রকাশ পায়।"],"related_hadiths":[{"id":"50","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"8","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর চিহ্নে উম্মতকে চেনা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি কিয়ামতে তাঁর উম্মতকে ওযুর উজ্জ্বল চিহ্নে চিনবেন এবং হাওযে আগে থাকবেন।"},"heading":{"title":"ওযুর চিহ্নে নবীজির উম্মতকে চেনা ও হাওযে কাওসারের আশা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম কবরস্থানে গিয়ে মুমিন কবরবাসীদের সালাম দেন এবং বলেন, আল্লাহ চাইলে আমরাও তোমাদের সাথে মিলিত হব। এরপর তিনি বলেন, তাঁর ইচ্ছে ছিল তিনি তাঁর ভাইদের দেখতে পেতেন। সাহাবীগণ জিজ্ঞেস করলে তিনি বলেন, সাহাবীরা তাঁর সাথী, আর যারা পরে আসবে তারা তাঁর ভাই। তারপর প্রশ্ন ওঠে, তিনি না দেখা উম্মতকে কীভাবে চিনবেন। নবীজি উদাহরণ দেন—কালো ঘোড়ার দলে সাদা কপাল ও সাদা পা-ওয়ালা ঘোড়া যেমন আলাদা চেনা যায়, তেমনি তাঁর উম্মত ওযুর কারণে উজ্জ্বল চিহ্ন নিয়ে আসবে। তিনি হাওযে তাদের অগ্রগামী থাকবেন। এই হাদিস ওযুর মর্যাদা ও উম্মতের প্রতি নবীজির মমতা শেখায়।"},"teachings":["কবরবাসী মুমিনদের সালাম দেয়া নবীজির আমল হিসেবে এসেছে।","পরে আসা উম্মতের প্রতি নবীজির ভালোবাসা এই হাদিসে প্রকাশ পায়।","ওযুর চিহ্ন কিয়ামতে উম্মতের পরিচয়ের কারণ হবে।","হাওযে কাওসারের আশা মুসলিমকে আমলে যত্নবান করে।"],"related_hadiths":[{"id":"136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"246","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5868","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E78" s="4" t="n"/>
@@ -2294,12 +2290,12 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>178</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর চিহ্নে উম্মতকে চেনা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজি কিয়ামতে তাঁর উম্মতকে ওযুর উজ্জ্বল চিহ্নে চিনবেন এবং হাওযে আগে থাকবেন।"},"heading":{"title":"ওযুর চিহ্নে নবীজির উম্মতকে চেনা ও হাওযে কাওসারের আশা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম কবরস্থানে গিয়ে মুমিন কবরবাসীদের সালাম দেন এবং বলেন, আল্লাহ চাইলে আমরাও তোমাদের সাথে মিলিত হব। এরপর তিনি বলেন, তাঁর ইচ্ছে ছিল তিনি তাঁর ভাইদের দেখতে পেতেন। সাহাবীগণ জিজ্ঞেস করলে তিনি বলেন, সাহাবীরা তাঁর সাথী, আর যারা পরে আসবে তারা তাঁর ভাই। তারপর প্রশ্ন ওঠে, তিনি না দেখা উম্মতকে কীভাবে চিনবেন। নবীজি উদাহরণ দেন—কালো ঘোড়ার দলে সাদা কপাল ও সাদা পা-ওয়ালা ঘোড়া যেমন আলাদা চেনা যায়, তেমনি তাঁর উম্মত ওযুর কারণে উজ্জ্বল চিহ্ন নিয়ে আসবে। তিনি হাওযে তাদের অগ্রগামী থাকবেন। এই হাদিস ওযুর মর্যাদা ও উম্মতের প্রতি নবীজির মমতা শেখায়।"},"teachings":["কবরবাসী মুমিনদের সালাম দেয়া নবীজির আমল হিসেবে এসেছে।","পরে আসা উম্মতের প্রতি নবীজির ভালোবাসা এই হাদিসে প্রকাশ পায়।","ওযুর চিহ্ন কিয়ামতে উম্মতের পরিচয়ের কারণ হবে।","হাওযে কাওসারের আশা মুসলিমকে আমলে যত্নবান করে।"],"related_hadiths":[{"id":"136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"246","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5868","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর প্রভাবে উজ্জ্বল উম্মত","description":"$book_name$ $hadith_number$ - $chapter_name$. যাদের নবীজি দেখেননি, তাদেরও তিনি ওযুর উজ্জ্বল চিহ্নের মাধ্যমে চিনবেন—এটাই মূল শিক্ষা।"},"heading":{"title":"ওযুর প্রভাব: না দেখা উম্মতকেও চেনার আলামত","description":"এই হাদিসে সাহাবীগণ প্রশ্ন করেন, হে আল্লাহর রাসূল, আপনার উম্মতের মধ্যে যাদের আপনি দেখেননি, তাদেরকে কীভাবে চিনবেন। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উত্তরে বলেন, ওযুর প্রভাবে তাদের মুখমণ্ডল ও হাত-পা উজ্জ্বল হবে, তাদেরকে সাদা-কাল অবস্থায় দেখা যাবে। এই বর্ণনা আগের হাদিসগুলোর সাথে একই মূল শিক্ষা দেয়—ওযু কিয়ামতের দিনে উম্মতের পরিচয়ের বড় চিহ্ন হবে। একজন মুসলিম দুনিয়ায় যখন ওযু করে, তখন সে শুধু বাহ্যিক পবিত্রতা অর্জন করে না; আখিরাতে এই আমলের একটি আলাদা মর্যাদাও প্রকাশ পাবে। তাই ওযুতে অবহেলা করা উচিত নয়। প্রতিটি অঙ্গ ঠিকভাবে ধোয়া, নামাজের আগে পবিত্র হওয়া এবং পবিত্রতার প্রতি ভালোবাসা রাখা এই হাদিসের বাস্তব শিক্ষা।"},"teachings":["ওযু কিয়ামতে উম্মতের পরিচয়ের চিহ্ন হবে।","নবীজি তাঁর না দেখা উম্মতকেও আলাদা চিহ্নে চিনবেন।","ওযু শুধু বাহ্যিক পরিচ্ছন্নতা নয়, আখিরাতের মর্যাদার আমল।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়ার প্রতি যত্ন দরকার।"],"related_hadiths":[{"id":"136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"246","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5868","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E79" s="4" t="n"/>
@@ -2317,12 +2313,12 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর প্রভাবে উজ্জ্বল উম্মত","description":"$book_name$ $hadith_number$ - $chapter_name$. যাদের নবীজি দেখেননি, তাদেরও তিনি ওযুর উজ্জ্বল চিহ্নের মাধ্যমে চিনবেন—এটাই মূল শিক্ষা।"},"heading":{"title":"ওযুর প্রভাব: না দেখা উম্মতকেও চেনার আলামত","description":"এই হাদিসে সাহাবীগণ প্রশ্ন করেন, হে আল্লাহর রাসূল, আপনার উম্মতের মধ্যে যাদের আপনি দেখেননি, তাদেরকে কীভাবে চিনবেন। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উত্তরে বলেন, ওযুর প্রভাবে তাদের মুখমণ্ডল ও হাত-পা উজ্জ্বল হবে, তাদেরকে সাদা-কাল অবস্থায় দেখা যাবে। এই বর্ণনা আগের হাদিসগুলোর সাথে একই মূল শিক্ষা দেয়—ওযু কিয়ামতের দিনে উম্মতের পরিচয়ের বড় চিহ্ন হবে। একজন মুসলিম দুনিয়ায় যখন ওযু করে, তখন সে শুধু বাহ্যিক পবিত্রতা অর্জন করে না; আখিরাতে এই আমলের একটি আলাদা মর্যাদাও প্রকাশ পাবে। তাই ওযুতে অবহেলা করা উচিত নয়। প্রতিটি অঙ্গ ঠিকভাবে ধোয়া, নামাজের আগে পবিত্র হওয়া এবং পবিত্রতার প্রতি ভালোবাসা রাখা এই হাদিসের বাস্তব শিক্ষা।"},"teachings":["ওযু কিয়ামতে উম্মতের পরিচয়ের চিহ্ন হবে।","নবীজি তাঁর না দেখা উম্মতকেও আলাদা চিহ্নে চিনবেন।","ওযু শুধু বাহ্যিক পরিচ্ছন্নতা নয়, আখিরাতের মর্যাদার আমল।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়ার প্রতি যত্ন দরকার।"],"related_hadiths":[{"id":"136","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"246","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5868","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভালো ইচ্ছা ও মন্দ থেকে ফিরে আসা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ ফেরেশতাদের বলেন, বান্দা পাপ না করা পর্যন্ত তা লিখো না; নেক ইচ্ছা নেকি হিসেবে লিখো।"},"heading":{"title":"ভালো ইচ্ছা, পাপ ছেড়ে দেওয়া ও আল্লাহর দয়া","description":"এই হাদিসে আল্লাহর পক্ষ থেকে ফেরেশতাদের উদ্দেশে নির্দেশের কথা এসেছে। বান্দা যখন কোনো খারাপ কাজের ইচ্ছা করে, তা বাস্তবায়ন না করা পর্যন্ত লিখতে বলা হয় না। যদি সে পাপ করে, তার অনুরূপ পাপ লেখা হয়। আর যদি আল্লাহর কারণে তা ছেড়ে দেয়, তাহলে তার জন্য একটি নেকি লেখা হয়। অন্যদিকে বান্দা যদি কোনো ভালো কাজের ইচ্ছা করে কিন্তু করতে না পারে, তবু একটি নেকি লেখা হয়। আর যদি তা করে, তাহলে দশ থেকে সাতশত গুণ পর্যন্ত লেখা হয়। মুসলিমের বর্ণনাগুলোতেও একই অর্থ এসেছে—নেক ইচ্ছা মূল্যবান, আর পাপ ছেড়ে দেওয়া বিশেষ করে আল্লাহর জন্য হলে তা নেকির কারণ হতে পারে। এই হাদিস মানুষকে আল্লাহর দয়ার দিকে আশা দেয় এবং একই সাথে নিজের চিন্তা ও ইচ্ছাকে ভালো পথে চালানোর শিক্ষা দেয়।"},"teachings":["ভালো কাজের ইচ্ছা আল্লাহর কাছে মূল্যবান।","আল্লাহর কারণে পাপ ছেড়ে দেওয়া নেকির কারণ হতে পারে।","পাপ কাজ না করা পর্যন্ত তা লেখা হয় না—এতে আল্লাহর দয়া প্রকাশ পায়।","নেক কাজ করলে প্রতিদান অনেক গুণে বাড়তে পারে।"],"related_hadiths":[{"id":"6491","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"237","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E80" s="4" t="n"/>
@@ -2340,12 +2336,12 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>181</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভালো ইচ্ছা ও মন্দ থেকে ফিরে আসা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ ফেরেশতাদের বলেন, বান্দা পাপ না করা পর্যন্ত তা লিখো না; নেক ইচ্ছা নেকি হিসেবে লিখো।"},"heading":{"title":"ভালো ইচ্ছা, পাপ ছেড়ে দেওয়া ও আল্লাহর দয়া","description":"এই হাদিসে আল্লাহর পক্ষ থেকে ফেরেশতাদের উদ্দেশে নির্দেশের কথা এসেছে। বান্দা যখন কোনো খারাপ কাজের ইচ্ছা করে, তা বাস্তবায়ন না করা পর্যন্ত লিখতে বলা হয় না। যদি সে পাপ করে, তার অনুরূপ পাপ লেখা হয়। আর যদি আল্লাহর কারণে তা ছেড়ে দেয়, তাহলে তার জন্য একটি নেকি লেখা হয়। অন্যদিকে বান্দা যদি কোনো ভালো কাজের ইচ্ছা করে কিন্তু করতে না পারে, তবু একটি নেকি লেখা হয়। আর যদি তা করে, তাহলে দশ থেকে সাতশত গুণ পর্যন্ত লেখা হয়। মুসলিমের বর্ণনাগুলোতেও একই অর্থ এসেছে—নেক ইচ্ছা মূল্যবান, আর পাপ ছেড়ে দেওয়া বিশেষ করে আল্লাহর জন্য হলে তা নেকির কারণ হতে পারে। এই হাদিস মানুষকে আল্লাহর দয়ার দিকে আশা দেয় এবং একই সাথে নিজের চিন্তা ও ইচ্ছাকে ভালো পথে চালানোর শিক্ষা দেয়।"},"teachings":["ভালো কাজের ইচ্ছা আল্লাহর কাছে মূল্যবান।","আল্লাহর কারণে পাপ ছেড়ে দেওয়া নেকির কারণ হতে পারে।","পাপ কাজ না করা পর্যন্ত তা লেখা হয় না—এতে আল্লাহর দয়া প্রকাশ পায়।","নেক কাজ করলে প্রতিদান অনেক গুণে বাড়তে পারে।"],"related_hadiths":[{"id":"6491","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"237","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর ফজিলত ও পাপ মোচন","description":"$book_name$ $hadith_number$ - $chapter_name$. ওযুর অঙ্গ ধোয়ার সাথে চোখ, হাত ও পায়ের পাপ ঝরে যায়—হাদিসটি পবিত্রতার গভীর ফজিলত শেখায়।"},"heading":{"title":"ওযুর ফজিলত: অঙ্গ ধোয়ার সাথে পাপ মোচনের শিক্ষা","description":"এই হাদিসে ওযুর ফজিলত খুব সহজভাবে বোঝানো হয়েছে। একজন মুসলিম বা মুমিন বান্দা যখন ওযু করে, তখন শুধু বাহ্যিক ময়লা দূর হয় না; আল্লাহর দয়ায় তার পাপও ঝরে যায়। মুখ ধোয়ার সময় চোখ দিয়ে করা ভুল কাজের পাপ বের হয়ে যায়। হাত ধোয়ার সময় হাতে করা ভুল কাজের পাপ দূর হয়। পা ধোয়ার সময় পা দিয়ে যে ভুল পথে চলা হয়েছে, তার পাপও ঝরে যায়। তাই ওযু কেবল সালাতের প্রস্তুতি নয়, এটি পাপ মোচনের একটি বড় মাধ্যম। তবে হাদিসের ভাষা থেকে বুঝি, ওযু সুন্দরভাবে ও মনোযোগ দিয়ে করা উচিত, যেন বান্দা পবিত্র অবস্থায় ইবাদতের দিকে এগিয়ে যায়।"},"teachings":["ওযু বাহ্যিক পবিত্রতার পাশাপাশি পাপ মোচনের কারণ হয়।","চোখ, হাত ও পা দিয়ে করা ভুলের ব্যাপারে সতর্ক থাকা দরকার।","সালাতের আগে সুন্দরভাবে ওযু করা মুমিনের জন্য বড় কল্যাণের কাজ।","পবিত্রতা অর্জনের সময় আল্লাহর দয়ার আশা রাখা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E81" s="4" t="n"/>
@@ -2363,12 +2359,12 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>182</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযুর ফজিলত ও পাপ মোচন","description":"$book_name$ $hadith_number$ - $chapter_name$. ওযুর অঙ্গ ধোয়ার সাথে চোখ, হাত ও পায়ের পাপ ঝরে যায়—হাদিসটি পবিত্রতার গভীর ফজিলত শেখায়।"},"heading":{"title":"ওযুর ফজিলত: অঙ্গ ধোয়ার সাথে পাপ মোচনের শিক্ষা","description":"এই হাদিসে ওযুর ফজিলত খুব সহজভাবে বোঝানো হয়েছে। একজন মুসলিম বা মুমিন বান্দা যখন ওযু করে, তখন শুধু বাহ্যিক ময়লা দূর হয় না; আল্লাহর দয়ায় তার পাপও ঝরে যায়। মুখ ধোয়ার সময় চোখ দিয়ে করা ভুল কাজের পাপ বের হয়ে যায়। হাত ধোয়ার সময় হাতে করা ভুল কাজের পাপ দূর হয়। পা ধোয়ার সময় পা দিয়ে যে ভুল পথে চলা হয়েছে, তার পাপও ঝরে যায়। তাই ওযু কেবল সালাতের প্রস্তুতি নয়, এটি পাপ মোচনের একটি বড় মাধ্যম। তবে হাদিসের ভাষা থেকে বুঝি, ওযু সুন্দরভাবে ও মনোযোগ দিয়ে করা উচিত, যেন বান্দা পবিত্র অবস্থায় ইবাদতের দিকে এগিয়ে যায়।"},"teachings":["ওযু বাহ্যিক পবিত্রতার পাশাপাশি পাপ মোচনের কারণ হয়।","চোখ, হাত ও পা দিয়ে করা ভুলের ব্যাপারে সতর্ক থাকা দরকার।","সালাতের আগে সুন্দরভাবে ওযু করা মুমিনের জন্য বড় কল্যাণের কাজ।","পবিত্রতা অর্জনের সময় আল্লাহর দয়ার আশা রাখা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওযু ও গুনাহ মাফ","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরভাবে ওযু করলে শরীরের পাপ দূর হয়; এমনকি নখের নিচ থেকেও পাপ বের হওয়ার কথা হাদিসে এসেছে।"},"heading":{"title":"সুন্দরভাবে ওযু করলে পাপ মাফ হওয়ার ফজিলত","description":"এই হাদিসে সুন্দরভাবে ওযু করার গুরুত্ব এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি ওযু করে এবং তা সুন্দরভাবে শেষ করে, তার পাপ শরীর থেকে বের হয়ে যায়, এমনকি নখের নিচ থেকেও। একই বিষয়ের আরেক বর্ণনায় উসমান (রাঃ) নবীজির ওযুর মতো ওযু করে জানান, এভাবে ওযু করলে পূর্বের পাপ ক্ষমা করা হয় এবং সালাত ও মসজিদে যাওয়ার আমল অতিরিক্ত সওয়াবের কারণ হয়। নাসাঈর বর্ণনায় সালাত থেকে পরবর্তী সালাত পর্যন্ত মাঝের পাপ ক্ষমার কথা এসেছে। তাই ওযু করার নিয়ম শুধু বাহ্যিক কাজ নয়; এতে মনোযোগ, সুন্দরভাবে ধোয়া এবং আল্লাহর আদেশ মেনে চলার শিক্ষা আছে।"},"teachings":["সুন্দরভাবে ওযু করা পাপ মাফের কারণ হিসেবে এসেছে।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়ার প্রতি যত্ন নেওয়া উচিত।","সালাত ও মসজিদে গমন আলাদা নফল সওয়াবের কারণ হতে পারে।","হাদিসে সতর্ক করা হয়েছে—ফজিলত শুনে ধোকায় পড়া উচিত নয়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E82" s="4" t="n"/>
@@ -2386,12 +2382,12 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>183</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওযু ও গুনাহ মাফ","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্দরভাবে ওযু করলে শরীরের পাপ দূর হয়; এমনকি নখের নিচ থেকেও পাপ বের হওয়ার কথা হাদিসে এসেছে।"},"heading":{"title":"সুন্দরভাবে ওযু করলে পাপ মাফ হওয়ার ফজিলত","description":"এই হাদিসে সুন্দরভাবে ওযু করার গুরুত্ব এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি ওযু করে এবং তা সুন্দরভাবে শেষ করে, তার পাপ শরীর থেকে বের হয়ে যায়, এমনকি নখের নিচ থেকেও। একই বিষয়ের আরেক বর্ণনায় উসমান (রাঃ) নবীজির ওযুর মতো ওযু করে জানান, এভাবে ওযু করলে পূর্বের পাপ ক্ষমা করা হয় এবং সালাত ও মসজিদে যাওয়ার আমল অতিরিক্ত সওয়াবের কারণ হয়। নাসাঈর বর্ণনায় সালাত থেকে পরবর্তী সালাত পর্যন্ত মাঝের পাপ ক্ষমার কথা এসেছে। তাই ওযু করার নিয়ম শুধু বাহ্যিক কাজ নয়; এতে মনোযোগ, সুন্দরভাবে ধোয়া এবং আল্লাহর আদেশ মেনে চলার শিক্ষা আছে।"},"teachings":["সুন্দরভাবে ওযু করা পাপ মাফের কারণ হিসেবে এসেছে।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়ার প্রতি যত্ন নেওয়া উচিত।","সালাত ও মসজিদে গমন আলাদা নফল সওয়াবের কারণ হতে পারে।","হাদিসে সতর্ক করা হয়েছে—ফজিলত শুনে ধোকায় পড়া উচিত নয়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীজির মতো ওযু ও দুই রাকাআত সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজির মতো সুন্দরভাবে ওযু করে মসজিদে গিয়ে দুই রাকাআত সালাত আদায়ের ফজিলত এ হাদিসে এসেছে।"},"heading":{"title":"নবীজির মতো ওযু করে দুই রাকাআত সালাতের ফজিলত","description":"এই হাদিসে উসমান (রাঃ) নিজের দেখা একটি আমল শিক্ষা দিয়েছেন। তিনি মসজিদে নববীর পাশে বসে পানি নিয়ে সুন্দরভাবে ওযু করেন। এরপর বলেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে একই স্থানে এভাবে ওযু করতে দেখেছেন। নবীজি বলেছেন, যে ব্যক্তি এ ধরনের ওযু করে, তারপর মসজিদে এসে দুই রাকাআত সালাত পড়ে এবং বসে, তার পূর্বের পাপ ক্ষমা করা হয়। এখানে ওযু, মসজিদে আসা এবং সালাত—তিনটি বিষয় একসাথে এসেছে। তবে শেষে “তোমরা ধোকায় পড় না” বলা হয়েছে। তাই এই ফজিলত শুনে অবহেলা নয়; বরং সতর্কতা, আন্তরিকতা ও নিয়ম মেনে আমল করা দরকার।"},"teachings":["নবীজির মতো ওযু করার চেষ্টা করা একটি উত্তম আমল।","ওযুর পর দুই রাকাআত সালাত আদায়ের ফজিলত আছে।","মসজিদে গিয়ে সালাত আদায় করা এই বর্ণনায় বিশেষভাবে এসেছে।","ফজিলতের ওপর ভর করে পাপে ঢিলে হওয়া ঠিক নয়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"887","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E83" s="4" t="n"/>
@@ -2409,12 +2405,12 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>184</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীজির মতো ওযু ও দুই রাকাআত সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজির মতো সুন্দরভাবে ওযু করে মসজিদে গিয়ে দুই রাকাআত সালাত আদায়ের ফজিলত এ হাদিসে এসেছে।"},"heading":{"title":"নবীজির মতো ওযু করে দুই রাকাআত সালাতের ফজিলত","description":"এই হাদিসে উসমান (রাঃ) নিজের দেখা একটি আমল শিক্ষা দিয়েছেন। তিনি মসজিদে নববীর পাশে বসে পানি নিয়ে সুন্দরভাবে ওযু করেন। এরপর বলেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে একই স্থানে এভাবে ওযু করতে দেখেছেন। নবীজি বলেছেন, যে ব্যক্তি এ ধরনের ওযু করে, তারপর মসজিদে এসে দুই রাকাআত সালাত পড়ে এবং বসে, তার পূর্বের পাপ ক্ষমা করা হয়। এখানে ওযু, মসজিদে আসা এবং সালাত—তিনটি বিষয় একসাথে এসেছে। তবে শেষে “তোমরা ধোকায় পড় না” বলা হয়েছে। তাই এই ফজিলত শুনে অবহেলা নয়; বরং সতর্কতা, আন্তরিকতা ও নিয়ম মেনে আমল করা দরকার।"},"teachings":["নবীজির মতো ওযু করার চেষ্টা করা একটি উত্তম আমল।","ওযুর পর দুই রাকাআত সালাত আদায়ের ফজিলত আছে।","মসজিদে গিয়ে সালাত আদায় করা এই বর্ণনায় বিশেষভাবে এসেছে।","ফজিলতের ওপর ভর করে পাপে ঢিলে হওয়া ঠিক নয়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"887","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অঙ্গ ধোয়ার সাথে পাপ মোচন","description":"$book_name$ $hadith_number$ - $chapter_name$. মুখ, হাত, মাথা ও পা ধোয়া বা মাসেহ করার সাথে সংশ্লিষ্ট পাপ মোচনের কথা এই হাদিসে এসেছে।"},"heading":{"title":"ওযুর অঙ্গ ধোয়ার সাথে গুনাহ মাফের শিক্ষা","description":"এই হাদিসে উসমান (রাঃ)-এর একটি সুন্দর ঘটনা এসেছে। তিনি পানি আনিয়ে ওযু করলেন এবং হাসলেন। সাথীরা কারণ জানতে চাইলে তিনি বললেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে এভাবেই ওযু করতে ও হাসতে দেখেছেন। এরপর নবীজি বলেছেন, বান্দা যখন ওযুর পানি আনে এবং মুখ ধোয়, তখন মুখের মাধ্যমে করা পাপ আল্লাহ মুছে দেন। হাত ধুলে হাতের পাপ দূর হয়। পা ধুলেও একইভাবে পাপ মোচন হয়। বাযযারের বর্ণনায় মাথা মাসেহ করলেও এমন হওয়ার কথা এসেছে। এই হাদিসে ওযুকে পবিত্রতা ও গুনাহ মাফের মাধ্যম হিসেবে দেখানো হয়েছে। তাই ওযুর প্রতিটি অঙ্গ ধোয়ার সময় বান্দার উচিত নিজের ভুলের কথা মনে করে আল্লাহর দয়া আশা করা।"},"teachings":["ওযুর প্রতিটি ধাপে আল্লাহর দয়ার আশা করা যায়।","মুখ, হাত, মাথা ও পা দিয়ে করা ভুল থেকে সাবধান থাকা দরকার।","ওযু শুধু পানি ব্যবহার নয়; এটি বান্দার জন্য পাপ মোচনের সুযোগ।","সাহাবারা নবীজির আমল দেখে তা শেখাতেন।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E84" s="4" t="n"/>
@@ -2432,12 +2428,12 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>185</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অঙ্গ ধোয়ার সাথে পাপ মোচন","description":"$book_name$ $hadith_number$ - $chapter_name$. মুখ, হাত, মাথা ও পা ধোয়া বা মাসেহ করার সাথে সংশ্লিষ্ট পাপ মোচনের কথা এই হাদিসে এসেছে।"},"heading":{"title":"ওযুর অঙ্গ ধোয়ার সাথে গুনাহ মাফের শিক্ষা","description":"এই হাদিসে উসমান (রাঃ)-এর একটি সুন্দর ঘটনা এসেছে। তিনি পানি আনিয়ে ওযু করলেন এবং হাসলেন। সাথীরা কারণ জানতে চাইলে তিনি বললেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে এভাবেই ওযু করতে ও হাসতে দেখেছেন। এরপর নবীজি বলেছেন, বান্দা যখন ওযুর পানি আনে এবং মুখ ধোয়, তখন মুখের মাধ্যমে করা পাপ আল্লাহ মুছে দেন। হাত ধুলে হাতের পাপ দূর হয়। পা ধুলেও একইভাবে পাপ মোচন হয়। বাযযারের বর্ণনায় মাথা মাসেহ করলেও এমন হওয়ার কথা এসেছে। এই হাদিসে ওযুকে পবিত্রতা ও গুনাহ মাফের মাধ্যম হিসেবে দেখানো হয়েছে। তাই ওযুর প্রতিটি অঙ্গ ধোয়ার সময় বান্দার উচিত নিজের ভুলের কথা মনে করে আল্লাহর দয়া আশা করা।"},"teachings":["ওযুর প্রতিটি ধাপে আল্লাহর দয়ার আশা করা যায়।","মুখ, হাত, মাথা ও পা দিয়ে করা ভুল থেকে সাবধান থাকা দরকার।","ওযু শুধু পানি ব্যবহার নয়; এটি বান্দার জন্য পাপ মোচনের সুযোগ।","সাহাবারা নবীজির আমল দেখে তা শেখাতেন।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুলি, নাক ঝাড়া ও পূর্ণ ওযুর ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. কুলি, নাকে পানি, মুখ, হাত, মাথা ও পা—ওযুর প্রতিটি ধাপে পাপ ঝরে যাওয়ার শিক্ষা এ হাদিসে এসেছে।"},"heading":{"title":"পূর্ণ ওযুর ফজিলত: কুলি থেকে পা ধোয়া পর্যন্ত পাপ মোচন","description":"এই হাদিসে ওযুর ধাপগুলো আলাদা করে উল্লেখ করা হয়েছে। বান্দা যখন কুলি করে, মুখের পাপ বের হয়। নাকে পানি দিয়ে নাক ঝাড়লে নাকের পাপ ঝরে পড়ে। মুখ ধোয়ার সময় চোখের পাতার প্রান্ত পর্যন্ত পাপ বের হওয়ার কথা এসেছে। হাত ধোয়ার সময় হাতের নখের নিচ থেকেও পাপ বের হয়। মাথা মাসেহ করলে মাথা ও কান সম্পর্কিত পাপ দূর হয়। পা ধুলে পায়ের নখের নিচ থেকেও পাপ ঝরে যায়। এরপর মসজিদে যাওয়া ও সালাত তার জন্য নফল বা অতিরিক্ত হয়। এ হাদিস ওযুর ফজিলতকে খুব পরিষ্কারভাবে তুলে ধরে। তাই পূর্ণ ওযু করার সময় প্রতিটি অংশে যত্ন নেওয়া দরকার।"},"teachings":["কুলি, নাক পরিষ্কার, মুখ, হাত, মাথা ও পা—সব ধাপে ওযুর গুরুত্ব আছে।","ওযু পাপ মোচনের কারণ হিসেবে হাদিসে এসেছে।","মসজিদে গমন ও সালাত আলাদা নফল সওয়াবের কারণ হতে পারে।","ওযুর ছোট অংশগুলো অবহেলা না করে সুন্দরভাবে করা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E85" s="4" t="n"/>
@@ -2455,12 +2451,12 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>186</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুলি, নাক ঝাড়া ও পূর্ণ ওযুর ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. কুলি, নাকে পানি, মুখ, হাত, মাথা ও পা—ওযুর প্রতিটি ধাপে পাপ ঝরে যাওয়ার শিক্ষা এ হাদিসে এসেছে।"},"heading":{"title":"পূর্ণ ওযুর ফজিলত: কুলি থেকে পা ধোয়া পর্যন্ত পাপ মোচন","description":"এই হাদিসে ওযুর ধাপগুলো আলাদা করে উল্লেখ করা হয়েছে। বান্দা যখন কুলি করে, মুখের পাপ বের হয়। নাকে পানি দিয়ে নাক ঝাড়লে নাকের পাপ ঝরে পড়ে। মুখ ধোয়ার সময় চোখের পাতার প্রান্ত পর্যন্ত পাপ বের হওয়ার কথা এসেছে। হাত ধোয়ার সময় হাতের নখের নিচ থেকেও পাপ বের হয়। মাথা মাসেহ করলে মাথা ও কান সম্পর্কিত পাপ দূর হয়। পা ধুলে পায়ের নখের নিচ থেকেও পাপ ঝরে যায়। এরপর মসজিদে যাওয়া ও সালাত তার জন্য নফল বা অতিরিক্ত হয়। এ হাদিস ওযুর ফজিলতকে খুব পরিষ্কারভাবে তুলে ধরে। তাই পূর্ণ ওযু করার সময় প্রতিটি অংশে যত্ন নেওয়া দরকার।"},"teachings":["কুলি, নাক পরিষ্কার, মুখ, হাত, মাথা ও পা—সব ধাপে ওযুর গুরুত্ব আছে।","ওযু পাপ মোচনের কারণ হিসেবে হাদিসে এসেছে।","মসজিদে গমন ও সালাত আলাদা নফল সওয়াবের কারণ হতে পারে।","ওযুর ছোট অংশগুলো অবহেলা না করে সুন্দরভাবে করা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযু, একাগ্র সালাত ও নিষ্পাপ হওয়ার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. আদেশমতো ওযু করে একাগ্র মনে সালাত আদায় করলে পাপ থেকে পবিত্র হওয়ার বড় ফজিলত এ হাদিসে এসেছে।"},"heading":{"title":"ওযু ও একাগ্র সালাত: পাপ থেকে পবিত্র হওয়ার পথ","description":"এই হাদিসে আমর ইবনু আবাসা (রাঃ)-এর প্রশ্নের উত্তরে ওযুর ফজিলত বলা হয়েছে। তিনি নবীজির কাছে ওযু সম্পর্কে জানতে চান। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেন, কুলি, নাকে পানি দেওয়া ও নাক ঝাড়ার মাধ্যমে মুখ ও নাকের পাপ ঝরে পড়ে। আল্লাহর আদেশ অনুযায়ী মুখ, হাত, মাথা ও পা ধুলে বা মাসেহ করলে অঙ্গগুলোর পাপ পানির সাথে পড়ে যায়। এরপর যদি বান্দা দাঁড়িয়ে সালাত পড়ে, আল্লাহর প্রশংসা করে এবং মনকে শুধু আল্লাহর জন্য খালি রাখে, তাহলে সে পাপ থেকে এমনভাবে ফিরে আসে যেন মায়ের গর্ভ থেকে জন্মের দিনের মতো। এখানে ওযু ও মনোযোগী সালাত একসাথে এসেছে। তাই বাহ্যিক পবিত্রতার সাথে অন্তরের একাগ্রতাও জরুরি।"},"teachings":["আল্লাহর আদেশ অনুযায়ী ওযু করা বড় ফজিলতের কাজ।","ওযুর পর মনোযোগী সালাত পাপ মোচনের কারণ হিসেবে এসেছে।","সালাতে আল্লাহর প্রশংসা ও অন্তরের একাগ্রতা গুরুত্বপূর্ণ।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়া উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E86" s="4" t="n"/>
@@ -2478,12 +2474,12 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>187</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ওযু, একাগ্র সালাত ও নিষ্পাপ হওয়ার শিক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. আদেশমতো ওযু করে একাগ্র মনে সালাত আদায় করলে পাপ থেকে পবিত্র হওয়ার বড় ফজিলত এ হাদিসে এসেছে।"},"heading":{"title":"ওযু ও একাগ্র সালাত: পাপ থেকে পবিত্র হওয়ার পথ","description":"এই হাদিসে আমর ইবনু আবাসা (রাঃ)-এর প্রশ্নের উত্তরে ওযুর ফজিলত বলা হয়েছে। তিনি নবীজির কাছে ওযু সম্পর্কে জানতে চান। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেন, কুলি, নাকে পানি দেওয়া ও নাক ঝাড়ার মাধ্যমে মুখ ও নাকের পাপ ঝরে পড়ে। আল্লাহর আদেশ অনুযায়ী মুখ, হাত, মাথা ও পা ধুলে বা মাসেহ করলে অঙ্গগুলোর পাপ পানির সাথে পড়ে যায়। এরপর যদি বান্দা দাঁড়িয়ে সালাত পড়ে, আল্লাহর প্রশংসা করে এবং মনকে শুধু আল্লাহর জন্য খালি রাখে, তাহলে সে পাপ থেকে এমনভাবে ফিরে আসে যেন মায়ের গর্ভ থেকে জন্মের দিনের মতো। এখানে ওযু ও মনোযোগী সালাত একসাথে এসেছে। তাই বাহ্যিক পবিত্রতার সাথে অন্তরের একাগ্রতাও জরুরি।"},"teachings":["আল্লাহর আদেশ অনুযায়ী ওযু করা বড় ফজিলতের কাজ।","ওযুর পর মনোযোগী সালাত পাপ মোচনের কারণ হিসেবে এসেছে।","সালাতে আল্লাহর প্রশংসা ও অন্তরের একাগ্রতা গুরুত্বপূর্ণ।","ওযুর অঙ্গগুলো ঠিকভাবে ধোয়া উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাতের জন্য ওযু ও মর্যাদা বৃদ্ধি","description":"$book_name$ $hadith_number$ - $chapter_name$. সালাতের ইচ্ছায় ওযু করলে অঙ্গগুলোর পাপ ঝরে যায় এবং সালাতে দাঁড়ালে মর্যাদা বাড়ে—এ শিক্ষা এসেছে।"},"heading":{"title":"সালাতের জন্য ওযু: পাপ মোচন ও মর্যাদা বৃদ্ধির হাদিস","description":"এই হাদিসে সালাতের উদ্দেশ্যে ওযু করার বিশেষ ফজিলত বলা হয়েছে। একজন ব্যক্তি যখন সালাতের জন্য ওযুতে দাঁড়ায়, হাত ধোয়ার শুরুতেই হাতের পাপ নেমে যায়। কুলি, নাকে পানি দেওয়া ও নাক ঝাড়ার সময় জিহ্বা ও ঠোঁটের পাপ ঝরে পড়ে। মুখ ধুলে কান ও চোখের পাপ দূর হয়। হাত ও পা ধোয়ার পর সে পাপ থেকে পবিত্র হওয়ার বড় ফজিলত পায়। হাদিসে আরও এসেছে, সালাতে দাঁড়ালে আল্লাহ তার মর্যাদা বাড়িয়ে দেন, আর সালাত শেষে বসলে সে ক্ষমাপ্রাপ্ত অবস্থায় বসে। অন্য বর্ণনাগুলোও ওযুকে পূর্বের পাপের কাফফারা হিসেবে উল্লেখ করেছে। তাই ওযু ও সালাতকে হালকা করে দেখা ঠিক নয়।"},"teachings":["সালাতের নিয়তে ওযু করা পাপ মোচনের কারণ হয়।","জিহ্বা, চোখ, কান, হাত ও পা—সব অঙ্গের ব্যবহার নিয়ে সতর্ক থাকা দরকার।","সালাতে দাঁড়ানো মর্যাদা বৃদ্ধির কারণ হিসেবে এসেছে।","ওযু শেষে সালাত আদায় করা বড় ফজিলতের আমল।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E87" s="4" t="n"/>
@@ -2501,12 +2497,12 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>188</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাতের জন্য ওযু ও মর্যাদা বৃদ্ধি","description":"$book_name$ $hadith_number$ - $chapter_name$. সালাতের ইচ্ছায় ওযু করলে অঙ্গগুলোর পাপ ঝরে যায় এবং সালাতে দাঁড়ালে মর্যাদা বাড়ে—এ শিক্ষা এসেছে।"},"heading":{"title":"সালাতের জন্য ওযু: পাপ মোচন ও মর্যাদা বৃদ্ধির হাদিস","description":"এই হাদিসে সালাতের উদ্দেশ্যে ওযু করার বিশেষ ফজিলত বলা হয়েছে। একজন ব্যক্তি যখন সালাতের জন্য ওযুতে দাঁড়ায়, হাত ধোয়ার শুরুতেই হাতের পাপ নেমে যায়। কুলি, নাকে পানি দেওয়া ও নাক ঝাড়ার সময় জিহ্বা ও ঠোঁটের পাপ ঝরে পড়ে। মুখ ধুলে কান ও চোখের পাপ দূর হয়। হাত ও পা ধোয়ার পর সে পাপ থেকে পবিত্র হওয়ার বড় ফজিলত পায়। হাদিসে আরও এসেছে, সালাতে দাঁড়ালে আল্লাহ তার মর্যাদা বাড়িয়ে দেন, আর সালাত শেষে বসলে সে ক্ষমাপ্রাপ্ত অবস্থায় বসে। অন্য বর্ণনাগুলোও ওযুকে পূর্বের পাপের কাফফারা হিসেবে উল্লেখ করেছে। তাই ওযু ও সালাতকে হালকা করে দেখা ঠিক নয়।"},"teachings":["সালাতের নিয়তে ওযু করা পাপ মোচনের কারণ হয়।","জিহ্বা, চোখ, কান, হাত ও পা—সব অঙ্গের ব্যবহার নিয়ে সতর্ক থাকা দরকার।","সালাতে দাঁড়ানো মর্যাদা বৃদ্ধির কারণ হিসেবে এসেছে।","ওযু শেষে সালাত আদায় করা বড় ফজিলতের আমল।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওযু ও সালাতের ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. মুখ, হাত ও পা ভালোভাবে ধুয়ে সালাত আদায় করলে পূর্বের পাপ ক্ষমার কথা এই হাদিসে এসেছে।"},"heading":{"title":"সুন্দর ওযু করে সালাত আদায়ের ফজিলত","description":"এই হাদিসে সুন্দরভাবে ওযু করার একটি সহজ ছবি পাওয়া যায়। বর্ণনাকারী বলেন, রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কতবার এই কথা বলেছেন তিনি জানেন না। নবীজি বলেছেন, বান্দা যখন সুন্দরভাবে ওযু করে, মুখ ধোয় এমনভাবে যে পানি চিবুক পর্যন্ত বয়ে যায়, হাত ধোয় এমনভাবে যে পানি কনুই পর্যন্ত পৌঁছে, পা ধোয় এমনভাবে যে পানি টাখনু পর্যন্ত বয়ে যায়, তারপর দাঁড়িয়ে সালাত আদায় করে, তখন তার আগের পাপ ক্ষমা করা হয়। এখানে ওযুর অঙ্গগুলোতে পানি পৌঁছানোর বিষয়টি স্পষ্টভাবে এসেছে। তাই ওযুতে তাড়াহুড়া না করে, অঙ্গগুলো ঠিকভাবে ধোয়া এবং এরপর সালাত আদায় করা—এটাই মূল শিক্ষা।"},"teachings":["সুন্দরভাবে ওযু করার জন্য অঙ্গে পানি পৌঁছানো দরকার।","ওযুর পর সালাত আদায় পাপ ক্ষমার কারণ হিসেবে এসেছে।","ওযুর সময় মুখ, হাত ও পা ধোয়ায় যত্ন নেওয়া উচিত।","নবীজি একই শিক্ষা বারবার বলেছেন—এতে বিষয়টির গুরুত্ব বোঝা যায়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E88" s="4" t="n"/>
@@ -2524,12 +2520,12 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>189</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্দর ওযু ও সালাতের ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. মুখ, হাত ও পা ভালোভাবে ধুয়ে সালাত আদায় করলে পূর্বের পাপ ক্ষমার কথা এই হাদিসে এসেছে।"},"heading":{"title":"সুন্দর ওযু করে সালাত আদায়ের ফজিলত","description":"এই হাদিসে সুন্দরভাবে ওযু করার একটি সহজ ছবি পাওয়া যায়। বর্ণনাকারী বলেন, রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কতবার এই কথা বলেছেন তিনি জানেন না। নবীজি বলেছেন, বান্দা যখন সুন্দরভাবে ওযু করে, মুখ ধোয় এমনভাবে যে পানি চিবুক পর্যন্ত বয়ে যায়, হাত ধোয় এমনভাবে যে পানি কনুই পর্যন্ত পৌঁছে, পা ধোয় এমনভাবে যে পানি টাখনু পর্যন্ত বয়ে যায়, তারপর দাঁড়িয়ে সালাত আদায় করে, তখন তার আগের পাপ ক্ষমা করা হয়। এখানে ওযুর অঙ্গগুলোতে পানি পৌঁছানোর বিষয়টি স্পষ্টভাবে এসেছে। তাই ওযুতে তাড়াহুড়া না করে, অঙ্গগুলো ঠিকভাবে ধোয়া এবং এরপর সালাত আদায় করা—এটাই মূল শিক্ষা।"},"teachings":["সুন্দরভাবে ওযু করার জন্য অঙ্গে পানি পৌঁছানো দরকার।","ওযুর পর সালাত আদায় পাপ ক্ষমার কারণ হিসেবে এসেছে।","ওযুর সময় মুখ, হাত ও পা ধোয়ায় যত্ন নেওয়া উচিত।","নবীজি একই শিক্ষা বারবার বলেছেন—এতে বিষয়টির গুরুত্ব বোঝা যায়।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পবিত্রতা ঈমানের অর্ধেক","description":"$book_name$ $hadith_number$ - $chapter_name$. পবিত্রতা, আল্লাহর প্রশংসা, সালাত, সদকা, ধৈর্য ও কুরআনের দায়িত্ব—সবই মুমিন জীবনের বড় শিক্ষা।"},"heading":{"title":"পবিত্রতা ঈমানের অর্ধেক: আমল, সালাত ও কুরআনের শিক্ষা","description":"এই হাদিসে মুমিন জীবনের কয়েকটি বড় বিষয় একসাথে এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, পবিত্রতা ঈমানের অর্ধেক। এর মাধ্যমে তাহারাত বা পাক-পবিত্রতার গুরুত্ব বোঝা যায়। “আলহামদু লিল্লাহ” মীযানকে ভারী করে, আর “সুবহানাল্লাহ” ও “আলহামদু লিল্লাহ” আসমান ও জমিনের মাঝের স্থান পূর্ণ করে—এতে যিকিরের মর্যাদা বোঝানো হয়েছে। সালাতকে নূর বলা হয়েছে, দান-সাদকাকে দলীল বলা হয়েছে, ধৈর্যকে উজ্জ্বলতা বলা হয়েছে। কুরআন মানুষের পক্ষে বা বিপক্ষে দলীল হবে। শেষে বলা হয়েছে, প্রত্যেক মানুষ সকাল করে নিজের জন্য কাজ করে; কেউ নিজেকে মুক্তির পথে নেয়, কেউ ধ্বংসের পথে। তাই পবিত্রতা, যিকির, সালাত, সদকা, ধৈর্য ও কুরআনের সাথে জীবন গড়া দরকার।"},"teachings":["পবিত্রতা মুমিন জীবনের খুব গুরুত্বপূর্ণ অংশ।","আলহামদু লিল্লাহ ও সুবহানাল্লাহ যিকিরের বড় ফজিলত আছে।","সালাত, সদকা ও ধৈর্য বান্দার আমলে বিশেষ স্থান রাখে।","কুরআন মানুষের পক্ষে বা বিপক্ষে দলীল হতে পারে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E89" s="4" t="n"/>
@@ -2547,12 +2543,12 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পবিত্রতা ঈমানের অর্ধেক","description":"$book_name$ $hadith_number$ - $chapter_name$. পবিত্রতা, আল্লাহর প্রশংসা, সালাত, সদকা, ধৈর্য ও কুরআনের দায়িত্ব—সবই মুমিন জীবনের বড় শিক্ষা।"},"heading":{"title":"পবিত্রতা ঈমানের অর্ধেক: আমল, সালাত ও কুরআনের শিক্ষা","description":"এই হাদিসে মুমিন জীবনের কয়েকটি বড় বিষয় একসাথে এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, পবিত্রতা ঈমানের অর্ধেক। এর মাধ্যমে তাহারাত বা পাক-পবিত্রতার গুরুত্ব বোঝা যায়। “আলহামদু লিল্লাহ” মীযানকে ভারী করে, আর “সুবহানাল্লাহ” ও “আলহামদু লিল্লাহ” আসমান ও জমিনের মাঝের স্থান পূর্ণ করে—এতে যিকিরের মর্যাদা বোঝানো হয়েছে। সালাতকে নূর বলা হয়েছে, দান-সাদকাকে দলীল বলা হয়েছে, ধৈর্যকে উজ্জ্বলতা বলা হয়েছে। কুরআন মানুষের পক্ষে বা বিপক্ষে দলীল হবে। শেষে বলা হয়েছে, প্রত্যেক মানুষ সকাল করে নিজের জন্য কাজ করে; কেউ নিজেকে মুক্তির পথে নেয়, কেউ ধ্বংসের পথে। তাই পবিত্রতা, যিকির, সালাত, সদকা, ধৈর্য ও কুরআনের সাথে জীবন গড়া দরকার।"},"teachings":["পবিত্রতা মুমিন জীবনের খুব গুরুত্বপূর্ণ অংশ।","আলহামদু লিল্লাহ ও সুবহানাল্লাহ যিকিরের বড় ফজিলত আছে।","সালাত, সদকা ও ধৈর্য বান্দার আমলে বিশেষ স্থান রাখে।","কুরআন মানুষের পক্ষে বা বিপক্ষে দলীল হতে পারে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সদকার নিয়ত ও প্রাপকের অধিকার","description":"$book_name$ $hadith_number$ - $chapter_name$. ইয়াযীদ রাঃ দান করতে চেয়েছিলেন; নবীজি জানান, তিনি নিয়তের সওয়াব পাবেন আর মা’ন যা নিয়েছেন তা তাঁর।"},"heading":{"title":"সদকার নিয়ত: দাতার সওয়াব ও গ্রহণকারীর অধিকার","description":"এই হাদিসে মান ইবনে ইয়াযীদের একটি ঘটনা এসেছে। তাঁর পিতা ইয়াযীদ কিছু দীনার দান করার উদ্দেশ্যে বের করেন এবং মসজিদে একজনের কাছে রেখে দেন। ঘটনাক্রমে মান তা নিয়ে পিতার কাছে ফিরে আসেন। পিতা বলেন, তিনি মানকে উদ্দেশ্য করেননি। তখন বিষয়টি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে পেশ করা হয়। তিনি বলেন, হে ইয়াযীদ, তুমি যা নিয়ত করেছ তার সওয়াব পাবে; আর হে মান, যা তোমার হাতে এসেছে তা তোমার। এই হাদিস সদকার নিয়ত ও বাস্তব ফলের সুন্দর দিক দেখায়। দাতার উদ্দেশ্য যদি দান হয়, সে তার নিয়তের প্রতিদান পাবে। আর যে ব্যক্তি গ্রহণ করেছে, তার হাতে যা বৈধভাবে এসেছে, তা তার জন্য সাব্যস্ত হতে পারে। হাদিসটি শেখায়, আল্লাহ বান্দার নিয়ত জানেন এবং মানুষের লেনদেনে ন্যায়ভিত্তিক ফয়সালা জরুরি।"},"teachings":["সদকার ক্ষেত্রে দাতার নিয়ত আল্লাহর কাছে গুরুত্বপূর্ণ।","বাস্তব ঘটনার ফয়সালায় ন্যায় ও স্পষ্টতা দরকার।","দানকারীর উদ্দেশ্য ভালো হলে সে নিয়তের সওয়াব পেতে পারে।","কোনো বিরোধ হলে নবীর নির্দেশিত ন্যায়ের পথে ফয়সালা করা উচিত।"],"related_hadiths":[{"id":"1422","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E90" s="4" t="n"/>
@@ -2570,12 +2566,12 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>190</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সদকার নিয়ত ও প্রাপকের অধিকার","description":"$book_name$ $hadith_number$ - $chapter_name$. ইয়াযীদ রাঃ দান করতে চেয়েছিলেন; নবীজি জানান, তিনি নিয়তের সওয়াব পাবেন আর মা’ন যা নিয়েছেন তা তাঁর।"},"heading":{"title":"সদকার নিয়ত: দাতার সওয়াব ও গ্রহণকারীর অধিকার","description":"এই হাদিসে মান ইবনে ইয়াযীদের একটি ঘটনা এসেছে। তাঁর পিতা ইয়াযীদ কিছু দীনার দান করার উদ্দেশ্যে বের করেন এবং মসজিদে একজনের কাছে রেখে দেন। ঘটনাক্রমে মান তা নিয়ে পিতার কাছে ফিরে আসেন। পিতা বলেন, তিনি মানকে উদ্দেশ্য করেননি। তখন বিষয়টি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে পেশ করা হয়। তিনি বলেন, হে ইয়াযীদ, তুমি যা নিয়ত করেছ তার সওয়াব পাবে; আর হে মান, যা তোমার হাতে এসেছে তা তোমার। এই হাদিস সদকার নিয়ত ও বাস্তব ফলের সুন্দর দিক দেখায়। দাতার উদ্দেশ্য যদি দান হয়, সে তার নিয়তের প্রতিদান পাবে। আর যে ব্যক্তি গ্রহণ করেছে, তার হাতে যা বৈধভাবে এসেছে, তা তার জন্য সাব্যস্ত হতে পারে। হাদিসটি শেখায়, আল্লাহ বান্দার নিয়ত জানেন এবং মানুষের লেনদেনে ন্যায়ভিত্তিক ফয়সালা জরুরি।"},"teachings":["সদকার ক্ষেত্রে দাতার নিয়ত আল্লাহর কাছে গুরুত্বপূর্ণ।","বাস্তব ঘটনার ফয়সালায় ন্যায় ও স্পষ্টতা দরকার।","দানকারীর উদ্দেশ্য ভালো হলে সে নিয়তের সওয়াব পেতে পারে।","কোনো বিরোধ হলে নবীর নির্দেশিত ন্যায়ের পথে ফয়সালা করা উচিত।"],"related_hadiths":[{"id":"1422","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পূর্ণ ওযু ও সচেতন সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. পরিপূর্ণ ওযু করে সালাতে কী বলা হচ্ছে তা বুঝে দাঁড়ালে পাপ থেকে পবিত্র হওয়ার ফজিলত এসেছে।"},"heading":{"title":"পূর্ণ ওযু ও সচেতন সালাত: কী বলছি তা জানার গুরুত্ব","description":"এই হাদিসে দুইটি বিষয় একসাথে এসেছে—পরিপূর্ণ ওযু এবং সচেতন সালাত। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে মুসলিম ব্যক্তি ওযু করে এবং তা পরিপূর্ণভাবে সম্পন্ন করে, তারপর সালাতে দাঁড়ায়, আর সে জানে সে সালাতে কী বলছে, সে সালাত থেকে ফিরে আসে এমন পবিত্র অবস্থায়, যেমন তার মা তাকে জন্ম দিয়েছিল। এখানে শুধু ওযু করাই বলা হয়নি; ওযু সুন্দরভাবে করা এবং সালাতে মনোযোগ রাখার কথা এসেছে। সালাতে কী বলা হচ্ছে তা জানা মানে মনোযোগ, বুঝে পড়া এবং আল্লাহর সামনে দাঁড়ানোর অনুভব। তাই এই হাদিস নামাজের ফজিলতের পাশাপাশি নামাজে খুশু বা একাগ্রতার দিকেও ইঙ্গিত করে।"},"teachings":["পূর্ণ ওযু করা সালাতের গুরুত্বপূর্ণ প্রস্তুতি।","সালাতে কী বলা হচ্ছে তা বুঝে পড়ার গুরুত্ব আছে।","মনোযোগী সালাত পাপ থেকে পবিত্র হওয়ার কারণ হিসেবে এসেছে।","ওযু ও সালাতকে একসাথে যত্নের সাথে করা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E91" s="4" t="n"/>
@@ -2593,12 +2589,12 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>191</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পূর্ণ ওযু ও সচেতন সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. পরিপূর্ণ ওযু করে সালাতে কী বলা হচ্ছে তা বুঝে দাঁড়ালে পাপ থেকে পবিত্র হওয়ার ফজিলত এসেছে।"},"heading":{"title":"পূর্ণ ওযু ও সচেতন সালাত: কী বলছি তা জানার গুরুত্ব","description":"এই হাদিসে দুইটি বিষয় একসাথে এসেছে—পরিপূর্ণ ওযু এবং সচেতন সালাত। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে মুসলিম ব্যক্তি ওযু করে এবং তা পরিপূর্ণভাবে সম্পন্ন করে, তারপর সালাতে দাঁড়ায়, আর সে জানে সে সালাতে কী বলছে, সে সালাত থেকে ফিরে আসে এমন পবিত্র অবস্থায়, যেমন তার মা তাকে জন্ম দিয়েছিল। এখানে শুধু ওযু করাই বলা হয়নি; ওযু সুন্দরভাবে করা এবং সালাতে মনোযোগ রাখার কথা এসেছে। সালাতে কী বলা হচ্ছে তা জানা মানে মনোযোগ, বুঝে পড়া এবং আল্লাহর সামনে দাঁড়ানোর অনুভব। তাই এই হাদিস নামাজের ফজিলতের পাশাপাশি নামাজে খুশু বা একাগ্রতার দিকেও ইঙ্গিত করে।"},"teachings":["পূর্ণ ওযু করা সালাতের গুরুত্বপূর্ণ প্রস্তুতি।","সালাতে কী বলা হচ্ছে তা বুঝে পড়ার গুরুত্ব আছে।","মনোযোগী সালাত পাপ থেকে পবিত্র হওয়ার কারণ হিসেবে এসেছে।","ওযু ও সালাতকে একসাথে যত্নের সাথে করা উচিত।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কষ্টে ওযু, মসজিদে যাওয়া ও সালাতের অপেক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঠান্ডার কষ্টে পূর্ণ ওযু, মসজিদে হাঁটা ও পরের সালাতের অপেক্ষা পাপ ধুয়ে দেয়—এ শিক্ষা এসেছে।"},"heading":{"title":"কষ্টে ওযু ও মসজিদে হাঁটার ফজিলত","description":"এই হাদিসে তিনটি আমলকে পাপ ধুয়ে পরিষ্কার করার কারণ বলা হয়েছে। প্রথমটি হলো কষ্টের সময়, বিশেষ করে প্রচণ্ড ঠান্ডার কষ্ট সহ্য করে পরিপূর্ণ ওযু করা। দ্বিতীয়টি হলো পদযুগলকে মসজিদের দিকে ব্যবহার করা, অর্থাৎ মসজিদে গিয়ে সালাত আদায়ের চেষ্টা করা। তৃতীয়টি হলো এক সালাতের পর আরেক সালাতের জন্য অপেক্ষা করা। এখানে আমলের কষ্টকে গুরুত্ব দেওয়া হয়েছে, কিন্তু কষ্ট খোঁজার কথা বলা হয়নি; বরং কষ্ট থাকা সত্ত্বেও ইবাদত ঠিকভাবে করার ফজিলত বোঝানো হয়েছে। তাই মুসলিমের উচিত ওযু, মসজিদে যাওয়া এবং সালাতের সময়ের প্রতি যত্নবান থাকা। এই তিনটি আমল বান্দাকে নিয়মিত ইবাদতের পথে রাখে।"},"teachings":["কষ্টের সময়ও পরিপূর্ণ ওযু করার ফজিলত আছে।","মসজিদের দিকে হাঁটা নেকির কাজ হিসেবে এসেছে।","এক সালাতের পর আরেক সালাতের অপেক্ষা পাপ ধোয়ার কারণ।","ইবাদতে নিয়মিত থাকা বান্দার জন্য কল্যাণের পথ।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E92" s="4" t="n"/>
@@ -2616,12 +2612,12 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>192</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কষ্টে ওযু, মসজিদে যাওয়া ও সালাতের অপেক্ষা","description":"$book_name$ $hadith_number$ - $chapter_name$. ঠান্ডার কষ্টে পূর্ণ ওযু, মসজিদে হাঁটা ও পরের সালাতের অপেক্ষা পাপ ধুয়ে দেয়—এ শিক্ষা এসেছে।"},"heading":{"title":"কষ্টে ওযু ও মসজিদে হাঁটার ফজিলত","description":"এই হাদিসে তিনটি আমলকে পাপ ধুয়ে পরিষ্কার করার কারণ বলা হয়েছে। প্রথমটি হলো কষ্টের সময়, বিশেষ করে প্রচণ্ড ঠান্ডার কষ্ট সহ্য করে পরিপূর্ণ ওযু করা। দ্বিতীয়টি হলো পদযুগলকে মসজিদের দিকে ব্যবহার করা, অর্থাৎ মসজিদে গিয়ে সালাত আদায়ের চেষ্টা করা। তৃতীয়টি হলো এক সালাতের পর আরেক সালাতের জন্য অপেক্ষা করা। এখানে আমলের কষ্টকে গুরুত্ব দেওয়া হয়েছে, কিন্তু কষ্ট খোঁজার কথা বলা হয়নি; বরং কষ্ট থাকা সত্ত্বেও ইবাদত ঠিকভাবে করার ফজিলত বোঝানো হয়েছে। তাই মুসলিমের উচিত ওযু, মসজিদে যাওয়া এবং সালাতের সময়ের প্রতি যত্নবান থাকা। এই তিনটি আমল বান্দাকে নিয়মিত ইবাদতের পথে রাখে।"},"teachings":["কষ্টের সময়ও পরিপূর্ণ ওযু করার ফজিলত আছে।","মসজিদের দিকে হাঁটা নেকির কাজ হিসেবে এসেছে।","এক সালাতের পর আরেক সালাতের অপেক্ষা পাপ ধোয়ার কারণ।","ইবাদতে নিয়মিত থাকা বান্দার জন্য কল্যাণের পথ।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পাপ মোচন ও মর্যাদা বৃদ্ধির তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টে পূর্ণ ওযু, মসজিদে বেশি পদচারণা ও সালাতের অপেক্ষাকে পাপ মোচন ও মর্যাদা বৃদ্ধির কারণ বলা হয়েছে।"},"heading":{"title":"পাপ মোচন ও মর্যাদা বৃদ্ধির আমল: কষ্টে ওযু, মসজিদে হাঁটা, সালাতের অপেক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) সাহাবাদের জিজ্ঞেস করেন, তিনি কি এমন কাজ জানাবেন যা আল্লাহ পাপ মুছে দেন এবং মর্যাদা বাড়িয়ে দেন? তাঁরা জানতে চাইলে তিনি তিনটি কাজ বলেন। প্রথমত, কষ্টের সময়ও পরিপূর্ণভাবে ওযু করা। দ্বিতীয়ত, মসজিদের দিকে বেশি বেশি পদচারণা করা। তৃতীয়ত, এক সালাতের পর অন্য সালাতের জন্য অপেক্ষা করা। এরপর তিনি বলেন, এগুলোই তোমাদের জন্য “রিবাত” বা সীমান্ত পাহারার মতো। হাদিসের ভাষা থেকে বোঝা যায়, নিয়মিত ইবাদত, মসজিদের সাথে সম্পর্ক এবং সালাতের অপেক্ষা—এসব কাজ বান্দার মর্যাদা বাড়ার কারণ। তাই সহজ সময়ে যেমন, কষ্টের সময়ও ওযু ও সালাতের প্রতি যত্ন রাখা উচিত।"},"teachings":["কষ্টের সময় পূর্ণ ওযু করা পাপ মোচনের কারণ।","মসজিদে বেশি পদক্ষেপে যাওয়ার ফজিলত আছে।","সালাতের পর পরবর্তী সালাতের অপেক্ষা মর্যাদা বৃদ্ধির কারণ।","নিয়মিত ইবাদতকে হাদিসে রিবাতের সাথে তুলনা করা হয়েছে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E93" s="4" t="n"/>
@@ -2639,12 +2635,12 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>193</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পাপ মোচন ও মর্যাদা বৃদ্ধির তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টে পূর্ণ ওযু, মসজিদে বেশি পদচারণা ও সালাতের অপেক্ষাকে পাপ মোচন ও মর্যাদা বৃদ্ধির কারণ বলা হয়েছে।"},"heading":{"title":"পাপ মোচন ও মর্যাদা বৃদ্ধির আমল: কষ্টে ওযু, মসজিদে হাঁটা, সালাতের অপেক্ষা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) সাহাবাদের জিজ্ঞেস করেন, তিনি কি এমন কাজ জানাবেন যা আল্লাহ পাপ মুছে দেন এবং মর্যাদা বাড়িয়ে দেন? তাঁরা জানতে চাইলে তিনি তিনটি কাজ বলেন। প্রথমত, কষ্টের সময়ও পরিপূর্ণভাবে ওযু করা। দ্বিতীয়ত, মসজিদের দিকে বেশি বেশি পদচারণা করা। তৃতীয়ত, এক সালাতের পর অন্য সালাতের জন্য অপেক্ষা করা। এরপর তিনি বলেন, এগুলোই তোমাদের জন্য “রিবাত” বা সীমান্ত পাহারার মতো। হাদিসের ভাষা থেকে বোঝা যায়, নিয়মিত ইবাদত, মসজিদের সাথে সম্পর্ক এবং সালাতের অপেক্ষা—এসব কাজ বান্দার মর্যাদা বাড়ার কারণ। তাই সহজ সময়ে যেমন, কষ্টের সময়ও ওযু ও সালাতের প্রতি যত্ন রাখা উচিত।"},"teachings":["কষ্টের সময় পূর্ণ ওযু করা পাপ মোচনের কারণ।","মসজিদে বেশি পদক্ষেপে যাওয়ার ফজিলত আছে।","সালাতের পর পরবর্তী সালাতের অপেক্ষা মর্যাদা বৃদ্ধির কারণ।","নিয়মিত ইবাদতকে হাদিসে রিবাতের সাথে তুলনা করা হয়েছে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কষ্টে পূর্ণ ওযু ও নেকি বৃদ্ধি","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টকর অবস্থায় পূর্ণ ওযু, মসজিদে বেশি হাঁটা ও সালাতের অপেক্ষাকে নেকি বৃদ্ধি ও গুনাহের কাফফারা বলা হয়েছে।"},"heading":{"title":"কষ্টে ওযু, মসজিদে হাঁটা ও সালাতের অপেক্ষায় নেকি বৃদ্ধি","description":"এই বর্ণনায় একই মূল শিক্ষাকে আরেক ভাষায় বলা হয়েছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) জিজ্ঞেস করেন, তিনি কি এমন কাজ জানাবেন যার মাধ্যমে আল্লাহ পাপ মোচন করেন, নেকীর পাল্লা ভারী করেন এবং গুনাহের কাফফারা করেন? উত্তরে তিনি বলেন, কষ্টকর অবস্থায় পরিপূর্ণ ওযু করা, মসজিদের দিকে বেশি বেশি পদচারণা করা এবং এক সালাতের পর অন্য সালাতের জন্য অপেক্ষা করা। এগুলোকে শত্রুর বিরুদ্ধে সীমান্তে জিহাদে লিপ্ত থাকার সমতুল্য বলা হয়েছে। এখানে মূল শিক্ষা হলো, ধারাবাহিক ইবাদত ও সালাতের সাথে সম্পর্ক বান্দার জন্য বড় নেকির দরজা খুলে দেয়। তবে হাদিসে যেটুকু বলা হয়েছে, আমরা সেটুকুতেই সীমাবদ্ধ থাকি।"},"teachings":["কষ্টের সময়ও ওযু পূর্ণ করা নেকির কাজ।","মসজিদে বেশি পদচারণা গুনাহের কাফফারা হিসেবে এসেছে।","সালাতের অপেক্ষা বান্দাকে ইবাদতের সাথে যুক্ত রাখে।","হাদিসে এসব আমলকে সীমান্ত পাহারার মতো মর্যাদাপূর্ণ বলা হয়েছে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E94" s="4" t="n"/>
@@ -2662,12 +2658,12 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>194</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কষ্টে পূর্ণ ওযু ও নেকি বৃদ্ধি","description":"$book_name$ $hadith_number$ - $chapter_name$. কষ্টকর অবস্থায় পূর্ণ ওযু, মসজিদে বেশি হাঁটা ও সালাতের অপেক্ষাকে নেকি বৃদ্ধি ও গুনাহের কাফফারা বলা হয়েছে।"},"heading":{"title":"কষ্টে ওযু, মসজিদে হাঁটা ও সালাতের অপেক্ষায় নেকি বৃদ্ধি","description":"এই বর্ণনায় একই মূল শিক্ষাকে আরেক ভাষায় বলা হয়েছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) জিজ্ঞেস করেন, তিনি কি এমন কাজ জানাবেন যার মাধ্যমে আল্লাহ পাপ মোচন করেন, নেকীর পাল্লা ভারী করেন এবং গুনাহের কাফফারা করেন? উত্তরে তিনি বলেন, কষ্টকর অবস্থায় পরিপূর্ণ ওযু করা, মসজিদের দিকে বেশি বেশি পদচারণা করা এবং এক সালাতের পর অন্য সালাতের জন্য অপেক্ষা করা। এগুলোকে শত্রুর বিরুদ্ধে সীমান্তে জিহাদে লিপ্ত থাকার সমতুল্য বলা হয়েছে। এখানে মূল শিক্ষা হলো, ধারাবাহিক ইবাদত ও সালাতের সাথে সম্পর্ক বান্দার জন্য বড় নেকির দরজা খুলে দেয়। তবে হাদিসে যেটুকু বলা হয়েছে, আমরা সেটুকুতেই সীমাবদ্ধ থাকি।"},"teachings":["কষ্টের সময়ও ওযু পূর্ণ করা নেকির কাজ।","মসজিদে বেশি পদচারণা গুনাহের কাফফারা হিসেবে এসেছে।","সালাতের অপেক্ষা বান্দাকে ইবাদতের সাথে যুক্ত রাখে।","হাদিসে এসব আমলকে সীমান্ত পাহারার মতো মর্যাদাপূর্ণ বলা হয়েছে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মর্যাদা বৃদ্ধি ও পাপ মোচনের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. জামাআতের জন্য মসজিদে হাঁটা, ঠান্ডায় পূর্ণ ওযু ও সালাতের অপেক্ষাকে পাপ মোচন ও মর্যাদা বৃদ্ধির কারণ বলা হয়েছে।"},"heading":{"title":"মর্যাদা বৃদ্ধি ও পাপ মোচন: জামাআত, পূর্ণ ওযু ও সালাতের অপেক্ষা","description":"এই হাদিসে স্বপ্নযোগে পাওয়া এক কথোপকথনের বর্ণনা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেন, তাঁর পালনকর্তা তাঁকে জিজ্ঞেস করেন, নৈকট্যপ্রাপ্ত ফেরেশতারা কোন বিষয়ে আলোচনা করছে। উত্তরে তিনি বলেন, তা হলো মর্যাদা উন্নীতকরণ ও পাপ মোচনের আমল: জামাআতে সালাতের জন্য মসজিদে যাওয়ার পদক্ষেপ, কঠিন ঠান্ডার সময় পরিপূর্ণ ওযু এবং এক সালাতের পর পরবর্তী সালাতের অপেক্ষা। হাদিসে বলা হয়েছে, যে ব্যক্তি এসবের যত্ন নেবে সে কল্যাণের সাথে বাঁচবে, কল্যাণের মাঝে মৃত্যুবরণ করবে এবং পাপ থেকে পবিত্র হবে। এখানে মূল শিক্ষা হলো, জামাআত, ওযু ও সালাতের অপেক্ষা বান্দাকে আল্লাহর আনুগত্যের পথে রাখে।"},"teachings":["জামাআতে সালাতের জন্য মসজিদে যাওয়া মর্যাদার আমল।","ঠান্ডার কষ্টেও পূর্ণ ওযু করার ফজিলত আছে।","এক সালাতের পর অন্য সালাতের অপেক্ষা পাপ মোচনের কারণ।","নিয়মিত ইবাদতের যত্ন মানুষকে কল্যাণের পথে রাখে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E95" s="4" t="n"/>
@@ -2685,12 +2681,12 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>195</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মর্যাদা বৃদ্ধি ও পাপ মোচনের আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. জামাআতের জন্য মসজিদে হাঁটা, ঠান্ডায় পূর্ণ ওযু ও সালাতের অপেক্ষাকে পাপ মোচন ও মর্যাদা বৃদ্ধির কারণ বলা হয়েছে।"},"heading":{"title":"মর্যাদা বৃদ্ধি ও পাপ মোচন: জামাআত, পূর্ণ ওযু ও সালাতের অপেক্ষা","description":"এই হাদিসে স্বপ্নযোগে পাওয়া এক কথোপকথনের বর্ণনা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেন, তাঁর পালনকর্তা তাঁকে জিজ্ঞেস করেন, নৈকট্যপ্রাপ্ত ফেরেশতারা কোন বিষয়ে আলোচনা করছে। উত্তরে তিনি বলেন, তা হলো মর্যাদা উন্নীতকরণ ও পাপ মোচনের আমল: জামাআতে সালাতের জন্য মসজিদে যাওয়ার পদক্ষেপ, কঠিন ঠান্ডার সময় পরিপূর্ণ ওযু এবং এক সালাতের পর পরবর্তী সালাতের অপেক্ষা। হাদিসে বলা হয়েছে, যে ব্যক্তি এসবের যত্ন নেবে সে কল্যাণের সাথে বাঁচবে, কল্যাণের মাঝে মৃত্যুবরণ করবে এবং পাপ থেকে পবিত্র হবে। এখানে মূল শিক্ষা হলো, জামাআত, ওযু ও সালাতের অপেক্ষা বান্দাকে আল্লাহর আনুগত্যের পথে রাখে।"},"teachings":["জামাআতে সালাতের জন্য মসজিদে যাওয়া মর্যাদার আমল।","ঠান্ডার কষ্টেও পূর্ণ ওযু করার ফজিলত আছে।","এক সালাতের পর অন্য সালাতের অপেক্ষা পাপ মোচনের কারণ।","নিয়মিত ইবাদতের যত্ন মানুষকে কল্যাণের পথে রাখে।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1399","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আদেশমতো ওযু ও ফরয সালাতের কাফফারা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহর আদেশমতো ওযু করলে ফরয সালাতগুলোর মধ্যবর্তী সময়ের পাপের কাফফারা হওয়ার কথা এসেছে।"},"heading":{"title":"আদেশমতো ওযু: ফরয সালাতগুলোর মাঝের পাপের কাফফারা","description":"এই হাদিসে ওযু ও ফরয সালাতের সম্পর্ক খুব সংক্ষিপ্তভাবে বলা হয়েছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি আল্লাহ যেভাবে আদেশ করেছেন সেভাবে ওযু সম্পন্ন করবে, তার ফরয সালাতসমূহ একটির পর আরেকটির মাঝের সময়ের জন্য কাফফারা হবে। এখানে দুটি বিষয় স্পষ্ট। প্রথমত, ওযু নিজের মতো নয়; আল্লাহর আদেশ অনুযায়ী করতে হবে। দ্বিতীয়ত, ফরয সালাত নিয়মিত আদায় করা মুমিনের জীবনে পাপ মোচনের একটি বড় পথ। এই হাদিস মানুষকে শিখায়, ওযু ও সালাতকে আলাদা আলাদা ছোট কাজ হিসেবে না দেখে, একসাথে পবিত্র জীবন গড়ার আমল হিসেবে দেখতে। তাই প্রতিটি সালাতের আগে ওযু সুন্দরভাবে করা এবং ফরয সালাতের সময় রক্ষা করা জরুরি।"},"teachings":["আল্লাহর আদেশ অনুযায়ী ওযু করা জরুরি।","ফরয সালাতগুলো মধ্যবর্তী পাপের কাফফারা হিসেবে এসেছে।","ওযু ও সালাত পরস্পর গভীরভাবে যুক্ত।","সালাতের সময়গুলো নিয়মিত রক্ষা করা দরকার।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E96" s="4" t="n"/>
@@ -2708,12 +2704,12 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>196</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আদেশমতো ওযু ও ফরয সালাতের কাফফারা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহর আদেশমতো ওযু করলে ফরয সালাতগুলোর মধ্যবর্তী সময়ের পাপের কাফফারা হওয়ার কথা এসেছে।"},"heading":{"title":"আদেশমতো ওযু: ফরয সালাতগুলোর মাঝের পাপের কাফফারা","description":"এই হাদিসে ওযু ও ফরয সালাতের সম্পর্ক খুব সংক্ষিপ্তভাবে বলা হয়েছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি আল্লাহ যেভাবে আদেশ করেছেন সেভাবে ওযু সম্পন্ন করবে, তার ফরয সালাতসমূহ একটির পর আরেকটির মাঝের সময়ের জন্য কাফফারা হবে। এখানে দুটি বিষয় স্পষ্ট। প্রথমত, ওযু নিজের মতো নয়; আল্লাহর আদেশ অনুযায়ী করতে হবে। দ্বিতীয়ত, ফরয সালাত নিয়মিত আদায় করা মুমিনের জীবনে পাপ মোচনের একটি বড় পথ। এই হাদিস মানুষকে শিখায়, ওযু ও সালাতকে আলাদা আলাদা ছোট কাজ হিসেবে না দেখে, একসাথে পবিত্র জীবন গড়ার আমল হিসেবে দেখতে। তাই প্রতিটি সালাতের আগে ওযু সুন্দরভাবে করা এবং ফরয সালাতের সময় রক্ষা করা জরুরি।"},"teachings":["আল্লাহর আদেশ অনুযায়ী ওযু করা জরুরি।","ফরয সালাতগুলো মধ্যবর্তী পাপের কাফফারা হিসেবে এসেছে।","ওযু ও সালাত পরস্পর গভীরভাবে যুক্ত।","সালাতের সময়গুলো নিয়মিত রক্ষা করা দরকার।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নির্দেশমতো ওযু ও সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. নির্দেশমতো ওযু ও সালাত আদায় করলে পূর্বকৃত আমলের পাপ ক্ষমার কথা এই হাদিসে এসেছে।"},"heading":{"title":"নির্দেশমতো ওযু ও সালাত: পূর্বের পাপ ক্ষমার শিক্ষা","description":"এই হাদিসে আবু আইয়ুব (রাঃ) বলেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে বলতে শুনেছেন: যে ব্যক্তি নির্দেশ দেওয়া হয়েছে যেভাবে, সেভাবে ওযু করবে এবং নির্দেশ দেওয়া হয়েছে যেভাবে, সেভাবে সালাত আদায় করবে, তার পূর্বকৃত আমলের পাপ ক্ষমা করা হবে। এখানে শুধু ওযু বা শুধু সালাত নয়, দুটোই নির্দেশমতো করার কথা এসেছে। অর্থাৎ ইবাদতকে নিজের ইচ্ছামতো নয়, নবীজির শেখানো পথে করা দরকার। ওযুতে অঙ্গ ধোয়ার যত্ন, আর সালাতে নিয়ম, সময় ও মনোযোগ—সবই এই শিক্ষার অংশ। হাদিসটি মুমিনকে সহজ ভাষায় মনে করিয়ে দেয়, সঠিক পদ্ধতিতে করা ছোট আমলও আল্লাহর কাছে বড় ফজিলতের কারণ হতে পারে।"},"teachings":["ওযু ও সালাত নির্দেশমতো করা উচিত।","পূর্বের পাপ ক্ষমার ফজিলত হাদিসে এসেছে।","ইবাদতে নিজের ইচ্ছা নয়, শেখানো পদ্ধতি মানা দরকার।","ওযু ও সালাত—দুয়ের প্রতিই যত্নবান হওয়া দরকার।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E97" s="4" t="n"/>
@@ -2731,12 +2727,12 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>197</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নির্দেশমতো ওযু ও সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. নির্দেশমতো ওযু ও সালাত আদায় করলে পূর্বকৃত আমলের পাপ ক্ষমার কথা এই হাদিসে এসেছে।"},"heading":{"title":"নির্দেশমতো ওযু ও সালাত: পূর্বের পাপ ক্ষমার শিক্ষা","description":"এই হাদিসে আবু আইয়ুব (রাঃ) বলেন, তিনি রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-কে বলতে শুনেছেন: যে ব্যক্তি নির্দেশ দেওয়া হয়েছে যেভাবে, সেভাবে ওযু করবে এবং নির্দেশ দেওয়া হয়েছে যেভাবে, সেভাবে সালাত আদায় করবে, তার পূর্বকৃত আমলের পাপ ক্ষমা করা হবে। এখানে শুধু ওযু বা শুধু সালাত নয়, দুটোই নির্দেশমতো করার কথা এসেছে। অর্থাৎ ইবাদতকে নিজের ইচ্ছামতো নয়, নবীজির শেখানো পথে করা দরকার। ওযুতে অঙ্গ ধোয়ার যত্ন, আর সালাতে নিয়ম, সময় ও মনোযোগ—সবই এই শিক্ষার অংশ। হাদিসটি মুমিনকে সহজ ভাষায় মনে করিয়ে দেয়, সঠিক পদ্ধতিতে করা ছোট আমলও আল্লাহর কাছে বড় ফজিলতের কারণ হতে পারে।"},"teachings":["ওযু ও সালাত নির্দেশমতো করা উচিত।","পূর্বের পাপ ক্ষমার ফজিলত হাদিসে এসেছে।","ইবাদতে নিজের ইচ্ছা নয়, শেখানো পদ্ধতি মানা দরকার।","ওযু ও সালাত—দুয়ের প্রতিই যত্নবান হওয়া দরকার।"],"related_hadiths":[{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাত শ্রেষ্ঠ আমল ও ওযুর যত্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. সঠিক পথে অটল থাকা, সালাতের মর্যাদা এবং মুমিনের ওযুর প্রতি যত্ন—এই তিনটি শিক্ষা হাদিসে এসেছে।"},"heading":{"title":"সালাত শ্রেষ্ঠ আমল: মুমিনের ওযুর প্রতি যত্ন","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কয়েকটি গুরুত্বপূর্ণ শিক্ষা দিয়েছেন। তিনি বলেছেন, তোমরা সত্য ও সঠিক পথের উপর অটল থাক। আমলের সওয়াব গুনে শেষ করা সম্ভব নয়—এ কথার মাধ্যমে আমলের ব্যাপারে বিনয় শেখানো হয়েছে। এরপর বলা হয়েছে, তোমাদের উত্তম আমল হলো সালাত। আর মুমিন ব্যক্তি ছাড়া কেউ ওযুর প্রতি যত্নশীল হয় না। সহীহ ইবনু হিব্বানের বর্ণনায় বাড়াবাড়ি ও শিথিলতা পরিহার করে সঠিক পথের কাছাকাছি থাকার কথাও এসেছে। তাই এই হাদিসের মূল শিক্ষা হলো, সালাতকে জীবনের বড় আমল হিসেবে গ্রহণ করা, ওযুর প্রতি যত্ন রাখা এবং ইবাদতে ভারসাম্য বজায় রাখা।"},"teachings":["সঠিক পথে অটল থাকার চেষ্টা করা দরকার।","সালাতকে উত্তম আমল হিসেবে গুরুত্ব দেওয়া হয়েছে।","ওযুর প্রতি যত্ন মুমিনের পরিচয়ের সাথে যুক্ত।","ইবাদতে বাড়াবাড়ি ও শিথিলতা এড়িয়ে চলা উচিত।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E98" s="4" t="n"/>
@@ -2754,12 +2750,12 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাত শ্রেষ্ঠ আমল ও ওযুর যত্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. সঠিক পথে অটল থাকা, সালাতের মর্যাদা এবং মুমিনের ওযুর প্রতি যত্ন—এই তিনটি শিক্ষা হাদিসে এসেছে।"},"heading":{"title":"সালাত শ্রেষ্ঠ আমল: মুমিনের ওযুর প্রতি যত্ন","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) কয়েকটি গুরুত্বপূর্ণ শিক্ষা দিয়েছেন। তিনি বলেছেন, তোমরা সত্য ও সঠিক পথের উপর অটল থাক। আমলের সওয়াব গুনে শেষ করা সম্ভব নয়—এ কথার মাধ্যমে আমলের ব্যাপারে বিনয় শেখানো হয়েছে। এরপর বলা হয়েছে, তোমাদের উত্তম আমল হলো সালাত। আর মুমিন ব্যক্তি ছাড়া কেউ ওযুর প্রতি যত্নশীল হয় না। সহীহ ইবনু হিব্বানের বর্ণনায় বাড়াবাড়ি ও শিথিলতা পরিহার করে সঠিক পথের কাছাকাছি থাকার কথাও এসেছে। তাই এই হাদিসের মূল শিক্ষা হলো, সালাতকে জীবনের বড় আমল হিসেবে গ্রহণ করা, ওযুর প্রতি যত্ন রাখা এবং ইবাদতে ভারসাম্য বজায় রাখা।"},"teachings":["সঠিক পথে অটল থাকার চেষ্টা করা দরকার।","সালাতকে উত্তম আমল হিসেবে গুরুত্ব দেওয়া হয়েছে।","ওযুর প্রতি যত্ন মুমিনের পরিচয়ের সাথে যুক্ত।","ইবাদতে বাড়াবাড়ি ও শিথিলতা এড়িয়ে চলা উচিত।"],"related_hadiths":[{"id":"475","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"422","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"443","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোপন সদকা ও ভালো ফলের আশা","description":"$book_name$ $hadith_number$ - $chapter_name$. চোর, ব্যভিচারিণী ও ধনী ব্যক্তির কাছে সদকা পৌঁছালেও আল্লাহ চাইলে তাতে কল্যাণ হতে পারে।"},"heading":{"title":"গোপন সদকা: ভুল হাতে গেলেও আল্লাহ কল্যাণ দিতে পারেন","description":"এই হাদিসে এক ব্যক্তির সদকার ঘটনা এসেছে। তিনি রাতে দান করতে বের হন। প্রথম রাতে তাঁর দান এক চোরের হাতে যায়। মানুষ তা নিয়ে আলোচনা করলে তিনি আল্লাহর প্রশংসা করেন এবং আবার দান করার সিদ্ধান্ত নেন। দ্বিতীয় রাতে তা এক ব্যভিচারিণীর হাতে যায়। তৃতীয় রাতে তা এক ধনী ব্যক্তির হাতে যায়। প্রতিবারই তিনি আল্লাহর প্রশংসা করেন। পরে স্বপ্নের মাধ্যমে তাকে জানানো হয়, চোর হয়তো এই দানের কারণে চুরি থেকে বিরত থাকবে; ব্যভিচারিণী হয়তো এ কারণে পাপ থেকে পবিত্রতার পথে ফিরবে; আর ধনী ব্যক্তি হয়তো শিক্ষা নিয়ে নিজের সম্পদ থেকে দান করবে। মুসলিম ও নাসাঈর বর্ণনায় সদকা কবুল হওয়ার কথাও এসেছে। এই হাদিস সদকার নিয়ত, আল্লাহর অদৃশ্য হিকমত এবং মানুষের সীমিত ধারণার কথা শেখায়। বাহ্যিকভাবে ফল অপ্রত্যাশিত হলেও আল্লাহ তাতে কল্যাণ রাখতে পারেন।"},"teachings":["সদকায় নিয়ত খাঁটি হলে আল্লাহ তাতে কল্যাণ দিতে পারেন।","মানুষ বাহ্যিক দিক দেখে, কিন্তু আল্লাহ ফলের পথ জানেন।","দান কারও জীবনে ভালো পরিবর্তনের কারণ হতে পারে।","অপ্রত্যাশিত ফল দেখেও আল্লাহর প্রশংসা করা সুন্দর আচরণ।"],"related_hadiths":[{"id":"1421","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1422","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E99" s="4" t="n"/>
@@ -2777,12 +2773,12 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোপন সদকা ও ভালো ফলের আশা","description":"$book_name$ $hadith_number$ - $chapter_name$. চোর, ব্যভিচারিণী ও ধনী ব্যক্তির কাছে সদকা পৌঁছালেও আল্লাহ চাইলে তাতে কল্যাণ হতে পারে।"},"heading":{"title":"গোপন সদকা: ভুল হাতে গেলেও আল্লাহ কল্যাণ দিতে পারেন","description":"এই হাদিসে এক ব্যক্তির সদকার ঘটনা এসেছে। তিনি রাতে দান করতে বের হন। প্রথম রাতে তাঁর দান এক চোরের হাতে যায়। মানুষ তা নিয়ে আলোচনা করলে তিনি আল্লাহর প্রশংসা করেন এবং আবার দান করার সিদ্ধান্ত নেন। দ্বিতীয় রাতে তা এক ব্যভিচারিণীর হাতে যায়। তৃতীয় রাতে তা এক ধনী ব্যক্তির হাতে যায়। প্রতিবারই তিনি আল্লাহর প্রশংসা করেন। পরে স্বপ্নের মাধ্যমে তাকে জানানো হয়, চোর হয়তো এই দানের কারণে চুরি থেকে বিরত থাকবে; ব্যভিচারিণী হয়তো এ কারণে পাপ থেকে পবিত্রতার পথে ফিরবে; আর ধনী ব্যক্তি হয়তো শিক্ষা নিয়ে নিজের সম্পদ থেকে দান করবে। মুসলিম ও নাসাঈর বর্ণনায় সদকা কবুল হওয়ার কথাও এসেছে। এই হাদিস সদকার নিয়ত, আল্লাহর অদৃশ্য হিকমত এবং মানুষের সীমিত ধারণার কথা শেখায়। বাহ্যিকভাবে ফল অপ্রত্যাশিত হলেও আল্লাহ তাতে কল্যাণ রাখতে পারেন।"},"teachings":["সদকায় নিয়ত খাঁটি হলে আল্লাহ তাতে কল্যাণ দিতে পারেন।","মানুষ বাহ্যিক দিক দেখে, কিন্তু আল্লাহ ফলের পথ জানেন।","দান কারও জীবনে ভালো পরিবর্তনের কারণ হতে পারে।","অপ্রত্যাশিত ফল দেখেও আল্লাহর প্রশংসা করা সুন্দর আচরণ।"],"related_hadiths":[{"id":"1421","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1422","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | প্রতি সালাতে ওযু ও মেসওয়াকের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. উম্মতের কষ্টের কথা ভেবে প্রতি সালাতে ওযু ও প্রতি ওযুতে মেসওয়াক বাধ্যতামূলক করা হয়নি—তবু এর গুরুত্ব বোঝানো হয়েছে।"},"heading":{"title":"মেসওয়াক ও ওযুর গুরুত্ব: উম্মতের প্রতি নবীজির মমতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর উম্মতের প্রতি মমতা স্পষ্টভাবে দেখা যায়। তিনি বলেছেন, যদি উম্মতের উপর কঠিন মনে না করতেন, তবে প্রত্যেক সালাতের সময় ওযু করার আদেশ দিতেন এবং প্রত্যেক ওযুর সাথে মেসওয়াক করার নির্দেশ দিতেন। এখানে বোঝা যায়, ওযু ও মেসওয়াক দুটিই গুরুত্বপূর্ণ আমল। তবে নবীজি উম্মতের কষ্টের দিকও বিবেচনা করেছেন। তাই এই হাদিস থেকে আমরা মেসওয়াকের ফজিলত এবং ওযুর প্রতি নবীজির উৎসাহ বুঝি, কিন্তু এটিকে এমনভাবে বলা ঠিক নয় যে প্রত্যেক ওযুতে মেসওয়াক বাধ্যতামূলক। বরং হাদিসের ভাষা অনুযায়ী, এটি একটি গুরুত্ববহ ও প্রিয় আমল, যা মুসলিমের পবিত্রতা ও পরিচ্ছন্নতার সাথে জড়িত।"},"teachings":["মেসওয়াক ওযুর সাথে গুরুত্বপূর্ণ আমল হিসেবে এসেছে।","নবীজি উম্মতের কষ্টের কথা বিবেচনা করেছেন।","প্রত্যেক সালাতে নতুন ওযুর প্রতি উৎসাহ বোঝা যায়, তবে কষ্টকর বাধ্যবাধকতা করা হয়নি।","পবিত্রতা ও মুখের পরিচ্ছন্নতার দিকে যত্ন নেওয়া উচিত।"],"related_hadiths":[{"id":"887","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1934","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E100" s="4" t="n"/>
@@ -2800,12 +2796,12 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | প্রতি সালাতে ওযু ও মেসওয়াকের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. উম্মতের কষ্টের কথা ভেবে প্রতি সালাতে ওযু ও প্রতি ওযুতে মেসওয়াক বাধ্যতামূলক করা হয়নি—তবু এর গুরুত্ব বোঝানো হয়েছে।"},"heading":{"title":"মেসওয়াক ও ওযুর গুরুত্ব: উম্মতের প্রতি নবীজির মমতা","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর উম্মতের প্রতি মমতা স্পষ্টভাবে দেখা যায়। তিনি বলেছেন, যদি উম্মতের উপর কঠিন মনে না করতেন, তবে প্রত্যেক সালাতের সময় ওযু করার আদেশ দিতেন এবং প্রত্যেক ওযুর সাথে মেসওয়াক করার নির্দেশ দিতেন। এখানে বোঝা যায়, ওযু ও মেসওয়াক দুটিই গুরুত্বপূর্ণ আমল। তবে নবীজি উম্মতের কষ্টের দিকও বিবেচনা করেছেন। তাই এই হাদিস থেকে আমরা মেসওয়াকের ফজিলত এবং ওযুর প্রতি নবীজির উৎসাহ বুঝি, কিন্তু এটিকে এমনভাবে বলা ঠিক নয় যে প্রত্যেক ওযুতে মেসওয়াক বাধ্যতামূলক। বরং হাদিসের ভাষা অনুযায়ী, এটি একটি গুরুত্ববহ ও প্রিয় আমল, যা মুসলিমের পবিত্রতা ও পরিচ্ছন্নতার সাথে জড়িত।"},"teachings":["মেসওয়াক ওযুর সাথে গুরুত্বপূর্ণ আমল হিসেবে এসেছে।","নবীজি উম্মতের কষ্টের কথা বিবেচনা করেছেন।","প্রত্যেক সালাতে নতুন ওযুর প্রতি উৎসাহ বোঝা যায়, তবে কষ্টকর বাধ্যবাধকতা করা হয়নি।","পবিত্রতা ও মুখের পরিচ্ছন্নতার দিকে যত্ন নেওয়া উচিত।"],"related_hadiths":[{"id":"887","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1934","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কিয়ামুল লাইলের নিয়ত ও ঘুমের রহমত","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতে নফল সালাতের নিয়ত করেও ঘুমিয়ে পড়লে নিয়তের সওয়াব লেখা হয় এবং ঘুম রবের পক্ষ থেকে দয়া হয়।"},"heading":{"title":"কিয়ামুল লাইলের নিয়ত: ঘুমিয়ে পড়লেও নেক নিয়তের মূল্য","description":"এই হাদিসে নিয়তের গুরুত্ব খুব কোমলভাবে বোঝানো হয়েছে। একজন মানুষ রাতে কিয়ামুল লাইল বা নফল সালাত আদায়ের নিয়ত করে বিছানায় গেল। কিন্তু ঘুম তাকে পরাজিত করল, ফলে সে জাগতে পারল না। এখানে তার অলসতা বা ইচ্ছাকৃত অবহেলার কথা বলা হয়নি; বরং সে সত্যিই রাতের সালাতের নিয়ত করেছিল। তাই তার জন্য সে নিয়ত লিখে দেওয়া হয়। একই সঙ্গে তার ঘুমকে তার রবের পক্ষ থেকে সাদকা বলা হয়েছে। এই শিক্ষা আমাদের মনে করায়, ইবাদতের ক্ষেত্রে অন্তরের সত্য ইচ্ছা খুব মূল্যবান। তবে হাদিসটি ইচ্ছাকৃতভাবে সালাত ছেড়ে দেওয়ার অনুমতি দেয় না; বরং সৎ নিয়ত থাকা সত্ত্বেও ঘুমের কারণে অপারগ হয়ে গেলে আল্লাহর দয়ার কথা জানায়।"},"teachings":["সৎ নিয়ত আল্লাহর কাছে মূল্যবান, এমনকি কাজটি বাধার কারণে সম্পন্ন না হলেও।","কিয়ামুল লাইলের ইচ্ছা নিয়ে ঘুমানো একটি সুন্দর নেক নিয়তের পরিচয়।","ইবাদতে অপারগতা আর ইচ্ছাকৃত অবহেলা এক বিষয় নয়।","বান্দার প্রতি আল্লাহর দয়া অনেক সময় তার অক্ষমতার অবস্থাতেও প্রকাশ পায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1907","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"23","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E101" s="4" t="n"/>
@@ -2823,12 +2819,12 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কিয়ামুল লাইলের নিয়ত ও ঘুমের রহমত","description":"$book_name$ $hadith_number$ - $chapter_name$. রাতে নফল সালাতের নিয়ত করেও ঘুমিয়ে পড়লে নিয়তের সওয়াব লেখা হয় এবং ঘুম রবের পক্ষ থেকে দয়া হয়।"},"heading":{"title":"কিয়ামুল লাইলের নিয়ত: ঘুমিয়ে পড়লেও নেক নিয়তের মূল্য","description":"এই হাদিসে নিয়তের গুরুত্ব খুব কোমলভাবে বোঝানো হয়েছে। একজন মানুষ রাতে কিয়ামুল লাইল বা নফল সালাত আদায়ের নিয়ত করে বিছানায় গেল। কিন্তু ঘুম তাকে পরাজিত করল, ফলে সে জাগতে পারল না। এখানে তার অলসতা বা ইচ্ছাকৃত অবহেলার কথা বলা হয়নি; বরং সে সত্যিই রাতের সালাতের নিয়ত করেছিল। তাই তার জন্য সে নিয়ত লিখে দেওয়া হয়। একই সঙ্গে তার ঘুমকে তার রবের পক্ষ থেকে সাদকা বলা হয়েছে। এই শিক্ষা আমাদের মনে করায়, ইবাদতের ক্ষেত্রে অন্তরের সত্য ইচ্ছা খুব মূল্যবান। তবে হাদিসটি ইচ্ছাকৃতভাবে সালাত ছেড়ে দেওয়ার অনুমতি দেয় না; বরং সৎ নিয়ত থাকা সত্ত্বেও ঘুমের কারণে অপারগ হয়ে গেলে আল্লাহর দয়ার কথা জানায়।"},"teachings":["সৎ নিয়ত আল্লাহর কাছে মূল্যবান, এমনকি কাজটি বাধার কারণে সম্পন্ন না হলেও।","কিয়ামুল লাইলের ইচ্ছা নিয়ে ঘুমানো একটি সুন্দর নেক নিয়তের পরিচয়।","ইবাদতে অপারগতা আর ইচ্ছাকৃত অবহেলা এক বিষয় নয়।","বান্দার প্রতি আল্লাহর দয়া অনেক সময় তার অক্ষমতার অবস্থাতেও প্রকাশ পায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1907","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"23","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও লোক দেখানো আমলের ভয়াবহ পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. শহীদ, আলেম ও দানশীলের আমলও যদি লোক দেখানোর জন্য হয়, কিয়ামতে তা কঠিন জবাবদিহির কারণ হবে।"},"heading":{"title":"রিয়া ও ইখলাস: বড় আমলও নিয়ত নষ্ট হলে বিপদের কারণ","description":"এই হাদিসে রিয়া বা লোক দেখানো আমলের ভয়াবহ দিক তুলে ধরা হয়েছে। বাহ্যিকভাবে তিনটি কাজ খুব বড়: আল্লাহর পথে নিহত হওয়া, জ্ঞান শেখা ও কুরআন পড়া, আর সম্পদ দান করা। কিন্তু হাদিসে দেখা যায়, এসব কাজ যদি আল্লাহর সন্তুষ্টির বদলে মানুষের প্রশংসার জন্য করা হয়, তবে তা গ্রহণযোগ্য আমলের রূপ ধরে না। একজন চেয়েছিল তাকে বীর বলা হোক, একজন চেয়েছিল তাকে আলেম বা ক্বারী বলা হোক, আর একজন চেয়েছিল তাকে দানশীল বলা হোক। দুনিয়ায় সেই প্রশংসা তারা পেয়েছে। তাই কিয়ামতের দিনে তাদের সামনে আসল নিয়ত প্রকাশ করা হবে। এই হাদিস আমাদের শেখায়, আমলের আকার বড় হলেই যথেষ্ট নয়; ইখলাস বা আল্লাহর জন্য করা নিয়তই আসল।"},"teachings":["বড় আমলও লোক দেখানোর জন্য হলে কঠিন জবাবদিহির কারণ হতে পারে।","মানুষের প্রশংসা পাওয়া আমল গ্রহণের প্রমাণ নয়।","জ্ঞান, দান ও সাহস—সব ক্ষেত্রেই ইখলাস দরকার।","কিয়ামতের বিচার বাহ্যিক পরিচয় নয়, আসল নিয়ত অনুযায়ী হবে।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E102" s="4" t="n"/>
@@ -2846,12 +2842,12 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও লোক দেখানো আমলের ভয়াবহ পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. শহীদ, আলেম ও দানশীলের আমলও যদি লোক দেখানোর জন্য হয়, কিয়ামতে তা কঠিন জবাবদিহির কারণ হবে।"},"heading":{"title":"রিয়া ও ইখলাস: বড় আমলও নিয়ত নষ্ট হলে বিপদের কারণ","description":"এই হাদিসে রিয়া বা লোক দেখানো আমলের ভয়াবহ দিক তুলে ধরা হয়েছে। বাহ্যিকভাবে তিনটি কাজ খুব বড়: আল্লাহর পথে নিহত হওয়া, জ্ঞান শেখা ও কুরআন পড়া, আর সম্পদ দান করা। কিন্তু হাদিসে দেখা যায়, এসব কাজ যদি আল্লাহর সন্তুষ্টির বদলে মানুষের প্রশংসার জন্য করা হয়, তবে তা গ্রহণযোগ্য আমলের রূপ ধরে না। একজন চেয়েছিল তাকে বীর বলা হোক, একজন চেয়েছিল তাকে আলেম বা ক্বারী বলা হোক, আর একজন চেয়েছিল তাকে দানশীল বলা হোক। দুনিয়ায় সেই প্রশংসা তারা পেয়েছে। তাই কিয়ামতের দিনে তাদের সামনে আসল নিয়ত প্রকাশ করা হবে। এই হাদিস আমাদের শেখায়, আমলের আকার বড় হলেই যথেষ্ট নয়; ইখলাস বা আল্লাহর জন্য করা নিয়তই আসল।"},"teachings":["বড় আমলও লোক দেখানোর জন্য হলে কঠিন জবাবদিহির কারণ হতে পারে।","মানুষের প্রশংসা পাওয়া আমল গ্রহণের প্রমাণ নয়।","জ্ঞান, দান ও সাহস—সব ক্ষেত্রেই ইখলাস দরকার।","কিয়ামতের বিচার বাহ্যিক পরিচয় নয়, আসল নিয়ত অনুযায়ী হবে।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আখেরাতের আমল দুনিয়ার জন্য নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. এই উম্মতের মর্যাদার সুসংবাদ আছে, তবে আখেরাতের আমল দুনিয়ার উদ্দেশ্যে করলে পরকালের অংশ নষ্ট হয়।"},"heading":{"title":"আখেরাতের আমল দুনিয়ার লাভের জন্য করলে কী ক্ষতি","description":"এই হাদিসে উম্মতে মুহাম্মদীর জন্য সুসংবাদ আছে—দ্বীনের মাধ্যমে সম্মান, মর্যাদা এবং পৃথিবীতে প্রতিষ্ঠার কথা বলা হয়েছে। কিন্তু এই সুসংবাদের পরই একটি বড় সতর্কতা এসেছে। যে ব্যক্তি আখেরাতের কাজ দুনিয়ার উদ্দেশ্যে করে, তার জন্য পরকালে কোনো অংশ থাকবে না। অর্থাৎ ইবাদত, দ্বীনি কাজ, কুরআন, দান বা অন্য নেক আমল যদি শুধু দুনিয়ার নাম, লাভ, প্রভাব বা বাহ্যিক সুবিধার জন্য করা হয়, তাহলে তা বিপদের বিষয়। হাদিসটি আমাদের শেখায় যে দুনিয়া পাওয়া মুমিনের প্রধান লক্ষ্য হতে পারে না। আখেরাতের আমল আখেরাতের জন্যই হওয়া উচিত। দুনিয়ার সুযোগ আসতে পারে, কিন্তু উদ্দেশ্য হওয়া উচিত আল্লাহর সন্তুষ্টি।"},"teachings":["এই উম্মতের জন্য দ্বীনের মাধ্যমে সম্মান ও প্রতিষ্ঠার সুসংবাদ আছে।","আখেরাতের আমল দুনিয়ার লাভের জন্য করা ঠিক নয়।","ইবাদতের উদ্দেশ্য মানুষ, নাম বা সুবিধা নয়; আল্লাহর সন্তুষ্টি হওয়া দরকার।","দুনিয়ার উদ্দেশ্য আমলের আখেরাতের ফলকে ক্ষতিগ্রস্ত করতে পারে।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E103" s="4" t="n"/>
@@ -2869,12 +2865,12 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আখেরাতের আমল দুনিয়ার জন্য নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. এই উম্মতের মর্যাদার সুসংবাদ আছে, তবে আখেরাতের আমল দুনিয়ার উদ্দেশ্যে করলে পরকালের অংশ নষ্ট হয়।"},"heading":{"title":"আখেরাতের আমল দুনিয়ার লাভের জন্য করলে কী ক্ষতি","description":"এই হাদিসে উম্মতে মুহাম্মদীর জন্য সুসংবাদ আছে—দ্বীনের মাধ্যমে সম্মান, মর্যাদা এবং পৃথিবীতে প্রতিষ্ঠার কথা বলা হয়েছে। কিন্তু এই সুসংবাদের পরই একটি বড় সতর্কতা এসেছে। যে ব্যক্তি আখেরাতের কাজ দুনিয়ার উদ্দেশ্যে করে, তার জন্য পরকালে কোনো অংশ থাকবে না। অর্থাৎ ইবাদত, দ্বীনি কাজ, কুরআন, দান বা অন্য নেক আমল যদি শুধু দুনিয়ার নাম, লাভ, প্রভাব বা বাহ্যিক সুবিধার জন্য করা হয়, তাহলে তা বিপদের বিষয়। হাদিসটি আমাদের শেখায় যে দুনিয়া পাওয়া মুমিনের প্রধান লক্ষ্য হতে পারে না। আখেরাতের আমল আখেরাতের জন্যই হওয়া উচিত। দুনিয়ার সুযোগ আসতে পারে, কিন্তু উদ্দেশ্য হওয়া উচিত আল্লাহর সন্তুষ্টি।"},"teachings":["এই উম্মতের জন্য দ্বীনের মাধ্যমে সম্মান ও প্রতিষ্ঠার সুসংবাদ আছে।","আখেরাতের আমল দুনিয়ার লাভের জন্য করা ঠিক নয়।","ইবাদতের উদ্দেশ্য মানুষ, নাম বা সুবিধা নয়; আল্লাহর সন্তুষ্টি হওয়া দরকার।","দুনিয়ার উদ্দেশ্য আমলের আখেরাতের ফলকে ক্ষতিগ্রস্ত করতে পারে।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও সুমআহর গোপন উদ্দেশ্য প্রকাশ","description":"$book_name$ $hadith_number$ - $chapter_name$. রিয়া ও মানুষের কাছে নাম শোনানোর উদ্দেশ্যে আমল করলে কিয়ামতে আল্লাহ সেই গোপন উদ্দেশ্য প্রকাশ করবেন।"},"heading":{"title":"রিয়া ও সুমআহ: লোক দেখানো আমলের গোপন বিপদ","description":"এই হাদিসে রিয়া এবং সুমআহ বা নিজের আমলের কথা মানুষের কাছে শোনানোর উদ্দেশ্য সম্পর্কে সতর্ক করা হয়েছে। কেউ যদি কোনো আমল করে মানুষের চোখে ভালো দেখাতে চায়, বা এমনভাবে কাজ করে যেন মানুষ তার প্রশংসা করে, তবে কিয়ামতের দিনে আল্লাহ তার সেই অসৎ উদ্দেশ্য প্রকাশ করবেন। হাদিসে বলা হয়েছে, আল্লাহ তাকে সবার সামনে লাঞ্ছিত করবেন। এর মূল শিক্ষা হলো, ইবাদত বা নেক কাজ মানুষের সামনে প্রকাশ পেলেই সমস্যা নয়; সমস্যা হলো অন্তরের উদ্দেশ্য যদি মানুষের প্রশংসা হয়। তাই নামাজ, দান, কুরআন তিলাওয়াত, দাওয়াত—সব কাজে নিজের নিয়ত পরীক্ষা করা দরকার। আমল ছোট হোক বা বড়, তা আল্লাহর জন্য হলে মূল্যবান; মানুষের জন্য হলে বিপদের কারণ হতে পারে।"},"teachings":["রিয়া ও সুমআহ আমলের নিয়তকে নষ্ট করে দিতে পারে।","মানুষের প্রশংসার জন্য আমল করলে কিয়ামতে গোপন উদ্দেশ্য প্রকাশ হতে পারে।","নেক কাজের আগে ও পরে নিয়ত পরীক্ষা করা দরকার।","ইবাদতের আসল লক্ষ্য মানুষের চোখে বড় হওয়া নয়।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2986","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E104" s="4" t="n"/>
@@ -2892,12 +2888,12 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও সুমআহর গোপন উদ্দেশ্য প্রকাশ","description":"$book_name$ $hadith_number$ - $chapter_name$. রিয়া ও মানুষের কাছে নাম শোনানোর উদ্দেশ্যে আমল করলে কিয়ামতে আল্লাহ সেই গোপন উদ্দেশ্য প্রকাশ করবেন।"},"heading":{"title":"রিয়া ও সুমআহ: লোক দেখানো আমলের গোপন বিপদ","description":"এই হাদিসে রিয়া এবং সুমআহ বা নিজের আমলের কথা মানুষের কাছে শোনানোর উদ্দেশ্য সম্পর্কে সতর্ক করা হয়েছে। কেউ যদি কোনো আমল করে মানুষের চোখে ভালো দেখাতে চায়, বা এমনভাবে কাজ করে যেন মানুষ তার প্রশংসা করে, তবে কিয়ামতের দিনে আল্লাহ তার সেই অসৎ উদ্দেশ্য প্রকাশ করবেন। হাদিসে বলা হয়েছে, আল্লাহ তাকে সবার সামনে লাঞ্ছিত করবেন। এর মূল শিক্ষা হলো, ইবাদত বা নেক কাজ মানুষের সামনে প্রকাশ পেলেই সমস্যা নয়; সমস্যা হলো অন্তরের উদ্দেশ্য যদি মানুষের প্রশংসা হয়। তাই নামাজ, দান, কুরআন তিলাওয়াত, দাওয়াত—সব কাজে নিজের নিয়ত পরীক্ষা করা দরকার। আমল ছোট হোক বা বড়, তা আল্লাহর জন্য হলে মূল্যবান; মানুষের জন্য হলে বিপদের কারণ হতে পারে।"},"teachings":["রিয়া ও সুমআহ আমলের নিয়তকে নষ্ট করে দিতে পারে।","মানুষের প্রশংসার জন্য আমল করলে কিয়ামতে গোপন উদ্দেশ্য প্রকাশ হতে পারে।","নেক কাজের আগে ও পরে নিয়ত পরীক্ষা করা দরকার।","ইবাদতের আসল লক্ষ্য মানুষের চোখে বড় হওয়া নয়।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2986","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আমল প্রচার করে বেড়ানোর বিপদ","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি নিজের আমলের কথা মানুষকে শোনাতে চায়, আল্লাহ তাকে সৃষ্টির সামনে ছোট ও লাঞ্ছিত করবেন।"},"heading":{"title":"নিজের আমল শুনিয়ে বেড়ানো: সুমআহ থেকে সতর্কতা","description":"এই হাদিসে এমন ব্যক্তির কথা বলা হয়েছে, যে নিজের আমলের কথা মানুষের সামনে শুনিয়ে বেড়ায়। তার উদ্দেশ্য হলো মানুষ যেন তাকে ধার্মিক, দানশীল বা ভালো আমলকারী বলে। হাদিসে সতর্ক করা হয়েছে, আল্লাহ সৃষ্টিকুলের সামনে তার বিষয় প্রকাশ করবেন এবং তাকে ছোট ও লাঞ্ছিত করবেন। এখানে মূল শিক্ষা হলো, নেক আমল করার পর সেটাকে আত্মপ্রচারের জিনিস বানানো উচিত নয়। কোনো ভালো কাজ মানুষের জানা দরকার হলে সেটি আলাদা বিষয়; কিন্তু নিজের মর্যাদা বাড়ানোর জন্য আমল প্রচার করা সুমআহর অন্তর্ভুক্ত হতে পারে। তাই মুমিনের উচিত নীরবে নেক কাজ করা, আর প্রকাশ পেলেও অন্তরকে আল্লাহর জন্য রাখার চেষ্টা করা। আমলের সৌন্দর্য তার প্রচারে নয়, নিয়তের সত্যতায়।"},"teachings":["নিজের আমল প্রচার করা অন্তরের নিয়তকে ঝুঁকিতে ফেলতে পারে।","মানুষের প্রশংসা পাওয়ার ইচ্ছা সুমআহর কারণ হতে পারে।","নেক কাজের পরে বিনয় ধরে রাখা জরুরি।","আল্লাহর জন্য করা আমল আত্মপ্রচারের উপকরণ হওয়া উচিত নয়।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"24","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"27","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E105" s="4" t="n"/>
@@ -2915,12 +2911,12 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আমল প্রচার করে বেড়ানোর বিপদ","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি নিজের আমলের কথা মানুষকে শোনাতে চায়, আল্লাহ তাকে সৃষ্টির সামনে ছোট ও লাঞ্ছিত করবেন।"},"heading":{"title":"নিজের আমল শুনিয়ে বেড়ানো: সুমআহ থেকে সতর্কতা","description":"এই হাদিসে এমন ব্যক্তির কথা বলা হয়েছে, যে নিজের আমলের কথা মানুষের সামনে শুনিয়ে বেড়ায়। তার উদ্দেশ্য হলো মানুষ যেন তাকে ধার্মিক, দানশীল বা ভালো আমলকারী বলে। হাদিসে সতর্ক করা হয়েছে, আল্লাহ সৃষ্টিকুলের সামনে তার বিষয় প্রকাশ করবেন এবং তাকে ছোট ও লাঞ্ছিত করবেন। এখানে মূল শিক্ষা হলো, নেক আমল করার পর সেটাকে আত্মপ্রচারের জিনিস বানানো উচিত নয়। কোনো ভালো কাজ মানুষের জানা দরকার হলে সেটি আলাদা বিষয়; কিন্তু নিজের মর্যাদা বাড়ানোর জন্য আমল প্রচার করা সুমআহর অন্তর্ভুক্ত হতে পারে। তাই মুমিনের উচিত নীরবে নেক কাজ করা, আর প্রকাশ পেলেও অন্তরকে আল্লাহর জন্য রাখার চেষ্টা করা। আমলের সৌন্দর্য তার প্রচারে নয়, নিয়তের সত্যতায়।"},"teachings":["নিজের আমল প্রচার করা অন্তরের নিয়তকে ঝুঁকিতে ফেলতে পারে।","মানুষের প্রশংসা পাওয়ার ইচ্ছা সুমআহর কারণ হতে পারে।","নেক কাজের পরে বিনয় ধরে রাখা জরুরি।","আল্লাহর জন্য করা আমল আত্মপ্রচারের উপকরণ হওয়া উচিত নয়।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"24","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"27","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | লোক দেখানো আমল ও প্রশংসার লোভ","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রশংসা শোনার জন্য বা মানুষকে দেখানোর জন্য আমল করলে কিয়ামতে সেই খারাপ নিয়ত প্রকাশ হবে।"},"heading":{"title":"লোক দেখানো আমল: প্রশংসার লোভ থেকে নিয়ত বাঁচানো","description":"এই হাদিসে দুই ধরনের বিপদ স্পষ্ট করা হয়েছে। প্রথমত, কেউ নিজের আমল মানুষের সামনে প্রকাশ করে যেন তার প্রশংসা শোনা যায়। দ্বিতীয়ত, কেউ মানুষকে দেখানোর জন্য আমল করে। উভয় অবস্থায় কিয়ামতের দিনে আল্লাহ তার খারাপ নিয়ত প্রকাশ করবেন এবং তাকে মানুষের সামনে লাঞ্ছিত করবেন। এখানে আমল প্রকাশ পাওয়া নয়, বরং প্রশংসা পাওয়ার উদ্দেশ্যই মূল সমস্যা। একজন মানুষ নামাজ পড়তে পারে, দান করতে পারে, কুরআন পড়তে পারে; কিন্তু অন্তরে যদি মানুষের দৃষ্টি ও নাম কামনার ইচ্ছা ঢুকে যায়, তবে তা রিয়া হয়ে যায়। তাই হাদিসটি আমাদের নীরবে নিজের অন্তরকে প্রশ্ন করতে শেখায়—আমি এই কাজটি কার জন্য করছি? আল্লাহর জন্য, নাকি মানুষের চোখে বড় হওয়ার জন্য?"},"teachings":["প্রশংসা পাওয়ার উদ্দেশ্যে আমল করা সুমআহর দিকে নিয়ে যায়।","মানুষকে দেখানোর জন্য আমল করা রিয়ার অন্তর্ভুক্ত।","কিয়ামতে আমলের পেছনের উদ্দেশ্য প্রকাশিত হতে পারে।","প্রতিটি নেক কাজের আগে নিজের নিয়ত যাচাই করা দরকার।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2986","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E106" s="4" t="n"/>
@@ -2938,12 +2934,12 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | লোক দেখানো আমল ও প্রশংসার লোভ","description":"$book_name$ $hadith_number$ - $chapter_name$. প্রশংসা শোনার জন্য বা মানুষকে দেখানোর জন্য আমল করলে কিয়ামতে সেই খারাপ নিয়ত প্রকাশ হবে।"},"heading":{"title":"লোক দেখানো আমল: প্রশংসার লোভ থেকে নিয়ত বাঁচানো","description":"এই হাদিসে দুই ধরনের বিপদ স্পষ্ট করা হয়েছে। প্রথমত, কেউ নিজের আমল মানুষের সামনে প্রকাশ করে যেন তার প্রশংসা শোনা যায়। দ্বিতীয়ত, কেউ মানুষকে দেখানোর জন্য আমল করে। উভয় অবস্থায় কিয়ামতের দিনে আল্লাহ তার খারাপ নিয়ত প্রকাশ করবেন এবং তাকে মানুষের সামনে লাঞ্ছিত করবেন। এখানে আমল প্রকাশ পাওয়া নয়, বরং প্রশংসা পাওয়ার উদ্দেশ্যই মূল সমস্যা। একজন মানুষ নামাজ পড়তে পারে, দান করতে পারে, কুরআন পড়তে পারে; কিন্তু অন্তরে যদি মানুষের দৃষ্টি ও নাম কামনার ইচ্ছা ঢুকে যায়, তবে তা রিয়া হয়ে যায়। তাই হাদিসটি আমাদের নীরবে নিজের অন্তরকে প্রশ্ন করতে শেখায়—আমি এই কাজটি কার জন্য করছি? আল্লাহর জন্য, নাকি মানুষের চোখে বড় হওয়ার জন্য?"},"teachings":["প্রশংসা পাওয়ার উদ্দেশ্যে আমল করা সুমআহর দিকে নিয়ে যায়।","মানুষকে দেখানোর জন্য আমল করা রিয়ার অন্তর্ভুক্ত।","কিয়ামতে আমলের পেছনের উদ্দেশ্য প্রকাশিত হতে পারে।","প্রতিটি নেক কাজের আগে নিজের নিয়ত যাচাই করা দরকার।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2986","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও সুমআহর অপমানজনক পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. লোক দেখানো বা প্রশংসা শোনার উদ্দেশ্যে আমল করলে আল্লাহ কিয়ামতে তা প্রকাশ করে অপমানিত করবেন।"},"heading":{"title":"রিয়া ও সুমআহ: ইবাদতে মানুষের দৃষ্টি খোঁজার ক্ষতি","description":"এই হাদিসে রিয়া এবং সুমআহকে খুব সরাসরি ভাষায় সতর্ক করা হয়েছে। কেউ যদি লোক দেখানোর উদ্দেশ্যে আমল করে, আল্লাহ তার সেই আমল দেখিয়ে দেবেন। আর কেউ যদি মানুষের প্রশংসা শোনার উদ্দেশ্যে আমল করে, আল্লাহ তার কথা সৃষ্টিকুলকে শুনিয়ে দেবেন এবং তাকে অপমানিত করবেন। হাদিসটি আমাদের শেখায়, মানুষের চোখে ধার্মিক দেখানো আর আল্লাহর কাছে গ্রহণযোগ্য হওয়া এক জিনিস নয়। অনেক সময় মানুষ বাহ্যিক কাজ দেখে প্রশংসা করে, কিন্তু আল্লাহ অন্তরের উদ্দেশ্য জানেন। তাই মুমিনের উচিত নিজের আমলকে আল্লাহর জন্য রাখা। প্রকাশ্য আমল করলেও অন্তর যেন মানুষের হাততালি বা নামের পেছনে না যায়। এই সতর্কতা বিশেষ করে ইবাদত, দান, জ্ঞানচর্চা এবং ভালো কাজের ক্ষেত্রে খুব প্রয়োজন।"},"teachings":["লোক দেখানো আমল কিয়ামতে অপমানের কারণ হতে পারে।","সুমআহ মানে মানুষের কাছে নিজের আমলের কথা শোনানোর মানসিকতা।","আল্লাহ অন্তরের উদ্দেশ্য জানেন, তাই বাহ্যিক প্রশংসায় ভরসা করা ঠিক নয়।","ইবাদতে মানুষের দৃষ্টি নয়, আল্লাহর সন্তুষ্টি কামনা করা দরকার।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"24","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E107" s="4" t="n"/>
@@ -2961,12 +2957,12 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ও সুমআহর অপমানজনক পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. লোক দেখানো বা প্রশংসা শোনার উদ্দেশ্যে আমল করলে আল্লাহ কিয়ামতে তা প্রকাশ করে অপমানিত করবেন।"},"heading":{"title":"রিয়া ও সুমআহ: ইবাদতে মানুষের দৃষ্টি খোঁজার ক্ষতি","description":"এই হাদিসে রিয়া এবং সুমআহকে খুব সরাসরি ভাষায় সতর্ক করা হয়েছে। কেউ যদি লোক দেখানোর উদ্দেশ্যে আমল করে, আল্লাহ তার সেই আমল দেখিয়ে দেবেন। আর কেউ যদি মানুষের প্রশংসা শোনার উদ্দেশ্যে আমল করে, আল্লাহ তার কথা সৃষ্টিকুলকে শুনিয়ে দেবেন এবং তাকে অপমানিত করবেন। হাদিসটি আমাদের শেখায়, মানুষের চোখে ধার্মিক দেখানো আর আল্লাহর কাছে গ্রহণযোগ্য হওয়া এক জিনিস নয়। অনেক সময় মানুষ বাহ্যিক কাজ দেখে প্রশংসা করে, কিন্তু আল্লাহ অন্তরের উদ্দেশ্য জানেন। তাই মুমিনের উচিত নিজের আমলকে আল্লাহর জন্য রাখা। প্রকাশ্য আমল করলেও অন্তর যেন মানুষের হাততালি বা নামের পেছনে না যায়। এই সতর্কতা বিশেষ করে ইবাদত, দান, জ্ঞানচর্চা এবং ভালো কাজের ক্ষেত্রে খুব প্রয়োজন।"},"teachings":["লোক দেখানো আমল কিয়ামতে অপমানের কারণ হতে পারে।","সুমআহ মানে মানুষের কাছে নিজের আমলের কথা শোনানোর মানসিকতা।","আল্লাহ অন্তরের উদ্দেশ্য জানেন, তাই বাহ্যিক প্রশংসায় ভরসা করা ঠিক নয়।","ইবাদতে মানুষের দৃষ্টি নয়, আল্লাহর সন্তুষ্টি কামনা করা দরকার।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"24","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শ্রুতি ও প্রদর্শনের আমলের পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. পৃথিবীতে শ্রুতি ও প্রদর্শনের জন্য আমল করলে কিয়ামতে আল্লাহ সেই অসৎ নিয়ত সৃষ্টির সামনে প্রকাশ করবেন।"},"heading":{"title":"শ্রুতি ও প্রদর্শনের জন্য আমল: কিয়ামতের দিনের সতর্কতা","description":"এই হাদিসে বলা হয়েছে, যে বান্দা দুনিয়াতে শ্রুতি ও প্রদর্শনের জন্য কোনো আমল করে, আল্লাহ কিয়ামতের দিন সমস্ত সৃষ্টির সামনে তার অসৎ নিয়ত প্রকাশ করবেন। শ্রুতি মানে নিজের আমলের কথা মানুষের কানে পৌঁছানো, আর প্রদর্শন মানে মানুষের চোখে ভালো দেখানোর জন্য কাজ করা। দুটোর মূল রোগ একই—মানুষের প্রশংসা কামনা করা। এই হাদিস আমাদের শেখায়, দুনিয়ার সাময়িক নাম বা পরিচিতি আমলের আসল লক্ষ্য হতে পারে না। নেক কাজের সৌন্দর্য তখনই থাকে, যখন তা আল্লাহর জন্য হয়। তাই প্রকাশ্য কাজ করলেও অন্তরের লক্ষ্য পরিষ্কার রাখা দরকার। মানুষ জানুক বা না জানুক, আল্লাহ যেন সন্তুষ্ট হন—এই চিন্তাই ইখলাসের পথে সাহায্য করে।"},"teachings":["শ্রুতি ও প্রদর্শন আমলের ইখলাসকে নষ্ট করতে পারে।","দুনিয়ার পরিচিতি আখেরাতের নিরাপত্তার নিশ্চয়তা নয়।","কিয়ামতে গোপন উদ্দেশ্য প্রকাশ পাওয়ার আশঙ্কা আছে।","নেক কাজের লক্ষ্য হওয়া উচিত আল্লাহর সন্তুষ্টি।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"33","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E108" s="4" t="n"/>
@@ -2984,12 +2980,12 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | শ্রুতি ও প্রদর্শনের আমলের পরিণতি","description":"$book_name$ $hadith_number$ - $chapter_name$. পৃথিবীতে শ্রুতি ও প্রদর্শনের জন্য আমল করলে কিয়ামতে আল্লাহ সেই অসৎ নিয়ত সৃষ্টির সামনে প্রকাশ করবেন।"},"heading":{"title":"শ্রুতি ও প্রদর্শনের জন্য আমল: কিয়ামতের দিনের সতর্কতা","description":"এই হাদিসে বলা হয়েছে, যে বান্দা দুনিয়াতে শ্রুতি ও প্রদর্শনের জন্য কোনো আমল করে, আল্লাহ কিয়ামতের দিন সমস্ত সৃষ্টির সামনে তার অসৎ নিয়ত প্রকাশ করবেন। শ্রুতি মানে নিজের আমলের কথা মানুষের কানে পৌঁছানো, আর প্রদর্শন মানে মানুষের চোখে ভালো দেখানোর জন্য কাজ করা। দুটোর মূল রোগ একই—মানুষের প্রশংসা কামনা করা। এই হাদিস আমাদের শেখায়, দুনিয়ার সাময়িক নাম বা পরিচিতি আমলের আসল লক্ষ্য হতে পারে না। নেক কাজের সৌন্দর্য তখনই থাকে, যখন তা আল্লাহর জন্য হয়। তাই প্রকাশ্য কাজ করলেও অন্তরের লক্ষ্য পরিষ্কার রাখা দরকার। মানুষ জানুক বা না জানুক, আল্লাহ যেন সন্তুষ্ট হন—এই চিন্তাই ইখলাসের পথে সাহায্য করে।"},"teachings":["শ্রুতি ও প্রদর্শন আমলের ইখলাসকে নষ্ট করতে পারে।","দুনিয়ার পরিচিতি আখেরাতের নিরাপত্তার নিশ্চয়তা নয়।","কিয়ামতে গোপন উদ্দেশ্য প্রকাশ পাওয়ার আশঙ্কা আছে।","নেক কাজের লক্ষ্য হওয়া উচিত আল্লাহর সন্তুষ্টি।"],"related_hadiths":[{"id":"6499","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"26","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"33","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মানুষকে দেখানোর আমলের অসারতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়ায় মানুষকে দেখানোর জন্য করা আমল কিয়ামতে উপকার করবে কি না—এই প্রশ্নেই তার অসারতা প্রকাশ পাবে।"},"heading":{"title":"মানুষকে দেখানোর আমল: কিয়ামতে কী উপকার দেবে?","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তি দুনিয়াতে কোনো আমল মানুষকে দেখানোর জন্য করেছে, কিয়ামতের দিন আল্লাহ তাকে সেই আমলের দিকে সোপর্দ করবেন এবং বলবেন, দেখো তো তা তোমার কোনো উপকারে আসে কি না। এই কথার মধ্যে বড় শিক্ষা আছে। মানুষকে দেখানোর জন্য করা আমল দুনিয়ায় প্রশংসা এনে দিতে পারে, কিন্তু আখেরাতের দরকারের সময় তা সহায়ক হবে কি না—এটাই ভয়ের বিষয়। বর্ণনাটি মাওকুফ হলেও এর বার্তা রিয়া সম্পর্কে অন্যান্য হাদিসের সঙ্গে মিলে যায়। এখানে আমলের বাহ্যিক রূপের চেয়ে উদ্দেশ্যকে বেশি গুরুত্ব দেওয়া হয়েছে। তাই মুমিনের উচিত নেক কাজকে মানুষের চোখের জন্য না বানানো। আল্লাহর জন্য করা কাজই আখেরাতের আশার কারণ হতে পারে।"},"teachings":["মানুষকে দেখানোর জন্য করা আমল আখেরাতে উপকারহীন হতে পারে।","দুনিয়ার প্রশংসা আমলের আসল ফল নয়।","নেক আমলে নিয়ত ঠিক রাখা দরকার।","কিয়ামতের হিসাব মানুষের দৃষ্টির ভিত্তিতে নয়, আল্লাহর জ্ঞানের ভিত্তিতে হবে।"],"related_hadiths":[{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E109" s="4" t="n"/>
@@ -3007,12 +3003,12 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মানুষকে দেখানোর আমলের অসারতা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়ায় মানুষকে দেখানোর জন্য করা আমল কিয়ামতে উপকার করবে কি না—এই প্রশ্নেই তার অসারতা প্রকাশ পাবে।"},"heading":{"title":"মানুষকে দেখানোর আমল: কিয়ামতে কী উপকার দেবে?","description":"এই বর্ণনায় বলা হয়েছে, যে ব্যক্তি দুনিয়াতে কোনো আমল মানুষকে দেখানোর জন্য করেছে, কিয়ামতের দিন আল্লাহ তাকে সেই আমলের দিকে সোপর্দ করবেন এবং বলবেন, দেখো তো তা তোমার কোনো উপকারে আসে কি না। এই কথার মধ্যে বড় শিক্ষা আছে। মানুষকে দেখানোর জন্য করা আমল দুনিয়ায় প্রশংসা এনে দিতে পারে, কিন্তু আখেরাতের দরকারের সময় তা সহায়ক হবে কি না—এটাই ভয়ের বিষয়। বর্ণনাটি মাওকুফ হলেও এর বার্তা রিয়া সম্পর্কে অন্যান্য হাদিসের সঙ্গে মিলে যায়। এখানে আমলের বাহ্যিক রূপের চেয়ে উদ্দেশ্যকে বেশি গুরুত্ব দেওয়া হয়েছে। তাই মুমিনের উচিত নেক কাজকে মানুষের চোখের জন্য না বানানো। আল্লাহর জন্য করা কাজই আখেরাতের আশার কারণ হতে পারে।"},"teachings":["মানুষকে দেখানোর জন্য করা আমল আখেরাতে উপকারহীন হতে পারে।","দুনিয়ার প্রশংসা আমলের আসল ফল নয়।","নেক আমলে নিয়ত ঠিক রাখা দরকার।","কিয়ামতের হিসাব মানুষের দৃষ্টির ভিত্তিতে নয়, আল্লাহর জ্ঞানের ভিত্তিতে হবে।"],"related_hadiths":[{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোপন শির্ক ও সাজানো সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের দৃষ্টি আকর্ষণের জন্য সালাত সুন্দর করে পড়া গোপন শির্কের উদাহরণ হিসেবে সতর্ক করা হয়েছে।"},"heading":{"title":"গোপন শির্ক: মানুষের জন্য সালাত সাজানোর বিপদ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের এমন এক বিষয়ের কথা জানালেন, যা তিনি দাজ্জালের চেয়েও বেশি ভয় করতেন। সেটি হলো গোপন শির্ক। এর উদাহরণ হিসেবে বলা হয়েছে, একজন ব্যক্তি সালাতে দাঁড়ায়, তারপর মানুষের দৃষ্টি দেখে নিজের সালাতকে সাজিয়ে তোলে। অর্থাৎ সালাতের সৌন্দর্য আল্লাহর জন্য নয়, মানুষের দেখার জন্য বাড়িয়ে দেয়। এই হাদিস আমাদের খুব সূক্ষ্ম একটি রোগের দিকে সতর্ক করে। বাহ্যিকভাবে কাজটি নামাজ, কিন্তু অন্তরের উদ্দেশ্যে মানুষের দৃষ্টি ঢুকে গেলে তা বিপজ্জনক হয়ে যায়। তাই সালাতে খুশু, রুকু, সিজদা—সবকিছু আল্লাহর জন্য হওয়া দরকার। মানুষ দেখছে কি না, তা যেন আমলের মান পরিবর্তনের কারণ না হয়।"},"teachings":["মানুষের দৃষ্টি দেখে সালাত সাজানো গোপন শির্কের উদাহরণ।","ইবাদতের বাহ্যিক সৌন্দর্যের সঙ্গে অন্তরের ইখলাস থাকা দরকার।","গোপন শির্ক খুব সূক্ষ্ম, তাই আত্মপরীক্ষা জরুরি।","সালাতের লক্ষ্য আল্লাহর সন্তুষ্টি, মানুষের প্রশংসা নয়।"],"related_hadiths":[{"id":"31","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"36","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E110" s="4" t="n"/>
@@ -3030,12 +3026,12 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গোপন শির্ক ও সাজানো সালাত","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের দৃষ্টি আকর্ষণের জন্য সালাত সুন্দর করে পড়া গোপন শির্কের উদাহরণ হিসেবে সতর্ক করা হয়েছে।"},"heading":{"title":"গোপন শির্ক: মানুষের জন্য সালাত সাজানোর বিপদ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের এমন এক বিষয়ের কথা জানালেন, যা তিনি দাজ্জালের চেয়েও বেশি ভয় করতেন। সেটি হলো গোপন শির্ক। এর উদাহরণ হিসেবে বলা হয়েছে, একজন ব্যক্তি সালাতে দাঁড়ায়, তারপর মানুষের দৃষ্টি দেখে নিজের সালাতকে সাজিয়ে তোলে। অর্থাৎ সালাতের সৌন্দর্য আল্লাহর জন্য নয়, মানুষের দেখার জন্য বাড়িয়ে দেয়। এই হাদিস আমাদের খুব সূক্ষ্ম একটি রোগের দিকে সতর্ক করে। বাহ্যিকভাবে কাজটি নামাজ, কিন্তু অন্তরের উদ্দেশ্যে মানুষের দৃষ্টি ঢুকে গেলে তা বিপজ্জনক হয়ে যায়। তাই সালাতে খুশু, রুকু, সিজদা—সবকিছু আল্লাহর জন্য হওয়া দরকার। মানুষ দেখছে কি না, তা যেন আমলের মান পরিবর্তনের কারণ না হয়।"},"teachings":["মানুষের দৃষ্টি দেখে সালাত সাজানো গোপন শির্কের উদাহরণ।","ইবাদতের বাহ্যিক সৌন্দর্যের সঙ্গে অন্তরের ইখলাস থাকা দরকার।","গোপন শির্ক খুব সূক্ষ্ম, তাই আত্মপরীক্ষা জরুরি।","সালাতের লক্ষ্য আল্লাহর সন্তুষ্টি, মানুষের প্রশংসা নয়।"],"related_hadiths":[{"id":"31","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"36","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাতে গোপন শির্ক থেকে সাবধান","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের নজর দেখে রুকু-সিজদা সুন্দর করা গোপন শির্ক; তাই সালাতে ইখলাস রক্ষা জরুরি।"},"heading":{"title":"সালাতে গোপন শির্ক: মানুষের নজর দেখে ইবাদত বদলানো","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম মানুষকে গোপন শির্ক থেকে সাবধান করেছেন। সাহাবীরা জিজ্ঞেস করলেন, গোপন শির্ক কী? উত্তরে বলা হলো, একজন ব্যক্তি সালাতে দাঁড়ায় এবং মানুষের চোখের দৃষ্টি দেখে ইচ্ছাকৃতভাবে রুকু ও সিজদা সুন্দর করে। এতে বোঝা যায়, ইবাদতের ভেতরে মানুষের প্রশংসা বা দৃষ্টি খোঁজা কত সূক্ষ্মভাবে ঢুকে যেতে পারে। সালাত আল্লাহর সামনে দাঁড়ানোর আমল। তাই একজন মুমিন একা থাকুক বা মানুষের সামনে থাকুক, তার ইবাদতের উদ্দেশ্য একই হওয়া উচিত। হাদিসটি আমাদের শেখায়, বাহ্যিক ভঙ্গি সুন্দর করা যথেষ্ট নয়; অন্তরের লক্ষ্যও পরিষ্কার থাকা দরকার। মানুষের জন্য নয়, আল্লাহর জন্য সালাতকে সুন্দর করতে হবে।"},"teachings":["মানুষের নজর দেখে সালাতের ভঙ্গি বদলানো গোপন শির্কের লক্ষণ হতে পারে।","রুকু ও সিজদা আল্লাহর জন্য সুন্দর হওয়া উচিত।","ইবাদতে ইচ্ছাকৃত আত্মপ্রদর্শন থেকে সতর্ক থাকা দরকার।","সালাতে ইখলাস রক্ষা করা মুমিনের বড় দায়িত্ব।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"35","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E111" s="4" t="n"/>
@@ -3053,15 +3049,19 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সালাতে গোপন শির্ক থেকে সাবধান","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষের নজর দেখে রুকু-সিজদা সুন্দর করা গোপন শির্ক; তাই সালাতে ইখলাস রক্ষা জরুরি।"},"heading":{"title":"সালাতে গোপন শির্ক: মানুষের নজর দেখে ইবাদত বদলানো","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম মানুষকে গোপন শির্ক থেকে সাবধান করেছেন। সাহাবীরা জিজ্ঞেস করলেন, গোপন শির্ক কী? উত্তরে বলা হলো, একজন ব্যক্তি সালাতে দাঁড়ায় এবং মানুষের চোখের দৃষ্টি দেখে ইচ্ছাকৃতভাবে রুকু ও সিজদা সুন্দর করে। এতে বোঝা যায়, ইবাদতের ভেতরে মানুষের প্রশংসা বা দৃষ্টি খোঁজা কত সূক্ষ্মভাবে ঢুকে যেতে পারে। সালাত আল্লাহর সামনে দাঁড়ানোর আমল। তাই একজন মুমিন একা থাকুক বা মানুষের সামনে থাকুক, তার ইবাদতের উদ্দেশ্য একই হওয়া উচিত। হাদিসটি আমাদের শেখায়, বাহ্যিক ভঙ্গি সুন্দর করা যথেষ্ট নয়; অন্তরের লক্ষ্যও পরিষ্কার থাকা দরকার। মানুষের জন্য নয়, আল্লাহর জন্য সালাতকে সুন্দর করতে হবে।"},"teachings":["মানুষের নজর দেখে সালাতের ভঙ্গি বদলানো গোপন শির্কের লক্ষণ হতে পারে।","রুকু ও সিজদা আল্লাহর জন্য সুন্দর হওয়া উচিত।","ইবাদতে ইচ্ছাকৃত আত্মপ্রদর্শন থেকে সতর্ক থাকা দরকার।","সালাতে ইখলাস রক্ষা করা মুমিনের বড় দায়িত্ব।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"35","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="n"/>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ছোট শির্ক রিয়া থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ছোট শির্ক হলো রিয়া; যারা দেখানোর জন্য আমল করে তাদের বলা হবে, যাদের দেখিয়েছিলে তাদের কাছেই প্রতিদান খোঁজো।"},"heading":{"title":"ছোট শির্ক রিয়া: আমলের প্রতিদান কোথায় খুঁজবে?","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর উম্মতের জন্য যে বিষয়টি নিয়ে গভীর আশঙ্কা করেছেন, সেটি হলো শির্ক আসগার বা ছোট শির্ক। সাহাবীরা জিজ্ঞেস করলে তিনি বলেন, সেটি রিয়া। এরপর কিয়ামতের একটি দৃশ্য বলা হয়েছে। যখন মানুষকে তাদের আমলের প্রতিদান দেওয়া হবে, তখন রিয়াকারীদের বলা হবে, দুনিয়ায় যাদের দেখানোর জন্য তোমরা আমল করতে, তাদের কাছে যাও এবং দেখো তাদের কাছে কোনো প্রতিদান পাও কি না। এই হাদিস খুব স্পষ্ট করে দেয় যে ইবাদত মানুষের জন্য হলে তা আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা হয়। তাই সালাত, দান, জ্ঞান, কুরআন—সব আমলে নিয়ত আল্লাহর জন্য রাখা দরকার। মানুষের প্রশংসা সাময়িক; আখেরাতের প্রতিদান আল্লাহর কাছেই।"},"teachings":["রিয়া ছোট শির্ক হিসেবে উল্লেখ করা হয়েছে।","মানুষকে দেখানোর জন্য আমল করলে আখেরাতে প্রতিদান হারানোর আশঙ্কা আছে।","আমলের আসল উদ্দেশ্য আল্লাহর সন্তুষ্টি হওয়া জরুরি।","মানুষের প্রশংসা আখেরাতের প্রতিদানের বিকল্প নয়।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>related_hadiths[2]: unknown book label "সহিহ হাদিসে কুদসি ৭"</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="46" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
@@ -3076,19 +3076,15 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ছোট শির্ক রিয়া থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ছোট শির্ক হলো রিয়া; যারা দেখানোর জন্য আমল করে তাদের বলা হবে, যাদের দেখিয়েছিলে তাদের কাছেই প্রতিদান খোঁজো।"},"heading":{"title":"ছোট শির্ক রিয়া: আমলের প্রতিদান কোথায় খুঁজবে?","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর উম্মতের জন্য যে বিষয়টি নিয়ে গভীর আশঙ্কা করেছেন, সেটি হলো শির্ক আসগার বা ছোট শির্ক। সাহাবীরা জিজ্ঞেস করলে তিনি বলেন, সেটি রিয়া। এরপর কিয়ামতের একটি দৃশ্য বলা হয়েছে। যখন মানুষকে তাদের আমলের প্রতিদান দেওয়া হবে, তখন রিয়াকারীদের বলা হবে, দুনিয়ায় যাদের দেখানোর জন্য তোমরা আমল করতে, তাদের কাছে যাও এবং দেখো তাদের কাছে কোনো প্রতিদান পাও কি না। এই হাদিস খুব স্পষ্ট করে দেয় যে ইবাদত মানুষের জন্য হলে তা আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা হয়। তাই সালাত, দান, জ্ঞান, কুরআন—সব আমলে নিয়ত আল্লাহর জন্য রাখা দরকার। মানুষের প্রশংসা সাময়িক; আখেরাতের প্রতিদান আল্লাহর কাছেই।"},"teachings":["রিয়া ছোট শির্ক হিসেবে উল্লেখ করা হয়েছে।","মানুষকে দেখানোর জন্য আমল করলে আখেরাতে প্রতিদান হারানোর আশঙ্কা আছে।","আমলের আসল উদ্দেশ্য আল্লাহর সন্তুষ্টি হওয়া জরুরি।","মানুষের প্রশংসা আখেরাতের প্রতিদানের বিকল্প নয়।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[2]: unknown book label "সহিহ হাদিসে কুদসি ৭"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আমলে আল্লাহর সাথে অংশীদার করা","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি আল্লাহর জন্য করা আমলে অন্যকে অংশীদার করে, তাকে তার প্রতিদান সেই অংশীদারের কাছেই চাইতে বলা হবে।"},"heading":{"title":"আমলে অংশীদার করা: রিয়ার গভীর সতর্কবার্তা","description":"এই হাদিসে কিয়ামতের দিনের একটি ঘোষণা সম্পর্কে বলা হয়েছে। যখন আল্লাহ সব মানুষকে একত্রিত করবেন, তখন একজন ঘোষণাকারী বলবে, যে ব্যক্তি আল্লাহর জন্য করা কোনো আমলে অন্য কাউকে অংশীদার করেছে, সে যেন তার প্রতিদান সেই ব্যক্তির কাছেই চায়। কারণ আল্লাহ অংশীদারদের অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত। এর অর্থ হলো, ইবাদত বা নেক কাজ যদি আল্লাহর সঙ্গে মানুষের প্রশংসা, নাম বা স্বীকৃতিকে উদ্দেশ্য বানায়, তবে তা বড় ক্ষতির কারণ। হাদিসটি আমাদের শেখায়, আমল দেখতে ভালো হলেও নিয়ত যদি মিশ্র হয়, তা বিপজ্জনক হতে পারে। আল্লাহর জন্য করা কাজে আল্লাহকেই উদ্দেশ্য করা দরকার। মানুষের কাছে মর্যাদা চাইলে মানুষ সাময়িক কিছু দিতে পারে, কিন্তু আখেরাতের প্রতিদান আল্লাহর হাতে।"},"teachings":["আল্লাহর জন্য করা আমলে অন্য উদ্দেশ্য মিশানো বিপজ্জনক।","রিয়া আমলকে আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা দিতে পারে।","কিয়ামতে প্রতিদান আল্লাহর কাছেই কামনা করতে হবে।","আল্লাহ অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="n"/>
     </row>
     <row r="114" ht="46" customHeight="1">
       <c r="A114" s="4" t="inlineStr">
@@ -3103,15 +3099,19 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আমলে আল্লাহর সাথে অংশীদার করা","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি আল্লাহর জন্য করা আমলে অন্যকে অংশীদার করে, তাকে তার প্রতিদান সেই অংশীদারের কাছেই চাইতে বলা হবে।"},"heading":{"title":"আমলে অংশীদার করা: রিয়ার গভীর সতর্কবার্তা","description":"এই হাদিসে কিয়ামতের দিনের একটি ঘোষণা সম্পর্কে বলা হয়েছে। যখন আল্লাহ সব মানুষকে একত্রিত করবেন, তখন একজন ঘোষণাকারী বলবে, যে ব্যক্তি আল্লাহর জন্য করা কোনো আমলে অন্য কাউকে অংশীদার করেছে, সে যেন তার প্রতিদান সেই ব্যক্তির কাছেই চায়। কারণ আল্লাহ অংশীদারদের অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত। এর অর্থ হলো, ইবাদত বা নেক কাজ যদি আল্লাহর সঙ্গে মানুষের প্রশংসা, নাম বা স্বীকৃতিকে উদ্দেশ্য বানায়, তবে তা বড় ক্ষতির কারণ। হাদিসটি আমাদের শেখায়, আমল দেখতে ভালো হলেও নিয়ত যদি মিশ্র হয়, তা বিপজ্জনক হতে পারে। আল্লাহর জন্য করা কাজে আল্লাহকেই উদ্দেশ্য করা দরকার। মানুষের কাছে মর্যাদা চাইলে মানুষ সাময়িক কিছু দিতে পারে, কিন্তু আখেরাতের প্রতিদান আল্লাহর হাতে।"},"teachings":["আল্লাহর জন্য করা আমলে অন্য উদ্দেশ্য মিশানো বিপজ্জনক।","রিয়া আমলকে আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা দিতে পারে।","কিয়ামতে প্রতিদান আল্লাহর কাছেই কামনা করতে হবে।","আল্লাহ অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"34","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"22","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
-        </is>
-      </c>
-      <c r="E114" s="4" t="n"/>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য আমলে রিয়া মেশানোর ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ বলেন, যে আমার জন্য আমল করে তাতে অন্যকে শরীক করে, আমি সেই আমল থেকে সম্পূর্ণ মুক্ত।"},"heading":{"title":"রিয়া মেশানো আমল: আল্লাহ অংশীদারিত্ব থেকে মুক্ত","description":"এই হাদিসে কুদসির ভাষায় আল্লাহর পক্ষ থেকে এক বড় সতর্কতা এসেছে। আল্লাহ বলেন, তিনি অংশীদারদের অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত। কেউ যদি আল্লাহর জন্য কোনো আমল করে, কিন্তু তাতে অন্য কাউকে অংশীদার করে, তবে আল্লাহ সেই আমল থেকে মুক্ত। অর্থাৎ আমলটি আল্লাহর জন্য খাঁটি থাকল না। এখানে রিয়ার মূল সমস্যা স্পষ্ট হয়—মানুষের প্রশংসা, সম্মান বা দৃষ্টি যদি আমলের উদ্দেশ্যে ঢুকে যায়, তবে ইখলাস নষ্ট হয়। এই হাদিস আমাদের শেখায়, ইবাদত শুধু বাহ্যিক কাজের নাম নয়; এটি অন্তরের সত্য দিকও দাবি করে। আল্লাহর জন্য নামাজ, দান, কুরআন, জ্ঞান বা অন্য যে আমলই করা হোক, তা আল্লাহর জন্যই রাখা দরকার।"},"teachings":["আল্লাহ অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত।","আল্লাহর জন্য করা আমলে অন্য উদ্দেশ্য মেশানো বিপজ্জনক।","রিয়া আমলের ইখলাস নষ্ট করতে পারে।","প্রতিটি নেক কাজ আল্লাহর সন্তুষ্টির জন্য হওয়া উচিত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"33","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>related_hadiths[0]: unknown book label "সহিহ হাদিসে কুদসি ৭"</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="46" customHeight="1">
       <c r="A115" s="4" t="inlineStr">
@@ -3126,19 +3126,15 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য আমলে রিয়া মেশানোর ক্ষতি","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ বলেন, যে আমার জন্য আমল করে তাতে অন্যকে শরীক করে, আমি সেই আমল থেকে সম্পূর্ণ মুক্ত।"},"heading":{"title":"রিয়া মেশানো আমল: আল্লাহ অংশীদারিত্ব থেকে মুক্ত","description":"এই হাদিসে কুদসির ভাষায় আল্লাহর পক্ষ থেকে এক বড় সতর্কতা এসেছে। আল্লাহ বলেন, তিনি অংশীদারদের অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত। কেউ যদি আল্লাহর জন্য কোনো আমল করে, কিন্তু তাতে অন্য কাউকে অংশীদার করে, তবে আল্লাহ সেই আমল থেকে মুক্ত। অর্থাৎ আমলটি আল্লাহর জন্য খাঁটি থাকল না। এখানে রিয়ার মূল সমস্যা স্পষ্ট হয়—মানুষের প্রশংসা, সম্মান বা দৃষ্টি যদি আমলের উদ্দেশ্যে ঢুকে যায়, তবে ইখলাস নষ্ট হয়। এই হাদিস আমাদের শেখায়, ইবাদত শুধু বাহ্যিক কাজের নাম নয়; এটি অন্তরের সত্য দিকও দাবি করে। আল্লাহর জন্য নামাজ, দান, কুরআন, জ্ঞান বা অন্য যে আমলই করা হোক, তা আল্লাহর জন্যই রাখা দরকার।"},"teachings":["আল্লাহ অংশীদারিত্ব থেকে সম্পূর্ণ মুক্ত।","আল্লাহর জন্য করা আমলে অন্য উদ্দেশ্য মেশানো বিপজ্জনক।","রিয়া আমলের ইখলাস নষ্ট করতে পারে।","প্রতিটি নেক কাজ আল্লাহর সন্তুষ্টির জন্য হওয়া উচিত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"33","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[0]: unknown book label "সহিহ হাদিসে কুদসি ৭"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ছোট শির্ক হিসেবে গণ্য","description":"$book_name$ $hadith_number$ - $chapter_name$. সাহাবীদের সময়ে রিয়াকে ছোট শির্ক হিসেবে গণ্য করা হতো; তাই ইবাদতে ইখলাস রক্ষা জরুরি।"},"heading":{"title":"রিয়া ছোট শির্ক: সাহাবীদের দৃষ্টিতে ইখলাসের গুরুত্ব","description":"এই বর্ণনায় শাদ্দাদ রাদিয়াল্লাহু আনহু বলেন, নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের যুগে তারা রিয়াকে ছোট শির্ক হিসেবে গণ্য করতেন। বাক্যটি ছোট, কিন্তু শিক্ষা খুব গভীর। রিয়া মানে মানুষের সামনে নিজেকে দেখানোর জন্য ইবাদত বা নেক কাজ করা। সাহাবীরা এটিকে হালকা বিষয় মনে করেননি; বরং শির্ক আসগারের অন্তর্ভুক্ত হিসেবে দেখতেন। এতে বোঝা যায়, ইবাদতের বাহ্যিক রূপ যেমন গুরুত্বপূর্ণ, তেমনি অন্তরের উদ্দেশ্যও গুরুত্বপূর্ণ। কেউ নামাজ পড়ছে, দান করছে বা জ্ঞান শিখছে—এসব ভালো কাজ। কিন্তু যদি উদ্দেশ্য হয় মানুষ যেন দেখে, প্রশংসা করে বা মর্যাদা দেয়, তাহলে সেই আমল বিপদের মুখে পড়ে। তাই মুমিনের উচিত রিয়া সম্পর্কে ভয় রাখা এবং ইখলাসের জন্য দোয়া করা।"},"teachings":["সাহাবীরা রিয়াকে ছোট শির্ক হিসেবে গণ্য করতেন।","রিয়াকে ছোট বিষয় মনে করা উচিত নয়।","ইবাদতের বাহ্যিক রূপের সঙ্গে অন্তরের ইখলাস দরকার।","মানুষের প্রশংসা নয়, আল্লাহর সন্তুষ্টিই আমলের লক্ষ্য হওয়া উচিত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"36","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="n"/>
     </row>
     <row r="116" ht="46" customHeight="1">
       <c r="A116" s="4" t="inlineStr">
@@ -3153,12 +3149,12 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রিয়া ছোট শির্ক হিসেবে গণ্য","description":"$book_name$ $hadith_number$ - $chapter_name$. সাহাবীদের সময়ে রিয়াকে ছোট শির্ক হিসেবে গণ্য করা হতো; তাই ইবাদতে ইখলাস রক্ষা জরুরি।"},"heading":{"title":"রিয়া ছোট শির্ক: সাহাবীদের দৃষ্টিতে ইখলাসের গুরুত্ব","description":"এই বর্ণনায় শাদ্দাদ রাদিয়াল্লাহু আনহু বলেন, নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের যুগে তারা রিয়াকে ছোট শির্ক হিসেবে গণ্য করতেন। বাক্যটি ছোট, কিন্তু শিক্ষা খুব গভীর। রিয়া মানে মানুষের সামনে নিজেকে দেখানোর জন্য ইবাদত বা নেক কাজ করা। সাহাবীরা এটিকে হালকা বিষয় মনে করেননি; বরং শির্ক আসগারের অন্তর্ভুক্ত হিসেবে দেখতেন। এতে বোঝা যায়, ইবাদতের বাহ্যিক রূপ যেমন গুরুত্বপূর্ণ, তেমনি অন্তরের উদ্দেশ্যও গুরুত্বপূর্ণ। কেউ নামাজ পড়ছে, দান করছে বা জ্ঞান শিখছে—এসব ভালো কাজ। কিন্তু যদি উদ্দেশ্য হয় মানুষ যেন দেখে, প্রশংসা করে বা মর্যাদা দেয়, তাহলে সেই আমল বিপদের মুখে পড়ে। তাই মুমিনের উচিত রিয়া সম্পর্কে ভয় রাখা এবং ইখলাসের জন্য দোয়া করা।"},"teachings":["সাহাবীরা রিয়াকে ছোট শির্ক হিসেবে গণ্য করতেন।","রিয়াকে ছোট বিষয় মনে করা উচিত নয়।","ইবাদতের বাহ্যিক রূপের সঙ্গে অন্তরের ইখলাস দরকার।","মানুষের প্রশংসা নয়, আল্লাহর সন্তুষ্টিই আমলের লক্ষ্য হওয়া উচিত।"],"related_hadiths":[{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"36","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সূক্ষ্ম শির্ক থেকে বাঁচার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. শির্ক পিপিলিকার চলার শব্দের চেয়েও সূক্ষ্ম; তাই জানা-অজানা শির্ক থেকে আশ্রয় ও ক্ষমা চাইতে শেখানো হয়েছে।"},"heading":{"title":"গোপন শির্ক থেকে বাঁচার দোয়া ও সতর্কতা","description":"এই হাদিসে শির্কের সূক্ষ্মতা খুব শক্তভাবে বোঝানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, শির্ক পিপিলিকার চলার শব্দ থেকেও গোপন হতে পারে। সাহাবীদের পক্ষ থেকে প্রশ্ন আসে, এত সূক্ষ্ম বিষয় থেকে কীভাবে বাঁচা যাবে? উত্তরে একটি দোয়া শেখানো হয়েছে: হে আল্লাহ, আমরা জেনে তোমার সাথে কোনো কিছুকে শরীক করা থেকে তোমার আশ্রয় চাই এবং যা আমরা জানি না, তার জন্য তোমার কাছে ক্ষমা চাই। এই দোয়া আমাদের শেখায়, মানুষ নিজের অন্তরের সব সূক্ষ্ম রোগ সব সময় বুঝতে পারে না। তাই সতর্কতা, আত্মপরীক্ষা এবং আল্লাহর কাছে আশ্রয়—সবই দরকার। বিশেষ করে রিয়া, আত্মপ্রদর্শন ও প্রশংসার আকাঙ্ক্ষা থেকে বাঁচতে এই হাদিস খুব প্রাসঙ্গিক।"},"teachings":["শির্ক কখনো খুব সূক্ষ্মভাবে অন্তরে ঢুকতে পারে।","জানা ও অজানা ভুলের জন্য আল্লাহর কাছে আশ্রয় ও ক্ষমা চাওয়া দরকার।","রিয়া থেকে বাঁচতে দোয়া ও আত্মপরীক্ষা জরুরি।","মানুষ নিজের সব গোপন দুর্বলতা বুঝতে পারে না, তাই আল্লাহর সাহায্য দরকার।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"31","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E116" s="4" t="n"/>
@@ -3176,12 +3172,12 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সূক্ষ্ম শির্ক থেকে বাঁচার দোয়া","description":"$book_name$ $hadith_number$ - $chapter_name$. শির্ক পিপিলিকার চলার শব্দের চেয়েও সূক্ষ্ম; তাই জানা-অজানা শির্ক থেকে আশ্রয় ও ক্ষমা চাইতে শেখানো হয়েছে।"},"heading":{"title":"গোপন শির্ক থেকে বাঁচার দোয়া ও সতর্কতা","description":"এই হাদিসে শির্কের সূক্ষ্মতা খুব শক্তভাবে বোঝানো হয়েছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, শির্ক পিপিলিকার চলার শব্দ থেকেও গোপন হতে পারে। সাহাবীদের পক্ষ থেকে প্রশ্ন আসে, এত সূক্ষ্ম বিষয় থেকে কীভাবে বাঁচা যাবে? উত্তরে একটি দোয়া শেখানো হয়েছে: হে আল্লাহ, আমরা জেনে তোমার সাথে কোনো কিছুকে শরীক করা থেকে তোমার আশ্রয় চাই এবং যা আমরা জানি না, তার জন্য তোমার কাছে ক্ষমা চাই। এই দোয়া আমাদের শেখায়, মানুষ নিজের অন্তরের সব সূক্ষ্ম রোগ সব সময় বুঝতে পারে না। তাই সতর্কতা, আত্মপরীক্ষা এবং আল্লাহর কাছে আশ্রয়—সবই দরকার। বিশেষ করে রিয়া, আত্মপ্রদর্শন ও প্রশংসার আকাঙ্ক্ষা থেকে বাঁচতে এই হাদিস খুব প্রাসঙ্গিক।"},"teachings":["শির্ক কখনো খুব সূক্ষ্মভাবে অন্তরে ঢুকতে পারে।","জানা ও অজানা ভুলের জন্য আল্লাহর কাছে আশ্রয় ও ক্ষমা চাওয়া দরকার।","রিয়া থেকে বাঁচতে দোয়া ও আত্মপরীক্ষা জরুরি।","মানুষ নিজের সব গোপন দুর্বলতা বুঝতে পারে না, তাই আল্লাহর সাহায্য দরকার।"],"related_hadiths":[{"id":"30","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"31","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"32","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নাত আঁকড়ে ধরা ও বিদআত থেকে সাবধান","description":"$book_name$ $hadith_number$ - $chapter_name$. মতভেদের সময় নবীর সুন্নাত ও খোলাফায়ে রাশেদার পথ আঁকড়ে ধরতে এবং বিদআত থেকে বাঁচতে বলা হয়েছে।"},"heading":{"title":"সুন্নাত আঁকড়ে ধরা: মতভেদের সময় মুমিনের পথ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম এমন এক নসীহত দিয়েছেন, যা শুনে অন্তর ভীত হয়েছে এবং চোখ অশ্রুসিক্ত হয়েছে। তিনি তাকওয়া, নেতার কথা শোনা ও আনুগত্যের উপদেশ দিয়েছেন, যদিও নেতা একজন কৃতদাস হয়। এরপর তিনি জানিয়েছেন, তাঁর পর অনেক মতভেদ দেখা যাবে। সেই সময় করণীয় হলো তাঁর সুন্নাত এবং সুপথপ্রাপ্ত খোলাফায়ে রাশেদার সুন্নাত আঁকড়ে ধরা। হাদিসে মাড়ির দাঁত দিয়ে কামড়ে ধরার উপমা এসেছে, অর্থাৎ দৃঢ়ভাবে ধরে রাখা। একই সঙ্গে দ্বীনের মধ্যে নতুনত্ব থেকে সাবধান করা হয়েছে, কারণ প্রত্যেক বিদআত ভ্রষ্টতা। এই হাদিসের মূল শিক্ষা হলো, দ্বীনের নিরাপদ পথ হলো সুন্নাতের অনুসরণ, ব্যক্তিগত খেয়াল বা নতুন তৈরি পদ্ধতি নয়।"},"teachings":["মতভেদের সময় নবীর সুন্নাত আঁকড়ে ধরা দরকার।","খোলাফায়ে রাশেদার পথ সুপথপ্রাপ্ত পথ হিসেবে উল্লেখ হয়েছে।","তাকওয়া ও বৈধ নেতৃত্বের আনুগত্যের উপদেশ দেওয়া হয়েছে।","দ্বীনের নতুনত্ব বা বিদআত থেকে সতর্ক থাকতে বলা হয়েছে।"],"related_hadiths":[{"id":"4607","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2676","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"42","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E117" s="4" t="n"/>
@@ -3199,12 +3195,12 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নাত আঁকড়ে ধরা ও বিদআত থেকে সাবধান","description":"$book_name$ $hadith_number$ - $chapter_name$. মতভেদের সময় নবীর সুন্নাত ও খোলাফায়ে রাশেদার পথ আঁকড়ে ধরতে এবং বিদআত থেকে বাঁচতে বলা হয়েছে।"},"heading":{"title":"সুন্নাত আঁকড়ে ধরা: মতভেদের সময় মুমিনের পথ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম এমন এক নসীহত দিয়েছেন, যা শুনে অন্তর ভীত হয়েছে এবং চোখ অশ্রুসিক্ত হয়েছে। তিনি তাকওয়া, নেতার কথা শোনা ও আনুগত্যের উপদেশ দিয়েছেন, যদিও নেতা একজন কৃতদাস হয়। এরপর তিনি জানিয়েছেন, তাঁর পর অনেক মতভেদ দেখা যাবে। সেই সময় করণীয় হলো তাঁর সুন্নাত এবং সুপথপ্রাপ্ত খোলাফায়ে রাশেদার সুন্নাত আঁকড়ে ধরা। হাদিসে মাড়ির দাঁত দিয়ে কামড়ে ধরার উপমা এসেছে, অর্থাৎ দৃঢ়ভাবে ধরে রাখা। একই সঙ্গে দ্বীনের মধ্যে নতুনত্ব থেকে সাবধান করা হয়েছে, কারণ প্রত্যেক বিদআত ভ্রষ্টতা। এই হাদিসের মূল শিক্ষা হলো, দ্বীনের নিরাপদ পথ হলো সুন্নাতের অনুসরণ, ব্যক্তিগত খেয়াল বা নতুন তৈরি পদ্ধতি নয়।"},"teachings":["মতভেদের সময় নবীর সুন্নাত আঁকড়ে ধরা দরকার।","খোলাফায়ে রাশেদার পথ সুপথপ্রাপ্ত পথ হিসেবে উল্লেখ হয়েছে।","তাকওয়া ও বৈধ নেতৃত্বের আনুগত্যের উপদেশ দেওয়া হয়েছে।","দ্বীনের নতুনত্ব বা বিদআত থেকে সতর্ক থাকতে বলা হয়েছে।"],"related_hadiths":[{"id":"4607","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2676","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"42","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন আঁকড়ে ধরার সুসংবাদ","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআনকে দৃঢ়ভাবে আঁকড়ে ধরলে বিভ্রান্তি ও ধ্বংস থেকে বাঁচার সুসংবাদ দেওয়া হয়েছে।"},"heading":{"title":"কুরআন আঁকড়ে ধরা: হিদায়াতের নিরাপদ পথ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের সুসংবাদ দিয়েছেন। তিনি তাদের সাক্ষ্য সম্পর্কে জিজ্ঞেস করেছেন—আল্লাহ ছাড়া সত্য কোনো উপাস্য নেই এবং তিনি আল্লাহর রাসূল। তারা তা স্বীকার করলে তিনি কুরআনের মর্যাদা ও দায়িত্বের কথা বলেন। হাদিসে বলা হয়েছে, এই কুরআনের এক দিক আল্লাহর হাতে এবং অন্য দিক তোমাদের হাতে। তাই তোমরা এটিকে আঁকড়ে ধরো। এর ফলে বিভ্রান্তি ও ধ্বংস থেকে বাঁচার কথা বলা হয়েছে। এখানে কুরআনকে শুধু তিলাওয়াতের বই হিসেবে নয়, আঁকড়ে ধরার জীবনপথ হিসেবে দেখা যায়। কুরআন মানা, তার নির্দেশকে গুরুত্ব দেওয়া এবং তার সঙ্গে সম্পর্ক দৃঢ় রাখা—এই হাদিসের মূল বার্তা।"},"teachings":["কুরআন আল্লাহর পক্ষ থেকে হিদায়াতের শক্ত বন্ধন।","কুরআনকে আঁকড়ে ধরা বিভ্রান্তি থেকে বাঁচার কারণ।","ঈমানের সাক্ষ্যের সঙ্গে কুরআনের অনুসরণ জড়িত।","কুরআনের সঙ্গে সম্পর্ক শুধু পড়ায় নয়, মানায়ও প্রকাশ পায়।"],"related_hadiths":[{"id":"39","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"40","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"5027","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E118" s="4" t="n"/>
@@ -3222,12 +3218,12 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন আঁকড়ে ধরার সুসংবাদ","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআনকে দৃঢ়ভাবে আঁকড়ে ধরলে বিভ্রান্তি ও ধ্বংস থেকে বাঁচার সুসংবাদ দেওয়া হয়েছে।"},"heading":{"title":"কুরআন আঁকড়ে ধরা: হিদায়াতের নিরাপদ পথ","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের সুসংবাদ দিয়েছেন। তিনি তাদের সাক্ষ্য সম্পর্কে জিজ্ঞেস করেছেন—আল্লাহ ছাড়া সত্য কোনো উপাস্য নেই এবং তিনি আল্লাহর রাসূল। তারা তা স্বীকার করলে তিনি কুরআনের মর্যাদা ও দায়িত্বের কথা বলেন। হাদিসে বলা হয়েছে, এই কুরআনের এক দিক আল্লাহর হাতে এবং অন্য দিক তোমাদের হাতে। তাই তোমরা এটিকে আঁকড়ে ধরো। এর ফলে বিভ্রান্তি ও ধ্বংস থেকে বাঁচার কথা বলা হয়েছে। এখানে কুরআনকে শুধু তিলাওয়াতের বই হিসেবে নয়, আঁকড়ে ধরার জীবনপথ হিসেবে দেখা যায়। কুরআন মানা, তার নির্দেশকে গুরুত্ব দেওয়া এবং তার সঙ্গে সম্পর্ক দৃঢ় রাখা—এই হাদিসের মূল বার্তা।"},"teachings":["কুরআন আল্লাহর পক্ষ থেকে হিদায়াতের শক্ত বন্ধন।","কুরআনকে আঁকড়ে ধরা বিভ্রান্তি থেকে বাঁচার কারণ।","ঈমানের সাক্ষ্যের সঙ্গে কুরআনের অনুসরণ জড়িত।","কুরআনের সঙ্গে সম্পর্ক শুধু পড়ায় নয়, মানায়ও প্রকাশ পায়।"],"related_hadiths":[{"id":"39","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"40","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"5027","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন আল্লাহর পক্ষ থেকে এসেছে","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন আল্লাহর পক্ষ থেকে এসেছে—এই সাক্ষ্যের পর তাকে আঁকড়ে ধরলে বিভ্রান্তি থেকে বাঁচার সুসংবাদ আছে।"},"heading":{"title":"কুরআন আঁকড়ে ধরা: ধ্বংস ও বিভ্রান্তি থেকে বাঁচার উপায়","description":"এই হাদিসে জুহফা নামক স্থানে নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের কয়েকটি সাক্ষ্যের কথা জিজ্ঞেস করেন। তারা সাক্ষ্য দেন যে আল্লাহ ছাড়া সত্য কোনো উপাস্য নেই, তিনি একক, তাঁর কোনো শরীক নেই, নবী আল্লাহর রাসূল এবং কুরআন আল্লাহর নিকট থেকে এসেছে। এরপর তিনি বলেন, সুসংবাদ গ্রহণ করো; এই কুরআনের একাংশ আল্লাহর হাতে এবং আরেকাংশ তোমাদের হাতে। তাই তোমরা এটিকে আঁকড়ে ধরো। হাদিসে বলা হয়েছে, কুরআন আঁকড়ে ধরার পর তারা ধ্বংস ও বিভ্রান্তি থেকে বাঁচবে। এই বার্তায় কুরআনের সঙ্গে দৃঢ় সম্পর্কের কথা আছে। কুরআনকে মানা, তার নির্দেশে চলা এবং বিশ্বাসের সঙ্গে জীবন সাজানো—এটাই এই হাদিসের সহজ শিক্ষা।"},"teachings":["কুরআন আল্লাহর পক্ষ থেকে এসেছে—এটি ঈমানের গুরুত্বপূর্ণ সাক্ষ্য।","কুরআন আঁকড়ে ধরার মধ্যে হিদায়াতের পথ রয়েছে।","তাওহীদ, রিসালাত ও কুরআনের প্রতি বিশ্বাস একসঙ্গে উল্লেখ হয়েছে।","কুরআনের সঙ্গে দৃঢ় সম্পর্ক বিভ্রান্তি থেকে বাঁচার কারণ।"],"related_hadiths":[{"id":"38","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"40","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"37","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E119" s="4" t="n"/>
@@ -3245,15 +3241,19 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন আল্লাহর পক্ষ থেকে এসেছে","description":"$book_name$ $hadith_number$ - $chapter_name$. কুরআন আল্লাহর পক্ষ থেকে এসেছে—এই সাক্ষ্যের পর তাকে আঁকড়ে ধরলে বিভ্রান্তি থেকে বাঁচার সুসংবাদ আছে।"},"heading":{"title":"কুরআন আঁকড়ে ধরা: ধ্বংস ও বিভ্রান্তি থেকে বাঁচার উপায়","description":"এই হাদিসে জুহফা নামক স্থানে নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সাহাবীদের কয়েকটি সাক্ষ্যের কথা জিজ্ঞেস করেন। তারা সাক্ষ্য দেন যে আল্লাহ ছাড়া সত্য কোনো উপাস্য নেই, তিনি একক, তাঁর কোনো শরীক নেই, নবী আল্লাহর রাসূল এবং কুরআন আল্লাহর নিকট থেকে এসেছে। এরপর তিনি বলেন, সুসংবাদ গ্রহণ করো; এই কুরআনের একাংশ আল্লাহর হাতে এবং আরেকাংশ তোমাদের হাতে। তাই তোমরা এটিকে আঁকড়ে ধরো। হাদিসে বলা হয়েছে, কুরআন আঁকড়ে ধরার পর তারা ধ্বংস ও বিভ্রান্তি থেকে বাঁচবে। এই বার্তায় কুরআনের সঙ্গে দৃঢ় সম্পর্কের কথা আছে। কুরআনকে মানা, তার নির্দেশে চলা এবং বিশ্বাসের সঙ্গে জীবন সাজানো—এটাই এই হাদিসের সহজ শিক্ষা।"},"teachings":["কুরআন আল্লাহর পক্ষ থেকে এসেছে—এটি ঈমানের গুরুত্বপূর্ণ সাক্ষ্য।","কুরআন আঁকড়ে ধরার মধ্যে হিদায়াতের পথ রয়েছে।","তাওহীদ, রিসালাত ও কুরআনের প্রতি বিশ্বাস একসঙ্গে উল্লেখ হয়েছে।","কুরআনের সঙ্গে দৃঢ় সম্পর্ক বিভ্রান্তি থেকে বাঁচার কারণ।"],"related_hadiths":[{"id":"38","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"40","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"37","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
-        </is>
-      </c>
-      <c r="E120" s="4" t="n"/>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইখলাস, নসীহত ও জামাতের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদায় হজ্জের এই বাণীতে ইখলাস, মুসলিম নেতাদের নসীহত ও জামাত আঁকড়ে ধরার শিক্ষা এসেছে।"},"heading":{"title":"ইখলাস ও মুসলিম জামাত: বিদায় হজ্জের গুরুত্বপূর্ণ শিক্ষা","description":"এই হাদিসে নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের একটি গুরুত্বপূর্ণ বক্তব্য এসেছে। তিনি এমন ব্যক্তির জন্য আল্লাহর পক্ষ থেকে উজ্জ্বল মুখমণ্ডল বা সম্মানের দোয়া করেছেন, যে তাঁর কথা শুনে তা মনে রাখে। এরপর বলা হয়েছে, অনেকেই জ্ঞান বহন করে, কিন্তু সে নিজে গভীরভাবে বোঝে না। তারপর তিনটি বিষয় উল্লেখ করা হয়েছে, যেগুলোর উপর মুমিনের অন্তরে হিংসা বা খারাপ মনোভাব জমে না। প্রথমটি হলো আল্লাহর জন্য আমলকে একনিষ্ঠ করা। দ্বিতীয়টি মুসলমানদের নেতৃবৃন্দকে নসীহত করা। তৃতীয়টি মুসলমানদের জামাতকে আঁকড়ে ধরা। এই হাদিসে ইখলাস শুধু ব্যক্তিগত আমলের বিষয় নয়; মুসলিম সমাজের মঙ্গল, সঠিক উপদেশ এবং ঐক্যের সাথেও তা যুক্ত হয়েছে। তাই হাদিস শ্রবণ, মনে রাখা এবং সঠিকভাবে পৌঁছে দেওয়াও গুরুত্বপূর্ণ দায়িত্ব।"},"teachings":["নবীর কথা শুনে মনে রাখা ও পৌঁছে দেওয়া মূল্যবান কাজ।","আল্লাহর জন্য আমল একনিষ্ঠ করা মুমিনের অন্তরের বড় গুণ।","মুসলিম নেতৃবৃন্দকে সৎ নসীহত করা কল্যাণের অংশ।","মুসলিম জামাতের সাথে থাকা ঐক্যের শিক্ষা দেয়।"],"related_hadiths":[{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ২৩২ (প্রাসঙ্গিক বর্ণনা)"</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="46" customHeight="1">
       <c r="A121" s="4" t="inlineStr">
@@ -3268,19 +3268,15 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইখলাস, নসীহত ও জামাতের গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদায় হজ্জের এই বাণীতে ইখলাস, মুসলিম নেতাদের নসীহত ও জামাত আঁকড়ে ধরার শিক্ষা এসেছে।"},"heading":{"title":"ইখলাস ও মুসলিম জামাত: বিদায় হজ্জের গুরুত্বপূর্ণ শিক্ষা","description":"এই হাদিসে নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের একটি গুরুত্বপূর্ণ বক্তব্য এসেছে। তিনি এমন ব্যক্তির জন্য আল্লাহর পক্ষ থেকে উজ্জ্বল মুখমণ্ডল বা সম্মানের দোয়া করেছেন, যে তাঁর কথা শুনে তা মনে রাখে। এরপর বলা হয়েছে, অনেকেই জ্ঞান বহন করে, কিন্তু সে নিজে গভীরভাবে বোঝে না। তারপর তিনটি বিষয় উল্লেখ করা হয়েছে, যেগুলোর উপর মুমিনের অন্তরে হিংসা বা খারাপ মনোভাব জমে না। প্রথমটি হলো আল্লাহর জন্য আমলকে একনিষ্ঠ করা। দ্বিতীয়টি মুসলমানদের নেতৃবৃন্দকে নসীহত করা। তৃতীয়টি মুসলমানদের জামাতকে আঁকড়ে ধরা। এই হাদিসে ইখলাস শুধু ব্যক্তিগত আমলের বিষয় নয়; মুসলিম সমাজের মঙ্গল, সঠিক উপদেশ এবং ঐক্যের সাথেও তা যুক্ত হয়েছে। তাই হাদিস শ্রবণ, মনে রাখা এবং সঠিকভাবে পৌঁছে দেওয়াও গুরুত্বপূর্ণ দায়িত্ব।"},"teachings":["নবীর কথা শুনে মনে রাখা ও পৌঁছে দেওয়া মূল্যবান কাজ।","আল্লাহর জন্য আমল একনিষ্ঠ করা মুমিনের অন্তরের বড় গুণ।","মুসলিম নেতৃবৃন্দকে সৎ নসীহত করা কল্যাণের অংশ।","মুসলিম জামাতের সাথে থাকা ঐক্যের শিক্ষা দেয়।"],"related_hadiths":[{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
-        </is>
-      </c>
-      <c r="E121" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ২৩২ (প্রাসঙ্গিক বর্ণনা)"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর কিতাব ও নবীর সুন্নাত আঁকড়ে ধরা","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদায় হজ্জের খুতবায় আল্লাহর কিতাব ও নবীর সুন্নাত আঁকড়ে ধরলে পথভ্রষ্ট না হওয়ার শিক্ষা দেওয়া হয়েছে।"},"heading":{"title":"আল্লাহর কিতাব ও নবীর সুন্নাত: পথভ্রষ্টতা থেকে বাঁচার পথ","description":"এই হাদিসে বিদায় হজ্জের খুতবার একটি গুরুত্বপূর্ণ অংশ এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, শয়তান এই জমিনে সরাসরি ইবাদত পাওয়ার ব্যাপারে নিরাশ হয়ে গেছে। কিন্তু সে ছোটখাট তুচ্ছ মনে হওয়া কাজে আনুগত্য পেতে সন্তুষ্ট। তাই সতর্ক থাকতে বলা হয়েছে। এরপর তিনি বলেন, তিনি মানুষের মাঝে এমন বস্তু রেখে যাচ্ছেন, যা আঁকড়ে ধরলে তারা পথভ্রষ্ট হবে না—আল্লাহর কিতাব এবং তাঁর নবীর সুন্নাত। এই হাদিস আমাদের দুইটি বড় শিক্ষা দেয়। একদিকে ছোট মনে হওয়া পাপ ও শয়তানের পথ থেকে সাবধান থাকা দরকার। অন্যদিকে কুরআন ও সুন্নাহকে জীবনের মাপকাঠি বানানো দরকার। মত, অভ্যাস বা সমাজের চাপ নয়; নিরাপদ পথ হলো আল্লাহর কিতাব ও রাসূলের সুন্নাত।"},"teachings":["শয়তান ছোট মনে হওয়া কাজের মাধ্যমেও মানুষকে ভুল পথে নিতে পারে।","কুরআন ও সুন্নাহ আঁকড়ে ধরা পথভ্রষ্টতা থেকে বাঁচার কারণ।","ছোট পাপ বা তুচ্ছ মনে হওয়া ভুলকে হালকা করে দেখা উচিত নয়।","দ্বীনের নিরাপদ মাপকাঠি হলো আল্লাহর কিতাব ও নবীর সুন্নাত।"],"related_hadiths":[{"id":"37","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"38","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"39","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="n"/>
     </row>
     <row r="122" ht="46" customHeight="1">
       <c r="A122" s="4" t="inlineStr">
@@ -3295,12 +3291,12 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর কিতাব ও নবীর সুন্নাত আঁকড়ে ধরা","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদায় হজ্জের খুতবায় আল্লাহর কিতাব ও নবীর সুন্নাত আঁকড়ে ধরলে পথভ্রষ্ট না হওয়ার শিক্ষা দেওয়া হয়েছে।"},"heading":{"title":"আল্লাহর কিতাব ও নবীর সুন্নাত: পথভ্রষ্টতা থেকে বাঁচার পথ","description":"এই হাদিসে বিদায় হজ্জের খুতবার একটি গুরুত্বপূর্ণ অংশ এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, শয়তান এই জমিনে সরাসরি ইবাদত পাওয়ার ব্যাপারে নিরাশ হয়ে গেছে। কিন্তু সে ছোটখাট তুচ্ছ মনে হওয়া কাজে আনুগত্য পেতে সন্তুষ্ট। তাই সতর্ক থাকতে বলা হয়েছে। এরপর তিনি বলেন, তিনি মানুষের মাঝে এমন বস্তু রেখে যাচ্ছেন, যা আঁকড়ে ধরলে তারা পথভ্রষ্ট হবে না—আল্লাহর কিতাব এবং তাঁর নবীর সুন্নাত। এই হাদিস আমাদের দুইটি বড় শিক্ষা দেয়। একদিকে ছোট মনে হওয়া পাপ ও শয়তানের পথ থেকে সাবধান থাকা দরকার। অন্যদিকে কুরআন ও সুন্নাহকে জীবনের মাপকাঠি বানানো দরকার। মত, অভ্যাস বা সমাজের চাপ নয়; নিরাপদ পথ হলো আল্লাহর কিতাব ও রাসূলের সুন্নাত।"},"teachings":["শয়তান ছোট মনে হওয়া কাজের মাধ্যমেও মানুষকে ভুল পথে নিতে পারে।","কুরআন ও সুন্নাহ আঁকড়ে ধরা পথভ্রষ্টতা থেকে বাঁচার কারণ।","ছোট পাপ বা তুচ্ছ মনে হওয়া ভুলকে হালকা করে দেখা উচিত নয়।","দ্বীনের নিরাপদ মাপকাঠি হলো আল্লাহর কিতাব ও নবীর সুন্নাত।"],"related_hadiths":[{"id":"37","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"38","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"39","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নাত আঁকড়ে ধরা বিদআতের চেয়ে উত্তম","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্নাতকে যথেষ্ট মনে করা বিদআতে বেশি চেষ্টা করার চেয়ে উত্তম—এই হাদিসে দ্বীনে সঠিক পথ ধরার শিক্ষা রয়েছে।"},"heading":{"title":"সুন্নাত অনুসরণ কেন বিদআতের চেয়ে উত্তম","description":"এই হাদিসের মূল কথা হলো, দ্বীনের কাজে সুন্নাতকে যথেষ্ট মনে করা নিরাপদ ও উত্তম পথ। এখানে ইবনে মাসউদ (রাঃ) বলেছেন, বিদআতের মধ্যে বেশি গবেষণা বা বেশি চেষ্টা করার চেয়ে সুন্নাতের উপর সীমিত থাকা ভালো। সহজ ভাষায়, ইবাদত বা দ্বীনি কাজে নতুন নতুন পথ খোঁজার বদলে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম থেকে প্রমাণিত পথে থাকা উচিত। এই হাদিস সুন্নাত অনুসরণ, বিদআত থেকে বাঁচা এবং দ্বীনের কাজে ভারসাম্য রাখার শিক্ষা দেয়। তাই “সুন্নাত বনাম বিদআত” বিষয়ে যারা খোঁজ করেন, তাদের জন্য এই বর্ণনা খুব গুরুত্বপূর্ণ। এখানে কোনো অতিরিক্ত কথা নেই; মূল শিক্ষা হলো, সুন্নাত যথেষ্ট, বিদআতের চেষ্টা নয়।"},"teachings":["দ্বীনি কাজে সুন্নাতকে যথেষ্ট মনে করা নিরাপদ পথ।","বিদআতের মধ্যে বেশি চেষ্টা করাকে এই বর্ণনায় প্রশংসা করা হয়নি।","সাহাবিদের বুঝ অনুযায়ী সুন্নাত আঁকড়ে ধরা বড় শিক্ষা।","ইবাদতে নতুন পথের চেয়ে প্রমাণিত পথকে গুরুত্ব দিতে হবে।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E122" s="4" t="n"/>
@@ -3318,12 +3314,12 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সুন্নাত আঁকড়ে ধরা বিদআতের চেয়ে উত্তম","description":"$book_name$ $hadith_number$ - $chapter_name$. সুন্নাতকে যথেষ্ট মনে করা বিদআতে বেশি চেষ্টা করার চেয়ে উত্তম—এই হাদিসে দ্বীনে সঠিক পথ ধরার শিক্ষা রয়েছে।"},"heading":{"title":"সুন্নাত অনুসরণ কেন বিদআতের চেয়ে উত্তম","description":"এই হাদিসের মূল কথা হলো, দ্বীনের কাজে সুন্নাতকে যথেষ্ট মনে করা নিরাপদ ও উত্তম পথ। এখানে ইবনে মাসউদ (রাঃ) বলেছেন, বিদআতের মধ্যে বেশি গবেষণা বা বেশি চেষ্টা করার চেয়ে সুন্নাতের উপর সীমিত থাকা ভালো। সহজ ভাষায়, ইবাদত বা দ্বীনি কাজে নতুন নতুন পথ খোঁজার বদলে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম থেকে প্রমাণিত পথে থাকা উচিত। এই হাদিস সুন্নাত অনুসরণ, বিদআত থেকে বাঁচা এবং দ্বীনের কাজে ভারসাম্য রাখার শিক্ষা দেয়। তাই “সুন্নাত বনাম বিদআত” বিষয়ে যারা খোঁজ করেন, তাদের জন্য এই বর্ণনা খুব গুরুত্বপূর্ণ। এখানে কোনো অতিরিক্ত কথা নেই; মূল শিক্ষা হলো, সুন্নাত যথেষ্ট, বিদআতের চেষ্টা নয়।"},"teachings":["দ্বীনি কাজে সুন্নাতকে যথেষ্ট মনে করা নিরাপদ পথ।","বিদআতের মধ্যে বেশি চেষ্টা করাকে এই বর্ণনায় প্রশংসা করা হয়নি।","সাহাবিদের বুঝ অনুযায়ী সুন্নাত আঁকড়ে ধরা বড় শিক্ষা।","ইবাদতে নতুন পথের চেয়ে প্রমাণিত পথকে গুরুত্ব দিতে হবে।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর কিতাব আঁকড়ে ধরার নির্দেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের আনুগত্য, আল্লাহর কিতাব আঁকড়ে ধরা এবং হালাল-হারাম মানার সরল শিক্ষা এই হাদিসে এসেছে।"},"heading":{"title":"আল্লাহর কিতাব আঁকড়ে ধরা ও রাসূলের আনুগত্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর সাহাবিদের সামনে গুরুত্বপূর্ণ নির্দেশ দিয়েছেন। তিনি বলেন, তিনি যতক্ষণ তাদের মাঝে আছেন, তারা যেন তাঁর আনুগত্য করে। এরপর তিনি আল্লাহর কিতাব আঁকড়ে ধরার কথা বলেন। কুরআনে যে বিষয় হালাল বলা হয়েছে, সেটাকে হালাল মানতে হবে; আর যে বিষয় হারাম বলা হয়েছে, সেটাকে হারাম মানতে হবে। এই হাদিসের মূল বিষয় হলো কুরআন অনুসরণ, রাসূলের আনুগত্য এবং হালাল-হারাম বিষয়ে স্পষ্ট অবস্থান। এখানে কোনো বাড়তি ব্যাখ্যার দরকার নেই। বর্ণনাটি আমাদের শেখায়, দ্বীনের ক্ষেত্রে নিজের পছন্দ নয়, আল্লাহর কিতাব ও রাসূলের নির্দেশই মূল পথ।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর আনুগত্য ঈমানি দায়িত্ব।","আল্লাহর কিতাবকে দৃঢ়ভাবে আঁকড়ে ধরতে হবে।","হালালকে হালাল এবং হারামকে হারাম মানা জরুরি।","দ্বীনি বিষয়ে নিজের মতের আগে কুরআনের নির্দেশকে মানতে হবে।"],"related_hadiths":[{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
         </is>
       </c>
       <c r="E123" s="4" t="n"/>
@@ -3341,12 +3337,12 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর কিতাব আঁকড়ে ধরার নির্দেশ","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের আনুগত্য, আল্লাহর কিতাব আঁকড়ে ধরা এবং হালাল-হারাম মানার সরল শিক্ষা এই হাদিসে এসেছে।"},"heading":{"title":"আল্লাহর কিতাব আঁকড়ে ধরা ও রাসূলের আনুগত্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর সাহাবিদের সামনে গুরুত্বপূর্ণ নির্দেশ দিয়েছেন। তিনি বলেন, তিনি যতক্ষণ তাদের মাঝে আছেন, তারা যেন তাঁর আনুগত্য করে। এরপর তিনি আল্লাহর কিতাব আঁকড়ে ধরার কথা বলেন। কুরআনে যে বিষয় হালাল বলা হয়েছে, সেটাকে হালাল মানতে হবে; আর যে বিষয় হারাম বলা হয়েছে, সেটাকে হারাম মানতে হবে। এই হাদিসের মূল বিষয় হলো কুরআন অনুসরণ, রাসূলের আনুগত্য এবং হালাল-হারাম বিষয়ে স্পষ্ট অবস্থান। এখানে কোনো বাড়তি ব্যাখ্যার দরকার নেই। বর্ণনাটি আমাদের শেখায়, দ্বীনের ক্ষেত্রে নিজের পছন্দ নয়, আল্লাহর কিতাব ও রাসূলের নির্দেশই মূল পথ।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর আনুগত্য ঈমানি দায়িত্ব।","আল্লাহর কিতাবকে দৃঢ়ভাবে আঁকড়ে ধরতে হবে।","হালালকে হালাল এবং হারামকে হারাম মানা জরুরি।","দ্বীনি বিষয়ে নিজের মতের আগে কুরআনের নির্দেশকে মানতে হবে।"],"related_hadiths":[{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাজরে আসওয়াদ ও সুন্নাহ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. উমর (রাঃ) হাজরে আসওয়াদ চুম্বন করেন শুধু রাসূলকে তা করতে দেখেছিলেন বলে—এতে সুন্নাহ অনুসরণের শিক্ষা আছে।"},"heading":{"title":"হাজরে আসওয়াদ চুম্বন: সুন্নাহ অনুসরণের সরল শিক্ষা","description":"এই হাদিসে উমর বিন খাত্তাব (রাঃ)-এর একটি খুব স্পষ্ট কথা এসেছে। তিনি হাজরে আসওয়াদকে চুম্বন করছিলেন, কিন্তু একই সাথে বলেছিলেন, তিনি জানেন এটি একটি পাথর; এটি নিজে কোনো উপকার বা অপকার করতে পারে না। তিনি এটি চুম্বন করেছেন শুধু এ কারণে যে তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে তা করতে দেখেছেন। এই বর্ণনার মূল বিষয় হলো সুন্নাহ অনুসরণ এবং তাওহীদের পরিষ্কার ধারণা। হাজরে আসওয়াদকে সম্মান করা হয়, কিন্তু উপকার-অপকারের ক্ষমতা পাথরের নয়—এ কথা উমর (রাঃ) নিজেই বলেছেন। তাই এই হাদিস হাজরে আসওয়াদ, তাওয়াফ এবং সুন্নাহ মানার বিষয়ে গুরুত্বপূর্ণ শিক্ষা দেয়।"},"teachings":["সুন্নাহ অনুসরণ করা সাহাবিদের বড় বৈশিষ্ট্য ছিল।","হাজরে আসওয়াদ নিজে উপকার বা অপকার করতে পারে না।","ইবাদতের কাজ রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর অনুসরণে করতে হয়।","সম্মান ও বিশ্বাসের সীমা আলাদা করে বুঝতে হবে।"],"related_hadiths":[{"id":"1597","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
         </is>
       </c>
       <c r="E124" s="4" t="n"/>
@@ -3364,12 +3360,12 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাজরে আসওয়াদ ও সুন্নাহ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. উমর (রাঃ) হাজরে আসওয়াদ চুম্বন করেন শুধু রাসূলকে তা করতে দেখেছিলেন বলে—এতে সুন্নাহ অনুসরণের শিক্ষা আছে।"},"heading":{"title":"হাজরে আসওয়াদ চুম্বন: সুন্নাহ অনুসরণের সরল শিক্ষা","description":"এই হাদিসে উমর বিন খাত্তাব (রাঃ)-এর একটি খুব স্পষ্ট কথা এসেছে। তিনি হাজরে আসওয়াদকে চুম্বন করছিলেন, কিন্তু একই সাথে বলেছিলেন, তিনি জানেন এটি একটি পাথর; এটি নিজে কোনো উপকার বা অপকার করতে পারে না। তিনি এটি চুম্বন করেছেন শুধু এ কারণে যে তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে তা করতে দেখেছেন। এই বর্ণনার মূল বিষয় হলো সুন্নাহ অনুসরণ এবং তাওহীদের পরিষ্কার ধারণা। হাজরে আসওয়াদকে সম্মান করা হয়, কিন্তু উপকার-অপকারের ক্ষমতা পাথরের নয়—এ কথা উমর (রাঃ) নিজেই বলেছেন। তাই এই হাদিস হাজরে আসওয়াদ, তাওয়াফ এবং সুন্নাহ মানার বিষয়ে গুরুত্বপূর্ণ শিক্ষা দেয়।"},"teachings":["সুন্নাহ অনুসরণ করা সাহাবিদের বড় বৈশিষ্ট্য ছিল।","হাজরে আসওয়াদ নিজে উপকার বা অপকার করতে পারে না।","ইবাদতের কাজ রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর অনুসরণে করতে হয়।","সম্মান ও বিশ্বাসের সীমা আলাদা করে বুঝতে হবে।"],"related_hadiths":[{"id":"1597","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বায়আত ও মোহরে নবুওয়াত স্পর্শ","description":"$book_name$ $hadith_number$ - $chapter_name$. কুররা (রাঃ) বায়আতের সময় নবীর মোহরে নবুওয়াত স্পর্শ করেন; পরে পোশাকের একটি অভ্যাসেও অনুসরণ দেখা যায়।"},"heading":{"title":"মোহরে নবুওয়াত স্পর্শ ও সাহাবিদের অনুসরণের দৃষ্টান্ত","description":"এই হাদিসে কুররা (রাঃ)-এর ঘটনা এসেছে। তিনি মুযায়না গোত্রের একটি দলের সাথে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে আসেন এবং তাঁর হাতে বায়আত করেন। সে সময় রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর জামার গলাবন্দ খোলা ছিল। কুররা (রাঃ) হাত ঢুকিয়ে তাঁর পৃষ্ঠদেশে থাকা মোহরে নবুওয়াত স্পর্শ করেন। এরপর বর্ণনাকারী বলেন, মুআবিয়া বা তাঁর পুত্রকে শীত বা গ্রীষ্মে জামার গলাবন্দ খোলা ছাড়া দেখা যেত না। এই হাদিসে বায়আত, নবুওয়াতের নিদর্শন এবং সাহাবিদের অনুসরণের একটি ছবি দেখা যায়। তবে এখানে কোনো সাধারণ বিধান বানানো হয়নি; শুধু বর্ণিত ঘটনা ও আচরণকে তুলে ধরা হয়েছে।"},"teachings":["সাহাবিরা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে এসে বায়আত করতেন।","মোহরে নবুওয়াত তাঁর বিশেষ নিদর্শনের একটি হিসেবে বর্ণিত হয়েছে।","কিছু সাহাবি রাসূলের দেখা অভ্যাসকে ভালোবাসা থেকে অনুসরণ করতেন।","ঘটনা থেকে বাড়তি বিধান বানানোর আগে বর্ণনার সীমা মনে রাখা দরকার।"],"related_hadiths":[{"id":"190","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5670","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5981","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E125" s="4" t="n"/>
@@ -3387,12 +3383,12 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বায়আত ও মোহরে নবুওয়াত স্পর্শ","description":"$book_name$ $hadith_number$ - $chapter_name$. কুররা (রাঃ) বায়আতের সময় নবীর মোহরে নবুওয়াত স্পর্শ করেন; পরে পোশাকের একটি অভ্যাসেও অনুসরণ দেখা যায়।"},"heading":{"title":"মোহরে নবুওয়াত স্পর্শ ও সাহাবিদের অনুসরণের দৃষ্টান্ত","description":"এই হাদিসে কুররা (রাঃ)-এর ঘটনা এসেছে। তিনি মুযায়না গোত্রের একটি দলের সাথে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে আসেন এবং তাঁর হাতে বায়আত করেন। সে সময় রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর জামার গলাবন্দ খোলা ছিল। কুররা (রাঃ) হাত ঢুকিয়ে তাঁর পৃষ্ঠদেশে থাকা মোহরে নবুওয়াত স্পর্শ করেন। এরপর বর্ণনাকারী বলেন, মুআবিয়া বা তাঁর পুত্রকে শীত বা গ্রীষ্মে জামার গলাবন্দ খোলা ছাড়া দেখা যেত না। এই হাদিসে বায়আত, নবুওয়াতের নিদর্শন এবং সাহাবিদের অনুসরণের একটি ছবি দেখা যায়। তবে এখানে কোনো সাধারণ বিধান বানানো হয়নি; শুধু বর্ণিত ঘটনা ও আচরণকে তুলে ধরা হয়েছে।"},"teachings":["সাহাবিরা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে এসে বায়আত করতেন।","মোহরে নবুওয়াত তাঁর বিশেষ নিদর্শনের একটি হিসেবে বর্ণিত হয়েছে।","কিছু সাহাবি রাসূলের দেখা অভ্যাসকে ভালোবাসা থেকে অনুসরণ করতেন।","ঘটনা থেকে বাড়তি বিধান বানানোর আগে বর্ণনার সীমা মনে রাখা দরকার।"],"related_hadiths":[{"id":"190","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5670","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5981","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে নবীর কাজ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে উমর (রাঃ) সফরে রাসূলকে যে পথে যেতে দেখেছিলেন, সেই কাজ অনুসরণ করতেন—এতে সুন্নাহর ভালোবাসা ফুটে ওঠে।"},"heading":{"title":"সফরে সুন্নাহ অনুসরণে ইবনে উমর (রাঃ)-এর দৃষ্টান্ত","description":"এই হাদিসে ইবনে উমর (রাঃ)-এর সুন্নাহ অনুসরণের একটি বাস্তব ঘটনা এসেছে। সফরে তিনি একটি জায়গা দিয়ে যাওয়ার সময় একটু সরে ডান বা বাম দিক দিয়ে গেলেন। তাঁকে কারণ জিজ্ঞেস করা হলে তিনি বলেন, তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে এমন করতে দেখেছেন, তাই তিনিও তা করেছেন। এই বর্ণনার মূল শিক্ষা হলো, সাহাবিরা রাসূলের কাজকে কত মনোযোগ দিয়ে দেখতেন এবং ভালোবাসা নিয়ে অনুসরণ করতেন। এখানে কোনো বড় আলোচনা নেই; একটি ছোট কাজের মধ্যেও সুন্নাহর প্রতি ভালোবাসা প্রকাশ পেয়েছে। তাই “সুন্নাহ অনুসরণ” এবং “সাহাবিদের আমল” বিষয়ে এই হাদিস খুব সুন্দর উদাহরণ।"},"teachings":["সাহাবিরা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাজ মনোযোগ দিয়ে দেখতেন।","ছোট কাজেও সুন্নাহ অনুসরণের ভালোবাসা প্রকাশ পেতে পারে।","ইবনে উমর (রাঃ) নবীর দেখা কাজকে অনুসরণ করেছেন।","সুন্নাহর প্রতি শ্রদ্ধা শুধু কথায় নয়, কাজে দেখা যায়।"],"related_hadiths":[{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E126" s="4" t="n"/>
@@ -3410,12 +3406,12 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সফরে নবীর কাজ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে উমর (রাঃ) সফরে রাসূলকে যে পথে যেতে দেখেছিলেন, সেই কাজ অনুসরণ করতেন—এতে সুন্নাহর ভালোবাসা ফুটে ওঠে।"},"heading":{"title":"সফরে সুন্নাহ অনুসরণে ইবনে উমর (রাঃ)-এর দৃষ্টান্ত","description":"এই হাদিসে ইবনে উমর (রাঃ)-এর সুন্নাহ অনুসরণের একটি বাস্তব ঘটনা এসেছে। সফরে তিনি একটি জায়গা দিয়ে যাওয়ার সময় একটু সরে ডান বা বাম দিক দিয়ে গেলেন। তাঁকে কারণ জিজ্ঞেস করা হলে তিনি বলেন, তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামকে এমন করতে দেখেছেন, তাই তিনিও তা করেছেন। এই বর্ণনার মূল শিক্ষা হলো, সাহাবিরা রাসূলের কাজকে কত মনোযোগ দিয়ে দেখতেন এবং ভালোবাসা নিয়ে অনুসরণ করতেন। এখানে কোনো বড় আলোচনা নেই; একটি ছোট কাজের মধ্যেও সুন্নাহর প্রতি ভালোবাসা প্রকাশ পেয়েছে। তাই “সুন্নাহ অনুসরণ” এবং “সাহাবিদের আমল” বিষয়ে এই হাদিস খুব সুন্দর উদাহরণ।"},"teachings":["সাহাবিরা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাজ মনোযোগ দিয়ে দেখতেন।","ছোট কাজেও সুন্নাহ অনুসরণের ভালোবাসা প্রকাশ পেতে পারে।","ইবনে উমর (রাঃ) নবীর দেখা কাজকে অনুসরণ করেছেন।","সুন্নাহর প্রতি শ্রদ্ধা শুধু কথায় নয়, কাজে দেখা যায়।"],"related_hadiths":[{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গাছের নিচে বিশ্রাম ও সুন্নাহ ভালোবাসা","description":"$book_name$ $hadith_number$ - $chapter_name$. মক্কা-মদীনার মাঝের একটি গাছের নিচে ইবনে উমর (রাঃ) বিশ্রাম নিতেন, কারণ রাসূলও সেখানে বিশ্রাম করতেন।"},"heading":{"title":"গাছের নিচে বিশ্রাম: সুন্নাহ ভালোবাসার সরল উদাহরণ","description":"এই হাদিসে ইবনে উমর (রাঃ)-এর আরেকটি অনুসরণের ঘটনা এসেছে। মক্কা ও মদীনার মাঝে একটি গাছের কাছে এলে তিনি তার নিচে শুয়ে বিশ্রাম করতেন। তিনি বলতেন, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামও এমন করতেন। এই বর্ণনায় কোনো জটিল বিধান নেই। এখানে দেখা যায়, সাহাবিরা রাসূলের কাজকে শুধু বড় ইবাদতের মধ্যে সীমাবদ্ধ রাখেননি; তাঁরা তাঁর দেখা অভ্যাসও ভালোবাসা নিয়ে মনে রাখতেন। “সুন্নাহ অনুসরণ” বলতে শুধু মুখে বলা নয়, বরং নবীর পথকে সম্মান করার মনও বুঝায়। তবে এই হাদিস থেকে সবার জন্য আলাদা বাধ্যতামূলক আমল বানানো ঠিক নয়; এটি একটি বর্ণিত ঘটনা।"},"teachings":["ইবনে উমর (রাঃ) রাসূলের কাজকে ভালোবাসা দিয়ে অনুসরণ করতেন।","সাহাবিরা নবীর ছোট ছোট কাজও মনে রাখতেন।","সুন্নাহর প্রতি ভালোবাসা আচরণে প্রকাশ পেতে পারে।","বর্ণিত ঘটনা থেকে অতিরিক্ত বাধ্যতামূলক বিধান বানানো উচিত নয়।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E127" s="4" t="n"/>
@@ -3433,12 +3429,12 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | গাছের নিচে বিশ্রাম ও সুন্নাহ ভালোবাসা","description":"$book_name$ $hadith_number$ - $chapter_name$. মক্কা-মদীনার মাঝের একটি গাছের নিচে ইবনে উমর (রাঃ) বিশ্রাম নিতেন, কারণ রাসূলও সেখানে বিশ্রাম করতেন।"},"heading":{"title":"গাছের নিচে বিশ্রাম: সুন্নাহ ভালোবাসার সরল উদাহরণ","description":"এই হাদিসে ইবনে উমর (রাঃ)-এর আরেকটি অনুসরণের ঘটনা এসেছে। মক্কা ও মদীনার মাঝে একটি গাছের কাছে এলে তিনি তার নিচে শুয়ে বিশ্রাম করতেন। তিনি বলতেন, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লামও এমন করতেন। এই বর্ণনায় কোনো জটিল বিধান নেই। এখানে দেখা যায়, সাহাবিরা রাসূলের কাজকে শুধু বড় ইবাদতের মধ্যে সীমাবদ্ধ রাখেননি; তাঁরা তাঁর দেখা অভ্যাসও ভালোবাসা নিয়ে মনে রাখতেন। “সুন্নাহ অনুসরণ” বলতে শুধু মুখে বলা নয়, বরং নবীর পথকে সম্মান করার মনও বুঝায়। তবে এই হাদিস থেকে সবার জন্য আলাদা বাধ্যতামূলক আমল বানানো ঠিক নয়; এটি একটি বর্ণিত ঘটনা।"},"teachings":["ইবনে উমর (রাঃ) রাসূলের কাজকে ভালোবাসা দিয়ে অনুসরণ করতেন।","সাহাবিরা নবীর ছোট ছোট কাজও মনে রাখতেন।","সুন্নাহর প্রতি ভালোবাসা আচরণে প্রকাশ পেতে পারে।","বর্ণিত ঘটনা থেকে অতিরিক্ত বাধ্যতামূলক বিধান বানানো উচিত নয়।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আরাফাতে সুন্নাহ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. আরাফাত থেকে মুযদালিফার পথে ইবনে উমর (রাঃ) নবীর স্মৃতিতে একটি কাজ করতে পছন্দ করেন—এতে অনুসরণের শিক্ষা আছে।"},"heading":{"title":"আরাফাতের সফরে ইবনে উমর (রাঃ)-এর সুন্নাহ অনুসরণ","description":"এই হাদিসে আরাফাতের দিনের একটি সফর-ঘটনা এসেছে। ইবনে উমর (রাঃ) ইমামের সাথে যোহর ও আসর আদায় করলেন, আরাফাতে অবস্থান করলেন এবং ইমাম যখন মুযদালিফার দিকে রওনা হলেন, তিনিও সঙ্গে গেলেন। পথে একটি স্থানে তিনি উট থামালেন। সঙ্গীরা ভেবেছিলেন, তিনি হয়তো সালাত পড়বেন। কিন্তু তাঁর সেবক জানালেন, তিনি এখানে সালাতের জন্য থামেননি; বরং তাঁর মনে পড়েছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম এখানে প্রাকৃতিক প্রয়োজন পূরণ করেছিলেন, তাই তিনিও তা করতে পছন্দ করেছেন। এই বর্ণনায় সাহাবিদের সুন্নাহ অনুসরণের গভীরতা দেখা যায়। তবে এটিকে বাড়িয়ে নতুন বিধান বানানো নয়; ঘটনাটিকে ঘটনার মতোই বুঝতে হবে।"},"teachings":["আরাফাতের আমলে ইমামের অনুসরণ করার দিকটি বর্ণনায় এসেছে।","ইবনে উমর (রাঃ) রাসূলের কাজ স্মরণ করে অনুসরণ করতে পছন্দ করতেন।","সাহাবিদের কাছে সুন্নাহ ছিল জীবনের বাস্তব পথ।","ঘটনাকে তার সীমার মধ্যে রেখে বোঝা দরকার।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E128" s="4" t="n"/>
@@ -3456,12 +3452,12 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আরাফাতে সুন্নাহ অনুসরণ","description":"$book_name$ $hadith_number$ - $chapter_name$. আরাফাত থেকে মুযদালিফার পথে ইবনে উমর (রাঃ) নবীর স্মৃতিতে একটি কাজ করতে পছন্দ করেন—এতে অনুসরণের শিক্ষা আছে।"},"heading":{"title":"আরাফাতের সফরে ইবনে উমর (রাঃ)-এর সুন্নাহ অনুসরণ","description":"এই হাদিসে আরাফাতের দিনের একটি সফর-ঘটনা এসেছে। ইবনে উমর (রাঃ) ইমামের সাথে যোহর ও আসর আদায় করলেন, আরাফাতে অবস্থান করলেন এবং ইমাম যখন মুযদালিফার দিকে রওনা হলেন, তিনিও সঙ্গে গেলেন। পথে একটি স্থানে তিনি উট থামালেন। সঙ্গীরা ভেবেছিলেন, তিনি হয়তো সালাত পড়বেন। কিন্তু তাঁর সেবক জানালেন, তিনি এখানে সালাতের জন্য থামেননি; বরং তাঁর মনে পড়েছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম এখানে প্রাকৃতিক প্রয়োজন পূরণ করেছিলেন, তাই তিনিও তা করতে পছন্দ করেছেন। এই বর্ণনায় সাহাবিদের সুন্নাহ অনুসরণের গভীরতা দেখা যায়। তবে এটিকে বাড়িয়ে নতুন বিধান বানানো নয়; ঘটনাটিকে ঘটনার মতোই বুঝতে হবে।"},"teachings":["আরাফাতের আমলে ইমামের অনুসরণ করার দিকটি বর্ণনায় এসেছে।","ইবনে উমর (রাঃ) রাসূলের কাজ স্মরণ করে অনুসরণ করতে পছন্দ করতেন।","সাহাবিদের কাছে সুন্নাহ ছিল জীবনের বাস্তব পথ।","ঘটনাকে তার সীমার মধ্যে রেখে বোঝা দরকার।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্বীনে নতুন কাজ অগ্রহণযোগ্য","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের নির্দেশ ছাড়া দ্বীনে নতুন কিছু সৃষ্টি বা আমল করলে তা প্রত্যাখ্যাত—এই হাদিসে বিদআত থেকে সতর্ক করা হয়েছে।"},"heading":{"title":"দ্বীনে নতুন কাজ কেন অগ্রহণযোগ্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম খুব পরিষ্কারভাবে বলেছেন, যে ব্যক্তি এই দ্বীনের মধ্যে এমন নতুন কিছু সৃষ্টি করবে যা এর অন্তর্ভুক্ত নয়, তা প্রত্যাখ্যাত। অন্য বর্ণনায় এসেছে, তাঁর নির্দেশ ছাড়া কোনো কাজ করলে সেটিও প্রত্যাখ্যাত। তাই এই হাদিসের মূল বিষয় হলো বিদআত থেকে সতর্ক থাকা এবং আমলকে রাসূলের নির্দেশের সাথে মিলিয়ে দেখা। “দ্বীনে নতুন কাজ” বলতে এখানে ইবাদত ও দ্বীনি আমলের ক্ষেত্রে এমন কিছু বোঝানো হয়েছে, যার ভিত্তি রাসূলের নির্দেশে নেই। তাই ভালো মনে হলেই কোনো কাজ দ্বীনের অংশ হয়ে যায় না। এই হাদিস মুসলিমদের শেখায়, আমলের গ্রহণযোগ্যতার জন্য সুন্নাহর সাথে মিল থাকা জরুরি।"},"teachings":["দ্বীনের নামে নতুন কিছু যোগ করা গ্রহণযোগ্য নয়।","রাসূলের নির্দেশ ছাড়া করা আমল প্রত্যাখ্যাত হতে পারে।","ইবাদতে ভালো নিয়ত যথেষ্ট নয়; সুন্নাহর সাথে মিল দরকার।","বিদআত থেকে বাঁচা দ্বীনের সঠিক পথ রক্ষার অংশ।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
         </is>
       </c>
       <c r="E129" s="4" t="n"/>
@@ -3479,15 +3475,19 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্বীনে নতুন কাজ অগ্রহণযোগ্য","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের নির্দেশ ছাড়া দ্বীনে নতুন কিছু সৃষ্টি বা আমল করলে তা প্রত্যাখ্যাত—এই হাদিসে বিদআত থেকে সতর্ক করা হয়েছে।"},"heading":{"title":"দ্বীনে নতুন কাজ কেন অগ্রহণযোগ্য","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম খুব পরিষ্কারভাবে বলেছেন, যে ব্যক্তি এই দ্বীনের মধ্যে এমন নতুন কিছু সৃষ্টি করবে যা এর অন্তর্ভুক্ত নয়, তা প্রত্যাখ্যাত। অন্য বর্ণনায় এসেছে, তাঁর নির্দেশ ছাড়া কোনো কাজ করলে সেটিও প্রত্যাখ্যাত। তাই এই হাদিসের মূল বিষয় হলো বিদআত থেকে সতর্ক থাকা এবং আমলকে রাসূলের নির্দেশের সাথে মিলিয়ে দেখা। “দ্বীনে নতুন কাজ” বলতে এখানে ইবাদত ও দ্বীনি আমলের ক্ষেত্রে এমন কিছু বোঝানো হয়েছে, যার ভিত্তি রাসূলের নির্দেশে নেই। তাই ভালো মনে হলেই কোনো কাজ দ্বীনের অংশ হয়ে যায় না। এই হাদিস মুসলিমদের শেখায়, আমলের গ্রহণযোগ্যতার জন্য সুন্নাহর সাথে মিল থাকা জরুরি।"},"teachings":["দ্বীনের নামে নতুন কিছু যোগ করা গ্রহণযোগ্য নয়।","রাসূলের নির্দেশ ছাড়া করা আমল প্রত্যাখ্যাত হতে পারে।","ইবাদতে ভালো নিয়ত যথেষ্ট নয়; সুন্নাহর সাথে মিল দরকার।","বিদআত থেকে বাঁচা দ্বীনের সঠিক পথ রক্ষার অংশ।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
-        </is>
-      </c>
-      <c r="E130" s="4" t="n"/>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস শ্রবণ ও বর্ণনার গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. এই নোটে একই বাণীর একাধিক সাহাবী সূত্রের কথা এসেছে, যা হাদিস শ্রবণ ও সংরক্ষণের গুরুত্ব দেখায়।"},"heading":{"title":"হাদিস শ্রবণ ও সংরক্ষণ: বর্ণনার সূত্রের মূল্য","description":"এই অংশে পূর্ণ হাদিসের নতুন কোনো আলাদা বক্তব্য দেওয়া হয়নি। এখানে বলা হয়েছে, ইবনে হিব্বান তাঁর সহীহ গ্রন্থে যায়েদ বিন সাবেত রাদিয়াল্লাহু আনহু থেকে হাদিসটি বর্ণনা করেছেন এবং হাদিস শ্রবণ অনুচ্ছেদে এর বর্ণনা আসবে। এরপর হাফেজ আবদুল আযীম আল মুনযেরীর মন্তব্য এসেছে যে, এই হাদিস আরও অনেক সাহাবী থেকে বর্ণিত হয়েছে। তাদের মধ্যে ইবনে মাসউদ, মুআয বিন জাবাল, নূমান বিন বাশীর, জুবায়র বিন মুতঈম, আবু দারদা এবং আরও অনেক সাহাবীর নাম উল্লেখ হয়েছে। এই নোটের মূল শিক্ষা হলো, হাদিসের বর্ণনা ও সূত্রের গুরুত্ব অনেক। একই অর্থের বাণী বিভিন্ন সাহাবী থেকে আসলে তা সংরক্ষণের গুরুত্ব আরও স্পষ্ট হয়। তবে এখানে পূর্ণ হাদিস না থাকায় ব্যাখ্যায় অতিরিক্ত বিষয় যোগ করা উচিত নয়।"},"teachings":["হাদিসের সূত্র জানা ইলমের গুরুত্বপূর্ণ অংশ।","একই বাণী একাধিক সাহাবী থেকে আসতে পারে।","পূর্ণ পাঠ ছাড়া নতুন বিধান বা অতিরিক্ত ব্যাখ্যা দেওয়া ঠিক নয়।","হাদিস শ্রবণ ও সংরক্ষণ ইসলামী জ্ঞানের বড় দায়িত্ব।"],"related_hadiths":[{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ২৩২ (প্রাসঙ্গিক বর্ণনা)"</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="46" customHeight="1">
       <c r="A131" s="4" t="inlineStr">
@@ -3502,19 +3502,15 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস শ্রবণ ও বর্ণনার গুরুত্ব","description":"$book_name$ $hadith_number$ - $chapter_name$. এই নোটে একই বাণীর একাধিক সাহাবী সূত্রের কথা এসেছে, যা হাদিস শ্রবণ ও সংরক্ষণের গুরুত্ব দেখায়।"},"heading":{"title":"হাদিস শ্রবণ ও সংরক্ষণ: বর্ণনার সূত্রের মূল্য","description":"এই অংশে পূর্ণ হাদিসের নতুন কোনো আলাদা বক্তব্য দেওয়া হয়নি। এখানে বলা হয়েছে, ইবনে হিব্বান তাঁর সহীহ গ্রন্থে যায়েদ বিন সাবেত রাদিয়াল্লাহু আনহু থেকে হাদিসটি বর্ণনা করেছেন এবং হাদিস শ্রবণ অনুচ্ছেদে এর বর্ণনা আসবে। এরপর হাফেজ আবদুল আযীম আল মুনযেরীর মন্তব্য এসেছে যে, এই হাদিস আরও অনেক সাহাবী থেকে বর্ণিত হয়েছে। তাদের মধ্যে ইবনে মাসউদ, মুআয বিন জাবাল, নূমান বিন বাশীর, জুবায়র বিন মুতঈম, আবু দারদা এবং আরও অনেক সাহাবীর নাম উল্লেখ হয়েছে। এই নোটের মূল শিক্ষা হলো, হাদিসের বর্ণনা ও সূত্রের গুরুত্ব অনেক। একই অর্থের বাণী বিভিন্ন সাহাবী থেকে আসলে তা সংরক্ষণের গুরুত্ব আরও স্পষ্ট হয়। তবে এখানে পূর্ণ হাদিস না থাকায় ব্যাখ্যায় অতিরিক্ত বিষয় যোগ করা উচিত নয়।"},"teachings":["হাদিসের সূত্র জানা ইলমের গুরুত্বপূর্ণ অংশ।","একই বাণী একাধিক সাহাবী থেকে আসতে পারে।","পূর্ণ পাঠ ছাড়া নতুন বিধান বা অতিরিক্ত ব্যাখ্যা দেওয়া ঠিক নয়।","হাদিস শ্রবণ ও সংরক্ষণ ইসলামী জ্ঞানের বড় দায়িত্ব।"],"related_hadiths":[{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
-        </is>
-      </c>
-      <c r="E131" s="4" t="inlineStr">
-        <is>
-          <t>related_hadiths[1]: unknown book label "সুনান ইবন মাজাহ ২৩২ (প্রাসঙ্গিক বর্ণনা)"</t>
-        </is>
-      </c>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন সেরা বাণী, নবীর পথ সেরা পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. খুতবায় রাসূল কুরআনকে সেরা বাণী, নিজের হেদায়াতকে সেরা পথ এবং বিদআতকে ভ্রষ্টতা বলেছেন।"},"heading":{"title":"সেরা বাণী আল্লাহর কিতাব, সেরা পথ মুহাম্মাদের হেদায়াত","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর খুতবার একটি শক্তিশালী বর্ণনা এসেছে। খুতবার সময় তাঁর চোখ লাল হতো, কণ্ঠ উঁচু হতো এবং তিনি এমনভাবে সতর্ক করতেন যেন কোনো বাহিনীকে বিপদের খবর দিচ্ছেন। তিনি কিয়ামতের নিকটতা বোঝাতে দুই আঙুল মিলিয়ে দেখাতেন। এরপর তিনি বলেন, সর্বোত্তম বাণী আল্লাহর কিতাব, সর্বোত্তম হেদায়াত মুহাম্মাদের হেদায়াত, আর দ্বীনের মধ্যে নতুন সৃষ্টি নিকৃষ্ট বিষয়; প্রত্যেক বিদআত ভ্রষ্টতা। এই হাদিসে কুরআন, সুন্নাহ, বিদআত থেকে সতর্কতা এবং উম্মতের প্রতি নবীর দায়িত্ববোধ একসাথে এসেছে। তাই এটি খুতবা, কুরআন-সুন্নাহ এবং বিদআত বিষয়ে খুব গুরুত্বপূর্ণ হাদিস।"},"teachings":["আল্লাহর কিতাবকে সর্বোত্তম বাণী বলা হয়েছে।","মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর হেদায়াতকে সেরা পথ বলা হয়েছে।","দ্বীনের মধ্যে নতুন সৃষ্টি থেকে সতর্ক করা হয়েছে।","খুতবায় মানুষকে সতর্ক করা নববী শিক্ষার অংশ।"],"related_hadiths":[{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="n"/>
     </row>
     <row r="132" ht="46" customHeight="1">
       <c r="A132" s="4" t="inlineStr">
@@ -3529,12 +3525,12 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন সেরা বাণী, নবীর পথ সেরা পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. খুতবায় রাসূল কুরআনকে সেরা বাণী, নিজের হেদায়াতকে সেরা পথ এবং বিদআতকে ভ্রষ্টতা বলেছেন।"},"heading":{"title":"সেরা বাণী আল্লাহর কিতাব, সেরা পথ মুহাম্মাদের হেদায়াত","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর খুতবার একটি শক্তিশালী বর্ণনা এসেছে। খুতবার সময় তাঁর চোখ লাল হতো, কণ্ঠ উঁচু হতো এবং তিনি এমনভাবে সতর্ক করতেন যেন কোনো বাহিনীকে বিপদের খবর দিচ্ছেন। তিনি কিয়ামতের নিকটতা বোঝাতে দুই আঙুল মিলিয়ে দেখাতেন। এরপর তিনি বলেন, সর্বোত্তম বাণী আল্লাহর কিতাব, সর্বোত্তম হেদায়াত মুহাম্মাদের হেদায়াত, আর দ্বীনের মধ্যে নতুন সৃষ্টি নিকৃষ্ট বিষয়; প্রত্যেক বিদআত ভ্রষ্টতা। এই হাদিসে কুরআন, সুন্নাহ, বিদআত থেকে সতর্কতা এবং উম্মতের প্রতি নবীর দায়িত্ববোধ একসাথে এসেছে। তাই এটি খুতবা, কুরআন-সুন্নাহ এবং বিদআত বিষয়ে খুব গুরুত্বপূর্ণ হাদিস।"},"teachings":["আল্লাহর কিতাবকে সর্বোত্তম বাণী বলা হয়েছে।","মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর হেদায়াতকে সেরা পথ বলা হয়েছে।","দ্বীনের মধ্যে নতুন সৃষ্টি থেকে সতর্ক করা হয়েছে।","খুতবায় মানুষকে সতর্ক করা নববী শিক্ষার অংশ।"],"related_hadiths":[{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেট, যৌন লোভ ও প্রবৃত্তির ফিতনা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেট, যৌন চাহিদা ও প্রবৃত্তির অনুসরণে পথভ্রষ্ট হওয়ার ভয় রাসূল প্রকাশ করেছেন।"},"heading":{"title":"প্রবৃত্তির অনুসরণ থেকে সতর্ক থাকার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উম্মতের জন্য একটি বিশেষ আশঙ্কার কথা বলেছেন। তিনি পেটের লোভ, যৌনাঙ্গের বিষয়ে লোভে পড়ে পথভ্রষ্ট হওয়া এবং প্রবৃত্তির অনুসরণ করে বিভ্রান্ত হওয়ার কথা উল্লেখ করেছেন। ভাষাটি খুব সরাসরি। মানুষের খাবার, ভোগ ও যৌন চাহিদা যদি নিয়ন্ত্রণ ছাড়া চলে, তাহলে তা দ্বীনি ও নৈতিক ক্ষতির কারণ হতে পারে—হাদিসের বক্তব্য এতটুকুই। এখানে অতিরিক্ত কোনো গল্প বা আলাদা বিধান দেওয়া হয়নি। এই হাদিস “প্রবৃত্তির অনুসরণ”, “লোভ”, “পেটের ফিতনা” এবং “যৌন চাহিদা নিয়ন্ত্রণ” বিষয়ে গুরুত্বপূর্ণ। এটি আমাদের নিজের ভেতরের টানকে চিনতে ও সতর্ক হতে শেখায়।"},"teachings":["পেটের লোভ মানুষকে ভুল পথে নিতে পারে।","যৌন চাহিদার বিষয়ে সংযম দরকার।","প্রবৃত্তির অনুসরণ বিভ্রান্তির কারণ হতে পারে।","নিজের ভেতরের দুর্বলতা সম্পর্কে সতর্ক থাকা জরুরি।"],"related_hadiths":[{"id":"2466","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2597","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E132" s="4" t="n"/>
@@ -3552,12 +3548,12 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>56</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | পেট, যৌন লোভ ও প্রবৃত্তির ফিতনা","description":"$book_name$ $hadith_number$ - $chapter_name$. পেট, যৌন চাহিদা ও প্রবৃত্তির অনুসরণে পথভ্রষ্ট হওয়ার ভয় রাসূল প্রকাশ করেছেন।"},"heading":{"title":"প্রবৃত্তির অনুসরণ থেকে সতর্ক থাকার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উম্মতের জন্য একটি বিশেষ আশঙ্কার কথা বলেছেন। তিনি পেটের লোভ, যৌনাঙ্গের বিষয়ে লোভে পড়ে পথভ্রষ্ট হওয়া এবং প্রবৃত্তির অনুসরণ করে বিভ্রান্ত হওয়ার কথা উল্লেখ করেছেন। ভাষাটি খুব সরাসরি। মানুষের খাবার, ভোগ ও যৌন চাহিদা যদি নিয়ন্ত্রণ ছাড়া চলে, তাহলে তা দ্বীনি ও নৈতিক ক্ষতির কারণ হতে পারে—হাদিসের বক্তব্য এতটুকুই। এখানে অতিরিক্ত কোনো গল্প বা আলাদা বিধান দেওয়া হয়নি। এই হাদিস “প্রবৃত্তির অনুসরণ”, “লোভ”, “পেটের ফিতনা” এবং “যৌন চাহিদা নিয়ন্ত্রণ” বিষয়ে গুরুত্বপূর্ণ। এটি আমাদের নিজের ভেতরের টানকে চিনতে ও সতর্ক হতে শেখায়।"},"teachings":["পেটের লোভ মানুষকে ভুল পথে নিতে পারে।","যৌন চাহিদার বিষয়ে সংযম দরকার।","প্রবৃত্তির অনুসরণ বিভ্রান্তির কারণ হতে পারে।","নিজের ভেতরের দুর্বলতা সম্পর্কে সতর্ক থাকা জরুরি।"],"related_hadiths":[{"id":"2466","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2597","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উদ্দীপনার পর সুন্নাহর পথে থাকা","description":"$book_name$ $hadith_number$ - $chapter_name$. আমলের উৎসাহ কমে গেলেও যে সুন্নাহর পথে থাকে, সে সঠিক পথে থাকে—এই হাদিসে ভারসাম্যের শিক্ষা আছে।"},"heading":{"title":"উৎসাহ কমলেও সুন্নাহর পথে থাকা","description":"এই হাদিসে বলা হয়েছে, প্রতিটি কাজের একটি উৎসাহ-উদ্দীপনা থাকে। সেই উদ্দীপনার পর একসময় অবসন্নতা বা বিরতি আসে। তখন মানুষের পথ দুই রকম হতে পারে: সে সুন্নাহর দিকে ফিরে আসে, অথবা অন্য কিছুর দিকে যায়। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, যার বিরতি তাঁর সুন্নাত পর্যন্ত গিয়ে থামে, সে সঠিক পথ পেয়েছে; আর যার বিরতি অন্য কিছুর দিকে, সে ধ্বংসের পথে পড়ে। এই বর্ণনার মূল শিক্ষা হলো, ইবাদতে আবেগ থাকলেও শেষ আশ্রয় সুন্নাহ হওয়া চাই। অতিরিক্ত উৎসাহের পর ক্লান্তি আসতে পারে, কিন্তু সেই সময় বিদআত বা ভুল পথে যাওয়া নয়; সুন্নাহর সীমায় থাকা দরকার।"},"teachings":["আমলে উৎসাহ আসে, আবার ক্লান্তিও আসতে পারে।","ক্লান্তির সময় সুন্নাহর মধ্যে থাকা নিরাপদ পথ।","উদ্দীপনা কমলে বিদআতের দিকে যাওয়া বিপজ্জনক।","ইবাদতে আবেগের সাথে সুন্নাহর সীমা মানা দরকার।"],"related_hadiths":[{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E133" s="4" t="n"/>
@@ -3575,12 +3571,12 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>59</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উদ্দীপনার পর সুন্নাহর পথে থাকা","description":"$book_name$ $hadith_number$ - $chapter_name$. আমলের উৎসাহ কমে গেলেও যে সুন্নাহর পথে থাকে, সে সঠিক পথে থাকে—এই হাদিসে ভারসাম্যের শিক্ষা আছে।"},"heading":{"title":"উৎসাহ কমলেও সুন্নাহর পথে থাকা","description":"এই হাদিসে বলা হয়েছে, প্রতিটি কাজের একটি উৎসাহ-উদ্দীপনা থাকে। সেই উদ্দীপনার পর একসময় অবসন্নতা বা বিরতি আসে। তখন মানুষের পথ দুই রকম হতে পারে: সে সুন্নাহর দিকে ফিরে আসে, অথবা অন্য কিছুর দিকে যায়। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, যার বিরতি তাঁর সুন্নাত পর্যন্ত গিয়ে থামে, সে সঠিক পথ পেয়েছে; আর যার বিরতি অন্য কিছুর দিকে, সে ধ্বংসের পথে পড়ে। এই বর্ণনার মূল শিক্ষা হলো, ইবাদতে আবেগ থাকলেও শেষ আশ্রয় সুন্নাহ হওয়া চাই। অতিরিক্ত উৎসাহের পর ক্লান্তি আসতে পারে, কিন্তু সেই সময় বিদআত বা ভুল পথে যাওয়া নয়; সুন্নাহর সীমায় থাকা দরকার।"},"teachings":["আমলে উৎসাহ আসে, আবার ক্লান্তিও আসতে পারে।","ক্লান্তির সময় সুন্নাহর মধ্যে থাকা নিরাপদ পথ।","উদ্দীপনা কমলে বিদআতের দিকে যাওয়া বিপজ্জনক।","ইবাদতে আবেগের সাথে সুন্নাহর সীমা মানা দরকার।"],"related_hadiths":[{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বচ্ছ দ্বীনের পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূল এমন উজ্জ্বল পথে উম্মতকে রেখে গেছেন, যার রাতও দিনের মতো পরিষ্কার—এ পথ থেকে বক্র হওয়া ক্ষতির কারণ।"},"heading":{"title":"রাসূল যে স্বচ্ছ পথে উম্মতকে রেখে গেছেন","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, তিনি উম্মতকে এমন এক স্পষ্ট পথে রেখে গেছেন, যার শুভ্রতা ও উজ্জ্বলতা এত পরিষ্কার যে তার রাতও দিনের মতো। এরপর বলা হয়েছে, ধ্বংসপ্রাপ্ত ব্যক্তি ছাড়া কেউ এ পথ থেকে বক্র পথে যায় না। এই বর্ণনার মূল শিক্ষা হলো, দ্বীনের পথ অস্পষ্ট নয়; রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম আল্লাহর নির্দেশে পথ দেখিয়ে গেছেন। তাই বিভ্রান্তি, বিদআত বা নিজের খেয়ালকে পথ বানানোর বদলে সেই পরিষ্কার পথে থাকা দরকার। এখানে অতিরিক্ত কোনো ইতিহাস নেই; শুধু হাদিসের সরল কথা হলো, রাসূলের রেখে যাওয়া দ্বীন স্পষ্ট, আর তা থেকে সরে যাওয়া বিপদের বিষয়।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উম্মতের জন্য স্পষ্ট পথ রেখে গেছেন।","দ্বীনের পথকে রাত-দিনের মতো পরিষ্কার বলা হয়েছে।","সেই পথ থেকে বক্র হওয়া ক্ষতির কারণ হিসেবে এসেছে।","সঠিক পথ জানতে রাসূলের শিক্ষা আঁকড়ে ধরা দরকার।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E134" s="4" t="n"/>
@@ -3598,12 +3594,12 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | স্বচ্ছ দ্বীনের পথ","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূল এমন উজ্জ্বল পথে উম্মতকে রেখে গেছেন, যার রাতও দিনের মতো পরিষ্কার—এ পথ থেকে বক্র হওয়া ক্ষতির কারণ।"},"heading":{"title":"রাসূল যে স্বচ্ছ পথে উম্মতকে রেখে গেছেন","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, তিনি উম্মতকে এমন এক স্পষ্ট পথে রেখে গেছেন, যার শুভ্রতা ও উজ্জ্বলতা এত পরিষ্কার যে তার রাতও দিনের মতো। এরপর বলা হয়েছে, ধ্বংসপ্রাপ্ত ব্যক্তি ছাড়া কেউ এ পথ থেকে বক্র পথে যায় না। এই বর্ণনার মূল শিক্ষা হলো, দ্বীনের পথ অস্পষ্ট নয়; রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম আল্লাহর নির্দেশে পথ দেখিয়ে গেছেন। তাই বিভ্রান্তি, বিদআত বা নিজের খেয়ালকে পথ বানানোর বদলে সেই পরিষ্কার পথে থাকা দরকার। এখানে অতিরিক্ত কোনো ইতিহাস নেই; শুধু হাদিসের সরল কথা হলো, রাসূলের রেখে যাওয়া দ্বীন স্পষ্ট, আর তা থেকে সরে যাওয়া বিপদের বিষয়।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম উম্মতের জন্য স্পষ্ট পথ রেখে গেছেন।","দ্বীনের পথকে রাত-দিনের মতো পরিষ্কার বলা হয়েছে।","সেই পথ থেকে বক্র হওয়া ক্ষতির কারণ হিসেবে এসেছে।","সঠিক পথ জানতে রাসূলের শিক্ষা আঁকড়ে ধরা দরকার।"],"related_hadiths":[{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"7277","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5063","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুর্বলদের দোয়া ও ইখলাসে সাহায্য","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি জানায়, উম্মতের দুর্বলদের দোয়া, সালাত ও ইখলাস আল্লাহর সাহায্যের কারণ।"},"heading":{"title":"দুর্বলদের দোয়া, সালাত ও ইখলাস: সাহায্যের সুন্দর শিক্ষা","description":"এই হাদিসে সা’দ রাদিয়াল্লাহু আনহুর একটি ভাবনার কথা এসেছে। তিনি মনে করেছিলেন, গনীমতের মালে অন্যদের তুলনায় তাঁর বেশি অধিকার আছে। তখন নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁকে এমন শিক্ষা দেন, যা অহংকার কমায় এবং দুর্বলদের মর্যাদা বুঝতে সাহায্য করে। তিনি বলেন, আল্লাহ এই উম্মতকে তাদের দুর্বল ব্যক্তিদের মাধ্যমে সাহায্য করেন—তাদের দোয়া, সালাত এবং ইখলাসের মাধ্যমে। এখানে মূল বিষয় হলো, বাহ্যিক শক্তি, অবস্থান বা সামরিক যোগ্যতা একমাত্র মানদণ্ড নয়। আল্লাহর কাছে খাঁটি দোয়া, নিয়মিত সালাত এবং একনিষ্ঠ আমলের মূল্য আছে। তাই সমাজে যাদের দুর্বল মনে করা হয়, তাদেরকে ছোট করে দেখা ঠিক নয়। এই হাদিস ইখলাস, বিনয় এবং মুসলিম সমাজে সবার মর্যাদা বোঝার শিক্ষা দেয়।"},"teachings":["দুর্বল মুসলিমদের দোয়া ও সালাতকে ছোট করে দেখা উচিত নয়।","আল্লাহর সাহায্য বাহ্যিক শক্তির উপরই সীমাবদ্ধ নয়।","ইখলাস আমলকে মূল্যবান করে তোলে।","নিজের মর্যাদা নিয়ে অহংকার করা থেকে বাঁচা দরকার।"],"related_hadiths":[{"id":"2896","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E135" s="4" t="n"/>
@@ -3621,12 +3617,12 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুর্বলদের দোয়া ও ইখলাসে সাহায্য","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি জানায়, উম্মতের দুর্বলদের দোয়া, সালাত ও ইখলাস আল্লাহর সাহায্যের কারণ।"},"heading":{"title":"দুর্বলদের দোয়া, সালাত ও ইখলাস: সাহায্যের সুন্দর শিক্ষা","description":"এই হাদিসে সা’দ রাদিয়াল্লাহু আনহুর একটি ভাবনার কথা এসেছে। তিনি মনে করেছিলেন, গনীমতের মালে অন্যদের তুলনায় তাঁর বেশি অধিকার আছে। তখন নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁকে এমন শিক্ষা দেন, যা অহংকার কমায় এবং দুর্বলদের মর্যাদা বুঝতে সাহায্য করে। তিনি বলেন, আল্লাহ এই উম্মতকে তাদের দুর্বল ব্যক্তিদের মাধ্যমে সাহায্য করেন—তাদের দোয়া, সালাত এবং ইখলাসের মাধ্যমে। এখানে মূল বিষয় হলো, বাহ্যিক শক্তি, অবস্থান বা সামরিক যোগ্যতা একমাত্র মানদণ্ড নয়। আল্লাহর কাছে খাঁটি দোয়া, নিয়মিত সালাত এবং একনিষ্ঠ আমলের মূল্য আছে। তাই সমাজে যাদের দুর্বল মনে করা হয়, তাদেরকে ছোট করে দেখা ঠিক নয়। এই হাদিস ইখলাস, বিনয় এবং মুসলিম সমাজে সবার মর্যাদা বোঝার শিক্ষা দেয়।"},"teachings":["দুর্বল মুসলিমদের দোয়া ও সালাতকে ছোট করে দেখা উচিত নয়।","আল্লাহর সাহায্য বাহ্যিক শক্তির উপরই সীমাবদ্ধ নয়।","ইখলাস আমলকে মূল্যবান করে তোলে।","নিজের মর্যাদা নিয়ে অহংকার করা থেকে বাঁচা দরকার।"],"related_hadiths":[{"id":"2896","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে বিদআতী কিচ্ছা থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে মাসউদ (রাঃ) মসজিদে কিচ্ছা বয়ানকে পথভ্রষ্ট বিদআত বলে সতর্ক করেন; লোকেরা তা শুনে সরে যায়।"},"heading":{"title":"ইবনে মাসউদ (রাঃ)-এর বিদআত থেকে সতর্ক করার ঘটনা","description":"এই হাদিসে আমর বিন জুরারার ঘটনা এসেছে। তিনি মসজিদে কিচ্ছা-কাহিনী বয়ান করছিলেন। তখন আবদুল্লাহ ইবনে মাসউদ (রাঃ) তাঁর সামনে দাঁড়িয়ে বলেন, হে আমর! তুমি হয় পথভ্রষ্ট বিদআত আবিষ্কার করেছ, অথবা তুমি মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ও তাঁর সাহাবীদের চেয়ে বেশি হেদায়াতপ্রাপ্ত হয়ে গেছ। এই কথা শোনার পর বর্ণনাকারী দেখেন, শ্রোতারা সবাই সরে গেছে, কেউ আর রইল না। এই বর্ণনার মূল শিক্ষা হলো, দ্বীনের নামে নতুন পদ্ধতি চালু করার বিষয়ে সাহাবিরা সতর্ক ছিলেন। মসজিদে কথা বলার বিষয়টিও সুন্নাহর সীমার মধ্যে থাকা দরকার—এ কথা এই ঘটনার মাধ্যমে বোঝা যায়।"},"teachings":["সাহাবিরা বিদআত দেখলে সতর্ক করতেন।","দ্বীনের নামে নতুন পদ্ধতি চালু করা হালকা বিষয় নয়।","মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ও সাহাবিদের পথই হেদায়াতের মাপকাঠি।","সঠিক উপদেশ শুনে শ্রোতাদের ভুল কাজ থেকে সরে আসা উচিত।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
         </is>
       </c>
       <c r="E136" s="4" t="n"/>
@@ -3644,12 +3640,12 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>61</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে বিদআতী কিচ্ছা থেকে সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনে মাসউদ (রাঃ) মসজিদে কিচ্ছা বয়ানকে পথভ্রষ্ট বিদআত বলে সতর্ক করেন; লোকেরা তা শুনে সরে যায়।"},"heading":{"title":"ইবনে মাসউদ (রাঃ)-এর বিদআত থেকে সতর্ক করার ঘটনা","description":"এই হাদিসে আমর বিন জুরারার ঘটনা এসেছে। তিনি মসজিদে কিচ্ছা-কাহিনী বয়ান করছিলেন। তখন আবদুল্লাহ ইবনে মাসউদ (রাঃ) তাঁর সামনে দাঁড়িয়ে বলেন, হে আমর! তুমি হয় পথভ্রষ্ট বিদআত আবিষ্কার করেছ, অথবা তুমি মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ও তাঁর সাহাবীদের চেয়ে বেশি হেদায়াতপ্রাপ্ত হয়ে গেছ। এই কথা শোনার পর বর্ণনাকারী দেখেন, শ্রোতারা সবাই সরে গেছে, কেউ আর রইল না। এই বর্ণনার মূল শিক্ষা হলো, দ্বীনের নামে নতুন পদ্ধতি চালু করার বিষয়ে সাহাবিরা সতর্ক ছিলেন। মসজিদে কথা বলার বিষয়টিও সুন্নাহর সীমার মধ্যে থাকা দরকার—এ কথা এই ঘটনার মাধ্যমে বোঝা যায়।"},"teachings":["সাহাবিরা বিদআত দেখলে সতর্ক করতেন।","দ্বীনের নামে নতুন পদ্ধতি চালু করা হালকা বিষয় নয়।","মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম ও সাহাবিদের পথই হেদায়াতের মাপকাঠি।","সঠিক উপদেশ শুনে শ্রোতাদের ভুল কাজ থেকে সরে আসা উচিত।"],"related_hadiths":[{"id":"2697","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"161","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"},{"id":"1578","book_id":"3","slug":"nasai","label":"সুনান আন-নাসায়ী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উত্তম রীতি চালু করার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. অভাবী মানুষের পাশে দাঁড়ানো, দানের সূচনা করা এবং ভালো-মন্দ রীতি চালুর ফল এই হাদিসে স্পষ্ট হয়েছে।"},"heading":{"title":"উত্তম রীতি চালু করার ফজিলত ও দানের শিক্ষা","description":"এই হাদিসে দেখা যায়, কিছু অভাবী মানুষ রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর কাছে এলে তাদের কষ্ট দেখে তাঁর চেহারায় দুঃখের ছাপ ফুটে ওঠে। এরপর তিনি সালাত আদায় করে মানুষকে আল্লাহভীতি, আখেরাতের প্রস্তুতি এবং দানের দিকে ডাকেন। একজন আনসারী সাহাবী প্রথমে ভারী থলে নিয়ে দান করলে অন্যরাও তার অনুসরণ করে। এখানে মূল শিক্ষা হলো, ভালো কাজে প্রথম এগিয়ে আসা অনেক সময় অন্যদেরও উৎসাহ দেয়। তাই “উত্তম রীতি চালু করা” মানে ইসলামের ভেতরে নতুন বিদআত বানানো নয়; বরং বৈধ ভালো কাজের পথে মানুষকে আগে এগিয়ে দেওয়া। একইভাবে খারাপ প্রথা চালু করা ভয়ংকর, কারণ তার প্রভাব অন্যদের ওপরও পড়ে।"},"teachings":["অভাবী মানুষের কষ্ট দেখে উদাসীন না থেকে সাহায্যের চেষ্টা করা উচিত।","ভালো কাজে আগে এগিয়ে গেলে অন্যদের জন্য তা অনুপ্রেরণা হতে পারে।","সৎ কাজের প্রচলন প্রতিদানের কারণ, আর মন্দ কাজের প্রচলন পাপের কারণ।","সামান্য দানও মূল্যবান, এমনকি খেজুরের একটি অংশ হলেও।"],"related_hadiths":[{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1425","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E137" s="4" t="n"/>
@@ -3667,12 +3663,12 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | উত্তম রীতি চালু করার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. অভাবী মানুষের পাশে দাঁড়ানো, দানের সূচনা করা এবং ভালো-মন্দ রীতি চালুর ফল এই হাদিসে স্পষ্ট হয়েছে।"},"heading":{"title":"উত্তম রীতি চালু করার ফজিলত ও দানের শিক্ষা","description":"এই হাদিসে দেখা যায়, কিছু অভাবী মানুষ রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর কাছে এলে তাদের কষ্ট দেখে তাঁর চেহারায় দুঃখের ছাপ ফুটে ওঠে। এরপর তিনি সালাত আদায় করে মানুষকে আল্লাহভীতি, আখেরাতের প্রস্তুতি এবং দানের দিকে ডাকেন। একজন আনসারী সাহাবী প্রথমে ভারী থলে নিয়ে দান করলে অন্যরাও তার অনুসরণ করে। এখানে মূল শিক্ষা হলো, ভালো কাজে প্রথম এগিয়ে আসা অনেক সময় অন্যদেরও উৎসাহ দেয়। তাই “উত্তম রীতি চালু করা” মানে ইসলামের ভেতরে নতুন বিদআত বানানো নয়; বরং বৈধ ভালো কাজের পথে মানুষকে আগে এগিয়ে দেওয়া। একইভাবে খারাপ প্রথা চালু করা ভয়ংকর, কারণ তার প্রভাব অন্যদের ওপরও পড়ে।"},"teachings":["অভাবী মানুষের কষ্ট দেখে উদাসীন না থেকে সাহায্যের চেষ্টা করা উচিত।","ভালো কাজে আগে এগিয়ে গেলে অন্যদের জন্য তা অনুপ্রেরণা হতে পারে।","সৎ কাজের প্রচলন প্রতিদানের কারণ, আর মন্দ কাজের প্রচলন পাপের কারণ।","সামান্য দানও মূল্যবান, এমনকি খেজুরের একটি অংশ হলেও।"],"related_hadiths":[{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1425","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভালো কাজে পথ দেখানোর প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. একজনের দান অন্যদের দানে উৎসাহিত করে; ভালো কাজ চালু করলে অনুসারীদের নেকির মতো প্রতিদান পাওয়া যায়।"},"heading":{"title":"ভালো কাজে পথ দেখানোর প্রতিদান ও মন্দ প্রথার ভয়াবহতা","description":"এই হাদিসে একজন ভিক্ষুকের কথা এসেছে। প্রথমে লোকেরা তাকে দান করা থেকে বিরত ছিল। পরে একজন ব্যক্তি তাকে কিছু দিলে অন্যরাও দান করতে শুরু করে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এই ঘটনাকে কেন্দ্র করে বলেন, যে ব্যক্তি ভালো কাজ চালু করে এবং পরে মানুষ তা অনুসরণ করে, সে নিজের প্রতিদান পায় এবং অনুসরণকারীদের মতো প্রতিদানও পায়। তবে তাদের প্রতিদান কমে না। একইভাবে, কেউ মন্দ কাজ চালু করলে সে নিজের পাপ বহন করে এবং যারা তাকে অনুসরণ করে তাদের মতো পাপের ভারও তার ওপর আসে। এই শিক্ষা আমাদের আচরণকে দায়িত্বশীল করে। কারণ আমাদের একটি কাজ অন্যদের জন্য পথ খুলে দিতে পারে—ভালো দিকেও, মন্দ দিকেও।"},"teachings":["একজনের ভালো উদ্যোগ অনেক মানুষের ভালো কাজের কারণ হতে পারে।","ভালো কাজে পথ দেখানো নিজেও নেকির কাজ।","মন্দ কাজ শুরু করা শুধু নিজের ক্ষতি নয়; অন্যদের প্রভাবিত করলে তার দায়ও বাড়ে।","মানুষের সামনে কাজ করার সময় প্রভাবের দিকটি ভাবা দরকার।"],"related_hadiths":[{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E138" s="4" t="n"/>
@@ -3690,12 +3686,12 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ভালো কাজে পথ দেখানোর প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. একজনের দান অন্যদের দানে উৎসাহিত করে; ভালো কাজ চালু করলে অনুসারীদের নেকির মতো প্রতিদান পাওয়া যায়।"},"heading":{"title":"ভালো কাজে পথ দেখানোর প্রতিদান ও মন্দ প্রথার ভয়াবহতা","description":"এই হাদিসে একজন ভিক্ষুকের কথা এসেছে। প্রথমে লোকেরা তাকে দান করা থেকে বিরত ছিল। পরে একজন ব্যক্তি তাকে কিছু দিলে অন্যরাও দান করতে শুরু করে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) এই ঘটনাকে কেন্দ্র করে বলেন, যে ব্যক্তি ভালো কাজ চালু করে এবং পরে মানুষ তা অনুসরণ করে, সে নিজের প্রতিদান পায় এবং অনুসরণকারীদের মতো প্রতিদানও পায়। তবে তাদের প্রতিদান কমে না। একইভাবে, কেউ মন্দ কাজ চালু করলে সে নিজের পাপ বহন করে এবং যারা তাকে অনুসরণ করে তাদের মতো পাপের ভারও তার ওপর আসে। এই শিক্ষা আমাদের আচরণকে দায়িত্বশীল করে। কারণ আমাদের একটি কাজ অন্যদের জন্য পথ খুলে দিতে পারে—ভালো দিকেও, মন্দ দিকেও।"},"teachings":["একজনের ভালো উদ্যোগ অনেক মানুষের ভালো কাজের কারণ হতে পারে।","ভালো কাজে পথ দেখানো নিজেও নেকির কাজ।","মন্দ কাজ শুরু করা শুধু নিজের ক্ষতি নয়; অন্যদের প্রভাবিত করলে তার দায়ও বাড়ে।","মানুষের সামনে কাজ করার সময় প্রভাবের দিকটি ভাবা দরকার।"],"related_hadiths":[{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আবু হুরায়রা রা. থেকে বর্ণিত রেওয়ায়াত","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনু মাজাহ আবু হুরায়রা (রা.) থেকে উক্ত হাদিস বর্ণনা করেছেন—বর্ণনার সূত্র জানাও ইলমের অংশ।"},"heading":{"title":"আবু হুরায়রা রা. থেকে বর্ণিত হাদিসের সূত্র","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, ইবনু মাজাহ উক্ত হাদিসটি আবু হুরায়রা (রাঃ) থেকে বর্ণনা করেছেন। এখানে নতুন কোনো আলাদা ঘটনা বা নতুন বক্তব্য উল্লেখ করা হয়নি। তাই এই হাদিসের মূল গুরুত্ব হলো বর্ণনার সূত্রের দিকে মনোযোগ দেওয়া। হাদিস শেখার ক্ষেত্রে শুধু অর্থ জানা যথেষ্ট নয়; কে বর্ণনা করেছেন, কোন গ্রন্থে এসেছে—এসব তথ্যও গুরুত্বপূর্ণ। এটি দ্বীনি ইলম গ্রহণে সতর্কতা শেখায়। একই বিষয়ের হাদিস একাধিক সাহাবী থেকে আসতে পারে, আর তা বিষয়টির গুরুত্ব বোঝাতে সাহায্য করে। তবে এই নির্দিষ্ট পাঠে শুধু বর্ণনাকারী ও গ্রন্থের কথা এসেছে; তাই এর বাইরে কোনো অতিরিক্ত বিধান বা ঘটনা যোগ করা ঠিক হবে না।"},"teachings":["হাদিস শেখার সময় বর্ণনাকারীর নাম জানা গুরুত্বপূর্ণ।","একই বিষয়ের হাদিস ভিন্ন সাহাবী থেকেও বর্ণিত হতে পারে।","সংক্ষিপ্ত বর্ণনায় যা আছে, ব্যাখ্যায় তার সীমা রক্ষা করা উচিত।","দ্বীনি জ্ঞান গ্রহণে সূত্রের প্রতি যত্নবান হওয়া দরকার।"],"related_hadiths":[{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E139" s="4" t="n"/>
@@ -3713,12 +3709,12 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আবু হুরায়রা রা. থেকে বর্ণিত রেওয়ায়াত","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবনু মাজাহ আবু হুরায়রা (রা.) থেকে উক্ত হাদিস বর্ণনা করেছেন—বর্ণনার সূত্র জানাও ইলমের অংশ।"},"heading":{"title":"আবু হুরায়রা রা. থেকে বর্ণিত হাদিসের সূত্র","description":"এই সংক্ষিপ্ত বর্ণনায় বলা হয়েছে, ইবনু মাজাহ উক্ত হাদিসটি আবু হুরায়রা (রাঃ) থেকে বর্ণনা করেছেন। এখানে নতুন কোনো আলাদা ঘটনা বা নতুন বক্তব্য উল্লেখ করা হয়নি। তাই এই হাদিসের মূল গুরুত্ব হলো বর্ণনার সূত্রের দিকে মনোযোগ দেওয়া। হাদিস শেখার ক্ষেত্রে শুধু অর্থ জানা যথেষ্ট নয়; কে বর্ণনা করেছেন, কোন গ্রন্থে এসেছে—এসব তথ্যও গুরুত্বপূর্ণ। এটি দ্বীনি ইলম গ্রহণে সতর্কতা শেখায়। একই বিষয়ের হাদিস একাধিক সাহাবী থেকে আসতে পারে, আর তা বিষয়টির গুরুত্ব বোঝাতে সাহায্য করে। তবে এই নির্দিষ্ট পাঠে শুধু বর্ণনাকারী ও গ্রন্থের কথা এসেছে; তাই এর বাইরে কোনো অতিরিক্ত বিধান বা ঘটনা যোগ করা ঠিক হবে না।"},"teachings":["হাদিস শেখার সময় বর্ণনাকারীর নাম জানা গুরুত্বপূর্ণ।","একই বিষয়ের হাদিস ভিন্ন সাহাবী থেকেও বর্ণিত হতে পারে।","সংক্ষিপ্ত বর্ণনায় যা আছে, ব্যাখ্যায় তার সীমা রক্ষা করা উচিত।","দ্বীনি জ্ঞান গ্রহণে সূত্রের প্রতি যত্নবান হওয়া দরকার।"],"related_hadiths":[{"id":"203","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অন্যায় হত্যার পাপ ও প্রথম হত্যাকারীর দায়","description":"$book_name$ $hadith_number$ - $chapter_name$. অন্যায়ভাবে কেউ নিহত হলে প্রথম হত্যার রীতি চালুকারীর ওপরও পাপের অংশ পড়ে—এ হাদিসে তা বলা হয়েছে।"},"heading":{"title":"অন্যায় হত্যার পাপ ও খারাপ প্রথা চালুর ভয়","description":"এই হাদিসে অন্যায় হত্যার ভয়াবহ দিক তুলে ধরা হয়েছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, নাহকভাবে কোনো ব্যক্তি নিহত হলে তার খুনের পাপের একটি অংশ আদমের প্রথম সন্তানের ওপর বর্তাবে। কারণ সে-ই প্রথম হত্যা চালু করেছিল। এখানে মূল শিক্ষা হলো, মন্দ কাজ শুরু করার দায় শুধু একবারের কাজেই শেষ হয় না। যদি সেই কাজ পরে মানুষের মধ্যে চলতে থাকে, তাহলে তার প্রভাবের দায়ও ভয়ংকর হতে পারে। হাদিসটি হত্যার মতো বড় অপরাধের কথা বললেও এর ভেতরে খারাপ রীতি চালু করার সাধারণ সতর্কতাও আছে। মানুষকে ক্ষতি করা, অন্যায়ের পথ খুলে দেওয়া এবং পাপের দৃষ্টান্ত হওয়া—এসব থেকে একজন মুমিনের দূরে থাকা উচিত।"},"teachings":["নাহক হত্যা বড় পাপ এবং এর পরিণতি ভয়ংকর।","মন্দ কাজের পথ খুলে দিলে তার প্রভাবের দায় বাড়তে পারে।","অন্যায়ের দৃষ্টান্ত হওয়া থেকে নিজেকে বাঁচাতে হবে।","মানুষের জীবন ও নিরাপত্তার ব্যাপারে সতর্ক থাকা জরুরি।"],"related_hadiths":[{"id":"3335","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4473","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2616","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E140" s="4" t="n"/>
@@ -3736,12 +3732,12 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | অন্যায় হত্যার পাপ ও প্রথম হত্যাকারীর দায়","description":"$book_name$ $hadith_number$ - $chapter_name$. অন্যায়ভাবে কেউ নিহত হলে প্রথম হত্যার রীতি চালুকারীর ওপরও পাপের অংশ পড়ে—এ হাদিসে তা বলা হয়েছে।"},"heading":{"title":"অন্যায় হত্যার পাপ ও খারাপ প্রথা চালুর ভয়","description":"এই হাদিসে অন্যায় হত্যার ভয়াবহ দিক তুলে ধরা হয়েছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, নাহকভাবে কোনো ব্যক্তি নিহত হলে তার খুনের পাপের একটি অংশ আদমের প্রথম সন্তানের ওপর বর্তাবে। কারণ সে-ই প্রথম হত্যা চালু করেছিল। এখানে মূল শিক্ষা হলো, মন্দ কাজ শুরু করার দায় শুধু একবারের কাজেই শেষ হয় না। যদি সেই কাজ পরে মানুষের মধ্যে চলতে থাকে, তাহলে তার প্রভাবের দায়ও ভয়ংকর হতে পারে। হাদিসটি হত্যার মতো বড় অপরাধের কথা বললেও এর ভেতরে খারাপ রীতি চালু করার সাধারণ সতর্কতাও আছে। মানুষকে ক্ষতি করা, অন্যায়ের পথ খুলে দেওয়া এবং পাপের দৃষ্টান্ত হওয়া—এসব থেকে একজন মুমিনের দূরে থাকা উচিত।"},"teachings":["নাহক হত্যা বড় পাপ এবং এর পরিণতি ভয়ংকর।","মন্দ কাজের পথ খুলে দিলে তার প্রভাবের দায় বাড়তে পারে।","অন্যায়ের দৃষ্টান্ত হওয়া থেকে নিজেকে বাঁচাতে হবে।","মানুষের জীবন ও নিরাপত্তার ব্যাপারে সতর্ক থাকা জরুরি।"],"related_hadiths":[{"id":"3335","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4473","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2616","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জীবদ্দশা ও মৃত্যুর পর ভালো রীতির সওয়াব","description":"$book_name$ $hadith_number$ - $chapter_name$. উত্তম রীতি চালু করলে তা চলতে থাকা পর্যন্ত সওয়াব থাকে; মন্দ কাজ চালু করলে পাপের দায়ও চলতে থাকে।"},"heading":{"title":"উত্তম রীতির চলমান সওয়াব ও সীমান্ত পাহারার প্রতিদান","description":"এই হাদিসে তিনটি বিষয় এসেছে। প্রথমত, কেউ উত্তম রীতি চালু করলে জীবদ্দশায় এবং মৃত্যুর পরও সেই কাজ চলতে থাকলে সে প্রতিদান পেতে থাকে। দ্বিতীয়ত, কেউ মন্দ কাজ চালু করলে তা বন্ধ না হওয়া পর্যন্ত তার পাপের দায় থাকে। তৃতীয়ত, যে ব্যক্তি মুসলিম দেশের সীমানা পাহারা দিতে গিয়ে মৃত্যুবরণ করে, সে পুনরুত্থান পর্যন্ত পাহারারত মুজাহিদের মতো প্রতিদান পেতে থাকে। হাদিসটি মানুষকে দায়িত্বশীল জীবন শেখায়। আমাদের কাজ শুধু বর্তমান সময়ের জন্য নয়; কিছু কাজ মৃত্যুর পরও প্রভাব রেখে যায়। তাই ভালো পথ দেখানো, নিরাপত্তার কাজে থাকা এবং মন্দ কাজ বন্ধে সচেতন থাকা—এসব বিষয় এখানে গুরুত্ব পেয়েছে।"},"teachings":["ভালো কাজের প্রভাব চলতে থাকলে সওয়াবের আশা থাকে।","মন্দ কাজ চালু করলে তা বন্ধ না হওয়া পর্যন্ত দায় চলতে পারে।","দ্বীনের পথে সীমান্ত পাহারা একটি মর্যাদাপূর্ণ কাজ হিসেবে এসেছে।","নিজের কাজের দীর্ঘমেয়াদি প্রভাব নিয়ে ভাবা উচিত।"],"related_hadiths":[{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2500","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E141" s="4" t="n"/>
@@ -3759,12 +3755,12 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জীবদ্দশা ও মৃত্যুর পর ভালো রীতির সওয়াব","description":"$book_name$ $hadith_number$ - $chapter_name$. উত্তম রীতি চালু করলে তা চলতে থাকা পর্যন্ত সওয়াব থাকে; মন্দ কাজ চালু করলে পাপের দায়ও চলতে থাকে।"},"heading":{"title":"উত্তম রীতির চলমান সওয়াব ও সীমান্ত পাহারার প্রতিদান","description":"এই হাদিসে তিনটি বিষয় এসেছে। প্রথমত, কেউ উত্তম রীতি চালু করলে জীবদ্দশায় এবং মৃত্যুর পরও সেই কাজ চলতে থাকলে সে প্রতিদান পেতে থাকে। দ্বিতীয়ত, কেউ মন্দ কাজ চালু করলে তা বন্ধ না হওয়া পর্যন্ত তার পাপের দায় থাকে। তৃতীয়ত, যে ব্যক্তি মুসলিম দেশের সীমানা পাহারা দিতে গিয়ে মৃত্যুবরণ করে, সে পুনরুত্থান পর্যন্ত পাহারারত মুজাহিদের মতো প্রতিদান পেতে থাকে। হাদিসটি মানুষকে দায়িত্বশীল জীবন শেখায়। আমাদের কাজ শুধু বর্তমান সময়ের জন্য নয়; কিছু কাজ মৃত্যুর পরও প্রভাব রেখে যায়। তাই ভালো পথ দেখানো, নিরাপত্তার কাজে থাকা এবং মন্দ কাজ বন্ধে সচেতন থাকা—এসব বিষয় এখানে গুরুত্ব পেয়েছে।"},"teachings":["ভালো কাজের প্রভাব চলতে থাকলে সওয়াবের আশা থাকে।","মন্দ কাজ চালু করলে তা বন্ধ না হওয়া পর্যন্ত দায় চলতে পারে।","দ্বীনের পথে সীমান্ত পাহারা একটি মর্যাদাপূর্ণ কাজ হিসেবে এসেছে।","নিজের কাজের দীর্ঘমেয়াদি প্রভাব নিয়ে ভাবা উচিত।"],"related_hadiths":[{"id":"1017","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2500","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কল্যাণের চাবি ও অকল্যাণের তালা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ যাকে কল্যাণের চাবি ও অকল্যাণের তালা করেন, তার জন্য সুসংবাদ; বিপরীত অবস্থা দুঃখজনক।"},"heading":{"title":"কল্যাণের চাবি হওয়া: মুমিনের সুন্দর দায়িত্ব","description":"এই হাদিসে কল্যাণ ও নেক কাজকে ভান্ডারের সাথে তুলনা করা হয়েছে। প্রতিটি ভান্ডারের যেমন চাবি থাকে, তেমনি মানুষের মধ্যেও কেউ কেউ ভালো কাজের দরজা খুলে দেয়। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, সুসংবাদ সেই ব্যক্তির জন্য, যাকে আল্লাহ কল্যাণের চাবি এবং অকল্যাণের তালা করেছেন। অর্থাৎ তার মাধ্যমে ভালো কাজ সহজ হয় এবং মন্দ কাজের পথ বন্ধ হয়। আবার দুর্ভাগ্য সেই বান্দার জন্য, যে অকল্যাণের চাবি এবং কল্যাণের তালা হয়ে যায়। এই হাদিস আমাদের নিজের ভূমিকা নিয়ে ভাবতে শেখায়। আমরা কথা, আচরণ, পরামর্শ ও উদ্যোগের মাধ্যমে মানুষকে ভালো দিকে নিতে পারি, আবার অসতর্ক হলে খারাপ দিকেও ঠেলে দিতে পারি।"},"teachings":["মানুষের মাধ্যমে ভালো কাজের দরজা খুলতে পারে।","মন্দ কাজ বন্ধ করার চেষ্টা করাও কল্যাণের অংশ।","নিজের কথা ও কাজ অন্যদের ওপর প্রভাব ফেলে।","কল্যাণের চাবি হওয়া মুমিনের সুন্দর লক্ষ্য হতে পারে।"],"related_hadiths":[{"id":"237","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1425","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E142" s="4" t="n"/>
@@ -3782,12 +3778,12 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কল্যাণের চাবি ও অকল্যাণের তালা","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ যাকে কল্যাণের চাবি ও অকল্যাণের তালা করেন, তার জন্য সুসংবাদ; বিপরীত অবস্থা দুঃখজনক।"},"heading":{"title":"কল্যাণের চাবি হওয়া: মুমিনের সুন্দর দায়িত্ব","description":"এই হাদিসে কল্যাণ ও নেক কাজকে ভান্ডারের সাথে তুলনা করা হয়েছে। প্রতিটি ভান্ডারের যেমন চাবি থাকে, তেমনি মানুষের মধ্যেও কেউ কেউ ভালো কাজের দরজা খুলে দেয়। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, সুসংবাদ সেই ব্যক্তির জন্য, যাকে আল্লাহ কল্যাণের চাবি এবং অকল্যাণের তালা করেছেন। অর্থাৎ তার মাধ্যমে ভালো কাজ সহজ হয় এবং মন্দ কাজের পথ বন্ধ হয়। আবার দুর্ভাগ্য সেই বান্দার জন্য, যে অকল্যাণের চাবি এবং কল্যাণের তালা হয়ে যায়। এই হাদিস আমাদের নিজের ভূমিকা নিয়ে ভাবতে শেখায়। আমরা কথা, আচরণ, পরামর্শ ও উদ্যোগের মাধ্যমে মানুষকে ভালো দিকে নিতে পারি, আবার অসতর্ক হলে খারাপ দিকেও ঠেলে দিতে পারি।"},"teachings":["মানুষের মাধ্যমে ভালো কাজের দরজা খুলতে পারে।","মন্দ কাজ বন্ধ করার চেষ্টা করাও কল্যাণের অংশ।","নিজের কথা ও কাজ অন্যদের ওপর প্রভাব ফেলে।","কল্যাণের চাবি হওয়া মুমিনের সুন্দর লক্ষ্য হতে পারে।"],"related_hadiths":[{"id":"237","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1425","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্বীনের গভীর জ্ঞান আল্লাহর কল্যাণের চিহ্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ যার কল্যাণ চান, তাকে দ্বীনের গভীর জ্ঞান দেন; জ্ঞান শেখা ও ফিকহ অর্জনের গুরুত্ব এতে এসেছে।"},"heading":{"title":"দ্বীনের গভীর জ্ঞান লাভ আল্লাহর কল্যাণের নিদর্শন","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, আল্লাহ যার কল্যাণ চান, তাকে দ্বীনের গভীর জ্ঞান দান করেন। বর্ণনায় আরও এসেছে, জ্ঞান শেখার মাধ্যমে পাওয়া যায় এবং ফিকহ বা গভীর বুঝ অর্জিত হয় চেষ্টা ও অনুশীলনের মাধ্যমে। তাই দ্বীনি জ্ঞান কোনো হালকা বিষয় নয়; এটি শেখার, বুঝার এবং আল্লাহভীতির পথে চলার বিষয়। হাদিসে কুরআনের আয়াতও এসেছে যে, আল্লাহকে তাঁর বান্দাদের মধ্যে আলেমরাই ভয় করে চলে। এখানে আলেম বলতে শুধু তথ্য জানা নয়; বরং জ্ঞান থেকে আল্লাহভীতি জন্মানো গুরুত্বপূর্ণ। একজন মুসলিমের জন্য দ্বীনের হালাল-হারাম, আদব, ইবাদত ও দায়িত্ব শেখা জীবনের বড় কল্যাণ।"},"teachings":["দ্বীনের গভীর জ্ঞান আল্লাহর পক্ষ থেকে কল্যাণের বড় নিদর্শন।","জ্ঞান শেখার জন্য চেষ্টা, অধ্যয়ন ও বুঝার অভ্যাস দরকার।","সত্যিকারের জ্ঞান আল্লাহভীতির দিকে নিয়ে যায়।","দ্বীনি বিষয়ে না জেনে চলার বদলে শেখার পথ নেওয়া উচিত।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1037","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"220","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E143" s="4" t="n"/>
@@ -3805,12 +3801,12 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দ্বীনের গভীর জ্ঞান আল্লাহর কল্যাণের চিহ্ন","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহ যার কল্যাণ চান, তাকে দ্বীনের গভীর জ্ঞান দেন; জ্ঞান শেখা ও ফিকহ অর্জনের গুরুত্ব এতে এসেছে।"},"heading":{"title":"দ্বীনের গভীর জ্ঞান লাভ আল্লাহর কল্যাণের নিদর্শন","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, আল্লাহ যার কল্যাণ চান, তাকে দ্বীনের গভীর জ্ঞান দান করেন। বর্ণনায় আরও এসেছে, জ্ঞান শেখার মাধ্যমে পাওয়া যায় এবং ফিকহ বা গভীর বুঝ অর্জিত হয় চেষ্টা ও অনুশীলনের মাধ্যমে। তাই দ্বীনি জ্ঞান কোনো হালকা বিষয় নয়; এটি শেখার, বুঝার এবং আল্লাহভীতির পথে চলার বিষয়। হাদিসে কুরআনের আয়াতও এসেছে যে, আল্লাহকে তাঁর বান্দাদের মধ্যে আলেমরাই ভয় করে চলে। এখানে আলেম বলতে শুধু তথ্য জানা নয়; বরং জ্ঞান থেকে আল্লাহভীতি জন্মানো গুরুত্বপূর্ণ। একজন মুসলিমের জন্য দ্বীনের হালাল-হারাম, আদব, ইবাদত ও দায়িত্ব শেখা জীবনের বড় কল্যাণ।"},"teachings":["দ্বীনের গভীর জ্ঞান আল্লাহর পক্ষ থেকে কল্যাণের বড় নিদর্শন।","জ্ঞান শেখার জন্য চেষ্টা, অধ্যয়ন ও বুঝার অভ্যাস দরকার।","সত্যিকারের জ্ঞান আল্লাহভীতির দিকে নিয়ে যায়।","দ্বীনি বিষয়ে না জেনে চলার বদলে শেখার পথ নেওয়া উচিত।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1037","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"220","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের মর্যাদা ও পরহেজগারিতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবাদতের মর্যাদার চেয়ে বিদ্যার মর্যাদা বেশি বলা হয়েছে, আর দ্বীনের উত্তম বিষয় হিসেবে পরহেজগারিতা এসেছে।"},"heading":{"title":"ইলমের মর্যাদা ও পরহেজগারিতার গুরুত্ব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, ইবাদতের মর্যাদার চেয়ে বিদ্যার মর্যাদা অনেক বেশি। এর সঙ্গে তিনি বলেছেন, তোমাদের দ্বীনের মাঝে উত্তম বিষয় হলো পরহেজগারিতা। এখানে ইলম ও আমলকে আলাদা করে একটিকে বাদ দিয়ে অন্যটি ধরার কথা নয়; বরং সঠিক জ্ঞান ইবাদতকে ঠিক পথে চালায়। কেউ যদি জানে না কীভাবে ইবাদত করতে হয়, কী থেকে বাঁচতে হয়, কীভাবে আল্লাহকে ভয় করতে হয়—তাহলে তার ইবাদতও দুর্বল হতে পারে। আবার জ্ঞান থাকলেও পরহেজগারিতা না থাকলে সেই জ্ঞান জীবনে আলো দেয় না। তাই এই হাদিসে ইলম শেখা এবং হারাম-সন্দেহজনক বিষয় থেকে বাঁচার মানসিকতা—দুটিই গুরুত্বপূর্ণ হয়ে উঠেছে।"},"teachings":["সঠিক ইলম ইবাদতকে সঠিক পথে রাখতে সাহায্য করে।","পরহেজগারিতা দ্বীনি জীবনের গুরুত্বপূর্ণ গুণ।","জ্ঞান শুধু মুখের কথা নয়; তা আচরণে প্রভাব ফেলতে হবে।","ইবাদতের সঙ্গে সঠিক বুঝ ও সতর্কতা জরুরি।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E144" s="4" t="n"/>
@@ -3828,12 +3824,12 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের মর্যাদা ও পরহেজগারিতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইবাদতের মর্যাদার চেয়ে বিদ্যার মর্যাদা বেশি বলা হয়েছে, আর দ্বীনের উত্তম বিষয় হিসেবে পরহেজগারিতা এসেছে।"},"heading":{"title":"ইলমের মর্যাদা ও পরহেজগারিতার গুরুত্ব","description":"এই হাদিসে রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, ইবাদতের মর্যাদার চেয়ে বিদ্যার মর্যাদা অনেক বেশি। এর সঙ্গে তিনি বলেছেন, তোমাদের দ্বীনের মাঝে উত্তম বিষয় হলো পরহেজগারিতা। এখানে ইলম ও আমলকে আলাদা করে একটিকে বাদ দিয়ে অন্যটি ধরার কথা নয়; বরং সঠিক জ্ঞান ইবাদতকে ঠিক পথে চালায়। কেউ যদি জানে না কীভাবে ইবাদত করতে হয়, কী থেকে বাঁচতে হয়, কীভাবে আল্লাহকে ভয় করতে হয়—তাহলে তার ইবাদতও দুর্বল হতে পারে। আবার জ্ঞান থাকলেও পরহেজগারিতা না থাকলে সেই জ্ঞান জীবনে আলো দেয় না। তাই এই হাদিসে ইলম শেখা এবং হারাম-সন্দেহজনক বিষয় থেকে বাঁচার মানসিকতা—দুটিই গুরুত্বপূর্ণ হয়ে উঠেছে।"},"teachings":["সঠিক ইলম ইবাদতকে সঠিক পথে রাখতে সাহায্য করে।","পরহেজগারিতা দ্বীনি জীবনের গুরুত্বপূর্ণ গুণ।","জ্ঞান শুধু মুখের কথা নয়; তা আচরণে প্রভাব ফেলতে হবে।","ইবাদতের সঙ্গে সঠিক বুঝ ও সতর্কতা জরুরি।"],"related_hadiths":[{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মুসলিম ভাইকে সাহায্য ও ইলম অর্জনের ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. বিপদ দূর করা, দোষ গোপন রাখা, অভাবীকে সহজ করা, ইলম শেখা ও কুরআন অধ্যয়নের বড় ফজিলত এসেছে।"},"heading":{"title":"মুসলিম ভাইকে সাহায্য, ইলম অর্জন ও কুরআন অধ্যয়নের ফজিলত","description":"এই হাদিসে বহু গুরুত্বপূর্ণ শিক্ষা একসঙ্গে এসেছে। কোনো মুমিনের দুনিয়ার একটি বিপদ দূর করলে আল্লাহ কিয়ামতের বিপদ থেকে একটি বিপদ দূর করবেন। কোনো মুসলিমের দোষ গোপন রাখলে আল্লাহ দুনিয়া ও আখেরাতে তার দোষ গোপন রাখবেন। ঋণগ্রস্ত বা অভাবীকে সহজ করলে আল্লাহ তার জন্য সহজ করবেন। বান্দা যতক্ষণ ভাইকে সাহায্য করে, আল্লাহও তাকে সাহায্য করেন। এরপর ইলম অর্জনের ফজিলত এসেছে—যে ব্যক্তি বিদ্যা শেখার পথে চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করেন। আল্লাহর ঘরে কুরআন তিলাওয়াত ও অধ্যয়নে প্রশান্তি, রহমত ও ফেরেশতাদের ঘিরে রাখার কথা এসেছে। শেষে বলা হয়েছে, আমল পিছিয়ে দিলে বংশ মর্যাদা এগিয়ে দিতে পারবে না।"},"teachings":["মানুষের বিপদ দূর করা আল্লাহর রহমত লাভের কারণ।","মুসলিমের দোষ গোপন রাখা উত্তম চরিত্রের অংশ।","ইলম অর্জন জান্নাতের পথ সহজ হওয়ার কারণ হিসেবে এসেছে।","বংশ পরিচয় নয়, আমলই মানুষের অগ্রগতির আসল পথ।"],"related_hadiths":[{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"225","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"4946","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E145" s="4" t="n"/>
@@ -3851,12 +3847,12 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মুসলিম ভাইকে সাহায্য ও ইলম অর্জনের ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. বিপদ দূর করা, দোষ গোপন রাখা, অভাবীকে সহজ করা, ইলম শেখা ও কুরআন অধ্যয়নের বড় ফজিলত এসেছে।"},"heading":{"title":"মুসলিম ভাইকে সাহায্য, ইলম অর্জন ও কুরআন অধ্যয়নের ফজিলত","description":"এই হাদিসে বহু গুরুত্বপূর্ণ শিক্ষা একসঙ্গে এসেছে। কোনো মুমিনের দুনিয়ার একটি বিপদ দূর করলে আল্লাহ কিয়ামতের বিপদ থেকে একটি বিপদ দূর করবেন। কোনো মুসলিমের দোষ গোপন রাখলে আল্লাহ দুনিয়া ও আখেরাতে তার দোষ গোপন রাখবেন। ঋণগ্রস্ত বা অভাবীকে সহজ করলে আল্লাহ তার জন্য সহজ করবেন। বান্দা যতক্ষণ ভাইকে সাহায্য করে, আল্লাহও তাকে সাহায্য করেন। এরপর ইলম অর্জনের ফজিলত এসেছে—যে ব্যক্তি বিদ্যা শেখার পথে চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করেন। আল্লাহর ঘরে কুরআন তিলাওয়াত ও অধ্যয়নে প্রশান্তি, রহমত ও ফেরেশতাদের ঘিরে রাখার কথা এসেছে। শেষে বলা হয়েছে, আমল পিছিয়ে দিলে বংশ মর্যাদা এগিয়ে দিতে পারবে না।"},"teachings":["মানুষের বিপদ দূর করা আল্লাহর রহমত লাভের কারণ।","মুসলিমের দোষ গোপন রাখা উত্তম চরিত্রের অংশ।","ইলম অর্জন জান্নাতের পথ সহজ হওয়ার কারণ হিসেবে এসেছে।","বংশ পরিচয় নয়, আমলই মানুষের অগ্রগতির আসল পথ।"],"related_hadiths":[{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"225","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"4946","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য খাঁটি আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি সতর্ক করে, আমলে আল্লাহর সাথে অন্য উদ্দেশ্য মেশালে তা আল্লাহর জন্য খাঁটি থাকে না।"},"heading":{"title":"খাঁটি আমল ও ইখলাস: আল্লাহর জন্য কাজ করার শিক্ষা","description":"এই হাদিসে আল্লাহর জন্য আমল খাঁটি রাখার কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, আল্লাহ বলেন, আমি উত্তম শরীক। কেউ যদি কোনো আমলে আল্লাহর সাথে অন্য কাউকে শরীক করে, তাহলে তা সেই শরীকের জন্যই সাব্যস্ত হবে। এরপর মানুষকে বলা হয়েছে, তোমরা একনিষ্ঠভাবে আমল কর। কারণ আল্লাহ শুধু সেই আমল কবুল করেন, যা তাঁর জন্য খাঁটি করা হয়। হাদিসে উদাহরণ দেওয়া হয়েছে, কেউ যেন না বলে, এই আমল আল্লাহর জন্য এবং আত্মীয়ের জন্য, বা আল্লাহর জন্য এবং মানুষের সন্তুষ্টির জন্য। এই বর্ণনা আমাদের নিয়ত পরীক্ষা করতে শেখায়। বাহ্যিকভাবে কাজ ভালো হলেও যদি উদ্দেশ্যে আল্লাহর সন্তুষ্টির সাথে মানুষের প্রশংসা বা অন্য স্বার্থ মিশে যায়, তাহলে তা বিপদের কারণ হতে পারে। তাই প্রতিটি ইবাদত ও ভালো কাজে ইখলাস রাখা জরুরি।"},"teachings":["আমল আল্লাহর জন্য খাঁটি হওয়া দরকার।","মানুষের সন্তুষ্টি বা আত্মীয়তার উদ্দেশ্য মিশিয়ে আমল করা ঝুঁকিপূর্ণ।","আল্লাহ একনিষ্ঠভাবে করা আমল কবুল করেন।","প্রতিটি ভালো কাজের আগে নিয়ত যাচাই করা দরকার।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"8","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
         </is>
       </c>
       <c r="E146" s="4" t="n"/>
@@ -3874,12 +3870,12 @@
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>70</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আল্লাহর জন্য খাঁটি আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিসটি সতর্ক করে, আমলে আল্লাহর সাথে অন্য উদ্দেশ্য মেশালে তা আল্লাহর জন্য খাঁটি থাকে না।"},"heading":{"title":"খাঁটি আমল ও ইখলাস: আল্লাহর জন্য কাজ করার শিক্ষা","description":"এই হাদিসে আল্লাহর জন্য আমল খাঁটি রাখার কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, আল্লাহ বলেন, আমি উত্তম শরীক। কেউ যদি কোনো আমলে আল্লাহর সাথে অন্য কাউকে শরীক করে, তাহলে তা সেই শরীকের জন্যই সাব্যস্ত হবে। এরপর মানুষকে বলা হয়েছে, তোমরা একনিষ্ঠভাবে আমল কর। কারণ আল্লাহ শুধু সেই আমল কবুল করেন, যা তাঁর জন্য খাঁটি করা হয়। হাদিসে উদাহরণ দেওয়া হয়েছে, কেউ যেন না বলে, এই আমল আল্লাহর জন্য এবং আত্মীয়ের জন্য, বা আল্লাহর জন্য এবং মানুষের সন্তুষ্টির জন্য। এই বর্ণনা আমাদের নিয়ত পরীক্ষা করতে শেখায়। বাহ্যিকভাবে কাজ ভালো হলেও যদি উদ্দেশ্যে আল্লাহর সন্তুষ্টির সাথে মানুষের প্রশংসা বা অন্য স্বার্থ মিশে যায়, তাহলে তা বিপদের কারণ হতে পারে। তাই প্রতিটি ইবাদত ও ভালো কাজে ইখলাস রাখা জরুরি।"},"teachings":["আমল আল্লাহর জন্য খাঁটি হওয়া দরকার।","মানুষের সন্তুষ্টি বা আত্মীয়তার উদ্দেশ্য মিশিয়ে আমল করা ঝুঁকিপূর্ণ।","আল্লাহ একনিষ্ঠভাবে করা আমল কবুল করেন।","প্রতিটি ভালো কাজের আগে নিয়ত যাচাই করা দরকার।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"8","book_id":"8","slug":"riyadus-salihin","label":"রিয়াদুস সালেহীন"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তালেবে ইলম ও আলেমের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলমের পথে চলা, ফেরেশতাদের সম্মান, আলেমের মর্যাদা ও নবীদের উত্তরাধিকার হিসেবে জ্ঞানের কথা এসেছে।"},"heading":{"title":"তালেবে ইলমের মর্যাদা ও আলেমরা নবীদের উত্তরসূরী","description":"এই হাদিসে ইলম অর্জনের মর্যাদা খুব সুন্দরভাবে এসেছে। যে ব্যক্তি জ্ঞানার্জনের উদ্দেশ্যে পথে চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করে দেন। তালেবে ইলমের কাজে সন্তুষ্ট হয়ে ফেরেশতারা তাদের ডানা বিছিয়ে দেন। আসমান ও জমিনের সৃষ্টিরাও আলেমের জন্য ক্ষমা প্রার্থনা করে, এমনকি পানির মাছও। হাদিসে আলেমের মর্যাদাকে আবেদের ওপর চাঁদের মর্যাদার সঙ্গে তুলনা করা হয়েছে। আরও বলা হয়েছে, আলেমরা নবীদের উত্তরসূরী। নবীরা দীনার-দিরহাম রেখে যাননি; তাঁরা রেখে গেছেন ইলম। তাই যে ব্যক্তি এই ইলম গ্রহণ করে, সে বড় অংশ গ্রহণ করে। এখানে জ্ঞানকে দুনিয়াবি সম্পদের চেয়ে বড় উত্তরাধিকার হিসেবে দেখানো হয়েছে।"},"teachings":["ইলম অর্জনের পথ জান্নাতের পথ সহজ হওয়ার কারণ হিসেবে এসেছে।","তালেবে ইলমের মর্যাদা ফেরেশতাদের সম্মানের মাধ্যমে বোঝানো হয়েছে।","আলেমের জ্ঞান মানুষের উপকারে আসে, তাই তার মর্যাদা বড়।","নবীদের আসল উত্তরাধিকার হলো ইলম, অর্থ-সম্পদ নয়।"],"related_hadiths":[{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E147" s="4" t="n"/>
@@ -3897,12 +3893,12 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তালেবে ইলম ও আলেমের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলমের পথে চলা, ফেরেশতাদের সম্মান, আলেমের মর্যাদা ও নবীদের উত্তরাধিকার হিসেবে জ্ঞানের কথা এসেছে।"},"heading":{"title":"তালেবে ইলমের মর্যাদা ও আলেমরা নবীদের উত্তরসূরী","description":"এই হাদিসে ইলম অর্জনের মর্যাদা খুব সুন্দরভাবে এসেছে। যে ব্যক্তি জ্ঞানার্জনের উদ্দেশ্যে পথে চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করে দেন। তালেবে ইলমের কাজে সন্তুষ্ট হয়ে ফেরেশতারা তাদের ডানা বিছিয়ে দেন। আসমান ও জমিনের সৃষ্টিরাও আলেমের জন্য ক্ষমা প্রার্থনা করে, এমনকি পানির মাছও। হাদিসে আলেমের মর্যাদাকে আবেদের ওপর চাঁদের মর্যাদার সঙ্গে তুলনা করা হয়েছে। আরও বলা হয়েছে, আলেমরা নবীদের উত্তরসূরী। নবীরা দীনার-দিরহাম রেখে যাননি; তাঁরা রেখে গেছেন ইলম। তাই যে ব্যক্তি এই ইলম গ্রহণ করে, সে বড় অংশ গ্রহণ করে। এখানে জ্ঞানকে দুনিয়াবি সম্পদের চেয়ে বড় উত্তরাধিকার হিসেবে দেখানো হয়েছে।"},"teachings":["ইলম অর্জনের পথ জান্নাতের পথ সহজ হওয়ার কারণ হিসেবে এসেছে।","তালেবে ইলমের মর্যাদা ফেরেশতাদের সম্মানের মাধ্যমে বোঝানো হয়েছে।","আলেমের জ্ঞান মানুষের উপকারে আসে, তাই তার মর্যাদা বড়।","নবীদের আসল উত্তরাধিকার হলো ইলম, অর্থ-সম্পদ নয়।"],"related_hadiths":[{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান অনুসন্ধানকারীকে স্বাগতম","description":"$book_name$ $hadith_number$ - $chapter_name$. তালেবে ইলমকে রাসূলুল্লাহ স্বাগত জানিয়েছেন; ফেরেশতারা তাকে ঘিরে রাখে ও ডানা দিয়ে ছায়া দেয়।"},"heading":{"title":"জ্ঞান অনুসন্ধানকারীকে স্বাগতম: তালেবে ইলমের সম্মান","description":"এই হাদিসে একজন সাহাবী রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর কাছে এসে বলেন, তিনি জ্ঞানার্জনের উদ্দেশ্যে এসেছেন। তখন নবীজি তাঁকে বলেন, “তালেবে ইলম স্বাগতম।” এই একটি বাক্য থেকেই বোঝা যায়, জ্ঞান অর্জনের নিয়ত নিয়ে আসা ব্যক্তি সম্মান পাওয়ার যোগ্য। হাদিসে আরও বলা হয়েছে, ফেরেশতারা জ্ঞান অনুসন্ধানকারীকে ঘিরে রাখেন এবং তাদের ডানা দিয়ে ছায়া দেন। এমনকি সে যে জিনিস খুঁজছে—ইলম—তার ভালোবাসায় ফেরেশতারা একে অপরের ওপর উঠতে উঠতে দুনিয়ার আসমান পর্যন্ত পৌঁছে যান। এখানে তালেবে ইলমের মর্যাদা, ইলমের প্রতি ভালোবাসা এবং জ্ঞান শেখার জন্য নবীজির উৎসাহ স্পষ্ট হয়েছে।"},"teachings":["জ্ঞান অর্জনের উদ্দেশ্যে আসা ব্যক্তিকে সম্মান করা উচিত।","তালেবে ইলমের জন্য ফেরেশতাদের বিশেষ সম্মানের কথা এসেছে।","ইলম শেখার নিয়ত নিজেই মর্যাদাপূর্ণ কাজ।","দ্বীনি জ্ঞান খোঁজার পথে উৎসাহ দেওয়া নববী শিক্ষা।"],"related_hadiths":[{"id":"226","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E148" s="4" t="n"/>
@@ -3920,12 +3916,12 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞান অনুসন্ধানকারীকে স্বাগতম","description":"$book_name$ $hadith_number$ - $chapter_name$. তালেবে ইলমকে রাসূলুল্লাহ স্বাগত জানিয়েছেন; ফেরেশতারা তাকে ঘিরে রাখে ও ডানা দিয়ে ছায়া দেয়।"},"heading":{"title":"জ্ঞান অনুসন্ধানকারীকে স্বাগতম: তালেবে ইলমের সম্মান","description":"এই হাদিসে একজন সাহাবী রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম)-এর কাছে এসে বলেন, তিনি জ্ঞানার্জনের উদ্দেশ্যে এসেছেন। তখন নবীজি তাঁকে বলেন, “তালেবে ইলম স্বাগতম।” এই একটি বাক্য থেকেই বোঝা যায়, জ্ঞান অর্জনের নিয়ত নিয়ে আসা ব্যক্তি সম্মান পাওয়ার যোগ্য। হাদিসে আরও বলা হয়েছে, ফেরেশতারা জ্ঞান অনুসন্ধানকারীকে ঘিরে রাখেন এবং তাদের ডানা দিয়ে ছায়া দেন। এমনকি সে যে জিনিস খুঁজছে—ইলম—তার ভালোবাসায় ফেরেশতারা একে অপরের ওপর উঠতে উঠতে দুনিয়ার আসমান পর্যন্ত পৌঁছে যান। এখানে তালেবে ইলমের মর্যাদা, ইলমের প্রতি ভালোবাসা এবং জ্ঞান শেখার জন্য নবীজির উৎসাহ স্পষ্ট হয়েছে।"},"teachings":["জ্ঞান অর্জনের উদ্দেশ্যে আসা ব্যক্তিকে সম্মান করা উচিত।","তালেবে ইলমের জন্য ফেরেশতাদের বিশেষ সম্মানের কথা এসেছে।","ইলম শেখার নিয়ত নিজেই মর্যাদাপূর্ণ কাজ।","দ্বীনি জ্ঞান খোঁজার পথে উৎসাহ দেওয়া নববী শিক্ষা।"],"related_hadiths":[{"id":"226","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2682","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয","description":"$book_name$ $hadith_number$ - $chapter_name$. জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয—এই সংক্ষিপ্ত হাদিস দ্বীনি শিক্ষা গ্রহণের গুরুত্ব জানায়।"},"heading":{"title":"জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয: ইলম শেখার দায়িত্ব","description":"এই হাদিস খুব সংক্ষিপ্ত, কিন্তু এর শিক্ষা গভীর। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, জ্ঞানার্জন প্রত্যেক মুসলিম ব্যক্তির উপর ফরয। এখানে জ্ঞান বলতে এমন দ্বীনি জ্ঞান বোঝায়, যা একজন মুসলিমকে সঠিকভাবে চলতে সাহায্য করে—যেমন ঈমান, ইবাদত, হালাল-হারাম, ভালো-মন্দ এবং আল্লাহর আদেশ-নিষেধ জানা। হাদিসটি আমাদের শেখায়, অজ্ঞতার ওপর সন্তুষ্ট থাকা ঠিক নয়। প্রত্যেকের অবস্থান, দায়িত্ব ও প্রয়োজন অনুযায়ী দ্বীনি জ্ঞান শেখা দরকার। কেউ আলেম হবে, কেউ সাধারণভাবে জরুরি জ্ঞান শিখবে—কিন্তু শেখার দরজা সবার জন্য খোলা। তাই ইলম অর্জন শুধু মাদরাসার ছাত্রদের কাজ নয়; প্রত্যেক মুসলিমের জীবনের একটি মৌলিক দায়িত্ব।"},"teachings":["প্রত্যেক মুসলিমের জন্য প্রয়োজনীয় দ্বীনি জ্ঞান শেখা দায়িত্ব।","ইবাদত ও জীবন সঠিক করতে জ্ঞান দরকার।","অজ্ঞতার ওপর সন্তুষ্ট থাকা মুমিনের জন্য ভালো পথ নয়।","নিজ অবস্থান অনুযায়ী ইলম শেখার চেষ্টা করা উচিত।"],"related_hadiths":[{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E149" s="4" t="n"/>
@@ -3943,12 +3939,12 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয","description":"$book_name$ $hadith_number$ - $chapter_name$. জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয—এই সংক্ষিপ্ত হাদিস দ্বীনি শিক্ষা গ্রহণের গুরুত্ব জানায়।"},"heading":{"title":"জ্ঞানার্জন প্রত্যেক মুসলিমের উপর ফরয: ইলম শেখার দায়িত্ব","description":"এই হাদিস খুব সংক্ষিপ্ত, কিন্তু এর শিক্ষা গভীর। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, জ্ঞানার্জন প্রত্যেক মুসলিম ব্যক্তির উপর ফরয। এখানে জ্ঞান বলতে এমন দ্বীনি জ্ঞান বোঝায়, যা একজন মুসলিমকে সঠিকভাবে চলতে সাহায্য করে—যেমন ঈমান, ইবাদত, হালাল-হারাম, ভালো-মন্দ এবং আল্লাহর আদেশ-নিষেধ জানা। হাদিসটি আমাদের শেখায়, অজ্ঞতার ওপর সন্তুষ্ট থাকা ঠিক নয়। প্রত্যেকের অবস্থান, দায়িত্ব ও প্রয়োজন অনুযায়ী দ্বীনি জ্ঞান শেখা দরকার। কেউ আলেম হবে, কেউ সাধারণভাবে জরুরি জ্ঞান শিখবে—কিন্তু শেখার দরজা সবার জন্য খোলা। তাই ইলম অর্জন শুধু মাদরাসার ছাত্রদের কাজ নয়; প্রত্যেক মুসলিমের জীবনের একটি মৌলিক দায়িত্ব।"},"teachings":["প্রত্যেক মুসলিমের জন্য প্রয়োজনীয় দ্বীনি জ্ঞান শেখা দায়িত্ব।","ইবাদত ও জীবন সঠিক করতে জ্ঞান দরকার।","অজ্ঞতার ওপর সন্তুষ্ট থাকা মুমিনের জন্য ভালো পথ নয়।","নিজ অবস্থান অনুযায়ী ইলম শেখার চেষ্টা করা উচিত।"],"related_hadiths":[{"id":"224","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর জারি থাকা সাত আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদ্যা শিক্ষা, নদী-কূপ খনন, গাছ লাগানো, মসজিদ, কুরআন ও সন্তানের দোয়ার সওয়াব জারি থাকে।"},"heading":{"title":"মৃত্যুর পর জারি থাকা সাতটি নেক আমল","description":"এই হাদিসে এমন সাতটি কাজের কথা এসেছে, যার সওয়াব বান্দার মৃত্যুর পর কবরে থাকা অবস্থায়ও জারি থাকে। এগুলো হলো—কাউকে বিদ্যা শিক্ষা দেওয়া, নদী খনন করা, কূপ খনন করা, খেজুর গাছ লাগানো, মসজিদ তৈরি করা, পবিত্র কুরআনের উত্তরাধিকার রেখে যাওয়া এবং এমন সন্তান রেখে যাওয়া যে মৃত্যুর পর তার জন্য ক্ষমা প্রার্থনা করে। এই হাদিস আমাদের শেখায়, কিছু নেক কাজ শুধু এক মুহূর্তের জন্য নয়; মানুষের উপকারে চলতে থাকলে তার সওয়াবও চলতে থাকে। বিশেষ করে উপকারী বিদ্যা, পানির ব্যবস্থা, মসজিদ, কুরআন এবং সৎ সন্তানের দোয়া—এসব দীর্ঘস্থায়ী কল্যাণের পথ। তাই জীবিত অবস্থায় এমন কাজের প্রতি মনোযোগ দেওয়া বুদ্ধিমানের কাজ।"},"teachings":["উপকারী বিদ্যা শেখানো মৃত্যুর পরও সওয়াবের কারণ হতে পারে।","মানুষের পানির ব্যবস্থা করা বড় উপকারী কাজ।","মসজিদ, কুরআন ও সৎ সন্তানের দোয়া দীর্ঘস্থায়ী কল্যাণের পথ।","জীবনে এমন কাজ করা উচিত, যার উপকার মানুষ পেতে থাকে।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E150" s="4" t="n"/>
@@ -3966,12 +3962,12 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>74</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর জারি থাকা সাত আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. বিদ্যা শিক্ষা, নদী-কূপ খনন, গাছ লাগানো, মসজিদ, কুরআন ও সন্তানের দোয়ার সওয়াব জারি থাকে।"},"heading":{"title":"মৃত্যুর পর জারি থাকা সাতটি নেক আমল","description":"এই হাদিসে এমন সাতটি কাজের কথা এসেছে, যার সওয়াব বান্দার মৃত্যুর পর কবরে থাকা অবস্থায়ও জারি থাকে। এগুলো হলো—কাউকে বিদ্যা শিক্ষা দেওয়া, নদী খনন করা, কূপ খনন করা, খেজুর গাছ লাগানো, মসজিদ তৈরি করা, পবিত্র কুরআনের উত্তরাধিকার রেখে যাওয়া এবং এমন সন্তান রেখে যাওয়া যে মৃত্যুর পর তার জন্য ক্ষমা প্রার্থনা করে। এই হাদিস আমাদের শেখায়, কিছু নেক কাজ শুধু এক মুহূর্তের জন্য নয়; মানুষের উপকারে চলতে থাকলে তার সওয়াবও চলতে থাকে। বিশেষ করে উপকারী বিদ্যা, পানির ব্যবস্থা, মসজিদ, কুরআন এবং সৎ সন্তানের দোয়া—এসব দীর্ঘস্থায়ী কল্যাণের পথ। তাই জীবিত অবস্থায় এমন কাজের প্রতি মনোযোগ দেওয়া বুদ্ধিমানের কাজ।"},"teachings":["উপকারী বিদ্যা শেখানো মৃত্যুর পরও সওয়াবের কারণ হতে পারে।","মানুষের পানির ব্যবস্থা করা বড় উপকারী কাজ।","মসজিদ, কুরআন ও সৎ সন্তানের দোয়া দীর্ঘস্থায়ী কল্যাণের পথ।","জীবনে এমন কাজ করা উচিত, যার উপকার মানুষ পেতে থাকে।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া, যিকির ও ইলমের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া ও তার সবকিছুর নিন্দা এসেছে, তবে আল্লাহর যিকির, সংশ্লিষ্ট কাজ, আলেম ও শিক্ষার্থী ব্যতিক্রম।"},"heading":{"title":"দুনিয়ার নিন্দার মাঝে যিকির, আলেম ও শিক্ষার্থীর মর্যাদা","description":"এই হাদিসে দুনিয়ার ব্যাপারে কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুনিয়া অভিশপ্ত এবং এর মধ্যে যা আছে তাও অভিশপ্ত; তবে আল্লাহর যিকির, যিকিরের সঙ্গে সংশ্লিষ্ট বিষয়, আলেম এবং জ্ঞানার্জনকারী এর বাইরে। এই হাদিস দুনিয়াকে পুরোপুরি ছেড়ে দেওয়ার কথা নয়; বরং এমন দুনিয়াবি ব্যস্ততার ব্যাপারে সতর্ক করে, যা মানুষকে আল্লাহ থেকে দূরে নেয়। আল্লাহর স্মরণ, জ্ঞান, শিক্ষা ও আলেমদের কাজ মানুষকে আল্লাহর দিকে ফিরিয়ে নেয়। তাই দুনিয়ার কাজের ভেতরেও যদি আল্লাহর স্মরণ, দ্বীনি শিক্ষা ও উপকারী উদ্দেশ্য থাকে, তা ভিন্ন মর্যাদা পায়। একজন মুমিনের উচিত দুনিয়ার মোহে হারিয়ে না গিয়ে যিকির ও ইলমকে জীবনের আলো বানানো।"},"teachings":["দুনিয়ার মোহ মানুষকে আল্লাহ থেকে দূরে নিতে পারে।","আল্লাহর যিকির দুনিয়ার নিন্দিত ব্যস্ততা থেকে আলাদা মর্যাদার।","আলেম ও জ্ঞানার্জনকারীর বিশেষ মর্যাদা এসেছে।","দুনিয়ার কাজেও আল্লাহর স্মরণ ও সঠিক উদ্দেশ্য রাখা দরকার।"],"related_hadiths":[{"id":"2322","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4112","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"5176","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E151" s="4" t="n"/>
@@ -3989,12 +3985,12 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | দুনিয়া, যিকির ও ইলমের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুনিয়া ও তার সবকিছুর নিন্দা এসেছে, তবে আল্লাহর যিকির, সংশ্লিষ্ট কাজ, আলেম ও শিক্ষার্থী ব্যতিক্রম।"},"heading":{"title":"দুনিয়ার নিন্দার মাঝে যিকির, আলেম ও শিক্ষার্থীর মর্যাদা","description":"এই হাদিসে দুনিয়ার ব্যাপারে কঠিন সতর্কতা এসেছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুনিয়া অভিশপ্ত এবং এর মধ্যে যা আছে তাও অভিশপ্ত; তবে আল্লাহর যিকির, যিকিরের সঙ্গে সংশ্লিষ্ট বিষয়, আলেম এবং জ্ঞানার্জনকারী এর বাইরে। এই হাদিস দুনিয়াকে পুরোপুরি ছেড়ে দেওয়ার কথা নয়; বরং এমন দুনিয়াবি ব্যস্ততার ব্যাপারে সতর্ক করে, যা মানুষকে আল্লাহ থেকে দূরে নেয়। আল্লাহর স্মরণ, জ্ঞান, শিক্ষা ও আলেমদের কাজ মানুষকে আল্লাহর দিকে ফিরিয়ে নেয়। তাই দুনিয়ার কাজের ভেতরেও যদি আল্লাহর স্মরণ, দ্বীনি শিক্ষা ও উপকারী উদ্দেশ্য থাকে, তা ভিন্ন মর্যাদা পায়। একজন মুমিনের উচিত দুনিয়ার মোহে হারিয়ে না গিয়ে যিকির ও ইলমকে জীবনের আলো বানানো।"},"teachings":["দুনিয়ার মোহ মানুষকে আল্লাহ থেকে দূরে নিতে পারে।","আল্লাহর যিকির দুনিয়ার নিন্দিত ব্যস্ততা থেকে আলাদা মর্যাদার।","আলেম ও জ্ঞানার্জনকারীর বিশেষ মর্যাদা এসেছে।","দুনিয়ার কাজেও আল্লাহর স্মরণ ও সঠিক উদ্দেশ্য রাখা দরকার।"],"related_hadiths":[{"id":"2322","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"4112","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"5176","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সৎ ব্যয়ে সম্পদ ও হিকমতের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুই বিষয়ে ঈর্ষণীয় আগ্রহের কথা এসেছে—সত্য পথে সম্পদ ব্যয় এবং হিকমত দিয়ে বিচার ও শিক্ষা।"},"heading":{"title":"সৎ পথে সম্পদ ব্যয় ও হিকমত শেখানোর মর্যাদা","description":"এই হাদিসে “হিংসা” শব্দটি এমন অর্থে এসেছে, যেখানে অন্যের নেয়ামত দেখে তা নষ্ট হওয়ার কামনা নয়; বরং তার মতো ভালো কাজ করার আগ্রহ বোঝানো হয়েছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুটি ক্ষেত্রে এমন আগ্রহ বৈধ। প্রথমত, আল্লাহ কাউকে সম্পদ দিয়েছেন এবং সে তা সৎপথে ব্যয় করার শক্তি পেয়েছে। দ্বিতীয়ত, আল্লাহ কাউকে হিকমত বা প্রজ্ঞা দিয়েছেন; সে তা দিয়ে বিচার-ফয়সালা করে এবং অন্যকে শিক্ষা দেয়। এই হাদিস আমাদের শেখায়, সম্পদ ও জ্ঞান তখনই মূল্যবান, যখন তা আল্লাহর পছন্দনীয় কাজে ব্যবহৃত হয়। শুধু ধনী হওয়া বা জ্ঞানী হওয়া লক্ষ্য নয়; সঠিক ব্যয়, সঠিক সিদ্ধান্ত এবং শিক্ষা দেওয়াই আসল কল্যাণ।"},"teachings":["সম্পদ সৎ পথে ব্যয় করলে তা প্রশংসনীয় নেয়ামত।","হিকমত দিয়ে বিচার করা ও শিক্ষা দেওয়া মর্যাদাপূর্ণ কাজ।","অন্যের ভালো কাজ দেখে নিজেও ভালো করার আগ্রহ রাখা যায়।","নেয়ামতকে আল্লাহর পছন্দনীয় কাজে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"815","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1409","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E152" s="4" t="n"/>
@@ -4012,12 +4008,12 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সৎ ব্যয়ে সম্পদ ও হিকমতের মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. দুই বিষয়ে ঈর্ষণীয় আগ্রহের কথা এসেছে—সত্য পথে সম্পদ ব্যয় এবং হিকমত দিয়ে বিচার ও শিক্ষা।"},"heading":{"title":"সৎ পথে সম্পদ ব্যয় ও হিকমত শেখানোর মর্যাদা","description":"এই হাদিসে “হিংসা” শব্দটি এমন অর্থে এসেছে, যেখানে অন্যের নেয়ামত দেখে তা নষ্ট হওয়ার কামনা নয়; বরং তার মতো ভালো কাজ করার আগ্রহ বোঝানো হয়েছে। রাসূলুল্লাহ (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, দুটি ক্ষেত্রে এমন আগ্রহ বৈধ। প্রথমত, আল্লাহ কাউকে সম্পদ দিয়েছেন এবং সে তা সৎপথে ব্যয় করার শক্তি পেয়েছে। দ্বিতীয়ত, আল্লাহ কাউকে হিকমত বা প্রজ্ঞা দিয়েছেন; সে তা দিয়ে বিচার-ফয়সালা করে এবং অন্যকে শিক্ষা দেয়। এই হাদিস আমাদের শেখায়, সম্পদ ও জ্ঞান তখনই মূল্যবান, যখন তা আল্লাহর পছন্দনীয় কাজে ব্যবহৃত হয়। শুধু ধনী হওয়া বা জ্ঞানী হওয়া লক্ষ্য নয়; সঠিক ব্যয়, সঠিক সিদ্ধান্ত এবং শিক্ষা দেওয়াই আসল কল্যাণ।"},"teachings":["সম্পদ সৎ পথে ব্যয় করলে তা প্রশংসনীয় নেয়ামত।","হিকমত দিয়ে বিচার করা ও শিক্ষা দেওয়া মর্যাদাপূর্ণ কাজ।","অন্যের ভালো কাজ দেখে নিজেও ভালো করার আগ্রহ রাখা যায়।","নেয়ামতকে আল্লাহর পছন্দনীয় কাজে ব্যবহার করা উচিত।"],"related_hadiths":[{"id":"73","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"815","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1409","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম ও হেদায়াত বৃষ্টির মতো","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম ও হেদায়াতকে বৃষ্টির সঙ্গে তুলনা করে গ্রহণকারী, উপকারী ও অগ্রাহ্যকারীর অবস্থা বোঝানো হয়েছে।"},"heading":{"title":"ইলম ও হেদায়াত বৃষ্টির মতো: কারা উপকৃত হয়","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) আল্লাহর পাঠানো ইলম ও হেদায়াতকে বৃষ্টির সঙ্গে তুলনা করেছেন। বৃষ্টি সব জমিতে পড়ে, কিন্তু সব জমির ফল একরকম হয় না। ভালো মাটি পানি গ্রহণ করে এবং অনেক ঘাস-উদ্ভিদ জন্মায়। আরেক ধরনের মাটি পানি ধরে রাখে; নিজে ফসল না ফলালেও মানুষ সেই পানি পান করে, সেচ দেয় ও চাষ করে। তৃতীয় ধরনের মাটি পানি ধরে না এবং কিছু জন্মায়ও না। এই উদাহরণে প্রথম দুই ধরনের মানুষ হলো তারা, যারা দ্বীনের জ্ঞান বুঝে, উপকৃত হয়, শেখে এবং অন্যকে শেখায়। আর তৃতীয় ধরনের মানুষ হলো তারা, যারা হেদায়াত গ্রহণ করে না। হাদিসটি ইলম গ্রহণ, তা থেকে উপকৃত হওয়া এবং অন্যকে শেখানোর গুরুত্ব বোঝায়।"},"teachings":["ইলম ও হেদায়াত গ্রহণ করলে মানুষ নিজেও উপকৃত হয়।","শেখা জ্ঞান অন্যকে শেখানো বড় উপকারী কাজ।","হেদায়াত অগ্রাহ্য করলে মানুষ বৃষ্টিহীন জমির মতো অনুপকারী হয়ে পড়ে।","জ্ঞান শুধু রাখা নয়; তা কাজে লাগানোও জরুরি।"],"related_hadiths":[{"id":"79","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2282","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E153" s="4" t="n"/>
@@ -4035,12 +4031,12 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম ও হেদায়াত বৃষ্টির মতো","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম ও হেদায়াতকে বৃষ্টির সঙ্গে তুলনা করে গ্রহণকারী, উপকারী ও অগ্রাহ্যকারীর অবস্থা বোঝানো হয়েছে।"},"heading":{"title":"ইলম ও হেদায়াত বৃষ্টির মতো: কারা উপকৃত হয়","description":"এই হাদিসে নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) আল্লাহর পাঠানো ইলম ও হেদায়াতকে বৃষ্টির সঙ্গে তুলনা করেছেন। বৃষ্টি সব জমিতে পড়ে, কিন্তু সব জমির ফল একরকম হয় না। ভালো মাটি পানি গ্রহণ করে এবং অনেক ঘাস-উদ্ভিদ জন্মায়। আরেক ধরনের মাটি পানি ধরে রাখে; নিজে ফসল না ফলালেও মানুষ সেই পানি পান করে, সেচ দেয় ও চাষ করে। তৃতীয় ধরনের মাটি পানি ধরে না এবং কিছু জন্মায়ও না। এই উদাহরণে প্রথম দুই ধরনের মানুষ হলো তারা, যারা দ্বীনের জ্ঞান বুঝে, উপকৃত হয়, শেখে এবং অন্যকে শেখায়। আর তৃতীয় ধরনের মানুষ হলো তারা, যারা হেদায়াত গ্রহণ করে না। হাদিসটি ইলম গ্রহণ, তা থেকে উপকৃত হওয়া এবং অন্যকে শেখানোর গুরুত্ব বোঝায়।"},"teachings":["ইলম ও হেদায়াত গ্রহণ করলে মানুষ নিজেও উপকৃত হয়।","শেখা জ্ঞান অন্যকে শেখানো বড় উপকারী কাজ।","হেদায়াত অগ্রাহ্য করলে মানুষ বৃষ্টিহীন জমির মতো অনুপকারী হয়ে পড়ে।","জ্ঞান শুধু রাখা নয়; তা কাজে লাগানোও জরুরি।"],"related_hadiths":[{"id":"79","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2282","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"71","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর পৌঁছানো আমল ও নেকি","description":"$book_name$ $hadith_number$ - $chapter_name$. শেখানো ইলম, সৎ সন্তান, কুরআন, মসজিদ, মুসাফিরের ঘর, নদী ও সাদকার সওয়াব মৃত্যুর পরও পৌঁছে।"},"heading":{"title":"মৃত্যুর পর পৌঁছানো নেক আমল: ইলম, সাদকা ও সৎ সন্তান","description":"এই হাদিসে বলা হয়েছে, মুমিনের মৃত্যুর পরও কিছু আমল ও নেকির সওয়াব তার কাছে পৌঁছতে থাকে। এর মধ্যে আছে—যে ইলম সে শিক্ষা দিয়েছে ও প্রচার করেছে, সৎ সন্তান রেখে গেছে, এমন কুরআন রেখে গেছে যা মানুষ উপকারে নেয়, মসজিদ নির্মাণ করেছে, মুসাফিরদের জন্য ঘর তৈরি করেছে, নদী প্রবাহিত করেছে বা জীবিত ও সুস্থ অবস্থায় নিজের সম্পদ থেকে সাদকা করেছে। এই হাদিস মানুষকে দীর্ঘস্থায়ী নেক কাজের দিকে ডাকে। জীবনের সম্পদ, জ্ঞান ও সময় যদি এমন কাজে ব্যয় হয়, যা মানুষের উপকারে চলতে থাকে, তাহলে মৃত্যুর পরও তার কল্যাণ পৌঁছার আশা থাকে। তাই শুধু আজকের কাজ নয়, ভবিষ্যতের উপকারও ভাবা উচিত।"},"teachings":["শেখানো ও প্রচার করা উপকারী ইলম মৃত্যুর পরও সওয়াবের কারণ হতে পারে।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী।","মসজিদ, মুসাফিরের ঘর, নদী ও সাদকা দীর্ঘস্থায়ী নেক কাজ।","জীবিত অবস্থায় স্থায়ী কল্যাণের কাজ করা উচিত।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E154" s="4" t="n"/>
@@ -4058,12 +4054,12 @@
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর পৌঁছানো আমল ও নেকি","description":"$book_name$ $hadith_number$ - $chapter_name$. শেখানো ইলম, সৎ সন্তান, কুরআন, মসজিদ, মুসাফিরের ঘর, নদী ও সাদকার সওয়াব মৃত্যুর পরও পৌঁছে।"},"heading":{"title":"মৃত্যুর পর পৌঁছানো নেক আমল: ইলম, সাদকা ও সৎ সন্তান","description":"এই হাদিসে বলা হয়েছে, মুমিনের মৃত্যুর পরও কিছু আমল ও নেকির সওয়াব তার কাছে পৌঁছতে থাকে। এর মধ্যে আছে—যে ইলম সে শিক্ষা দিয়েছে ও প্রচার করেছে, সৎ সন্তান রেখে গেছে, এমন কুরআন রেখে গেছে যা মানুষ উপকারে নেয়, মসজিদ নির্মাণ করেছে, মুসাফিরদের জন্য ঘর তৈরি করেছে, নদী প্রবাহিত করেছে বা জীবিত ও সুস্থ অবস্থায় নিজের সম্পদ থেকে সাদকা করেছে। এই হাদিস মানুষকে দীর্ঘস্থায়ী নেক কাজের দিকে ডাকে। জীবনের সম্পদ, জ্ঞান ও সময় যদি এমন কাজে ব্যয় হয়, যা মানুষের উপকারে চলতে থাকে, তাহলে মৃত্যুর পরও তার কল্যাণ পৌঁছার আশা থাকে। তাই শুধু আজকের কাজ নয়, ভবিষ্যতের উপকারও ভাবা উচিত।"},"teachings":["শেখানো ও প্রচার করা উপকারী ইলম মৃত্যুর পরও সওয়াবের কারণ হতে পারে।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী।","মসজিদ, মুসাফিরের ঘর, নদী ও সাদকা দীর্ঘস্থায়ী নেক কাজ।","জীবিত অবস্থায় স্থায়ী কল্যাণের কাজ করা উচিত।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তিন আমল মৃত্যুর পরও বন্ধ হয় না","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ মারা গেলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া বাকি থাকে।"},"heading":{"title":"তিনটি আমল মৃত্যুর পরও জারি থাকে","description":"এই প্রসিদ্ধ হাদিসে বলা হয়েছে, আদম সন্তান যখন মারা যায়, তখন তার সব আমল বন্ধ হয়ে যায়—তিনটি ছাড়া। প্রথমটি সাদকায়ে জারিয়া, অর্থাৎ এমন সাদকা যার উপকার চলতে থাকে। দ্বিতীয়টি উপকারী বিদ্যা, যার মাধ্যমে মানুষ উপকার পায়। তৃতীয়টি সৎ সন্তান, যে তার জন্য দোয়া করে। এই হাদিস আমাদের জীবনকে লক্ষ্যভিত্তিক করে। মানুষ দুনিয়া থেকে চলে গেলেও কিছু কাজের প্রভাব থেকে যায়। তাই এমন সাদকা করা, এমন জ্ঞান শেখানো বা রেখে যাওয়া, এবং সন্তানকে নেক পথে গড়ে তোলার চেষ্টা করা—এসব বড় মূল্যবান কাজ। এখানে অতিরঞ্জিত আশ্বাস নয়; বরং হাদিসে যে তিন পথ বলা হয়েছে, সেগুলোর গুরুত্ব স্পষ্টভাবে বোঝানো হয়েছে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায়।","সাদকায়ে জারিয়া চলমান সওয়াবের একটি পথ।","উপকারী বিদ্যা মানুষের উপকারে থাকলে সওয়াবের কারণ হয়।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2880","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1376","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
         </is>
       </c>
       <c r="E155" s="4" t="n"/>
@@ -4081,12 +4077,12 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>79</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | তিন আমল মৃত্যুর পরও বন্ধ হয় না","description":"$book_name$ $hadith_number$ - $chapter_name$. মানুষ মারা গেলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া বাকি থাকে।"},"heading":{"title":"তিনটি আমল মৃত্যুর পরও জারি থাকে","description":"এই প্রসিদ্ধ হাদিসে বলা হয়েছে, আদম সন্তান যখন মারা যায়, তখন তার সব আমল বন্ধ হয়ে যায়—তিনটি ছাড়া। প্রথমটি সাদকায়ে জারিয়া, অর্থাৎ এমন সাদকা যার উপকার চলতে থাকে। দ্বিতীয়টি উপকারী বিদ্যা, যার মাধ্যমে মানুষ উপকার পায়। তৃতীয়টি সৎ সন্তান, যে তার জন্য দোয়া করে। এই হাদিস আমাদের জীবনকে লক্ষ্যভিত্তিক করে। মানুষ দুনিয়া থেকে চলে গেলেও কিছু কাজের প্রভাব থেকে যায়। তাই এমন সাদকা করা, এমন জ্ঞান শেখানো বা রেখে যাওয়া, এবং সন্তানকে নেক পথে গড়ে তোলার চেষ্টা করা—এসব বড় মূল্যবান কাজ। এখানে অতিরঞ্জিত আশ্বাস নয়; বরং হাদিসে যে তিন পথ বলা হয়েছে, সেগুলোর গুরুত্ব স্পষ্টভাবে বোঝানো হয়েছে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায়।","সাদকায়ে জারিয়া চলমান সওয়াবের একটি পথ।","উপকারী বিদ্যা মানুষের উপকারে থাকলে সওয়াবের কারণ হয়।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য উপকারী।"],"related_hadiths":[{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"2880","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"1376","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর রেখে যাওয়া সেরা তিন সম্পদ","description":"$book_name$ $hadith_number$ - $chapter_name$. নেক সন্তান, চলমান সাদকা এবং এমন ইলম যা মৃত্যুর পরও আমল করা হয়—এগুলো সেরা রেখে যাওয়া বিষয়।"},"heading":{"title":"মৃত্যুর পর রেখে যাওয়া সেরা তিন জিনিস","description":"এই হাদিসে বলা হয়েছে, একজন মানুষ মৃত্যুর পর যা রেখে যায়, তার মধ্যে উত্তম তিনটি বিষয় হলো—নেক সন্তান যে তার জন্য দোয়া করে, এমন সাদকা যার মাধ্যমে মানুষ উপকৃত হতে থাকে এবং এমন ইলম যার ওপর মৃত্যুর পরও আমল করা হয়। এই শিক্ষা আমাদের দুনিয়ার সম্পদ ও সাফল্যকে নতুনভাবে ভাবতে শেখায়। মানুষ অনেক কিছু রেখে যায়, কিন্তু সবকিছু তার আখেরাতের উপকারে আসে না। যে সন্তান দোয়া করে, যে সাদকা মানুষের কাজে লাগে এবং যে জ্ঞান মানুষকে ভালো পথে চালায়—এসব দীর্ঘস্থায়ী কল্যাণ। তাই জীবনে সম্পদ, সময় ও শিক্ষা এমনভাবে ব্যবহার করা দরকার, যাতে মৃত্যুর পরও মানুষের উপকারের দরজা খোলা থাকে।"},"teachings":["নেক সন্তান রেখে যাওয়া বড় কল্যাণের পথ।","চলমান সাদকা মানুষের উপকারে থাকলে প্রতিদানের কারণ হতে পারে।","যে ইলম অনুযায়ী মানুষ আমল করে, তা দীর্ঘস্থায়ী নেক কাজ।","মৃত্যুর পর কী রেখে যাচ্ছি—এটি একজন মুমিনের ভাবনার বিষয়।"],"related_hadiths":[{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E156" s="4" t="n"/>
@@ -4104,12 +4100,12 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পর রেখে যাওয়া সেরা তিন সম্পদ","description":"$book_name$ $hadith_number$ - $chapter_name$. নেক সন্তান, চলমান সাদকা এবং এমন ইলম যা মৃত্যুর পরও আমল করা হয়—এগুলো সেরা রেখে যাওয়া বিষয়।"},"heading":{"title":"মৃত্যুর পর রেখে যাওয়া সেরা তিন জিনিস","description":"এই হাদিসে বলা হয়েছে, একজন মানুষ মৃত্যুর পর যা রেখে যায়, তার মধ্যে উত্তম তিনটি বিষয় হলো—নেক সন্তান যে তার জন্য দোয়া করে, এমন সাদকা যার মাধ্যমে মানুষ উপকৃত হতে থাকে এবং এমন ইলম যার ওপর মৃত্যুর পরও আমল করা হয়। এই শিক্ষা আমাদের দুনিয়ার সম্পদ ও সাফল্যকে নতুনভাবে ভাবতে শেখায়। মানুষ অনেক কিছু রেখে যায়, কিন্তু সবকিছু তার আখেরাতের উপকারে আসে না। যে সন্তান দোয়া করে, যে সাদকা মানুষের কাজে লাগে এবং যে জ্ঞান মানুষকে ভালো পথে চালায়—এসব দীর্ঘস্থায়ী কল্যাণ। তাই জীবনে সম্পদ, সময় ও শিক্ষা এমনভাবে ব্যবহার করা দরকার, যাতে মৃত্যুর পরও মানুষের উপকারের দরজা খোলা থাকে।"},"teachings":["নেক সন্তান রেখে যাওয়া বড় কল্যাণের পথ।","চলমান সাদকা মানুষের উপকারে থাকলে প্রতিদানের কারণ হতে পারে।","যে ইলম অনুযায়ী মানুষ আমল করে, তা দীর্ঘস্থায়ী নেক কাজ।","মৃত্যুর পর কী রেখে যাচ্ছি—এটি একজন মুমিনের ভাবনার বিষয়।"],"related_hadiths":[{"id":"241","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"1631","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"242","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সওয়াবের জন্য খাঁটি নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. যুদ্ধের মতো বড় আমলেও প্রশংসার উদ্দেশ্য মিশলে প্রতিদান নষ্ট হতে পারে—এই হাদিস সেটিই শেখায়।"},"heading":{"title":"সওয়াব ও প্রশংসা: আমলে ইখলাসের কঠিন পরীক্ষা","description":"এই হাদিসে একজন ব্যক্তি নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে এমন একজনের ব্যাপারে জানতে চান, যে সওয়াব ও প্রশংসা পাওয়ার উদ্দেশ্যে যুদ্ধ করে। নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, তার জন্য কোনো প্রতিদান নেই। লোকটি তিনবার একই প্রশ্ন করে, আর প্রতিবারই একই উত্তর দেওয়া হয়। শেষে তিনি বলেন, আল্লাহ সেই আমলই কবুল করেন, যা তাঁর জন্য খাঁটি এবং তাঁর সন্তুষ্টির উদ্দেশ্যে করা হয়। এই হাদিস আমলের ভেতরের উদ্দেশ্যকে সামনে আনে। বাহ্যিকভাবে কাজ বড় হলেও, যদি নিয়তে মানুষের নাম, প্রশংসা বা পরিচিতি পাওয়ার আকাঙ্ক্ষা থাকে, তাহলে তা আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা হতে পারে। তাই ইখলাস শুধু ছোট আমলে নয়, বড় ত্যাগের কাজেও জরুরি।"},"teachings":["সওয়াবের সাথে মানুষের প্রশংসা চাওয়া আমলকে ক্ষতিগ্রস্ত করতে পারে।","আল্লাহর কাছে কবুল হওয়ার জন্য আমল খাঁটি হওয়া দরকার।","বড় কাজ হলেও নিয়ত ভুল হলে প্রতিদানের আশা দুর্বল হয়।","একই প্রশ্নে নবীর পুনরাবৃত্ত উত্তর বিষয়টির গুরুত্ব দেখায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E157" s="4" t="n"/>
@@ -4127,12 +4123,12 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>80</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | সওয়াবের জন্য খাঁটি নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. যুদ্ধের মতো বড় আমলেও প্রশংসার উদ্দেশ্য মিশলে প্রতিদান নষ্ট হতে পারে—এই হাদিস সেটিই শেখায়।"},"heading":{"title":"সওয়াব ও প্রশংসা: আমলে ইখলাসের কঠিন পরীক্ষা","description":"এই হাদিসে একজন ব্যক্তি নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লামের কাছে এমন একজনের ব্যাপারে জানতে চান, যে সওয়াব ও প্রশংসা পাওয়ার উদ্দেশ্যে যুদ্ধ করে। নবী সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেন, তার জন্য কোনো প্রতিদান নেই। লোকটি তিনবার একই প্রশ্ন করে, আর প্রতিবারই একই উত্তর দেওয়া হয়। শেষে তিনি বলেন, আল্লাহ সেই আমলই কবুল করেন, যা তাঁর জন্য খাঁটি এবং তাঁর সন্তুষ্টির উদ্দেশ্যে করা হয়। এই হাদিস আমলের ভেতরের উদ্দেশ্যকে সামনে আনে। বাহ্যিকভাবে কাজ বড় হলেও, যদি নিয়তে মানুষের নাম, প্রশংসা বা পরিচিতি পাওয়ার আকাঙ্ক্ষা থাকে, তাহলে তা আল্লাহর কাছে গ্রহণযোগ্যতার পথে বাধা হতে পারে। তাই ইখলাস শুধু ছোট আমলে নয়, বড় ত্যাগের কাজেও জরুরি।"},"teachings":["সওয়াবের সাথে মানুষের প্রশংসা চাওয়া আমলকে ক্ষতিগ্রস্ত করতে পারে।","আল্লাহর কাছে কবুল হওয়ার জন্য আমল খাঁটি হওয়া দরকার।","বড় কাজ হলেও নিয়ত ভুল হলে প্রতিদানের আশা দুর্বল হয়।","একই প্রশ্নে নবীর পুনরাবৃত্ত উত্তর বিষয়টির গুরুত্ব দেখায়।"],"related_hadiths":[{"id":"1","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"4821","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের জ্ঞান শিক্ষা দেওয়ার প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ইসলামের জ্ঞান শেখায়, আমলকারীর মতো প্রতিদান পায়; এতে আমলকারীর সওয়াব কমে না।"},"heading":{"title":"ইসলামের জ্ঞান শিক্ষা দেওয়ার প্রতিদান","description":"এই হাদিসে ইসলামের জ্ঞান শিক্ষা দেওয়ার বড় ফজিলত এসেছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি ইসলামের জ্ঞান শিক্ষা দেয়, সে সেই জ্ঞান অনুযায়ী আমলকারীর অনুরূপ প্রতিদান লাভ করবে। তবে আমলকারীর প্রতিদান কোনো অংশে কমে যাবে না। এই শিক্ষা খুব সুন্দর ও আশাব্যঞ্জক। একজন মানুষ নিজে ভালো কাজ করে সওয়াব পেতে পারে; আবার অন্যকে সঠিক জ্ঞান শেখালে, সে ব্যক্তি যখন আমল করে, শিক্ষাদানকারীও প্রতিদানের অংশ পায়। তাই দ্বীনি জ্ঞান শিখে তা নিরাপদ, সঠিক ও উপকারীভাবে অন্যকে শেখানো বড় কল্যাণের কাজ। তবে জ্ঞান শেখানোর ক্ষেত্রে সতর্কতা দরকার, যেন ভুল কথা আল্লাহর নামে বলা না হয়।"},"teachings":["ইসলামের জ্ঞান শেখানো বড় নেক কাজ।","শিক্ষার্থী সেই জ্ঞান অনুযায়ী আমল করলে শিক্ষকও প্রতিদানের আশা করতে পারে।","আমলকারীর সওয়াব কমে না; আল্লাহর দান প্রশস্ত।","দ্বীনি জ্ঞান শেখাতে হলে সঠিকতা ও সতর্কতা জরুরি।"],"related_hadiths":[{"id":"240","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E158" s="4" t="n"/>
@@ -4150,12 +4146,12 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইসলামের জ্ঞান শিক্ষা দেওয়ার প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ইসলামের জ্ঞান শেখায়, আমলকারীর মতো প্রতিদান পায়; এতে আমলকারীর সওয়াব কমে না।"},"heading":{"title":"ইসলামের জ্ঞান শিক্ষা দেওয়ার প্রতিদান","description":"এই হাদিসে ইসলামের জ্ঞান শিক্ষা দেওয়ার বড় ফজিলত এসেছে। নবী (সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম) বলেছেন, যে ব্যক্তি ইসলামের জ্ঞান শিক্ষা দেয়, সে সেই জ্ঞান অনুযায়ী আমলকারীর অনুরূপ প্রতিদান লাভ করবে। তবে আমলকারীর প্রতিদান কোনো অংশে কমে যাবে না। এই শিক্ষা খুব সুন্দর ও আশাব্যঞ্জক। একজন মানুষ নিজে ভালো কাজ করে সওয়াব পেতে পারে; আবার অন্যকে সঠিক জ্ঞান শেখালে, সে ব্যক্তি যখন আমল করে, শিক্ষাদানকারীও প্রতিদানের অংশ পায়। তাই দ্বীনি জ্ঞান শিখে তা নিরাপদ, সঠিক ও উপকারীভাবে অন্যকে শেখানো বড় কল্যাণের কাজ। তবে জ্ঞান শেখানোর ক্ষেত্রে সতর্কতা দরকার, যেন ভুল কথা আল্লাহর নামে বলা না হয়।"},"teachings":["ইসলামের জ্ঞান শেখানো বড় নেক কাজ।","শিক্ষার্থী সেই জ্ঞান অনুযায়ী আমল করলে শিক্ষকও প্রতিদানের আশা করতে পারে।","আমলকারীর সওয়াব কমে না; আল্লাহর দান প্রশস্ত।","দ্বীনি জ্ঞান শেখাতে হলে সঠিকতা ও সতর্কতা জরুরি।"],"related_hadiths":[{"id":"240","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"2699","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"1893","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আলেমের মর্যাদা ও কল্যাণ শেখানোর ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. আলেমের মর্যাদা, কল্যাণ শেখানোর মূল্য এবং সৃষ্টির দোয়ার কথা এই হাদিসে সুন্দরভাবে এসেছে।"},"heading":{"title":"আলেমের মর্যাদা: কল্যাণ শেখানোর বড় ফজিলত","description":"এই হাদিসের মূল শিক্ষা হলো ইলমের মর্যাদা এবং মানুষকে কল্যাণ শেখানোর ফজিলত। এখানে একজন সাধারণ আবেদ ও একজন আলেমের কথা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে উল্লেখ করা হয়। তিনি আলেমের মর্যাদাকে খুব উঁচু করে তুলে ধরেছেন। এরপর তিনি বলেন, আল্লাহ, ফেরেশতাগণ, আসমান-যমীনের অধিবাসী, এমনকি গর্তের পিঁপড়া ও পানির মাছও মানুষকে ভালো শিক্ষা দেওয়ার জন্য দোয়া করে। তাই এই হাদিস আমাদের শেখায়, শুধু নিজে ইবাদত করাই নয়; সঠিক জ্ঞান নিয়ে মানুষকে ভালো পথে ডাকা, হালাল-হারাম শেখানো এবং উপকারী কথা পৌঁছে দেওয়া বড় কল্যাণের কাজ।"},"teachings":["আলেমের মর্যাদা সাধারণ ইবাদতকারীর চেয়ে বেশি বলে হাদিসে এসেছে।","মানুষকে কল্যাণ শেখানো এমন কাজ, যার জন্য সৃষ্টিজগতের দোয়ার কথা বলা হয়েছে।","ইলম শুধু নিজের জন্য নয়; তা মানুষের উপকারে লাগানো উচিত।","ভালো শিক্ষা দেওয়া আল্লাহর কাছে প্রিয় ও সম্মানিত কাজ।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E159" s="4" t="n"/>
@@ -4173,12 +4169,12 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | আলেমের মর্যাদা ও কল্যাণ শেখানোর ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. আলেমের মর্যাদা, কল্যাণ শেখানোর মূল্য এবং সৃষ্টির দোয়ার কথা এই হাদিসে সুন্দরভাবে এসেছে।"},"heading":{"title":"আলেমের মর্যাদা: কল্যাণ শেখানোর বড় ফজিলত","description":"এই হাদিসের মূল শিক্ষা হলো ইলমের মর্যাদা এবং মানুষকে কল্যাণ শেখানোর ফজিলত। এখানে একজন সাধারণ আবেদ ও একজন আলেমের কথা রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর কাছে উল্লেখ করা হয়। তিনি আলেমের মর্যাদাকে খুব উঁচু করে তুলে ধরেছেন। এরপর তিনি বলেন, আল্লাহ, ফেরেশতাগণ, আসমান-যমীনের অধিবাসী, এমনকি গর্তের পিঁপড়া ও পানির মাছও মানুষকে ভালো শিক্ষা দেওয়ার জন্য দোয়া করে। তাই এই হাদিস আমাদের শেখায়, শুধু নিজে ইবাদত করাই নয়; সঠিক জ্ঞান নিয়ে মানুষকে ভালো পথে ডাকা, হালাল-হারাম শেখানো এবং উপকারী কথা পৌঁছে দেওয়া বড় কল্যাণের কাজ।"},"teachings":["আলেমের মর্যাদা সাধারণ ইবাদতকারীর চেয়ে বেশি বলে হাদিসে এসেছে।","মানুষকে কল্যাণ শেখানো এমন কাজ, যার জন্য সৃষ্টিজগতের দোয়ার কথা বলা হয়েছে।","ইলম শুধু নিজের জন্য নয়; তা মানুষের উপকারে লাগানো উচিত।","ভালো শিক্ষা দেওয়া আল্লাহর কাছে প্রিয় ও সম্মানিত কাজ।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কল্যাণের শিক্ষকের জন্য ক্ষমা প্রার্থনা","description":"$book_name$ $hadith_number$ - $chapter_name$. কল্যাণ শেখানো এমন উপকারী কাজ, যার জন্য সমুদ্রের মাছসহ সৃষ্টির ক্ষমা প্রার্থনার কথা এসেছে।"},"heading":{"title":"কল্যাণের শিক্ষক: সৃষ্টির ক্ষমা প্রার্থনার হাদিস","description":"এই হাদিসে খুব সংক্ষেপে কিন্তু গভীর একটি শিক্ষা আছে। যে ব্যক্তি মানুষকে কল্যাণ শেখায়, তার জন্য প্রত্যেক বস্তু ক্ষমা প্রার্থনা করে—এমনকি সমুদ্রের মাছও। এখানে মূল বিষয় হলো ভালো শিক্ষা, উপকারী ইলম এবং মানুষের কল্যাণে কথা বলা। কল্যাণের শিক্ষক শুধু বই পড়ানো ব্যক্তি নন; যে মানুষকে সৎ পথ, ভালো কাজ, হালাল-হারাম বা উপকারী জ্ঞান শেখায়, সে এই অর্থের মধ্যে আসে। তবে ব্যাখ্যাটি হাদিসের কথার মধ্যেই সীমিত রাখা উচিত। এই হাদিস আমাদের মনে করিয়ে দেয়, জ্ঞানকে ভালো কাজে ব্যবহার করলে তা শুধু নিজের জন্য নয়, অন্যদের জন্যও উপকারী হয়।"},"teachings":["কল্যাণ শেখানো ক্ষমা প্রার্থনার কারণ হিসেবে হাদিসে এসেছে।","উপকারী ইলম মানুষের জীবনে ভালো প্রভাব ফেলে।","ভালো কথা ও সঠিক শিক্ষা ছড়িয়ে দেওয়া সম্মানিত কাজ।","জ্ঞান যেন মানুষের ক্ষতি নয়, কল্যাণের জন্য ব্যবহার হয়।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E160" s="4" t="n"/>
@@ -4196,12 +4192,12 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কল্যাণের শিক্ষকের জন্য ক্ষমা প্রার্থনা","description":"$book_name$ $hadith_number$ - $chapter_name$. কল্যাণ শেখানো এমন উপকারী কাজ, যার জন্য সমুদ্রের মাছসহ সৃষ্টির ক্ষমা প্রার্থনার কথা এসেছে।"},"heading":{"title":"কল্যাণের শিক্ষক: সৃষ্টির ক্ষমা প্রার্থনার হাদিস","description":"এই হাদিসে খুব সংক্ষেপে কিন্তু গভীর একটি শিক্ষা আছে। যে ব্যক্তি মানুষকে কল্যাণ শেখায়, তার জন্য প্রত্যেক বস্তু ক্ষমা প্রার্থনা করে—এমনকি সমুদ্রের মাছও। এখানে মূল বিষয় হলো ভালো শিক্ষা, উপকারী ইলম এবং মানুষের কল্যাণে কথা বলা। কল্যাণের শিক্ষক শুধু বই পড়ানো ব্যক্তি নন; যে মানুষকে সৎ পথ, ভালো কাজ, হালাল-হারাম বা উপকারী জ্ঞান শেখায়, সে এই অর্থের মধ্যে আসে। তবে ব্যাখ্যাটি হাদিসের কথার মধ্যেই সীমিত রাখা উচিত। এই হাদিস আমাদের মনে করিয়ে দেয়, জ্ঞানকে ভালো কাজে ব্যবহার করলে তা শুধু নিজের জন্য নয়, অন্যদের জন্যও উপকারী হয়।"},"teachings":["কল্যাণ শেখানো ক্ষমা প্রার্থনার কারণ হিসেবে হাদিসে এসেছে।","উপকারী ইলম মানুষের জীবনে ভালো প্রভাব ফেলে।","ভালো কথা ও সঠিক শিক্ষা ছড়িয়ে দেওয়া সম্মানিত কাজ।","জ্ঞান যেন মানুষের ক্ষতি নয়, কল্যাণের জন্য ব্যবহার হয়।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীর মীরাস হলো ইলম","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে নামাজ, কুরআন পাঠ ও হালাল-হারামের আলোচনা—এগুলোই নবীজির মীরাস হিসেবে বোঝানো হয়েছে।"},"heading":{"title":"নবীর মীরাস: মসজিদে ইলম, কুরআন ও হালাল-হারাম শিক্ষা","description":"এই বর্ণনায় আবু হুরায়রা রাদিয়াল্লাহু আনহু মদীনার বাজারের লোকদের দৃষ্টি মসজিদের দিকে ফেরান। তিনি বলেন, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর মীরাস বণ্টন হচ্ছে। লোকেরা ভাবল হয়তো সম্পদ বণ্টন হচ্ছে। কিন্তু তারা মসজিদে গিয়ে দেখল, কেউ নামাজ পড়ছে, কেউ কুরআন পড়ছে, কেউ হালাল-হারাম নিয়ে আলোচনা করছে। তখন আবু হুরায়রা বুঝিয়ে দিলেন, এটাই মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর মীরাস। এই হাদিসে ইলম, কুরআন শিক্ষা, নামাজ এবং দ্বীনি আলোচনা—এসবের মূল্য ফুটে উঠেছে। বাজারের ব্যস্ততার মাঝেও দ্বীনের জ্ঞানকে গুরুত্ব দেওয়ার শিক্ষা এতে আছে।"},"teachings":["নবীজির মীরাস হিসেবে ইলম, কুরআন ও দ্বীনি শিক্ষার গুরুত্ব বোঝানো হয়েছে।","মসজিদ শুধু নামাজের জায়গা নয়; ইলম শেখারও জায়গা।","হালাল-হারাম শেখা একজন মুসলিমের জীবনে গুরুত্বপূর্ণ।","দুনিয়ার ব্যস্ততার মধ্যেও দ্বীনি জ্ঞানকে অবহেলা করা উচিত নয়।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E161" s="4" t="n"/>
@@ -4219,12 +4215,12 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীর মীরাস হলো ইলম","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে নামাজ, কুরআন পাঠ ও হালাল-হারামের আলোচনা—এগুলোই নবীজির মীরাস হিসেবে বোঝানো হয়েছে।"},"heading":{"title":"নবীর মীরাস: মসজিদে ইলম, কুরআন ও হালাল-হারাম শিক্ষা","description":"এই বর্ণনায় আবু হুরায়রা রাদিয়াল্লাহু আনহু মদীনার বাজারের লোকদের দৃষ্টি মসজিদের দিকে ফেরান। তিনি বলেন, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর মীরাস বণ্টন হচ্ছে। লোকেরা ভাবল হয়তো সম্পদ বণ্টন হচ্ছে। কিন্তু তারা মসজিদে গিয়ে দেখল, কেউ নামাজ পড়ছে, কেউ কুরআন পড়ছে, কেউ হালাল-হারাম নিয়ে আলোচনা করছে। তখন আবু হুরায়রা বুঝিয়ে দিলেন, এটাই মুহাম্মাদ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর মীরাস। এই হাদিসে ইলম, কুরআন শিক্ষা, নামাজ এবং দ্বীনি আলোচনা—এসবের মূল্য ফুটে উঠেছে। বাজারের ব্যস্ততার মাঝেও দ্বীনের জ্ঞানকে গুরুত্ব দেওয়ার শিক্ষা এতে আছে।"},"teachings":["নবীজির মীরাস হিসেবে ইলম, কুরআন ও দ্বীনি শিক্ষার গুরুত্ব বোঝানো হয়েছে।","মসজিদ শুধু নামাজের জায়গা নয়; ইলম শেখারও জায়গা।","হালাল-হারাম শেখা একজন মুসলিমের জীবনে গুরুত্বপূর্ণ।","দুনিয়ার ব্যস্ততার মধ্যেও দ্বীনি জ্ঞানকে অবহেলা করা উচিত নয়।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের পথে জান্নাতের পথ সহজ","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি ইলমের জন্য পথ চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করেন—এ হাদিসে এ বড় ফজিলত এসেছে।"},"heading":{"title":"ইলম অর্জনের ফজিলত: জান্নাতের পথ সহজ হওয়ার হাদিস","description":"এই হাদিসে ইলম অর্জনের গুরুত্ব খুব পরিষ্কারভাবে বলা হয়েছে। যে ব্যক্তি বিদ্যান্বেষণের জন্য পথ চলে, আল্লাহ তার জন্য জান্নাতের একটি পথ সহজ করে দেন। এখানে ‘পথ চলা’ শুধু শারীরিকভাবে কোথাও যাওয়া নয়; ইলম শেখার জন্য চেষ্টা, সময় দেওয়া, শেখার আগ্রহ রাখা—এসব অর্থও বোঝায় বলে ইসলামী স্কলারদের মতে আলোচনা করা হয়। তবে মূল কথাটি হলো, দ্বীনের উপকারী জ্ঞান অর্জন আল্লাহর কাছে বড় মূল্যবান কাজ। একজন মানুষ যখন সঠিক জ্ঞান খোঁজে, তখন সে নিজের জীবনকে আল্লাহর নির্দেশের কাছাকাছি আনতে চায়। তাই ইলমের পথে চলা মুসলিম জীবনের সুন্দর লক্ষ্য।"},"teachings":["ইলম অর্জনের উদ্দেশ্যে পথ চলা বড় ফজিলতের কাজ।","আল্লাহ এমন ব্যক্তির জন্য জান্নাতের পথ সহজ করার কথা বলেছেন।","জ্ঞান অর্জনে চেষ্টা ও আগ্রহ রাখা দরকার।","উপকারী দ্বীনি জ্ঞান মানুষকে ভালো আমলের দিকে নিয়ে যায়।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E162" s="4" t="n"/>
@@ -4242,12 +4238,12 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের পথে জান্নাতের পথ সহজ","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি ইলমের জন্য পথ চলে, আল্লাহ তার জন্য জান্নাতের পথ সহজ করেন—এ হাদিসে এ বড় ফজিলত এসেছে।"},"heading":{"title":"ইলম অর্জনের ফজিলত: জান্নাতের পথ সহজ হওয়ার হাদিস","description":"এই হাদিসে ইলম অর্জনের গুরুত্ব খুব পরিষ্কারভাবে বলা হয়েছে। যে ব্যক্তি বিদ্যান্বেষণের জন্য পথ চলে, আল্লাহ তার জন্য জান্নাতের একটি পথ সহজ করে দেন। এখানে ‘পথ চলা’ শুধু শারীরিকভাবে কোথাও যাওয়া নয়; ইলম শেখার জন্য চেষ্টা, সময় দেওয়া, শেখার আগ্রহ রাখা—এসব অর্থও বোঝায় বলে ইসলামী স্কলারদের মতে আলোচনা করা হয়। তবে মূল কথাটি হলো, দ্বীনের উপকারী জ্ঞান অর্জন আল্লাহর কাছে বড় মূল্যবান কাজ। একজন মানুষ যখন সঠিক জ্ঞান খোঁজে, তখন সে নিজের জীবনকে আল্লাহর নির্দেশের কাছাকাছি আনতে চায়। তাই ইলমের পথে চলা মুসলিম জীবনের সুন্দর লক্ষ্য।"},"teachings":["ইলম অর্জনের উদ্দেশ্যে পথ চলা বড় ফজিলতের কাজ।","আল্লাহ এমন ব্যক্তির জন্য জান্নাতের পথ সহজ করার কথা বলেছেন।","জ্ঞান অর্জনে চেষ্টা ও আগ্রহ রাখা দরকার।","উপকারী দ্বীনি জ্ঞান মানুষকে ভালো আমলের দিকে নিয়ে যায়।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম তলবে ফেরেশতাদের সম্মান","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম তলবের উদ্দেশ্যে বের হলে ফেরেশতারা সন্তুষ্ট হয়ে ডানা বিছিয়ে দেন—এই ফজিলত এখানে এসেছে।"},"heading":{"title":"ইলম তলবের মর্যাদা: ফেরেশতাদের ডানা বিছানোর হাদিস","description":"এই হাদিসে জ্ঞানার্জনের জন্য ঘর থেকে বের হওয়ার বড় মর্যাদা বলা হয়েছে। বর্ণনাকারী ছাফওয়ান বিন আসসাল রাদিয়াল্লাহু আনহুর কাছে ইলম অর্জনের উদ্দেশ্যে আসেন। তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর একটি বাণী শুনিয়ে বলেন, যে ব্যক্তি ইলম তলবের উদ্দেশ্যে ঘর থেকে বের হয়, ফেরেশতারা তার কাজের প্রতি সন্তুষ্ট হয়ে তার জন্য ডানা বিছিয়ে দেন। এই বক্তব্য ইলমের পথে বিনয়, নিয়ত ও চেষ্টা—সবকিছুকে মূল্যবান করে তোলে। এখানে উদ্দেশ্য গুরুত্বপূর্ণ: শুধু কল্যাণকর জ্ঞান শেখা। তাই একজন শিক্ষার্থীকে নিজের নিয়ত ঠিক রাখা, ভালো উৎস থেকে শেখা এবং শেখা জ্ঞান অনুযায়ী আমল করার চিন্তা রাখা উচিত।"},"teachings":["ইলম তলবের উদ্দেশ্যে ঘর থেকে বের হওয়া সম্মানিত কাজ।","ফেরেশতাদের সন্তুষ্টির কথা হাদিসে উল্লেখ আছে।","জ্ঞানার্জনে নিয়ত পরিষ্কার রাখা দরকার।","উপকারী জ্ঞান শেখার জন্য কষ্ট করাও মূল্যবান।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E163" s="4" t="n"/>
@@ -4265,12 +4261,12 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>86</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম তলবে ফেরেশতাদের সম্মান","description":"$book_name$ $hadith_number$ - $chapter_name$. ইলম তলবের উদ্দেশ্যে বের হলে ফেরেশতারা সন্তুষ্ট হয়ে ডানা বিছিয়ে দেন—এই ফজিলত এখানে এসেছে।"},"heading":{"title":"ইলম তলবের মর্যাদা: ফেরেশতাদের ডানা বিছানোর হাদিস","description":"এই হাদিসে জ্ঞানার্জনের জন্য ঘর থেকে বের হওয়ার বড় মর্যাদা বলা হয়েছে। বর্ণনাকারী ছাফওয়ান বিন আসসাল রাদিয়াল্লাহু আনহুর কাছে ইলম অর্জনের উদ্দেশ্যে আসেন। তিনি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর একটি বাণী শুনিয়ে বলেন, যে ব্যক্তি ইলম তলবের উদ্দেশ্যে ঘর থেকে বের হয়, ফেরেশতারা তার কাজের প্রতি সন্তুষ্ট হয়ে তার জন্য ডানা বিছিয়ে দেন। এই বক্তব্য ইলমের পথে বিনয়, নিয়ত ও চেষ্টা—সবকিছুকে মূল্যবান করে তোলে। এখানে উদ্দেশ্য গুরুত্বপূর্ণ: শুধু কল্যাণকর জ্ঞান শেখা। তাই একজন শিক্ষার্থীকে নিজের নিয়ত ঠিক রাখা, ভালো উৎস থেকে শেখা এবং শেখা জ্ঞান অনুযায়ী আমল করার চিন্তা রাখা উচিত।"},"teachings":["ইলম তলবের উদ্দেশ্যে ঘর থেকে বের হওয়া সম্মানিত কাজ।","ফেরেশতাদের সন্তুষ্টির কথা হাদিসে উল্লেখ আছে।","জ্ঞানার্জনে নিয়ত পরিষ্কার রাখা দরকার।","উপকারী জ্ঞান শেখার জন্য কষ্ট করাও মূল্যবান।"],"related_hadiths":[{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে ইলম শেখা ও শেখানোর প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে শুধু কল্যাণ শেখা বা শেখানোর উদ্দেশ্যে গেলে পূর্ণ হজ্জের মতো প্রতিদানের কথা এসেছে।"},"heading":{"title":"মসজিদে ইলম শেখা: কল্যাণ শেখা ও শেখানোর ফজিলত","description":"এই হাদিসে মসজিদে যাওয়ার একটি বিশেষ উদ্দেশ্যের কথা বলা হয়েছে। যে ব্যক্তি মসজিদে যায় শুধু কল্যাণ শিক্ষা লাভ বা কল্যাণ শিক্ষা দেওয়ার উদ্দেশ্যে, তার জন্য পূর্ণ হজ্জ পালনকারীর মতো প্রতিদানের কথা এসেছে। এখানে হাদিসটি আমাদের নিয়তকে গুরুত্ব দিতে শেখায়। মসজিদে যাওয়া শুধু উপস্থিত হওয়া নয়; সেখানে ভালো শেখা, ভালো শেখানো এবং নিজের জীবনকে কল্যাণের পথে নেওয়া বড় বিষয়। তবে হাদিসে যে প্রতিদানের কথা আছে, সেটি ওই নির্দিষ্ট উদ্দেশ্যের সঙ্গে যুক্ত। তাই মসজিদে কুরআন, হাদিস, হালাল-হারাম ও ভালো কাজের শিক্ষা গ্রহণ করা একজন মুসলিমের জন্য বিশেষ সুযোগ।"},"teachings":["মসজিদে কল্যাণ শেখা বা শেখানো বড় ফজিলতের কাজ।","এই হাদিসে নিয়তের গুরুত্ব স্পষ্টভাবে বোঝা যায়।","মসজিদ দ্বীনি শিক্ষা গ্রহণের সুন্দর স্থান।","ভালো উদ্দেশ্যে মসজিদে যাওয়া আমলের মান বাড়ায়।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E164" s="4" t="n"/>
@@ -4288,12 +4284,12 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে ইলম শেখা ও শেখানোর প্রতিদান","description":"$book_name$ $hadith_number$ - $chapter_name$. মসজিদে শুধু কল্যাণ শেখা বা শেখানোর উদ্দেশ্যে গেলে পূর্ণ হজ্জের মতো প্রতিদানের কথা এসেছে।"},"heading":{"title":"মসজিদে ইলম শেখা: কল্যাণ শেখা ও শেখানোর ফজিলত","description":"এই হাদিসে মসজিদে যাওয়ার একটি বিশেষ উদ্দেশ্যের কথা বলা হয়েছে। যে ব্যক্তি মসজিদে যায় শুধু কল্যাণ শিক্ষা লাভ বা কল্যাণ শিক্ষা দেওয়ার উদ্দেশ্যে, তার জন্য পূর্ণ হজ্জ পালনকারীর মতো প্রতিদানের কথা এসেছে। এখানে হাদিসটি আমাদের নিয়তকে গুরুত্ব দিতে শেখায়। মসজিদে যাওয়া শুধু উপস্থিত হওয়া নয়; সেখানে ভালো শেখা, ভালো শেখানো এবং নিজের জীবনকে কল্যাণের পথে নেওয়া বড় বিষয়। তবে হাদিসে যে প্রতিদানের কথা আছে, সেটি ওই নির্দিষ্ট উদ্দেশ্যের সঙ্গে যুক্ত। তাই মসজিদে কুরআন, হাদিস, হালাল-হারাম ও ভালো কাজের শিক্ষা গ্রহণ করা একজন মুসলিমের জন্য বিশেষ সুযোগ।"},"teachings":["মসজিদে কল্যাণ শেখা বা শেখানো বড় ফজিলতের কাজ।","এই হাদিসে নিয়তের গুরুত্ব স্পষ্টভাবে বোঝা যায়।","মসজিদ দ্বীনি শিক্ষা গ্রহণের সুন্দর স্থান।","ভালো উদ্দেশ্যে মসজিদে যাওয়া আমলের মান বাড়ায়।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে নববীতে ইলমের নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি শুধু কল্যাণ শেখা বা শেখানোর জন্য মসজিদে আসে, তার মর্যাদার কথা এই হাদিসে এসেছে।"},"heading":{"title":"মসজিদে নববীতে ইলম: নিয়ত ঠিক রাখার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর মসজিদে আগমনের উদ্দেশ্য নিয়ে কথা বলেছেন। যে ব্যক্তি শুধু কল্যাণ শেখা বা শেখানোর উদ্দেশ্যে আসবে, সে আল্লাহর পথে জিহাদকারীদের মর্যাদার অধিকারী হবে। আর যে অন্য উদ্দেশ্যে আসবে, তার উদাহরণ দেওয়া হয়েছে এমন ব্যক্তির মতো, যে অন্যের সম্পদের দিকে তাকিয়ে থাকে। এখানে মূল শিক্ষা হলো নিয়ত। মসজিদে আসা, ইলম শেখা, মানুষকে ভালো শেখানো—সবই মূল্যবান, তবে উদ্দেশ্য পরিষ্কার হওয়া দরকার। এই হাদিস আমাদের শেখায়, দ্বীনি পরিবেশে উপস্থিত হওয়া যেন নাম, দুনিয়াবি লাভ বা কৌতূহলের জন্য না হয়; বরং কল্যাণের জন্য হয়।"},"teachings":["মসজিদে ইলম শেখা বা শেখানোর উদ্দেশ্য খুব গুরুত্বপূর্ণ।","সঠিক নিয়ত আমলের মর্যাদা বাড়ায়।","দ্বীনি স্থানে দুনিয়াবি উদ্দেশ্যকে প্রাধান্য দেওয়া ঠিক নয়।","কল্যাণ শেখা ও শেখানো আল্লাহর পথে কাজের সঙ্গে তুলনা করা হয়েছে।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E165" s="4" t="n"/>
@@ -4311,12 +4307,12 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মসজিদে নববীতে ইলমের নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. যে ব্যক্তি শুধু কল্যাণ শেখা বা শেখানোর জন্য মসজিদে আসে, তার মর্যাদার কথা এই হাদিসে এসেছে।"},"heading":{"title":"মসজিদে নববীতে ইলম: নিয়ত ঠিক রাখার শিক্ষা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম তাঁর মসজিদে আগমনের উদ্দেশ্য নিয়ে কথা বলেছেন। যে ব্যক্তি শুধু কল্যাণ শেখা বা শেখানোর উদ্দেশ্যে আসবে, সে আল্লাহর পথে জিহাদকারীদের মর্যাদার অধিকারী হবে। আর যে অন্য উদ্দেশ্যে আসবে, তার উদাহরণ দেওয়া হয়েছে এমন ব্যক্তির মতো, যে অন্যের সম্পদের দিকে তাকিয়ে থাকে। এখানে মূল শিক্ষা হলো নিয়ত। মসজিদে আসা, ইলম শেখা, মানুষকে ভালো শেখানো—সবই মূল্যবান, তবে উদ্দেশ্য পরিষ্কার হওয়া দরকার। এই হাদিস আমাদের শেখায়, দ্বীনি পরিবেশে উপস্থিত হওয়া যেন নাম, দুনিয়াবি লাভ বা কৌতূহলের জন্য না হয়; বরং কল্যাণের জন্য হয়।"},"teachings":["মসজিদে ইলম শেখা বা শেখানোর উদ্দেশ্য খুব গুরুত্বপূর্ণ।","সঠিক নিয়ত আমলের মর্যাদা বাড়ায়।","দ্বীনি স্থানে দুনিয়াবি উদ্দেশ্যকে প্রাধান্য দেওয়া ঠিক নয়।","কল্যাণ শেখা ও শেখানো আল্লাহর পথে কাজের সঙ্গে তুলনা করা হয়েছে।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"3641","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের পথে থাকা আল্লাহর পথে থাকা","description":"$book_name$ $hadith_number$ - $chapter_name$. জ্ঞানার্জনের জন্য বের হওয়া ব্যক্তি ফিরে আসা পর্যন্ত আল্লাহর পথেই থাকে—এ হাদিসে এ মর্যাদা এসেছে।"},"heading":{"title":"ইলম অর্জনের পথে থাকা: আল্লাহর পথে থাকার ফজিলত","description":"এই হাদিসে জ্ঞানার্জনের জন্য বের হওয়ার মর্যাদা সংক্ষেপে বলা হয়েছে। যে ব্যক্তি ইলম তলব করার জন্য বের হয়, সে ফিরে আসা পর্যন্ত আল্লাহর পথে থাকে। এখানে ইলমের গুরুত্ব, শেখার চেষ্টা এবং সময় দেওয়ার মূল্য বোঝানো হয়েছে। একজন মানুষ যখন দ্বীনের উপকারী জ্ঞান শেখার জন্য ঘর থেকে বের হয়, তখন তার সময়, পথচলা ও কষ্ট—সবই মূল্যবান হয়ে যায়। তবে এই মর্যাদা সেই ইলমের সঙ্গে যুক্ত, যা কল্যাণের পথে নেয়। তাই ইলম অর্জনের সময় নিয়ত ঠিক রাখা, সঠিক জ্ঞান খোঁজা এবং শেখা কথাকে জীবনে কাজে লাগানো জরুরি। এই হাদিস শিক্ষার্থীকে উৎসাহ দেয়।"},"teachings":["ইলম তলবের জন্য বের হওয়া আল্লাহর পথে থাকার কারণ হিসেবে এসেছে।","জ্ঞানার্জনের কষ্ট ও সময় মূল্যবান।","উপকারী ইলম শেখার জন্য আগ্রহ রাখা দরকার।","ফিরে আসা পর্যন্ত ইলমের সফরের মর্যাদা বজায় থাকে।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E166" s="4" t="n"/>
@@ -4334,12 +4330,12 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলমের পথে থাকা আল্লাহর পথে থাকা","description":"$book_name$ $hadith_number$ - $chapter_name$. জ্ঞানার্জনের জন্য বের হওয়া ব্যক্তি ফিরে আসা পর্যন্ত আল্লাহর পথেই থাকে—এ হাদিসে এ মর্যাদা এসেছে।"},"heading":{"title":"ইলম অর্জনের পথে থাকা: আল্লাহর পথে থাকার ফজিলত","description":"এই হাদিসে জ্ঞানার্জনের জন্য বের হওয়ার মর্যাদা সংক্ষেপে বলা হয়েছে। যে ব্যক্তি ইলম তলব করার জন্য বের হয়, সে ফিরে আসা পর্যন্ত আল্লাহর পথে থাকে। এখানে ইলমের গুরুত্ব, শেখার চেষ্টা এবং সময় দেওয়ার মূল্য বোঝানো হয়েছে। একজন মানুষ যখন দ্বীনের উপকারী জ্ঞান শেখার জন্য ঘর থেকে বের হয়, তখন তার সময়, পথচলা ও কষ্ট—সবই মূল্যবান হয়ে যায়। তবে এই মর্যাদা সেই ইলমের সঙ্গে যুক্ত, যা কল্যাণের পথে নেয়। তাই ইলম অর্জনের সময় নিয়ত ঠিক রাখা, সঠিক জ্ঞান খোঁজা এবং শেখা কথাকে জীবনে কাজে লাগানো জরুরি। এই হাদিস শিক্ষার্থীকে উৎসাহ দেয়।"},"teachings":["ইলম তলবের জন্য বের হওয়া আল্লাহর পথে থাকার কারণ হিসেবে এসেছে।","জ্ঞানার্জনের কষ্ট ও সময় মূল্যবান।","উপকারী ইলম শেখার জন্য আগ্রহ রাখা দরকার।","ফিরে আসা পর্যন্ত ইলমের সফরের মর্যাদা বজায় থাকে।"],"related_hadiths":[{"id":"6746","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"212","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"},{"id":"223","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস শুনে ঠিকভাবে পৌঁছে দেওয়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. যে শুনে যেমন শুনেছে তেমনই পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া এসেছে।"},"heading":{"title":"হাদিস পৌঁছে দেওয়ার আদব: যেমন শুনেছে তেমন বলা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সেই ব্যক্তির জন্য দোয়া করেছেন, যে তাঁর কাছ থেকে কিছু শুনে, তারপর যেমন শুনেছে তেমনই অন্যের কাছে পৌঁছে দেয়। এখানে হাদিস বর্ণনার বড় আদব আছে। নিজের মতো করে কথা বাড়ানো, অর্থ বদলে দেওয়া বা নিশ্চিত না হয়ে বলা—এসব থেকে সাবধান থাকা দরকার। কারণ যাকে কথা পৌঁছে দেওয়া হয়, সে অনেক সময় সরাসরি শ্রোতার চেয়েও ভালোভাবে তা সংরক্ষণ করতে পারে। তাই হাদিস শেখা, মনে রাখা এবং সঠিকভাবে বলা—সবই দায়িত্বের বিষয়। এই হাদিস আমাদের সত্যনিষ্ঠ জ্ঞান প্রচার ও সতর্ক ভাষার শিক্ষা দেয়।"},"teachings":["হাদিস যেমন শোনা হয়েছে, তেমনই পৌঁছে দেওয়া উচিত।","হাদিস বর্ণনায় সতর্কতা ও সত্যনিষ্ঠা জরুরি।","কথা যার কাছে পৌঁছে, সে কখনো বেশি ভালোভাবে বুঝতে পারে।","দ্বীনি কথা প্রচারের আগে তা ঠিকভাবে জানা দরকার।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E167" s="4" t="n"/>
@@ -4357,12 +4353,12 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস শুনে ঠিকভাবে পৌঁছে দেওয়ার ফজিলত","description":"$book_name$ $hadith_number$ - $chapter_name$. যে শুনে যেমন শুনেছে তেমনই পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া এসেছে।"},"heading":{"title":"হাদিস পৌঁছে দেওয়ার আদব: যেমন শুনেছে তেমন বলা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সেই ব্যক্তির জন্য দোয়া করেছেন, যে তাঁর কাছ থেকে কিছু শুনে, তারপর যেমন শুনেছে তেমনই অন্যের কাছে পৌঁছে দেয়। এখানে হাদিস বর্ণনার বড় আদব আছে। নিজের মতো করে কথা বাড়ানো, অর্থ বদলে দেওয়া বা নিশ্চিত না হয়ে বলা—এসব থেকে সাবধান থাকা দরকার। কারণ যাকে কথা পৌঁছে দেওয়া হয়, সে অনেক সময় সরাসরি শ্রোতার চেয়েও ভালোভাবে তা সংরক্ষণ করতে পারে। তাই হাদিস শেখা, মনে রাখা এবং সঠিকভাবে বলা—সবই দায়িত্বের বিষয়। এই হাদিস আমাদের সত্যনিষ্ঠ জ্ঞান প্রচার ও সতর্ক ভাষার শিক্ষা দেয়।"},"teachings":["হাদিস যেমন শোনা হয়েছে, তেমনই পৌঁছে দেওয়া উচিত।","হাদিস বর্ণনায় সতর্কতা ও সত্যনিষ্ঠা জরুরি।","কথা যার কাছে পৌঁছে, সে কখনো বেশি ভালোভাবে বুঝতে পারে।","দ্বীনি কথা প্রচারের আগে তা ঠিকভাবে জানা দরকার।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস প্রচার, এখলাস ও আখেরাতের নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিস পৌঁছে দেওয়া, আমলে এখলাস, জামাআত আঁকড়ে থাকা এবং আখেরাতমুখী নিয়তের শিক্ষা এখানে এসেছে।"},"heading":{"title":"হাদিস প্রচার ও নিয়তের শিক্ষা: দুনিয়া নয়, আখেরাত লক্ষ্য","description":"এই হাদিসে কয়েকটি বড় শিক্ষা একসাথে এসেছে। প্রথমে বলা হয়েছে, যে ব্যক্তি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর একটি হাদিস শুনে অন্যের কাছে পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া করা হয়েছে। কারণ কখনো জ্ঞান বহনকারী এমন ব্যক্তির কাছে তা পৌঁছে দেয়, যে তার চেয়ে বেশি বুঝতে পারে। এরপর তিনটি বিষয়ে অন্তরকে পরিষ্কার রাখার কথা এসেছে: আমলকে আল্লাহর জন্য একনিষ্ঠ করা, নেতৃবৃন্দকে নসীহত করা এবং মুসলমানদের জামাআত আঁকড়ে থাকা। শেষে দুনিয়াকে একমাত্র উদ্দেশ্য বানানো ও আখেরাতকে উদ্দেশ্য বানানোর ভিন্ন ফল বলা হয়েছে। তাই এই হাদিস জ্ঞান, নিয়ত ও জীবনলক্ষ্য—তিনটিকেই শুদ্ধ করতে শেখায়।"},"teachings":["হাদিস শুনে সঠিকভাবে অন্যের কাছে পৌঁছে দেওয়া মূল্যবান কাজ।","আমল আল্লাহর জন্য একনিষ্ঠ করা অন্তরের শুদ্ধতার অংশ।","মুসলিম জামাআত আঁকড়ে থাকার গুরুত্ব হাদিসে এসেছে।","দুনিয়াকে একমাত্র লক্ষ্য না করে আখেরাতকে লক্ষ্য করা উচিত।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E168" s="4" t="n"/>
@@ -4380,12 +4376,12 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস প্রচার, এখলাস ও আখেরাতের নিয়ত","description":"$book_name$ $hadith_number$ - $chapter_name$. হাদিস পৌঁছে দেওয়া, আমলে এখলাস, জামাআত আঁকড়ে থাকা এবং আখেরাতমুখী নিয়তের শিক্ষা এখানে এসেছে।"},"heading":{"title":"হাদিস প্রচার ও নিয়তের শিক্ষা: দুনিয়া নয়, আখেরাত লক্ষ্য","description":"এই হাদিসে কয়েকটি বড় শিক্ষা একসাথে এসেছে। প্রথমে বলা হয়েছে, যে ব্যক্তি রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর একটি হাদিস শুনে অন্যের কাছে পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া করা হয়েছে। কারণ কখনো জ্ঞান বহনকারী এমন ব্যক্তির কাছে তা পৌঁছে দেয়, যে তার চেয়ে বেশি বুঝতে পারে। এরপর তিনটি বিষয়ে অন্তরকে পরিষ্কার রাখার কথা এসেছে: আমলকে আল্লাহর জন্য একনিষ্ঠ করা, নেতৃবৃন্দকে নসীহত করা এবং মুসলমানদের জামাআত আঁকড়ে থাকা। শেষে দুনিয়াকে একমাত্র উদ্দেশ্য বানানো ও আখেরাতকে উদ্দেশ্য বানানোর ভিন্ন ফল বলা হয়েছে। তাই এই হাদিস জ্ঞান, নিয়ত ও জীবনলক্ষ্য—তিনটিকেই শুদ্ধ করতে শেখায়।"},"teachings":["হাদিস শুনে সঠিকভাবে অন্যের কাছে পৌঁছে দেওয়া মূল্যবান কাজ।","আমল আল্লাহর জন্য একনিষ্ঠ করা অন্তরের শুদ্ধতার অংশ।","মুসলিম জামাআত আঁকড়ে থাকার গুরুত্ব হাদিসে এসেছে।","দুনিয়াকে একমাত্র লক্ষ্য না করে আখেরাতকে লক্ষ্য করা উচিত।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস মুখস্ত করে পৌঁছে দেওয়ার মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. যে নবীজির কথা শুনে মুখস্ত করে না-শোনা ব্যক্তির কাছে পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া এসেছে।"},"heading":{"title":"নবীজির কথা সংরক্ষণ: মুখস্ত করা ও পৌঁছে দেওয়ার ফজিলত","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম মিনার মসজিদে খায়ফে দেওয়া বক্তব্যে এমন ব্যক্তির জন্য দোয়া করেছেন, যে তাঁর কথা শুনে, মুখস্ত করে, ধারণ করে এবং যারা শোনেনি তাদের কাছে পৌঁছে দেয়। এখানে দ্বীনি জ্ঞান সংরক্ষণের দায়িত্ব বোঝানো হয়েছে। শুধু শুনলেই যথেষ্ট নয়; শোনা কথাকে ভালোভাবে রাখা এবং সততার সঙ্গে অন্যের কাছে পৌঁছে দেওয়া দরকার। হাদিসে আরও বলা হয়েছে, অনেক জ্ঞান বহনকারী নিজে গভীর জ্ঞানী না হলেও, সে হয়তো তার চেয়ে বেশি জ্ঞানী কারও কাছে সেই কথা পৌঁছে দেয়। তাই জ্ঞান প্রচারে আমানতদারি, সতর্কতা ও সঠিক ভাষা জরুরি।"},"teachings":["নবীজির কথা মুখস্ত ও সংরক্ষণ করা সম্মানিত কাজ।","যারা শোনেনি তাদের কাছে সঠিকভাবে পৌঁছে দেওয়া জরুরি।","জ্ঞান বহনকারী ব্যক্তি অন্যের উপকারের মাধ্যম হতে পারে।","দ্বীনি কথা বলার সময় আমানতদারি রাখা দরকার।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E169" s="4" t="n"/>
@@ -4403,12 +4399,12 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | হাদিস মুখস্ত করে পৌঁছে দেওয়ার মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. যে নবীজির কথা শুনে মুখস্ত করে না-শোনা ব্যক্তির কাছে পৌঁছে দেয়, তার জন্য উজ্জ্বলতার দোয়া এসেছে।"},"heading":{"title":"নবীজির কথা সংরক্ষণ: মুখস্ত করা ও পৌঁছে দেওয়ার ফজিলত","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম মিনার মসজিদে খায়ফে দেওয়া বক্তব্যে এমন ব্যক্তির জন্য দোয়া করেছেন, যে তাঁর কথা শুনে, মুখস্ত করে, ধারণ করে এবং যারা শোনেনি তাদের কাছে পৌঁছে দেয়। এখানে দ্বীনি জ্ঞান সংরক্ষণের দায়িত্ব বোঝানো হয়েছে। শুধু শুনলেই যথেষ্ট নয়; শোনা কথাকে ভালোভাবে রাখা এবং সততার সঙ্গে অন্যের কাছে পৌঁছে দেওয়া দরকার। হাদিসে আরও বলা হয়েছে, অনেক জ্ঞান বহনকারী নিজে গভীর জ্ঞানী না হলেও, সে হয়তো তার চেয়ে বেশি জ্ঞানী কারও কাছে সেই কথা পৌঁছে দেয়। তাই জ্ঞান প্রচারে আমানতদারি, সতর্কতা ও সঠিক ভাষা জরুরি।"},"teachings":["নবীজির কথা মুখস্ত ও সংরক্ষণ করা সম্মানিত কাজ।","যারা শোনেনি তাদের কাছে সঠিকভাবে পৌঁছে দেওয়া জরুরি।","জ্ঞান বহনকারী ব্যক্তি অন্যের উপকারের মাধ্যম হতে পারে।","দ্বীনি কথা বলার সময় আমানতদারি রাখা দরকার।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম পৌঁছে দেওয়া ও অন্তরের শুদ্ধতা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজির কথা শুনে সংরক্ষণ ও পৌঁছে দেওয়া, এখলাস, নসীহত ও জামাআতের শিক্ষা এসেছে।"},"heading":{"title":"ইলম পৌঁছে দেওয়া: এখলাস, নসীহত ও জামাআত আঁকড়ে থাকা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সেই বান্দার জন্য সৌন্দর্য ও উজ্জ্বলতার দোয়া করেছেন, যে তাঁর বক্তব্য শুনে, মুখস্ত করে, ভালোভাবে সংরক্ষণ করে এবং যে শুনেনি তার কাছে পৌঁছে দেয়। এরপর বলা হয়েছে, অনেক জ্ঞান বহনকারী নিজে জ্ঞানী নাও হতে পারে, আবার সে তার চেয়ে বেশি জ্ঞানীর কাছে জ্ঞান পৌঁছে দিতে পারে। এই কথার পর তিনটি বিষয়ে মুমিনের অন্তরে হিংসা-দ্বেষ না থাকার শিক্ষা এসেছে: আল্লাহর জন্য এখলাস, মুসলমানদের নেতৃবৃন্দকে নসীহত এবং তাদের জামাআতকে আঁকড়ে থাকা। তাই এই হাদিস জ্ঞান প্রচার ও অন্তরের শুদ্ধতা—দুই দিকেই দৃষ্টি দেয়।"},"teachings":["নবীজির বক্তব্য শুনে সংরক্ষণ ও পৌঁছে দেওয়া গুরুত্বপূর্ণ দায়িত্ব।","জ্ঞান অন্যের কাছে পৌঁছালে সে আরও ভালোভাবে বুঝতে পারে।","আমলকে আল্লাহর জন্য একনিষ্ঠ করা মুমিনের গুণ।","মুসলিম জামাআত আঁকড়ে থাকা ও নসীহত করার শিক্ষা এসেছে।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
         </is>
       </c>
       <c r="E170" s="4" t="n"/>
@@ -4426,12 +4422,12 @@
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | ইলম পৌঁছে দেওয়া ও অন্তরের শুদ্ধতা","description":"$book_name$ $hadith_number$ - $chapter_name$. নবীজির কথা শুনে সংরক্ষণ ও পৌঁছে দেওয়া, এখলাস, নসীহত ও জামাআতের শিক্ষা এসেছে।"},"heading":{"title":"ইলম পৌঁছে দেওয়া: এখলাস, নসীহত ও জামাআত আঁকড়ে থাকা","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম সেই বান্দার জন্য সৌন্দর্য ও উজ্জ্বলতার দোয়া করেছেন, যে তাঁর বক্তব্য শুনে, মুখস্ত করে, ভালোভাবে সংরক্ষণ করে এবং যে শুনেনি তার কাছে পৌঁছে দেয়। এরপর বলা হয়েছে, অনেক জ্ঞান বহনকারী নিজে জ্ঞানী নাও হতে পারে, আবার সে তার চেয়ে বেশি জ্ঞানীর কাছে জ্ঞান পৌঁছে দিতে পারে। এই কথার পর তিনটি বিষয়ে মুমিনের অন্তরে হিংসা-দ্বেষ না থাকার শিক্ষা এসেছে: আল্লাহর জন্য এখলাস, মুসলমানদের নেতৃবৃন্দকে নসীহত এবং তাদের জামাআতকে আঁকড়ে থাকা। তাই এই হাদিস জ্ঞান প্রচার ও অন্তরের শুদ্ধতা—দুই দিকেই দৃষ্টি দেয়।"},"teachings":["নবীজির বক্তব্য শুনে সংরক্ষণ ও পৌঁছে দেওয়া গুরুত্বপূর্ণ দায়িত্ব।","জ্ঞান অন্যের কাছে পৌঁছালে সে আরও ভালোভাবে বুঝতে পারে।","আমলকে আল্লাহর জন্য একনিষ্ঠ করা মুমিনের গুণ।","মুসলিম জামাআত আঁকড়ে থাকা ও নসীহত করার শিক্ষা এসেছে।"],"related_hadiths":[{"id":"3660","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"2656","book_id":"5","slug":"tirmidhi","label":"জামে আত-তিরমিজি"},{"id":"230","book_id":"6","slug":"majah","label":"সুনান ইবনে মাজাহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পরও চলমান তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মৃত্যু হলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া বাকি থাকে।"},"heading":{"title":"মৃত্যুর পরও উপকার দেয়: সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া","description":"এই হাদিসে মানুষের মৃত্যুর পর আমলের অবস্থা নিয়ে খুব গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, আদম সন্তান মারা গেলে তার সব আমল বন্ধ হয়ে যায়, তবে তিনটি ছাড়া: সাদকায়ে জারিয়া, উপকারী বিদ্যা এবং সৎ সন্তানের দোয়া। এখানে উপকারী বিদ্যার গুরুত্ব বিশেষভাবে বোঝা যায়। যে জ্ঞান মানুষকে ভালো পথে সাহায্য করে, তা মৃত্যুর পরও উপকারের কারণ হতে পারে। তবে হাদিসে অপকারী জ্ঞানের প্রশংসা নেই; বরং মূল কথা হলো এমন জ্ঞান, যা মানুষের কল্যাণে লাগে। এই হাদিস আমাদের শেখায়, জীবনে এমন কাজ রেখে যেতে হবে, যা অন্যের ভালোতে কাজে আসে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায় বলে হাদিসে এসেছে।","সাদকায়ে জারিয়া চলমান কল্যাণের একটি পথ।","উপকারী বিদ্যা মৃত্যুর পরও উপকারের কারণ হতে পারে।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য কল্যাণকর।"],"related_hadiths":[{"id":"78","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"4115","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"203","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E171" s="4" t="n"/>
@@ -4449,12 +4445,12 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মৃত্যুর পরও চলমান তিন আমল","description":"$book_name$ $hadith_number$ - $chapter_name$. মৃত্যু হলে আমল বন্ধ হয়, তবে সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া বাকি থাকে।"},"heading":{"title":"মৃত্যুর পরও উপকার দেয়: সাদকায়ে জারিয়া, উপকারী বিদ্যা ও সৎ সন্তানের দোয়া","description":"এই হাদিসে মানুষের মৃত্যুর পর আমলের অবস্থা নিয়ে খুব গুরুত্বপূর্ণ শিক্ষা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, আদম সন্তান মারা গেলে তার সব আমল বন্ধ হয়ে যায়, তবে তিনটি ছাড়া: সাদকায়ে জারিয়া, উপকারী বিদ্যা এবং সৎ সন্তানের দোয়া। এখানে উপকারী বিদ্যার গুরুত্ব বিশেষভাবে বোঝা যায়। যে জ্ঞান মানুষকে ভালো পথে সাহায্য করে, তা মৃত্যুর পরও উপকারের কারণ হতে পারে। তবে হাদিসে অপকারী জ্ঞানের প্রশংসা নেই; বরং মূল কথা হলো এমন জ্ঞান, যা মানুষের কল্যাণে লাগে। এই হাদিস আমাদের শেখায়, জীবনে এমন কাজ রেখে যেতে হবে, যা অন্যের ভালোতে কাজে আসে।"},"teachings":["মৃত্যুর পর সাধারণ আমল বন্ধ হয়ে যায় বলে হাদিসে এসেছে।","সাদকায়ে জারিয়া চলমান কল্যাণের একটি পথ।","উপকারী বিদ্যা মৃত্যুর পরও উপকারের কারণ হতে পারে।","সৎ সন্তানের দোয়া মৃত ব্যক্তির জন্য কল্যাণকর।"],"related_hadiths":[{"id":"78","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"4115","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"203","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাসূলের নামে মিথ্যা বলার ভয়াবহতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইচ্ছাকৃতভাবে রাসূলের নামে মিথ্যা বলার ভয়াবহ পরিণতির কথা এই হাদিসে কঠোরভাবে বলা হয়েছে।"},"heading":{"title":"রাসূলের নামে মিথ্যা বলা: কঠোর সতর্কবার্তার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে মিথ্যা বলার ভয়াবহতা স্পষ্টভাবে এসেছে। তিনি বলেছেন, যে ব্যক্তি ইচ্ছাকৃতভাবে তাঁর উপর মিথ্যারোপ করবে, সে যেন তার স্থায়ী ঠিকানা জাহান্নামে করে নেয়। এই হাদিস হাদিস বর্ণনা, দ্বীনি কথা বলা এবং ইসলামের নামে কোনো কথা প্রচারের ক্ষেত্রে খুব বড় সতর্কতা। কাউকে প্রভাবিত করার জন্য, আবেগে, বা না জেনে কোনো কথা রাসূলের নামে বলা নিরাপদ নয়। হাদিস বলার আগে উৎস যাচাই করা, শব্দের অর্থ বুঝে নেওয়া এবং সন্দেহ হলে চুপ থাকা—এগুলো প্রয়োজন। দ্বীনি জ্ঞান প্রচারে সত্যনিষ্ঠা এখানে মূল শিক্ষা।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে মিথ্যা বলা ভয়াবহ গুনাহ।","ইচ্ছাকৃত মিথ্যারোপের কঠোর পরিণতি হাদিসে বলা হয়েছে।","হাদিস বর্ণনার আগে উৎস যাচাই করা দরকার।","দ্বীনি কথায় সততা ও সাবধানতা রাখা জরুরি।"],"related_hadiths":[{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"108","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E172" s="4" t="n"/>
@@ -4472,12 +4468,12 @@
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | রাসূলের নামে মিথ্যা বলার ভয়াবহতা","description":"$book_name$ $hadith_number$ - $chapter_name$. ইচ্ছাকৃতভাবে রাসূলের নামে মিথ্যা বলার ভয়াবহ পরিণতির কথা এই হাদিসে কঠোরভাবে বলা হয়েছে।"},"heading":{"title":"রাসূলের নামে মিথ্যা বলা: কঠোর সতর্কবার্তার হাদিস","description":"এই হাদিসে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে মিথ্যা বলার ভয়াবহতা স্পষ্টভাবে এসেছে। তিনি বলেছেন, যে ব্যক্তি ইচ্ছাকৃতভাবে তাঁর উপর মিথ্যারোপ করবে, সে যেন তার স্থায়ী ঠিকানা জাহান্নামে করে নেয়। এই হাদিস হাদিস বর্ণনা, দ্বীনি কথা বলা এবং ইসলামের নামে কোনো কথা প্রচারের ক্ষেত্রে খুব বড় সতর্কতা। কাউকে প্রভাবিত করার জন্য, আবেগে, বা না জেনে কোনো কথা রাসূলের নামে বলা নিরাপদ নয়। হাদিস বলার আগে উৎস যাচাই করা, শব্দের অর্থ বুঝে নেওয়া এবং সন্দেহ হলে চুপ থাকা—এগুলো প্রয়োজন। দ্বীনি জ্ঞান প্রচারে সত্যনিষ্ঠা এখানে মূল শিক্ষা।"},"teachings":["রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে মিথ্যা বলা ভয়াবহ গুনাহ।","ইচ্ছাকৃত মিথ্যারোপের কঠোর পরিণতি হাদিসে বলা হয়েছে।","হাদিস বর্ণনার আগে উৎস যাচাই করা দরকার।","দ্বীনি কথায় সততা ও সাবধানতা রাখা জরুরি।"],"related_hadiths":[{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"108","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মিথ্যা সন্দেহের হাদিস বর্ণনার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কোনো হাদিস মিথ্যা মনে করেও তা বর্ণনা করলে সে মিথ্যাবাদীদের একজন—এ কঠোর সতর্কতা এসেছে।"},"heading":{"title":"মিথ্যা মনে হওয়া হাদিস প্রচার: সাবধানতার জরুরি শিক্ষা","description":"এই হাদিসে এমন ব্যক্তির বিষয়ে কঠোর সতর্কতা এসেছে, যে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে কোনো হাদিস বর্ণনা করে, অথচ সে মনে করে হাদিসটি মিথ্যা। এমন ব্যক্তি দুজন মিথ্যাবাদীর একজন বলে হাদিসে এসেছে। এর মানে, শুধু নিজের মুখে বানানো নয়; সন্দেহজনক বা মিথ্যা মনে হওয়া কথা প্রচার করাও বিপজ্জনক। আজকের সময়ে মানুষ অনেক কথা দ্রুত ছড়িয়ে দেয়। কিন্তু হাদিসের ক্ষেত্রে বেশি সতর্ক হওয়া দরকার। কোনো বর্ণনা নিশ্চিত না হলে তা যাচাই করা, আলেমদের কাছে জিজ্ঞেস করা বা না বলা—এটাই নিরাপদ পথ।"},"teachings":["মিথ্যা মনে হওয়া হাদিস প্রচার করা গুরুতর ভুল।","হাদিস বর্ণনার আগে সত্যতা যাচাই জরুরি।","শুধু ফরওয়ার্ড করা বা ছড়িয়ে দেওয়াও দায়িত্বের বাইরে নয়।","দ্বীনি কথায় সন্দেহ হলে সাবধান থাকা উচিত।"],"related_hadiths":[{"id":"1","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"108","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
         </is>
       </c>
       <c r="E173" s="4" t="n"/>
@@ -4495,12 +4491,12 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | মিথ্যা সন্দেহের হাদিস বর্ণনার সতর্কতা","description":"$book_name$ $hadith_number$ - $chapter_name$. কোনো হাদিস মিথ্যা মনে করেও তা বর্ণনা করলে সে মিথ্যাবাদীদের একজন—এ কঠোর সতর্কতা এসেছে।"},"heading":{"title":"মিথ্যা মনে হওয়া হাদিস প্রচার: সাবধানতার জরুরি শিক্ষা","description":"এই হাদিসে এমন ব্যক্তির বিষয়ে কঠোর সতর্কতা এসেছে, যে রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর নামে কোনো হাদিস বর্ণনা করে, অথচ সে মনে করে হাদিসটি মিথ্যা। এমন ব্যক্তি দুজন মিথ্যাবাদীর একজন বলে হাদিসে এসেছে। এর মানে, শুধু নিজের মুখে বানানো নয়; সন্দেহজনক বা মিথ্যা মনে হওয়া কথা প্রচার করাও বিপজ্জনক। আজকের সময়ে মানুষ অনেক কথা দ্রুত ছড়িয়ে দেয়। কিন্তু হাদিসের ক্ষেত্রে বেশি সতর্ক হওয়া দরকার। কোনো বর্ণনা নিশ্চিত না হলে তা যাচাই করা, আলেমদের কাছে জিজ্ঞেস করা বা না বলা—এটাই নিরাপদ পথ।"},"teachings":["মিথ্যা মনে হওয়া হাদিস প্রচার করা গুরুতর ভুল।","হাদিস বর্ণনার আগে সত্যতা যাচাই জরুরি।","শুধু ফরওয়ার্ড করা বা ছড়িয়ে দেওয়াও দায়িত্বের বাইরে নয়।","দ্বীনি কথায় সন্দেহ হলে সাবধান থাকা উচিত।"],"related_hadiths":[{"id":"1","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"},{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"108","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীর নামে মিথ্যা অন্য মিথ্যার মতো নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের নামে ইচ্ছাকৃত মিথ্যা অন্য কারও নামে মিথ্যার মতো নয়—এ হাদিসে কঠোর সতর্কতা এসেছে।"},"heading":{"title":"নবীর নামে মিথ্যা: কেন এটি আরও ভয়াবহ সতর্কবার্তা","description":"এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর প্রতি মিথ্যারোপ করা অন্য কারও প্রতি মিথ্যারোপ করার মতো নয়। কারণ তিনি আল্লাহর রাসূল; তাঁর নামে বলা কথা মানুষ দ্বীনের অংশ মনে করে। তাই তাঁর নামে ইচ্ছাকৃত মিথ্যা বলা শুধু একটি সাধারণ মিথ্যা নয়, বরং মানুষের দ্বীন বোঝার ওপর ক্ষতি আনতে পারে। হাদিসে এর পরিণতি হিসেবে জাহান্নামের বাসস্থানের কথা এসেছে। এই শিক্ষা আমাদের খুব সতর্ক করে: কোনো কথা সুন্দর শোনালেই তা হাদিস নয়। যাচাই ছাড়া নবীজির নামে কথা বলা থেকে বিরত থাকা ঈমানি দায়িত্বের অংশ।"},"teachings":["রাসূলের নামে মিথ্যা বলা সাধারণ মিথ্যার মতো নয়।","ইচ্ছাকৃত মিথ্যারোপের ভয়াবহ পরিণতি হাদিসে এসেছে।","দ্বীনি কথা বলার আগে যাচাই করা জরুরি।","সুন্দর শোনালেই কোনো কথা হাদিস হয়ে যায় না।"],"related_hadiths":[{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
         </is>
       </c>
       <c r="E174" s="4" t="n"/>
@@ -4518,12 +4514,12 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>97</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | নবীর নামে মিথ্যা অন্য মিথ্যার মতো নয়","description":"$book_name$ $hadith_number$ - $chapter_name$. রাসূলের নামে ইচ্ছাকৃত মিথ্যা অন্য কারও নামে মিথ্যার মতো নয়—এ হাদিসে কঠোর সতর্কতা এসেছে।"},"heading":{"title":"নবীর নামে মিথ্যা: কেন এটি আরও ভয়াবহ সতর্কবার্তা","description":"এই হাদিসে বলা হয়েছে, রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম-এর প্রতি মিথ্যারোপ করা অন্য কারও প্রতি মিথ্যারোপ করার মতো নয়। কারণ তিনি আল্লাহর রাসূল; তাঁর নামে বলা কথা মানুষ দ্বীনের অংশ মনে করে। তাই তাঁর নামে ইচ্ছাকৃত মিথ্যা বলা শুধু একটি সাধারণ মিথ্যা নয়, বরং মানুষের দ্বীন বোঝার ওপর ক্ষতি আনতে পারে। হাদিসে এর পরিণতি হিসেবে জাহান্নামের বাসস্থানের কথা এসেছে। এই শিক্ষা আমাদের খুব সতর্ক করে: কোনো কথা সুন্দর শোনালেই তা হাদিস নয়। যাচাই ছাড়া নবীজির নামে কথা বলা থেকে বিরত থাকা ঈমানি দায়িত্বের অংশ।"},"teachings":["রাসূলের নামে মিথ্যা বলা সাধারণ মিথ্যার মতো নয়।","ইচ্ছাকৃত মিথ্যারোপের ভয়াবহ পরিণতি হাদিসে এসেছে।","দ্বীনি কথা বলার আগে যাচাই করা জরুরি।","সুন্দর শোনালেই কোনো কথা হাদিস হয়ে যায় না।"],"related_hadiths":[{"id":"106","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"107","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"1","book_id":"2","slug":"muslim","label":"সহীহ মুসলিম"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন জানার মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ওহুদের শহীদদের দাফনের সময় বেশি কুরআন জানা ব্যক্তিকে আগে রাখার মাধ্যমে কুরআনের মর্যাদা বোঝানো হয়েছে।"},"heading":{"title":"কুরআন জানার মর্যাদা: ওহুদের শহীদদের দাফনের শিক্ষা","description":"এই হাদিসে ওহুদ যুদ্ধের শহীদদের দাফনের সময়ের একটি ঘটনা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম দুজন শহীদকে একসাথে কবরে রাখার সময় জিজ্ঞেস করতেন, দুজনের মধ্যে কে বেশি কুরআন জানত। যখন একজনের দিকে ইঙ্গিত করা হতো, তাঁকে কবরে আগে রাখা হতো। এখানে কুরআন জানার মর্যাদা খুব পরিষ্কার। এমনকি দাফনের মতো অবস্থাতেও কুরআনের জ্ঞানকে সম্মানের কারণ করা হয়েছে। এই হাদিস আমাদের কুরআন শেখা, পড়া, মুখস্ত করা এবং তা জীবনে গুরুত্ব দেওয়ার দিকে উৎসাহ দেয়। তবে শিক্ষা হাদিসের সীমার মধ্যেই: বেশি কুরআন জানা সম্মানের বিষয়।"},"teachings":["কুরআন জানা ব্যক্তির সম্মান হাদিসে স্পষ্ট হয়েছে।","ওহুদের শহীদদের দাফনে কুরআনজ্ঞানকে গুরুত্ব দেওয়া হয়েছে।","কুরআন শেখা ও সংরক্ষণ করা মর্যাদাপূর্ণ কাজ।","দ্বীনি জ্ঞান মানুষের সম্মানের কারণ হতে পারে।"],"related_hadiths":[{"id":"1343","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5027","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2109","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
         </is>
       </c>
       <c r="E175" s="4" t="n"/>
@@ -4541,12 +4537,12 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | কুরআন জানার মর্যাদা","description":"$book_name$ $hadith_number$ - $chapter_name$. ওহুদের শহীদদের দাফনের সময় বেশি কুরআন জানা ব্যক্তিকে আগে রাখার মাধ্যমে কুরআনের মর্যাদা বোঝানো হয়েছে।"},"heading":{"title":"কুরআন জানার মর্যাদা: ওহুদের শহীদদের দাফনের শিক্ষা","description":"এই হাদিসে ওহুদ যুদ্ধের শহীদদের দাফনের সময়ের একটি ঘটনা এসেছে। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম দুজন শহীদকে একসাথে কবরে রাখার সময় জিজ্ঞেস করতেন, দুজনের মধ্যে কে বেশি কুরআন জানত। যখন একজনের দিকে ইঙ্গিত করা হতো, তাঁকে কবরে আগে রাখা হতো। এখানে কুরআন জানার মর্যাদা খুব পরিষ্কার। এমনকি দাফনের মতো অবস্থাতেও কুরআনের জ্ঞানকে সম্মানের কারণ করা হয়েছে। এই হাদিস আমাদের কুরআন শেখা, পড়া, মুখস্ত করা এবং তা জীবনে গুরুত্ব দেওয়ার দিকে উৎসাহ দেয়। তবে শিক্ষা হাদিসের সীমার মধ্যেই: বেশি কুরআন জানা সম্মানের বিষয়।"},"teachings":["কুরআন জানা ব্যক্তির সম্মান হাদিসে স্পষ্ট হয়েছে।","ওহুদের শহীদদের দাফনে কুরআনজ্ঞানকে গুরুত্ব দেওয়া হয়েছে।","কুরআন শেখা ও সংরক্ষণ করা মর্যাদাপূর্ণ কাজ।","দ্বীনি জ্ঞান মানুষের সম্মানের কারণ হতে পারে।"],"related_hadiths":[{"id":"1343","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"5027","book_id":"1","slug":"bukhari","label":"সহীহ বুখারী"},{"id":"2109","book_id":"14","slug":"mishkatul-masabih","label":"মিশকাতুল মাসাবীহ"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃদ্ধ, কুরআনধারী ও ন্যায়পরায়ণ শাসকের সম্মান","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহকে মর্যাদা দেওয়ার অংশ হিসেবে বৃদ্ধ মুসলিম, ভারসাম্যপূর্ণ কুরআনধারী ও ন্যায়পরায়ণ শাসককে সম্মানের কথা এসেছে।"},"heading":{"title":"সম্মানের শিক্ষা: বৃদ্ধ মুসলিম, কুরআনধারী ও ন্যায়পরায়ণ শাসক","description":"এই হাদিসে তিন শ্রেণির মানুষকে সম্মান করার কথা বলা হয়েছে, এবং এটিকে আল্লাহকে মর্যাদা দেওয়ার অন্তর্ভুক্ত বলা হয়েছে। প্রথমত বৃদ্ধ মুসলিম ব্যক্তি, দ্বিতীয়ত কুরআন ধারণকারী—যিনি কুরআন নিয়ে অতিরঞ্জন করেন না এবং এর সঙ্গে রূঢ় আচরণও করেন না, তৃতীয়ত ন্যায়পরায়ণ শাসক। এখানে সম্মান মানে অন্ধ অনুসরণ নয়; বরং হাদিসের ভাষ্য অনুযায়ী মর্যাদা দেওয়া, ভালো আচরণ করা এবং যথাযথ সম্মান বজায় রাখা। কুরআনধারীর ক্ষেত্রে ভারসাম্যের কথা বিশেষভাবে এসেছে। তাই কুরআনের প্রতি ভালোবাসা যেন অতিরঞ্জন বা অবহেলা—কোনোটাতেই না যায়। এই হাদিস সামাজিক আদব শেখায়।"},"teachings":["বৃদ্ধ মুসলিম ব্যক্তিকে সম্মান করা আল্লাহকে মর্যাদা দেওয়ার অংশ হিসেবে এসেছে।","কুরআনধারীর সম্মান আছে, তবে ভারসাম্য জরুরি।","ন্যায়পরায়ণ শাসককে সম্মান করার শিক্ষা দেওয়া হয়েছে।","ইসলামে সামাজিক আদব ও সম্মানের বড় গুরুত্ব আছে।"],"related_hadiths":[{"id":"4843","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"99","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"100","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
         </is>
       </c>
       <c r="E176" s="4" t="n"/>
@@ -4564,38 +4560,15 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বৃদ্ধ, কুরআনধারী ও ন্যায়পরায়ণ শাসকের সম্মান","description":"$book_name$ $hadith_number$ - $chapter_name$. আল্লাহকে মর্যাদা দেওয়ার অংশ হিসেবে বৃদ্ধ মুসলিম, ভারসাম্যপূর্ণ কুরআনধারী ও ন্যায়পরায়ণ শাসককে সম্মানের কথা এসেছে।"},"heading":{"title":"সম্মানের শিক্ষা: বৃদ্ধ মুসলিম, কুরআনধারী ও ন্যায়পরায়ণ শাসক","description":"এই হাদিসে তিন শ্রেণির মানুষকে সম্মান করার কথা বলা হয়েছে, এবং এটিকে আল্লাহকে মর্যাদা দেওয়ার অন্তর্ভুক্ত বলা হয়েছে। প্রথমত বৃদ্ধ মুসলিম ব্যক্তি, দ্বিতীয়ত কুরআন ধারণকারী—যিনি কুরআন নিয়ে অতিরঞ্জন করেন না এবং এর সঙ্গে রূঢ় আচরণও করেন না, তৃতীয়ত ন্যায়পরায়ণ শাসক। এখানে সম্মান মানে অন্ধ অনুসরণ নয়; বরং হাদিসের ভাষ্য অনুযায়ী মর্যাদা দেওয়া, ভালো আচরণ করা এবং যথাযথ সম্মান বজায় রাখা। কুরআনধারীর ক্ষেত্রে ভারসাম্যের কথা বিশেষভাবে এসেছে। তাই কুরআনের প্রতি ভালোবাসা যেন অতিরঞ্জন বা অবহেলা—কোনোটাতেই না যায়। এই হাদিস সামাজিক আদব শেখায়।"},"teachings":["বৃদ্ধ মুসলিম ব্যক্তিকে সম্মান করা আল্লাহকে মর্যাদা দেওয়ার অংশ হিসেবে এসেছে।","কুরআনধারীর সম্মান আছে, তবে ভারসাম্য জরুরি।","ন্যায়পরায়ণ শাসককে সম্মান করার শিক্ষা দেওয়া হয়েছে।","ইসলামে সামাজিক আদব ও সম্মানের বড় গুরুত্ব আছে।"],"related_hadiths":[{"id":"4843","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"},{"id":"99","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"100","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"}]}</t>
+          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বয়স্কদের সঙ্গে বরকত","description":"$book_name$ $hadith_number$ - $chapter_name$. তোমাদের বয়স্কদের সঙ্গে বরকত রয়েছে—এই সংক্ষিপ্ত হাদিস বড়দের সম্মানের সুন্দর শিক্ষা দেয়।"},"heading":{"title":"বয়স্কদের সঙ্গে বরকত: বড়দের সম্মান করার হাদিস","description":"এই হাদিস খুব ছোট, কিন্তু এর শিক্ষা গভীর। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, তোমাদের বয়স্ক ব্যক্তিদের সঙ্গে বরকত রয়েছে। এখানে বয়স্কদের মর্যাদা, অভিজ্ঞতা এবং তাদের প্রতি সম্মান রাখার শিক্ষা আছে। বড়দের সঙ্গে ভালো আচরণ, তাদের কথা মনোযোগ দিয়ে শোনা, তাদের কষ্ট না দেওয়া এবং তাদের হক বোঝা—এসব আদবের মধ্যে পড়ে। হাদিসে নির্দিষ্টভাবে ‘বরকত’ শব্দ এসেছে, তাই আমরা এর চেয়ে বাড়তি দাবি না করে বলি: বয়স্কদের উপস্থিতি ও সঙ্গ মুসলিম সমাজে কল্যাণের কারণ হতে পারে। এই শিক্ষা পরিবার, মসজিদ, সমাজ—সব জায়গায় দরকার।"},"teachings":["বয়স্কদের সঙ্গে বরকতের কথা হাদিসে এসেছে।","বড়দের সম্মান করা ইসলামী আদবের অংশ।","পরিবার ও সমাজে বয়স্কদের মর্যাদা রাখা দরকার।","বড়দের সঙ্গে ভালো আচরণ কল্যাণের পথ হতে পারে।"],"related_hadiths":[{"id":"98","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"100","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"4843","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
         </is>
       </c>
       <c r="E177" s="4" t="n"/>
-    </row>
-    <row r="178" ht="46" customHeight="1">
-      <c r="A178" s="4" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B178" s="4" t="inlineStr">
-        <is>
-          <t>bn</t>
-        </is>
-      </c>
-      <c r="C178" s="4" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
-      </c>
-      <c r="D178" s="4" t="inlineStr">
-        <is>
-          <t>{"meta":{"title":"$book_name$ - $hadith_number$ ($publication$) | বয়স্কদের সঙ্গে বরকত","description":"$book_name$ $hadith_number$ - $chapter_name$. তোমাদের বয়স্কদের সঙ্গে বরকত রয়েছে—এই সংক্ষিপ্ত হাদিস বড়দের সম্মানের সুন্দর শিক্ষা দেয়।"},"heading":{"title":"বয়স্কদের সঙ্গে বরকত: বড়দের সম্মান করার হাদিস","description":"এই হাদিস খুব ছোট, কিন্তু এর শিক্ষা গভীর। রাসূলুল্লাহ সাল্লাল্লাহু আলাইহি ওয়াসাল্লাম বলেছেন, তোমাদের বয়স্ক ব্যক্তিদের সঙ্গে বরকত রয়েছে। এখানে বয়স্কদের মর্যাদা, অভিজ্ঞতা এবং তাদের প্রতি সম্মান রাখার শিক্ষা আছে। বড়দের সঙ্গে ভালো আচরণ, তাদের কথা মনোযোগ দিয়ে শোনা, তাদের কষ্ট না দেওয়া এবং তাদের হক বোঝা—এসব আদবের মধ্যে পড়ে। হাদিসে নির্দিষ্টভাবে ‘বরকত’ শব্দ এসেছে, তাই আমরা এর চেয়ে বাড়তি দাবি না করে বলি: বয়স্কদের উপস্থিতি ও সঙ্গ মুসলিম সমাজে কল্যাণের কারণ হতে পারে। এই শিক্ষা পরিবার, মসজিদ, সমাজ—সব জায়গায় দরকার।"},"teachings":["বয়স্কদের সঙ্গে বরকতের কথা হাদিসে এসেছে।","বড়দের সম্মান করা ইসলামী আদবের অংশ।","পরিবার ও সমাজে বয়স্কদের মর্যাদা রাখা দরকার।","বড়দের সঙ্গে ভালো আচরণ কল্যাণের পথ হতে পারে।"],"related_hadiths":[{"id":"98","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"100","book_id":"22","slug":"targib-wattahrib","label":"তারগিব ওয়াত তাহরিব"},{"id":"4843","book_id":"4","slug":"dawud","label":"সুনান আবু দাউদ"}]}</t>
-        </is>
-      </c>
-      <c r="E178" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>